<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-18T06:46:25.867Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34724,12 +34724,14 @@
         <v>18.0</v>
       </c>
       <c r="C11" s="36">
-        <v>15.0</v>
+        <v>20.0</v>
       </c>
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="24"/>
+      <c r="E11" s="25">
+        <v>46099.61556196759</v>
+      </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-18T06:46:29.765Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34699,13 +34699,13 @@
         <v>4.0</v>
       </c>
       <c r="C10" s="36">
-        <v>15.0</v>
+        <v>20.0</v>
       </c>
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
       <c r="E10" s="25">
-        <v>46009.0</v>
+        <v>46099.615610243054</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-18T07:07:20.404Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34639,7 +34639,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="8">
-        <v>20.0</v>
+        <v>10.0</v>
       </c>
       <c r="C7" s="8">
         <v>20.0</v>
@@ -34648,7 +34648,7 @@
         <v>1.0</v>
       </c>
       <c r="E7" s="25">
-        <v>45946.879225324075</v>
+        <v>46099.630087812504</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-19T12:03:49.709Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -1214,11 +1214,11 @@
         <v>2.0</v>
       </c>
       <c r="C28" s="8">
-        <v>300.0</v>
+        <v>100.0</v>
       </c>
       <c r="D28" s="17"/>
       <c r="E28" s="23">
-        <v>46051.96181112269</v>
+        <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-19T12:03:55.860Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -1238,11 +1238,11 @@
         <v>20.0</v>
       </c>
       <c r="C29" s="8">
-        <v>300.0</v>
+        <v>100.0</v>
       </c>
       <c r="D29" s="17"/>
       <c r="E29" s="23">
-        <v>46051.96188216435</v>
+        <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-25T09:34:15.957Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -699,7 +699,9 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="9">
+        <v>46106.732072326384</v>
+      </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-03-25T09:34:37.732Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34619,13 +34619,13 @@
         <v>10.0</v>
       </c>
       <c r="C6" s="8">
-        <v>100.0</v>
+        <v>45.0</v>
       </c>
       <c r="D6" s="8">
         <v>1.0</v>
       </c>
       <c r="E6" s="25">
-        <v>45946.87939769676</v>
+        <v>46106.73232292824</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -34641,7 +34641,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="8">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
       <c r="C7" s="8">
         <v>20.0</v>
@@ -34650,7 +34650,7 @@
         <v>1.0</v>
       </c>
       <c r="E7" s="25">
-        <v>46099.630087812504</v>
+        <v>46106.732369062505</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-04T08:18:37.228Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34599,7 +34599,9 @@
       <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="9">
+        <v>46116.65051717593</v>
+      </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -34680,13 +34682,13 @@
         <v>25.0</v>
       </c>
       <c r="C8" s="11">
-        <v>5.0</v>
+        <v>10.0</v>
       </c>
       <c r="D8" s="11">
         <v>1.0</v>
       </c>
       <c r="E8" s="14">
-        <v>45954.915123425926</v>
+        <v>46116.67957466435</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-04T08:26:51.389Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34679,7 +34679,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="11">
-        <v>25.0</v>
+        <v>20.0</v>
       </c>
       <c r="C8" s="11">
         <v>10.0</v>
@@ -34688,7 +34688,7 @@
         <v>1.0</v>
       </c>
       <c r="E8" s="14">
-        <v>46116.67957466435</v>
+        <v>46116.685309016204</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-05T13:37:13.834Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51208,13 +51208,13 @@
         <v>24</v>
       </c>
       <c r="C14" s="39">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="D14" s="39">
         <v>1.0</v>
       </c>
       <c r="E14" s="26">
-        <v>46006.93993954861</v>
+        <v>46117.900830185186</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-06T13:00:31.323Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51123,7 +51123,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="36">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="C10" s="36">
         <v>20.0</v>
@@ -51132,7 +51132,7 @@
         <v>1.0</v>
       </c>
       <c r="E10" s="25">
-        <v>46099.615610243054</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-23T16:18:12.047Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>刻線</t>
+  </si>
+  <si>
+    <t>柔光紙</t>
   </si>
 </sst>
 </file>
@@ -51862,7 +51865,9 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="35"/>
+      <c r="A45" s="34" t="s">
+        <v>37</v>
+      </c>
       <c r="B45" s="35"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-23T16:18:24.362Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="37">
   <si>
     <t>項目</t>
   </si>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>刻線</t>
-  </si>
-  <si>
-    <t>柔光紙</t>
   </si>
 </sst>
 </file>
@@ -51865,9 +51862,7 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="34" t="s">
-        <v>37</v>
-      </c>
+      <c r="A45" s="34"/>
       <c r="B45" s="35"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-04-23T16:18:30.132Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51610,14 +51610,14 @@
         <v>33</v>
       </c>
       <c r="B33" s="34">
-        <v>3.0</v>
+        <v>15.0</v>
       </c>
       <c r="C33" s="15">
-        <v>80.0</v>
+        <v>16.0</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="44">
-        <v>46042.92027434028</v>
+        <v>46136.0128342824</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:23:42.665Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34600,7 +34600,7 @@
         <v>1.0</v>
       </c>
       <c r="E4" s="9">
-        <v>46116.65051717593</v>
+        <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -51086,7 +51086,7 @@
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
-    <row r="8">
+    <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="5"/>
       <c r="B8" s="37"/>
       <c r="C8" s="37"/>
@@ -51102,13 +51102,11 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="24"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="38"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51119,21 +51117,13 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>6</v>
+      <c r="A10" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B10" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C10" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D10" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E10" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="24"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51145,10 +51135,10 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C11" s="36">
         <v>20.0</v>
@@ -51157,7 +51147,7 @@
         <v>1.0</v>
       </c>
       <c r="E11" s="25">
-        <v>46099.61556196759</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -51169,11 +51159,21 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="24"/>
+      <c r="A12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C12" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D12" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E12" s="25">
+        <v>46099.61556196759</v>
+      </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51184,13 +51184,11 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="27"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51201,21 +51199,13 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="s">
-        <v>6</v>
+      <c r="A14" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B14" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D14" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E14" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51227,10 +51217,10 @@
     </row>
     <row r="15">
       <c r="A15" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B15" s="39">
-        <v>30.0</v>
+      <c r="B15" s="39" t="s">
+        <v>24</v>
       </c>
       <c r="C15" s="39">
         <v>15.0</v>
@@ -51238,7 +51228,9 @@
       <c r="D15" s="39">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51249,11 +51241,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="16"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="24"/>
+      <c r="A16" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C16" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D16" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E16" s="27"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51264,9 +51264,7 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A17" s="16"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -51281,21 +51279,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B18" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C18" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D18" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51307,10 +51297,10 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C19" s="8">
         <v>20.0</v>
@@ -51319,7 +51309,7 @@
         <v>1.0</v>
       </c>
       <c r="E19" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51332,23 +51322,21 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B20" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C20" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F20" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -51358,14 +51346,24 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="40" t="s">
-        <v>26</v>
+      <c r="A21" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="4"/>
+      <c r="B21" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C21" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D21" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E21" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -51375,21 +51373,13 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>27</v>
+      <c r="A22" s="40" t="s">
+        <v>26</v>
       </c>
-      <c r="B22" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C22" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D22" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E22" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51401,19 +51391,19 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B23" s="36">
         <v>2.0</v>
       </c>
       <c r="C23" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D23" s="36">
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -51426,19 +51416,19 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B24" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C24" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D24" s="36">
         <v>1.0</v>
       </c>
       <c r="E24" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -51450,11 +51440,21 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="24"/>
+      <c r="A25" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C25" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D25" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51465,17 +51465,11 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>29</v>
-      </c>
+      <c r="A26" s="7"/>
+      <c r="B26" s="8"/>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
-      <c r="E26" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E26" s="24"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51486,16 +51480,16 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7">
-        <v>50.0</v>
+      <c r="A27" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="B27" s="8">
-        <v>100.0</v>
+      <c r="B27" s="8" t="s">
+        <v>29</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
       <c r="E27" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51507,13 +51501,17 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="41" t="s">
-        <v>30</v>
+      <c r="A28" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="43"/>
+      <c r="B28" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51524,21 +51522,13 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="34" t="s">
-        <v>31</v>
+      <c r="A29" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="B29" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C29" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D29" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E29" s="44">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="43"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51549,11 +51539,21 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="35"/>
-      <c r="B30" s="35"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="A30" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C30" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D30" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E30" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51564,9 +51564,7 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="34" t="s">
-        <v>32</v>
-      </c>
+      <c r="A31" s="35"/>
       <c r="B31" s="35"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -51581,21 +51579,13 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>7</v>
+      <c r="A32" s="34" t="s">
+        <v>32</v>
       </c>
-      <c r="B32" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C32" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D32" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E32" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B32" s="35"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51606,18 +51596,20 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="34" t="s">
-        <v>33</v>
+      <c r="A33" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B33" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C33" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D33" s="4"/>
+      <c r="D33" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E33" s="44">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51629,11 +51621,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="35"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="4"/>
+      <c r="A34" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C34" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="E34" s="44">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51644,17 +51644,11 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A35" s="35"/>
+      <c r="B35" s="35"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="44">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51666,19 +51660,15 @@
     </row>
     <row r="36">
       <c r="A36" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B36" s="34">
-        <v>5.0</v>
+      <c r="B36" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C36" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D36" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
       <c r="E36" s="44">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -51691,19 +51681,19 @@
     </row>
     <row r="37">
       <c r="A37" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C37" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D37" s="15">
         <v>1.0</v>
       </c>
       <c r="E37" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51716,10 +51706,10 @@
     </row>
     <row r="38">
       <c r="A38" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B38" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C38" s="15">
         <v>10.0</v>
@@ -51728,7 +51718,7 @@
         <v>1.0</v>
       </c>
       <c r="E38" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51740,11 +51730,21 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="35"/>
-      <c r="B39" s="35"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="A39" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C39" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D39" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E39" s="44">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51755,17 +51755,11 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40" s="34" t="s">
-        <v>26</v>
-      </c>
+      <c r="A40" s="35"/>
+      <c r="B40" s="35"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="44">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51777,18 +51771,16 @@
     </row>
     <row r="41">
       <c r="A41" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B41" s="34">
-        <v>5.0</v>
+      <c r="B41" s="34" t="s">
+        <v>26</v>
       </c>
-      <c r="C41" s="15">
-        <v>80.0</v>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D41" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51800,13 +51792,13 @@
     </row>
     <row r="42">
       <c r="A42" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B42" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C42" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D42" s="15">
         <v>1.0</v>
@@ -51823,20 +51815,18 @@
     </row>
     <row r="43">
       <c r="A43" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B43" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C43" s="15">
         <v>10.0</v>
       </c>
       <c r="D43" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E43" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51847,11 +51837,21 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="35"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="A44" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C44" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D44" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E44" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51862,7 +51862,7 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="34"/>
+      <c r="A45" s="35"/>
       <c r="B45" s="35"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -51877,7 +51877,7 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="35"/>
+      <c r="A46" s="34"/>
       <c r="B46" s="35"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -51892,8 +51892,8 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4"/>
+      <c r="A47" s="35"/>
+      <c r="B47" s="35"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
@@ -65961,6 +65961,21 @@
       <c r="L984" s="4"/>
       <c r="M984" s="4"/>
     </row>
+    <row r="985">
+      <c r="A985" s="4"/>
+      <c r="B985" s="4"/>
+      <c r="C985" s="4"/>
+      <c r="D985" s="4"/>
+      <c r="E985" s="4"/>
+      <c r="F985" s="4"/>
+      <c r="G985" s="4"/>
+      <c r="H985" s="4"/>
+      <c r="I985" s="4"/>
+      <c r="J985" s="4"/>
+      <c r="K985" s="4"/>
+      <c r="L985" s="4"/>
+      <c r="M985" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:23:45.982Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51101,7 +51101,7 @@
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
     </row>
-    <row r="9">
+    <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="5"/>
       <c r="B9" s="37"/>
       <c r="C9" s="37"/>
@@ -51116,14 +51116,12 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="24"/>
+    <row r="10" ht="16.5" customHeight="1">
+      <c r="A10" s="5"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="38"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51134,21 +51132,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C11" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E11" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="A11" s="5"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="38"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51159,21 +51147,13 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>7</v>
+      <c r="A12" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="36">
-        <v>18.0</v>
-      </c>
-      <c r="C12" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D12" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E12" s="25">
-        <v>46099.61556196759</v>
-      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="24"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51184,11 +51164,21 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="24"/>
+      <c r="A13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="C13" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D13" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E13" s="25">
+        <v>46118.87534236111</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51199,13 +51189,21 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="s">
-        <v>10</v>
+      <c r="A14" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="27"/>
+      <c r="B14" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C14" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E14" s="25">
+        <v>46099.61556196759</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51216,21 +51214,11 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D15" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="A15" s="7"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51241,18 +51229,12 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>7</v>
+      <c r="A16" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B16" s="39">
-        <v>30.0</v>
-      </c>
-      <c r="C16" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D16" s="39">
-        <v>1.0</v>
-      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
       <c r="E16" s="27"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -51264,11 +51246,21 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="16"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D17" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E17" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51279,13 +51271,19 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>11</v>
+      <c r="A18" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C18" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D18" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E18" s="27"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51296,21 +51294,11 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C19" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D19" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E19" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="24"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51321,21 +51309,13 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
+      <c r="A20" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B20" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C20" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D20" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E20" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="24"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51350,20 +51330,18 @@
         <v>6</v>
       </c>
       <c r="B21" s="8">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C21" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D21" s="8">
         <v>1.0</v>
       </c>
       <c r="E21" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95620635417</v>
       </c>
-      <c r="F21" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -51373,13 +51351,21 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="s">
-        <v>26</v>
+      <c r="A22" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="8">
+        <v>55.0</v>
+      </c>
+      <c r="C22" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D22" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E22" s="25">
+        <v>46006.95627618056</v>
+      </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51391,21 +51377,23 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
-      <c r="B23" s="36">
-        <v>2.0</v>
+      <c r="B23" s="8">
+        <v>10.0</v>
       </c>
-      <c r="C23" s="36">
-        <v>100.0</v>
+      <c r="C23" s="8">
+        <v>250.0</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="8">
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>45900.48749</v>
+        <v>46038.439073761576</v>
       </c>
-      <c r="F23" s="4"/>
+      <c r="F23" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -51415,21 +51403,13 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>6</v>
+      <c r="A24" s="40" t="s">
+        <v>26</v>
       </c>
-      <c r="B24" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C24" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D24" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E24" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="24"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51441,19 +51421,19 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B25" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C25" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D25" s="36">
         <v>1.0</v>
       </c>
       <c r="E25" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -51465,11 +51445,21 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="24"/>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C26" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D26" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E26" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51481,15 +51471,19 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>29</v>
+      <c r="B27" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
+      <c r="C27" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D27" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E27" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51501,17 +51495,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B28" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A28" s="7"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="24"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51522,13 +51510,17 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="41" t="s">
-        <v>30</v>
+      <c r="A29" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="43"/>
+      <c r="B29" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51539,20 +51531,16 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="34" t="s">
-        <v>31</v>
+      <c r="A30" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B30" s="34">
+      <c r="B30" s="8">
         <v>100.0</v>
       </c>
-      <c r="C30" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D30" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E30" s="44">
-        <v>46009.783484375</v>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -51564,11 +51552,13 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="35"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="A31" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="42"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="43"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51580,12 +51570,20 @@
     </row>
     <row r="32">
       <c r="A32" s="34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="B32" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C32" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D32" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E32" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51596,21 +51594,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B33" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C33" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D33" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E33" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A33" s="35"/>
+      <c r="B33" s="35"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51622,18 +51610,12 @@
     </row>
     <row r="34">
       <c r="A34" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
-      <c r="B34" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C34" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B34" s="35"/>
+      <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="44">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51644,11 +51626,21 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="35"/>
-      <c r="B35" s="35"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="A35" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C35" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D35" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E35" s="44">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51660,15 +51652,17 @@
     </row>
     <row r="36">
       <c r="A36" s="34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
-      <c r="B36" s="34" t="s">
-        <v>12</v>
+      <c r="B36" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D36" s="4"/>
       <c r="E36" s="44">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -51680,21 +51674,11 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C37" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D37" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E37" s="44">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A37" s="35"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51706,19 +51690,15 @@
     </row>
     <row r="38">
       <c r="A38" s="34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
-      <c r="B38" s="34">
-        <v>15.0</v>
+      <c r="B38" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C38" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D38" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
       <c r="E38" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51731,19 +51711,19 @@
     </row>
     <row r="39">
       <c r="A39" s="34" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B39" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C39" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D39" s="15">
         <v>1.0</v>
       </c>
       <c r="E39" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51755,11 +51735,21 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="35"/>
-      <c r="B40" s="35"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="A40" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C40" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D40" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E40" s="44">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51771,15 +51761,19 @@
     </row>
     <row r="41">
       <c r="A41" s="34" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
-      <c r="B41" s="34" t="s">
-        <v>26</v>
+      <c r="B41" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
+      <c r="C41" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D41" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E41" s="44">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51791,18 +51785,10 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B42" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C42" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D42" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A42" s="35"/>
+      <c r="B42" s="35"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -51815,18 +51801,16 @@
     </row>
     <row r="43">
       <c r="A43" s="34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
-      <c r="B43" s="34">
-        <v>15.0</v>
+      <c r="B43" s="34" t="s">
+        <v>26</v>
       </c>
-      <c r="C43" s="15">
-        <v>10.0</v>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D43" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51838,20 +51822,18 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B44" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C44" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D44" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E44" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51862,10 +51844,18 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="35"/>
-      <c r="B45" s="35"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
+      <c r="A45" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C45" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D45" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51877,11 +51867,21 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="34"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="A46" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C46" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D46" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E46" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51907,8 +51907,8 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="34"/>
+      <c r="B48" s="35"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
@@ -51922,8 +51922,8 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
+      <c r="A49" s="35"/>
+      <c r="B49" s="35"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
@@ -65976,6 +65976,36 @@
       <c r="L985" s="4"/>
       <c r="M985" s="4"/>
     </row>
+    <row r="986">
+      <c r="A986" s="4"/>
+      <c r="B986" s="4"/>
+      <c r="C986" s="4"/>
+      <c r="D986" s="4"/>
+      <c r="E986" s="4"/>
+      <c r="F986" s="4"/>
+      <c r="G986" s="4"/>
+      <c r="H986" s="4"/>
+      <c r="I986" s="4"/>
+      <c r="J986" s="4"/>
+      <c r="K986" s="4"/>
+      <c r="L986" s="4"/>
+      <c r="M986" s="4"/>
+    </row>
+    <row r="987">
+      <c r="A987" s="4"/>
+      <c r="B987" s="4"/>
+      <c r="C987" s="4"/>
+      <c r="D987" s="4"/>
+      <c r="E987" s="4"/>
+      <c r="F987" s="4"/>
+      <c r="G987" s="4"/>
+      <c r="H987" s="4"/>
+      <c r="I987" s="4"/>
+      <c r="J987" s="4"/>
+      <c r="K987" s="4"/>
+      <c r="L987" s="4"/>
+      <c r="M987" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:23:49.329Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51131,7 +51131,7 @@
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
-    <row r="11">
+    <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
       <c r="B11" s="37"/>
       <c r="C11" s="37"/>
@@ -51147,13 +51147,11 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="24"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="38"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51164,21 +51162,13 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>6</v>
+      <c r="A13" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C13" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D13" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E13" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51190,10 +51180,10 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C14" s="36">
         <v>20.0</v>
@@ -51202,7 +51192,7 @@
         <v>1.0</v>
       </c>
       <c r="E14" s="25">
-        <v>46099.61556196759</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -51214,11 +51204,21 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="24"/>
+      <c r="A15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C15" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D15" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E15" s="25">
+        <v>46099.61556196759</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51229,13 +51229,11 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="27"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="24"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51246,21 +51244,13 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>6</v>
+      <c r="A17" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B17" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D17" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E17" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="27"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51272,10 +51262,10 @@
     </row>
     <row r="18">
       <c r="A18" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B18" s="39">
-        <v>30.0</v>
+      <c r="B18" s="39" t="s">
+        <v>24</v>
       </c>
       <c r="C18" s="39">
         <v>15.0</v>
@@ -51283,7 +51273,9 @@
       <c r="D18" s="39">
         <v>1.0</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51294,11 +51286,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="24"/>
+      <c r="A19" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C19" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D19" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E19" s="27"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51309,9 +51309,7 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -51326,21 +51324,13 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>6</v>
+      <c r="A21" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B21" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C21" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D21" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E21" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51352,10 +51342,10 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C22" s="8">
         <v>20.0</v>
@@ -51364,7 +51354,7 @@
         <v>1.0</v>
       </c>
       <c r="E22" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51377,23 +51367,21 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B23" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C23" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D23" s="8">
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F23" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -51403,14 +51391,24 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="40" t="s">
-        <v>26</v>
+      <c r="A24" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="4"/>
+      <c r="B24" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C24" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D24" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -51420,21 +51418,13 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>27</v>
+      <c r="A25" s="40" t="s">
+        <v>26</v>
       </c>
-      <c r="B25" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C25" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D25" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E25" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51446,19 +51436,19 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B26" s="36">
         <v>2.0</v>
       </c>
       <c r="C26" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D26" s="36">
         <v>1.0</v>
       </c>
       <c r="E26" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -51471,19 +51461,19 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C27" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D27" s="36">
         <v>1.0</v>
       </c>
       <c r="E27" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51495,11 +51485,21 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="24"/>
+      <c r="A28" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C28" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D28" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51510,17 +51510,11 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>29</v>
-      </c>
+      <c r="A29" s="7"/>
+      <c r="B29" s="8"/>
       <c r="C29" s="8"/>
       <c r="D29" s="8"/>
-      <c r="E29" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51531,16 +51525,16 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7">
-        <v>50.0</v>
+      <c r="A30" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="B30" s="8">
-        <v>100.0</v>
+      <c r="B30" s="8" t="s">
+        <v>29</v>
       </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
       <c r="E30" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -51552,13 +51546,17 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="41" t="s">
-        <v>30</v>
+      <c r="A31" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B31" s="42"/>
-      <c r="C31" s="42"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="43"/>
+      <c r="B31" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51569,21 +51567,13 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="34" t="s">
-        <v>31</v>
+      <c r="A32" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="B32" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C32" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D32" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E32" s="44">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="42"/>
+      <c r="E32" s="43"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51594,11 +51584,21 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="35"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="A33" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C33" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D33" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E33" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51609,9 +51609,7 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="34" t="s">
-        <v>32</v>
-      </c>
+      <c r="A34" s="35"/>
       <c r="B34" s="35"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -51626,21 +51624,13 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="s">
-        <v>7</v>
+      <c r="A35" s="34" t="s">
+        <v>32</v>
       </c>
-      <c r="B35" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C35" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D35" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E35" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B35" s="35"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51651,18 +51641,20 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="34" t="s">
-        <v>33</v>
+      <c r="A36" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B36" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C36" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D36" s="4"/>
+      <c r="D36" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E36" s="44">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -51674,11 +51666,19 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="35"/>
-      <c r="B37" s="35"/>
-      <c r="C37" s="4"/>
+      <c r="A37" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C37" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="44">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51689,17 +51689,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A38" s="35"/>
+      <c r="B38" s="35"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="44">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51711,19 +51705,15 @@
     </row>
     <row r="39">
       <c r="A39" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B39" s="34">
-        <v>5.0</v>
+      <c r="B39" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C39" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D39" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
       <c r="E39" s="44">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51736,19 +51726,19 @@
     </row>
     <row r="40">
       <c r="A40" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B40" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C40" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D40" s="15">
         <v>1.0</v>
       </c>
       <c r="E40" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51761,10 +51751,10 @@
     </row>
     <row r="41">
       <c r="A41" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B41" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C41" s="15">
         <v>10.0</v>
@@ -51773,7 +51763,7 @@
         <v>1.0</v>
       </c>
       <c r="E41" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51785,11 +51775,21 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="35"/>
-      <c r="B42" s="35"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="A42" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C42" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D42" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E42" s="44">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51800,17 +51800,11 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B43" s="34" t="s">
-        <v>26</v>
-      </c>
+      <c r="A43" s="35"/>
+      <c r="B43" s="35"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="44">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51822,18 +51816,16 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B44" s="34">
-        <v>5.0</v>
+      <c r="B44" s="34" t="s">
+        <v>26</v>
       </c>
-      <c r="C44" s="15">
-        <v>80.0</v>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D44" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51845,13 +51837,13 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B45" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C45" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D45" s="15">
         <v>1.0</v>
@@ -51868,20 +51860,18 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B46" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C46" s="15">
         <v>10.0</v>
       </c>
       <c r="D46" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E46" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51892,11 +51882,21 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="35"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="A47" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C47" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D47" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E47" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51907,7 +51907,7 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="34"/>
+      <c r="A48" s="35"/>
       <c r="B48" s="35"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
@@ -51922,7 +51922,7 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="35"/>
+      <c r="A49" s="34"/>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -51937,8 +51937,8 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="35"/>
+      <c r="B50" s="35"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
@@ -66006,6 +66006,21 @@
       <c r="L987" s="4"/>
       <c r="M987" s="4"/>
     </row>
+    <row r="988">
+      <c r="A988" s="4"/>
+      <c r="B988" s="4"/>
+      <c r="C988" s="4"/>
+      <c r="D988" s="4"/>
+      <c r="E988" s="4"/>
+      <c r="F988" s="4"/>
+      <c r="G988" s="4"/>
+      <c r="H988" s="4"/>
+      <c r="I988" s="4"/>
+      <c r="J988" s="4"/>
+      <c r="K988" s="4"/>
+      <c r="L988" s="4"/>
+      <c r="M988" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:23:53.532Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>PS</t>
   </si>
   <si>
     <t>６</t>
@@ -51101,12 +51104,16 @@
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
     </row>
-    <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="5"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38"/>
+    <row r="9">
+      <c r="A9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="24"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51116,12 +51123,22 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
+    <row r="10">
+      <c r="A10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C10" s="8">
+        <v>45.0</v>
+      </c>
+      <c r="D10" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E10" s="25">
+        <v>46106.73232292824</v>
+      </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51131,12 +51148,22 @@
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
-    <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+    <row r="11">
+      <c r="A11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="8">
+        <v>11.0</v>
+      </c>
+      <c r="C11" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D11" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E11" s="25">
+        <v>46106.732369062505</v>
+      </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51265,7 +51292,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="39">
         <v>15.0</v>
@@ -51407,7 +51434,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51419,7 +51446,7 @@
     </row>
     <row r="25">
       <c r="A25" s="40" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -51436,7 +51463,7 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B26" s="36">
         <v>2.0</v>
@@ -51526,10 +51553,10 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -51568,7 +51595,7 @@
     </row>
     <row r="32">
       <c r="A32" s="41" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" s="42"/>
       <c r="C32" s="42"/>
@@ -51585,7 +51612,7 @@
     </row>
     <row r="33">
       <c r="A33" s="34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" s="34">
         <v>100.0</v>
@@ -51625,7 +51652,7 @@
     </row>
     <row r="35">
       <c r="A35" s="34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B35" s="35"/>
       <c r="C35" s="4"/>
@@ -51667,7 +51694,7 @@
     </row>
     <row r="37">
       <c r="A37" s="34" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B37" s="34">
         <v>15.0</v>
@@ -51705,7 +51732,7 @@
     </row>
     <row r="39">
       <c r="A39" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B39" s="34" t="s">
         <v>12</v>
@@ -51726,7 +51753,7 @@
     </row>
     <row r="40">
       <c r="A40" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B40" s="34">
         <v>5.0</v>
@@ -51751,7 +51778,7 @@
     </row>
     <row r="41">
       <c r="A41" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B41" s="34">
         <v>15.0</v>
@@ -51816,10 +51843,10 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B44" s="34" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -51837,7 +51864,7 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B45" s="34">
         <v>5.0</v>
@@ -51860,7 +51887,7 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B46" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:23:57.970Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51113,7 +51113,9 @@
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
-      <c r="E9" s="24"/>
+      <c r="E9" s="25">
+        <v>46155.84992496528</v>
+      </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51128,16 +51130,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="C10" s="8">
-        <v>45.0</v>
+        <v>30.0</v>
       </c>
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
       <c r="E10" s="25">
-        <v>46106.73232292824</v>
+        <v>46155.84996290509</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:09.279Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51155,16 +51155,16 @@
         <v>16</v>
       </c>
       <c r="B11" s="8">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="C11" s="8">
-        <v>20.0</v>
+        <v>11.0</v>
       </c>
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
       <c r="E11" s="25">
-        <v>46106.732369062505</v>
+        <v>46155.850098194445</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:13.615Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51155,16 +51155,16 @@
         <v>16</v>
       </c>
       <c r="B11" s="8">
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="C11" s="8">
-        <v>11.0</v>
+        <v>20.0</v>
       </c>
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
       <c r="E11" s="25">
-        <v>46155.85010083333</v>
+        <v>46155.85013017361</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:27.177Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51164,7 +51164,7 @@
         <v>1.0</v>
       </c>
       <c r="E11" s="25">
-        <v>46155.85013017361</v>
+        <v>46155.85015881945</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -51273,13 +51273,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="27"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51290,21 +51288,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="s">
-        <v>6</v>
+      <c r="A18" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B18" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D18" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="27"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51316,10 +51306,10 @@
     </row>
     <row r="19">
       <c r="A19" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B19" s="39">
-        <v>30.0</v>
+      <c r="B19" s="39" t="s">
+        <v>25</v>
       </c>
       <c r="C19" s="39">
         <v>15.0</v>
@@ -51327,7 +51317,9 @@
       <c r="D19" s="39">
         <v>1.0</v>
       </c>
-      <c r="E19" s="27"/>
+      <c r="E19" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51338,11 +51330,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="24"/>
+      <c r="A20" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C20" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D20" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E20" s="27"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51353,9 +51353,7 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A21" s="16"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
@@ -51370,21 +51368,13 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>6</v>
+      <c r="A22" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B22" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C22" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D22" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E22" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51396,10 +51386,10 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B23" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C23" s="8">
         <v>20.0</v>
@@ -51408,7 +51398,7 @@
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -51421,23 +51411,21 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B24" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C24" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
       <c r="E24" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -51447,14 +51435,24 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="40" t="s">
-        <v>27</v>
+      <c r="A25" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="4"/>
+      <c r="B25" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C25" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D25" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -51464,21 +51462,13 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>28</v>
+      <c r="A26" s="40" t="s">
+        <v>27</v>
       </c>
-      <c r="B26" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C26" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D26" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="24"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51490,19 +51480,19 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B27" s="36">
         <v>2.0</v>
       </c>
       <c r="C27" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D27" s="36">
         <v>1.0</v>
       </c>
       <c r="E27" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51515,19 +51505,19 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B28" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C28" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D28" s="36">
         <v>1.0</v>
       </c>
       <c r="E28" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -51539,11 +51529,21 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="24"/>
+      <c r="A29" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C29" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D29" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E29" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51554,17 +51554,11 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="A30" s="7"/>
+      <c r="B30" s="8"/>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
-      <c r="E30" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51575,16 +51569,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7">
-        <v>50.0</v>
+      <c r="A31" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B31" s="8">
-        <v>100.0</v>
+      <c r="B31" s="8" t="s">
+        <v>30</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
       <c r="E31" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -51596,13 +51590,17 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="41" t="s">
-        <v>31</v>
+      <c r="A32" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="43"/>
+      <c r="B32" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51613,21 +51611,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="34" t="s">
-        <v>32</v>
+      <c r="A33" s="41" t="s">
+        <v>31</v>
       </c>
-      <c r="B33" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C33" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D33" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E33" s="44">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B33" s="42"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="43"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51638,11 +51628,21 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="35"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="A34" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C34" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D34" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E34" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51653,9 +51653,7 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="34" t="s">
-        <v>33</v>
-      </c>
+      <c r="A35" s="35"/>
       <c r="B35" s="35"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -51670,21 +51668,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="s">
-        <v>7</v>
+      <c r="A36" s="34" t="s">
+        <v>33</v>
       </c>
-      <c r="B36" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C36" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D36" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E36" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B36" s="35"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51695,18 +51685,20 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="s">
-        <v>34</v>
+      <c r="A37" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B37" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C37" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D37" s="4"/>
+      <c r="D37" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E37" s="44">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51718,11 +51710,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="35"/>
-      <c r="B38" s="35"/>
-      <c r="C38" s="4"/>
+      <c r="A38" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C38" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="E38" s="44">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51733,17 +51733,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A39" s="35"/>
+      <c r="B39" s="35"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="44">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51755,19 +51749,15 @@
     </row>
     <row r="40">
       <c r="A40" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B40" s="34">
-        <v>5.0</v>
+      <c r="B40" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C40" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D40" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
       <c r="E40" s="44">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51780,19 +51770,19 @@
     </row>
     <row r="41">
       <c r="A41" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B41" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C41" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D41" s="15">
         <v>1.0</v>
       </c>
       <c r="E41" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51805,10 +51795,10 @@
     </row>
     <row r="42">
       <c r="A42" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B42" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C42" s="15">
         <v>10.0</v>
@@ -51817,7 +51807,7 @@
         <v>1.0</v>
       </c>
       <c r="E42" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -51829,11 +51819,21 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="35"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="A43" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C43" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D43" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E43" s="44">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51844,17 +51844,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="A44" s="35"/>
+      <c r="B44" s="35"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="44">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51866,18 +51860,16 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B45" s="34">
-        <v>5.0</v>
+      <c r="B45" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C45" s="15">
-        <v>80.0</v>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D45" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51889,13 +51881,13 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B46" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C46" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D46" s="15">
         <v>1.0</v>
@@ -51912,20 +51904,18 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B47" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C47" s="15">
         <v>10.0</v>
       </c>
       <c r="D47" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E47" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51936,11 +51926,21 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="35"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="A48" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C48" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D48" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E48" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51951,7 +51951,7 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="34"/>
+      <c r="A49" s="35"/>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -51966,7 +51966,7 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="35"/>
+      <c r="A50" s="34"/>
       <c r="B50" s="35"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
@@ -51981,8 +51981,8 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="35"/>
+      <c r="B51" s="35"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
@@ -66050,6 +66050,21 @@
       <c r="L988" s="4"/>
       <c r="M988" s="4"/>
     </row>
+    <row r="989">
+      <c r="A989" s="4"/>
+      <c r="B989" s="4"/>
+      <c r="C989" s="4"/>
+      <c r="D989" s="4"/>
+      <c r="E989" s="4"/>
+      <c r="F989" s="4"/>
+      <c r="G989" s="4"/>
+      <c r="H989" s="4"/>
+      <c r="I989" s="4"/>
+      <c r="J989" s="4"/>
+      <c r="K989" s="4"/>
+      <c r="L989" s="4"/>
+      <c r="M989" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:30.658Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51288,13 +51288,11 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="27"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51305,21 +51303,11 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D19" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E19" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="A19" s="7"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="24"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51330,18 +51318,12 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="s">
-        <v>7</v>
+      <c r="A20" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B20" s="39">
-        <v>30.0</v>
-      </c>
-      <c r="C20" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D20" s="39">
-        <v>1.0</v>
-      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
       <c r="E20" s="27"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -51353,11 +51335,21 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="16"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="24"/>
+      <c r="A21" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D21" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E21" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51368,13 +51360,19 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
-        <v>11</v>
+      <c r="A22" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C22" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D22" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51385,21 +51383,11 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C23" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D23" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E23" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="A23" s="16"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51410,21 +51398,13 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>7</v>
+      <c r="A24" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B24" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C24" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D24" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E24" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="24"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51439,20 +51419,18 @@
         <v>6</v>
       </c>
       <c r="B25" s="8">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C25" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D25" s="8">
         <v>1.0</v>
       </c>
       <c r="E25" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95620635417</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -51462,13 +51440,21 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="40" t="s">
-        <v>27</v>
+      <c r="A26" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="8">
+        <v>55.0</v>
+      </c>
+      <c r="C26" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D26" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E26" s="25">
+        <v>46006.95627618056</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51480,21 +51466,23 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
-      <c r="B27" s="36">
-        <v>2.0</v>
+      <c r="B27" s="8">
+        <v>10.0</v>
       </c>
-      <c r="C27" s="36">
-        <v>100.0</v>
+      <c r="C27" s="8">
+        <v>250.0</v>
       </c>
-      <c r="D27" s="36">
+      <c r="D27" s="8">
         <v>1.0</v>
       </c>
       <c r="E27" s="25">
-        <v>45900.48749</v>
+        <v>46038.439073761576</v>
       </c>
-      <c r="F27" s="4"/>
+      <c r="F27" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
@@ -51504,21 +51492,13 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>6</v>
+      <c r="A28" s="40" t="s">
+        <v>27</v>
       </c>
-      <c r="B28" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C28" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D28" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E28" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="24"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51530,19 +51510,19 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B29" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C29" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D29" s="36">
         <v>1.0</v>
       </c>
       <c r="E29" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -51554,11 +51534,21 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="24"/>
+      <c r="A30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C30" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D30" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E30" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51570,15 +51560,19 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>30</v>
+      <c r="B31" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
+      <c r="C31" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D31" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E31" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -51590,17 +51584,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B32" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="24"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51611,13 +51599,17 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="41" t="s">
-        <v>31</v>
+      <c r="A33" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
+      <c r="B33" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51628,20 +51620,16 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="34" t="s">
-        <v>32</v>
+      <c r="A34" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B34" s="34">
+      <c r="B34" s="8">
         <v>100.0</v>
       </c>
-      <c r="C34" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D34" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E34" s="44">
-        <v>46009.783484375</v>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -51653,11 +51641,13 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="35"/>
-      <c r="B35" s="35"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="A35" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="42"/>
+      <c r="C35" s="42"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="43"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51669,12 +51659,20 @@
     </row>
     <row r="36">
       <c r="A36" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
-      <c r="B36" s="35"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="B36" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C36" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D36" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E36" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51685,21 +51683,11 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C37" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D37" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E37" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A37" s="35"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51711,18 +51699,12 @@
     </row>
     <row r="38">
       <c r="A38" s="34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
-      <c r="B38" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C38" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B38" s="35"/>
+      <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="44">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51733,11 +51715,21 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="35"/>
-      <c r="B39" s="35"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="A39" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C39" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D39" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E39" s="44">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51749,15 +51741,17 @@
     </row>
     <row r="40">
       <c r="A40" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B40" s="34" t="s">
-        <v>12</v>
+      <c r="B40" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C40" s="4"/>
+      <c r="C40" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D40" s="4"/>
       <c r="E40" s="44">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51769,21 +51763,11 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B41" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C41" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D41" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E41" s="44">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A41" s="35"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51795,19 +51779,15 @@
     </row>
     <row r="42">
       <c r="A42" s="34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
-      <c r="B42" s="34">
-        <v>15.0</v>
+      <c r="B42" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C42" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D42" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
       <c r="E42" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -51820,19 +51800,19 @@
     </row>
     <row r="43">
       <c r="A43" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B43" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C43" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D43" s="15">
         <v>1.0</v>
       </c>
       <c r="E43" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -51844,11 +51824,21 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="35"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="A44" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C44" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D44" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E44" s="44">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51860,15 +51850,19 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
-      <c r="B45" s="34" t="s">
-        <v>27</v>
+      <c r="B45" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
+      <c r="C45" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D45" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E45" s="44">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51880,18 +51874,10 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B46" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C46" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D46" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A46" s="35"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51904,18 +51890,16 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
-      <c r="B47" s="34">
-        <v>15.0</v>
+      <c r="B47" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C47" s="15">
-        <v>10.0</v>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D47" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51927,20 +51911,18 @@
     </row>
     <row r="48">
       <c r="A48" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B48" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C48" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D48" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E48" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51951,10 +51933,18 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="35"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
+      <c r="A49" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C49" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D49" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -51966,11 +51956,21 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="34"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
+      <c r="A50" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C50" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D50" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E50" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -51996,8 +51996,8 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4"/>
+      <c r="A52" s="34"/>
+      <c r="B52" s="35"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
@@ -52011,8 +52011,8 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
@@ -66065,6 +66065,36 @@
       <c r="L989" s="4"/>
       <c r="M989" s="4"/>
     </row>
+    <row r="990">
+      <c r="A990" s="4"/>
+      <c r="B990" s="4"/>
+      <c r="C990" s="4"/>
+      <c r="D990" s="4"/>
+      <c r="E990" s="4"/>
+      <c r="F990" s="4"/>
+      <c r="G990" s="4"/>
+      <c r="H990" s="4"/>
+      <c r="I990" s="4"/>
+      <c r="J990" s="4"/>
+      <c r="K990" s="4"/>
+      <c r="L990" s="4"/>
+      <c r="M990" s="4"/>
+    </row>
+    <row r="991">
+      <c r="A991" s="4"/>
+      <c r="B991" s="4"/>
+      <c r="C991" s="4"/>
+      <c r="D991" s="4"/>
+      <c r="E991" s="4"/>
+      <c r="F991" s="4"/>
+      <c r="G991" s="4"/>
+      <c r="H991" s="4"/>
+      <c r="I991" s="4"/>
+      <c r="J991" s="4"/>
+      <c r="K991" s="4"/>
+      <c r="L991" s="4"/>
+      <c r="M991" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:34.663Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51318,13 +51318,11 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="27"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="24"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51335,21 +51333,13 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>6</v>
+      <c r="A21" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="D21" s="39">
-        <v>1.0</v>
-      </c>
-      <c r="E21" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51361,10 +51351,10 @@
     </row>
     <row r="22">
       <c r="A22" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B22" s="39">
-        <v>30.0</v>
+      <c r="B22" s="39" t="s">
+        <v>25</v>
       </c>
       <c r="C22" s="39">
         <v>15.0</v>
@@ -51372,7 +51362,9 @@
       <c r="D22" s="39">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51383,11 +51375,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="24"/>
+      <c r="A23" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C23" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="D23" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51398,9 +51398,7 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A24" s="16"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -51415,21 +51413,13 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>6</v>
+      <c r="A25" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B25" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C25" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D25" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E25" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51441,10 +51431,10 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B26" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C26" s="8">
         <v>20.0</v>
@@ -51453,7 +51443,7 @@
         <v>1.0</v>
       </c>
       <c r="E26" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -51466,23 +51456,21 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B27" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C27" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D27" s="8">
         <v>1.0</v>
       </c>
       <c r="E27" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F27" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
@@ -51492,14 +51480,24 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="40" t="s">
-        <v>27</v>
+      <c r="A28" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="4"/>
+      <c r="B28" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C28" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
@@ -51509,21 +51507,13 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>28</v>
+      <c r="A29" s="40" t="s">
+        <v>27</v>
       </c>
-      <c r="B29" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C29" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D29" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E29" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51535,19 +51525,19 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B30" s="36">
         <v>2.0</v>
       </c>
       <c r="C30" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D30" s="36">
         <v>1.0</v>
       </c>
       <c r="E30" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -51560,19 +51550,19 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B31" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C31" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D31" s="36">
         <v>1.0</v>
       </c>
       <c r="E31" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -51584,11 +51574,21 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="24"/>
+      <c r="A32" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C32" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D32" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E32" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51599,17 +51599,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="A33" s="7"/>
+      <c r="B33" s="8"/>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
-      <c r="E33" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E33" s="24"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51620,16 +51614,16 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="7">
-        <v>50.0</v>
+      <c r="A34" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B34" s="8">
-        <v>100.0</v>
+      <c r="B34" s="8" t="s">
+        <v>30</v>
       </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
       <c r="E34" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -51641,13 +51635,17 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="41" t="s">
-        <v>31</v>
+      <c r="A35" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B35" s="42"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="43"/>
+      <c r="B35" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51658,21 +51656,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="34" t="s">
-        <v>32</v>
+      <c r="A36" s="41" t="s">
+        <v>31</v>
       </c>
-      <c r="B36" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C36" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D36" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E36" s="44">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B36" s="42"/>
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="43"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51683,11 +51673,21 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="35"/>
-      <c r="B37" s="35"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="A37" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C37" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D37" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E37" s="44">
+        <v>46009.783484375</v>
+      </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51698,9 +51698,7 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="34" t="s">
-        <v>33</v>
-      </c>
+      <c r="A38" s="35"/>
       <c r="B38" s="35"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -51715,21 +51713,13 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="s">
-        <v>7</v>
+      <c r="A39" s="34" t="s">
+        <v>33</v>
       </c>
-      <c r="B39" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C39" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D39" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E39" s="44">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B39" s="35"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51740,18 +51730,20 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="34" t="s">
-        <v>34</v>
+      <c r="A40" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B40" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C40" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D40" s="4"/>
+      <c r="D40" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E40" s="44">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51763,11 +51755,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="35"/>
-      <c r="B41" s="35"/>
-      <c r="C41" s="4"/>
+      <c r="A41" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C41" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="E41" s="44">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51778,17 +51778,11 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B42" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A42" s="35"/>
+      <c r="B42" s="35"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="44">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51800,19 +51794,15 @@
     </row>
     <row r="43">
       <c r="A43" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B43" s="34">
-        <v>5.0</v>
+      <c r="B43" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C43" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D43" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
       <c r="E43" s="44">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -51825,19 +51815,19 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B44" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C44" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D44" s="15">
         <v>1.0</v>
       </c>
       <c r="E44" s="44">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51850,10 +51840,10 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B45" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C45" s="15">
         <v>10.0</v>
@@ -51862,7 +51852,7 @@
         <v>1.0</v>
       </c>
       <c r="E45" s="44">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51874,11 +51864,21 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="35"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="A46" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C46" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D46" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E46" s="44">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51889,17 +51889,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B47" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="A47" s="35"/>
+      <c r="B47" s="35"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
-      <c r="E47" s="44">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51911,18 +51905,16 @@
     </row>
     <row r="48">
       <c r="A48" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B48" s="34">
-        <v>5.0</v>
+      <c r="B48" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C48" s="15">
-        <v>80.0</v>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="44">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D48" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51934,13 +51926,13 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B49" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C49" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D49" s="15">
         <v>1.0</v>
@@ -51957,20 +51949,18 @@
     </row>
     <row r="50">
       <c r="A50" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B50" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C50" s="15">
         <v>10.0</v>
       </c>
       <c r="D50" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E50" s="44">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -51981,11 +51971,21 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="35"/>
-      <c r="B51" s="35"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="A51" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C51" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D51" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E51" s="44">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -51996,7 +51996,7 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="34"/>
+      <c r="A52" s="35"/>
       <c r="B52" s="35"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
@@ -52011,7 +52011,7 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="35"/>
+      <c r="A53" s="34"/>
       <c r="B53" s="35"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
@@ -52026,8 +52026,8 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
+      <c r="A54" s="35"/>
+      <c r="B54" s="35"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
@@ -66095,6 +66095,21 @@
       <c r="L991" s="4"/>
       <c r="M991" s="4"/>
     </row>
+    <row r="992">
+      <c r="A992" s="4"/>
+      <c r="B992" s="4"/>
+      <c r="C992" s="4"/>
+      <c r="D992" s="4"/>
+      <c r="E992" s="4"/>
+      <c r="F992" s="4"/>
+      <c r="G992" s="4"/>
+      <c r="H992" s="4"/>
+      <c r="I992" s="4"/>
+      <c r="J992" s="4"/>
+      <c r="K992" s="4"/>
+      <c r="L992" s="4"/>
+      <c r="M992" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:39.813Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -179,7 +179,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,6 +196,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF00FFFF"/>
         <bgColor rgb="FF00FFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE5CD"/>
+        <bgColor rgb="FFFCE5CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -287,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -401,6 +407,9 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -51108,7 +51117,7 @@
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="39" t="s">
         <v>24</v>
       </c>
       <c r="C9" s="8"/>
@@ -51353,13 +51362,13 @@
       <c r="A22" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="39">
+      <c r="C22" s="40">
         <v>15.0</v>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="40">
         <v>1.0</v>
       </c>
       <c r="E22" s="26">
@@ -51378,13 +51387,13 @@
       <c r="A23" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="39">
+      <c r="B23" s="40">
         <v>30.0</v>
       </c>
-      <c r="C23" s="39">
+      <c r="C23" s="40">
         <v>15.0</v>
       </c>
-      <c r="D23" s="39">
+      <c r="D23" s="40">
         <v>1.0</v>
       </c>
       <c r="E23" s="27"/>
@@ -51507,7 +51516,7 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="41" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="17"/>
@@ -51656,13 +51665,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="41" t="s">
+      <c r="A36" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="42"/>
-      <c r="C36" s="42"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="44"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51685,7 +51694,7 @@
       <c r="D37" s="15">
         <v>2.0</v>
       </c>
-      <c r="E37" s="44">
+      <c r="E37" s="45">
         <v>46009.783484375</v>
       </c>
       <c r="F37" s="4"/>
@@ -51742,7 +51751,7 @@
       <c r="D40" s="15">
         <v>1.0</v>
       </c>
-      <c r="E40" s="44">
+      <c r="E40" s="45">
         <v>46038.9559609375</v>
       </c>
       <c r="F40" s="4"/>
@@ -51765,7 +51774,7 @@
         <v>16.0</v>
       </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="44">
+      <c r="E41" s="45">
         <v>46136.01284993056</v>
       </c>
       <c r="F41" s="4"/>
@@ -51801,7 +51810,7 @@
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="44">
+      <c r="E43" s="45">
         <v>46044.0116671875</v>
       </c>
       <c r="F43" s="4"/>
@@ -51826,7 +51835,7 @@
       <c r="D44" s="15">
         <v>1.0</v>
       </c>
-      <c r="E44" s="44">
+      <c r="E44" s="45">
         <v>46044.01310700232</v>
       </c>
       <c r="F44" s="4"/>
@@ -51851,7 +51860,7 @@
       <c r="D45" s="15">
         <v>1.0</v>
       </c>
-      <c r="E45" s="44">
+      <c r="E45" s="45">
         <v>46044.013194907406</v>
       </c>
       <c r="F45" s="4"/>
@@ -51876,7 +51885,7 @@
       <c r="D46" s="15">
         <v>1.0</v>
       </c>
-      <c r="E46" s="44">
+      <c r="E46" s="45">
         <v>46056.701985011576</v>
       </c>
       <c r="F46" s="4"/>
@@ -51912,7 +51921,7 @@
       </c>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="44">
+      <c r="E48" s="45">
         <v>46044.0136399537</v>
       </c>
       <c r="F48" s="4"/>
@@ -51983,7 +51992,7 @@
       <c r="D51" s="15">
         <v>6.0</v>
       </c>
-      <c r="E51" s="44">
+      <c r="E51" s="45">
         <v>46044.014003055556</v>
       </c>
       <c r="F51" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:44.975Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -293,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -409,7 +409,10 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -51114,10 +51117,10 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="40" t="s">
         <v>24</v>
       </c>
       <c r="C9" s="8"/>
@@ -51362,13 +51365,13 @@
       <c r="A22" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="41">
         <v>15.0</v>
       </c>
-      <c r="D22" s="40">
+      <c r="D22" s="41">
         <v>1.0</v>
       </c>
       <c r="E22" s="26">
@@ -51387,13 +51390,13 @@
       <c r="A23" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="40">
+      <c r="B23" s="41">
         <v>30.0</v>
       </c>
-      <c r="C23" s="40">
+      <c r="C23" s="41">
         <v>15.0</v>
       </c>
-      <c r="D23" s="40">
+      <c r="D23" s="41">
         <v>1.0</v>
       </c>
       <c r="E23" s="27"/>
@@ -51516,7 +51519,7 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="41" t="s">
+      <c r="A29" s="42" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="17"/>
@@ -51665,13 +51668,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="42" t="s">
+      <c r="A36" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="43"/>
-      <c r="C36" s="43"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="44"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="45"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51694,7 +51697,7 @@
       <c r="D37" s="15">
         <v>2.0</v>
       </c>
-      <c r="E37" s="45">
+      <c r="E37" s="46">
         <v>46009.783484375</v>
       </c>
       <c r="F37" s="4"/>
@@ -51751,7 +51754,7 @@
       <c r="D40" s="15">
         <v>1.0</v>
       </c>
-      <c r="E40" s="45">
+      <c r="E40" s="46">
         <v>46038.9559609375</v>
       </c>
       <c r="F40" s="4"/>
@@ -51774,7 +51777,7 @@
         <v>16.0</v>
       </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="45">
+      <c r="E41" s="46">
         <v>46136.01284993056</v>
       </c>
       <c r="F41" s="4"/>
@@ -51810,7 +51813,7 @@
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="45">
+      <c r="E43" s="46">
         <v>46044.0116671875</v>
       </c>
       <c r="F43" s="4"/>
@@ -51835,7 +51838,7 @@
       <c r="D44" s="15">
         <v>1.0</v>
       </c>
-      <c r="E44" s="45">
+      <c r="E44" s="46">
         <v>46044.01310700232</v>
       </c>
       <c r="F44" s="4"/>
@@ -51860,7 +51863,7 @@
       <c r="D45" s="15">
         <v>1.0</v>
       </c>
-      <c r="E45" s="45">
+      <c r="E45" s="46">
         <v>46044.013194907406</v>
       </c>
       <c r="F45" s="4"/>
@@ -51885,7 +51888,7 @@
       <c r="D46" s="15">
         <v>1.0</v>
       </c>
-      <c r="E46" s="45">
+      <c r="E46" s="46">
         <v>46056.701985011576</v>
       </c>
       <c r="F46" s="4"/>
@@ -51921,7 +51924,7 @@
       </c>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="45">
+      <c r="E48" s="46">
         <v>46044.0136399537</v>
       </c>
       <c r="F48" s="4"/>
@@ -51992,7 +51995,7 @@
       <c r="D51" s="15">
         <v>6.0</v>
       </c>
-      <c r="E51" s="45">
+      <c r="E51" s="46">
         <v>46044.014003055556</v>
       </c>
       <c r="F51" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:50.333Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -200,8 +200,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE5CD"/>
-        <bgColor rgb="FFFCE5CD"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:24:58.086Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -200,8 +200,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:25:05.252Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51125,9 +51125,7 @@
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
-      <c r="E9" s="25">
-        <v>46155.84992496528</v>
-      </c>
+      <c r="E9" s="25"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51150,9 +51148,7 @@
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="25">
-        <v>46155.84996290509</v>
-      </c>
+      <c r="E10" s="25"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51175,9 +51171,7 @@
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="25">
-        <v>46155.85015881945</v>
-      </c>
+      <c r="E11" s="25"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:25:08.684Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -51279,7 +51279,9 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7"/>
+      <c r="A17" s="5" t="s">
+        <v>8</v>
+      </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -51294,10 +51296,18 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="C18" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D18" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -51309,10 +51319,18 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
+      <c r="A19" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C19" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D19" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E19" s="24"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:25:12.944Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -51282,10 +51282,14 @@
       <c r="A17" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="17"/>
+      <c r="B17" s="40" t="s">
+        <v>24</v>
+      </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="24"/>
+      <c r="E17" s="25">
+        <v>46155.850816817125</v>
+      </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:25:17.739Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51303,16 +51303,14 @@
       <c r="A18" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C18" s="36">
-        <v>20.0</v>
-      </c>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36"/>
       <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="24"/>
+      <c r="E18" s="25">
+        <v>46155.85087877315</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51326,12 +51324,8 @@
       <c r="A19" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="36">
-        <v>18.0</v>
-      </c>
-      <c r="C19" s="36">
-        <v>20.0</v>
-      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
       <c r="D19" s="8">
         <v>1.0</v>
       </c>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:30:52.180Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51300,17 +51300,11 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A18" s="7"/>
       <c r="B18" s="36"/>
       <c r="C18" s="36"/>
-      <c r="D18" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="25">
-        <v>46155.85087877315</v>
-      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="25"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51322,14 +51316,16 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" s="36"/>
       <c r="C19" s="36"/>
       <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="24"/>
+      <c r="E19" s="25">
+        <v>46155.85087877315</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51340,10 +51336,14 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
+      <c r="A20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E20" s="24"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -51355,13 +51355,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="27"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51372,21 +51370,13 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>6</v>
+      <c r="A22" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B22" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D22" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E22" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51398,10 +51388,10 @@
     </row>
     <row r="23">
       <c r="A23" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B23" s="41">
-        <v>30.0</v>
+      <c r="B23" s="41" t="s">
+        <v>25</v>
       </c>
       <c r="C23" s="41">
         <v>15.0</v>
@@ -51409,7 +51399,9 @@
       <c r="D23" s="41">
         <v>1.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51420,11 +51412,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="24"/>
+      <c r="A24" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C24" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D24" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="27"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51435,9 +51435,7 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A25" s="16"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
@@ -51452,21 +51450,13 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B26" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C26" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D26" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="24"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51478,10 +51468,10 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C27" s="8">
         <v>20.0</v>
@@ -51490,7 +51480,7 @@
         <v>1.0</v>
       </c>
       <c r="E27" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51503,23 +51493,21 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B28" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C28" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D28" s="8">
         <v>1.0</v>
       </c>
       <c r="E28" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F28" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
@@ -51529,14 +51517,24 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="42" t="s">
-        <v>27</v>
+      <c r="A29" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="4"/>
+      <c r="B29" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C29" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D29" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E29" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
@@ -51546,21 +51544,13 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>28</v>
+      <c r="A30" s="42" t="s">
+        <v>27</v>
       </c>
-      <c r="B30" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C30" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D30" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E30" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51572,19 +51562,19 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B31" s="36">
         <v>2.0</v>
       </c>
       <c r="C31" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D31" s="36">
         <v>1.0</v>
       </c>
       <c r="E31" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -51597,19 +51587,19 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B32" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C32" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D32" s="36">
         <v>1.0</v>
       </c>
       <c r="E32" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -51621,11 +51611,21 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="24"/>
+      <c r="A33" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C33" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E33" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51636,17 +51636,11 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="A34" s="7"/>
+      <c r="B34" s="8"/>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
-      <c r="E34" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E34" s="24"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51657,16 +51651,16 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="7">
-        <v>50.0</v>
+      <c r="A35" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B35" s="8">
-        <v>100.0</v>
+      <c r="B35" s="8" t="s">
+        <v>30</v>
       </c>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
       <c r="E35" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -51678,13 +51672,17 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="43" t="s">
-        <v>31</v>
+      <c r="A36" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B36" s="44"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="45"/>
+      <c r="B36" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51695,21 +51693,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="s">
-        <v>32</v>
+      <c r="A37" s="43" t="s">
+        <v>31</v>
       </c>
-      <c r="B37" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C37" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D37" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E37" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B37" s="44"/>
+      <c r="C37" s="44"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="45"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51720,11 +51710,21 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="35"/>
-      <c r="B38" s="35"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="A38" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C38" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D38" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E38" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51735,9 +51735,7 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="34" t="s">
-        <v>33</v>
-      </c>
+      <c r="A39" s="35"/>
       <c r="B39" s="35"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
@@ -51752,21 +51750,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>7</v>
+      <c r="A40" s="34" t="s">
+        <v>33</v>
       </c>
-      <c r="B40" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C40" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D40" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E40" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B40" s="35"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51777,18 +51767,20 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="34" t="s">
-        <v>34</v>
+      <c r="A41" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B41" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C41" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D41" s="4"/>
+      <c r="D41" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E41" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51800,11 +51792,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="35"/>
-      <c r="B42" s="35"/>
-      <c r="C42" s="4"/>
+      <c r="A42" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B42" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C42" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="E42" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51815,17 +51815,11 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B43" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A43" s="35"/>
+      <c r="B43" s="35"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51837,19 +51831,15 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B44" s="34">
-        <v>5.0</v>
+      <c r="B44" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C44" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D44" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
       <c r="E44" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51862,19 +51852,19 @@
     </row>
     <row r="45">
       <c r="A45" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B45" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C45" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D45" s="15">
         <v>1.0</v>
       </c>
       <c r="E45" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51887,10 +51877,10 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B46" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C46" s="15">
         <v>10.0</v>
@@ -51899,7 +51889,7 @@
         <v>1.0</v>
       </c>
       <c r="E46" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51911,11 +51901,21 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="35"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="A47" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C47" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D47" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E47" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51926,17 +51926,11 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B48" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="A48" s="35"/>
+      <c r="B48" s="35"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51948,18 +51942,16 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B49" s="34">
-        <v>5.0</v>
+      <c r="B49" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C49" s="15">
-        <v>80.0</v>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D49" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -51971,13 +51963,13 @@
     </row>
     <row r="50">
       <c r="A50" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B50" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C50" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D50" s="15">
         <v>1.0</v>
@@ -51994,20 +51986,18 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B51" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C51" s="15">
         <v>10.0</v>
       </c>
       <c r="D51" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E51" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52018,11 +52008,21 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="35"/>
-      <c r="B52" s="35"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
+      <c r="A52" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C52" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D52" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E52" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52033,7 +52033,7 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="34"/>
+      <c r="A53" s="35"/>
       <c r="B53" s="35"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
@@ -52048,7 +52048,7 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="35"/>
+      <c r="A54" s="34"/>
       <c r="B54" s="35"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
@@ -52063,8 +52063,8 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="4"/>
-      <c r="B55" s="4"/>
+      <c r="A55" s="35"/>
+      <c r="B55" s="35"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
@@ -66132,6 +66132,21 @@
       <c r="L992" s="4"/>
       <c r="M992" s="4"/>
     </row>
+    <row r="993">
+      <c r="A993" s="4"/>
+      <c r="B993" s="4"/>
+      <c r="C993" s="4"/>
+      <c r="D993" s="4"/>
+      <c r="E993" s="4"/>
+      <c r="F993" s="4"/>
+      <c r="G993" s="4"/>
+      <c r="H993" s="4"/>
+      <c r="I993" s="4"/>
+      <c r="J993" s="4"/>
+      <c r="K993" s="4"/>
+      <c r="L993" s="4"/>
+      <c r="M993" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:30:55.892Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -51300,8 +51300,12 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="36"/>
+      <c r="A18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="36">
+        <v>4.0</v>
+      </c>
       <c r="C18" s="36"/>
       <c r="D18" s="8"/>
       <c r="E18" s="25"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:30:57.721Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51306,9 +51306,13 @@
       <c r="B18" s="36">
         <v>4.0</v>
       </c>
-      <c r="C18" s="36"/>
+      <c r="C18" s="36">
+        <v>30.0</v>
+      </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="25"/>
+      <c r="E18" s="25">
+        <v>46155.85481211805</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:30:58.959Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51309,9 +51309,11 @@
       <c r="C18" s="36">
         <v>30.0</v>
       </c>
-      <c r="D18" s="8"/>
+      <c r="D18" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E18" s="25">
-        <v>46155.85481211805</v>
+        <v>46155.8548316088</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:31:35.928Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51313,7 +51313,7 @@
         <v>1.0</v>
       </c>
       <c r="E18" s="25">
-        <v>46155.8548316088</v>
+        <v>46155.854844050926</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -51328,13 +51328,17 @@
       <c r="A19" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
+      <c r="B19" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="C19" s="36">
+        <v>30.0</v>
+      </c>
       <c r="D19" s="8">
         <v>1.0</v>
       </c>
       <c r="E19" s="25">
-        <v>46155.85087877315</v>
+        <v>46155.85526246528</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:31:56.905Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51353,12 +51353,18 @@
       <c r="A20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
+      <c r="B20" s="36">
+        <v>30.0</v>
+      </c>
+      <c r="C20" s="36">
+        <v>20.0</v>
+      </c>
       <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="24"/>
+      <c r="E20" s="25">
+        <v>46155.85549109954</v>
+      </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:41:28.766Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51329,7 +51329,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="36">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="C19" s="36">
         <v>30.0</v>
@@ -51338,7 +51338,7 @@
         <v>1.0</v>
       </c>
       <c r="E19" s="25">
-        <v>46155.8552762037</v>
+        <v>46155.86212506944</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:49:22.370Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51304,10 +51304,10 @@
         <v>18</v>
       </c>
       <c r="B18" s="36">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="C18" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D18" s="8">
         <v>1.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T12:59:44.747Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51252,7 +51252,7 @@
         <v>1.0</v>
       </c>
       <c r="E15" s="25">
-        <v>46099.61556196759</v>
+        <v>46155.874796793985</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -51313,7 +51313,7 @@
         <v>1.0</v>
       </c>
       <c r="E18" s="25">
-        <v>46155.86763329861</v>
+        <v>46155.86764509259</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:03:14.395Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51354,10 +51354,10 @@
         <v>7</v>
       </c>
       <c r="B20" s="36">
-        <v>30.0</v>
+        <v>17.0</v>
       </c>
       <c r="C20" s="36">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="D20" s="8">
         <v>1.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:13:43.843Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51390,13 +51390,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="27"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51407,21 +51405,11 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D23" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E23" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="A23" s="7"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51432,18 +51420,12 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>7</v>
+      <c r="A24" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B24" s="41">
-        <v>30.0</v>
-      </c>
-      <c r="C24" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D24" s="41">
-        <v>1.0</v>
-      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
       <c r="E24" s="27"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -51455,11 +51437,21 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="24"/>
+      <c r="A25" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D25" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51470,13 +51462,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>11</v>
+      <c r="A26" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C26" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D26" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E26" s="27"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51487,21 +51485,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B27" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C27" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D27" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E27" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="A27" s="16"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51512,21 +51500,13 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>7</v>
+      <c r="A28" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B28" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C28" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D28" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E28" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="24"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51541,20 +51521,18 @@
         <v>6</v>
       </c>
       <c r="B29" s="8">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C29" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D29" s="8">
         <v>1.0</v>
       </c>
       <c r="E29" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95620635417</v>
       </c>
-      <c r="F29" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
@@ -51564,13 +51542,21 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="42" t="s">
-        <v>27</v>
+      <c r="A30" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="24"/>
+      <c r="B30" s="8">
+        <v>55.0</v>
+      </c>
+      <c r="C30" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D30" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E30" s="25">
+        <v>46006.95627618056</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51582,21 +51568,23 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
-      <c r="B31" s="36">
-        <v>2.0</v>
+      <c r="B31" s="8">
+        <v>10.0</v>
       </c>
-      <c r="C31" s="36">
-        <v>100.0</v>
+      <c r="C31" s="8">
+        <v>250.0</v>
       </c>
-      <c r="D31" s="36">
+      <c r="D31" s="8">
         <v>1.0</v>
       </c>
       <c r="E31" s="25">
-        <v>45900.48749</v>
+        <v>46038.439073761576</v>
       </c>
-      <c r="F31" s="4"/>
+      <c r="F31" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
@@ -51606,21 +51594,13 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>6</v>
+      <c r="A32" s="42" t="s">
+        <v>27</v>
       </c>
-      <c r="B32" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C32" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D32" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E32" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="24"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51632,19 +51612,19 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B33" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C33" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D33" s="36">
         <v>1.0</v>
       </c>
       <c r="E33" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51656,11 +51636,21 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="7"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="24"/>
+      <c r="A34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C34" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D34" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E34" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51672,15 +51662,19 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
-      <c r="B35" s="8" t="s">
-        <v>30</v>
+      <c r="B35" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
+      <c r="C35" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D35" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E35" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -51692,17 +51686,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B36" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A36" s="7"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51713,13 +51701,17 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="43" t="s">
-        <v>31</v>
+      <c r="A37" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B37" s="44"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="45"/>
+      <c r="B37" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51730,20 +51722,16 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="34" t="s">
-        <v>32</v>
+      <c r="A38" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B38" s="34">
+      <c r="B38" s="8">
         <v>100.0</v>
       </c>
-      <c r="C38" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D38" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E38" s="46">
-        <v>46009.783484375</v>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51755,11 +51743,13 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="35"/>
-      <c r="B39" s="35"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="A39" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" s="44"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="45"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51771,12 +51761,20 @@
     </row>
     <row r="40">
       <c r="A40" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
-      <c r="B40" s="35"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="B40" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C40" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D40" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E40" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51787,21 +51785,11 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B41" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C41" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D41" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E41" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A41" s="35"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51813,18 +51801,12 @@
     </row>
     <row r="42">
       <c r="A42" s="34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
-      <c r="B42" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C42" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B42" s="35"/>
+      <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="46">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51835,11 +51817,21 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="35"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="A43" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C43" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D43" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E43" s="46">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51851,15 +51843,17 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B44" s="34" t="s">
-        <v>12</v>
+      <c r="B44" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C44" s="4"/>
+      <c r="C44" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D44" s="4"/>
       <c r="E44" s="46">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51871,21 +51865,11 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B45" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C45" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D45" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E45" s="46">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A45" s="35"/>
+      <c r="B45" s="35"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51897,19 +51881,15 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
-      <c r="B46" s="34">
-        <v>15.0</v>
+      <c r="B46" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C46" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D46" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
       <c r="E46" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51922,19 +51902,19 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B47" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C47" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D47" s="15">
         <v>1.0</v>
       </c>
       <c r="E47" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -51946,11 +51926,21 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="35"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="A48" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C48" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D48" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E48" s="46">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51962,15 +51952,19 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
-      <c r="B49" s="34" t="s">
-        <v>27</v>
+      <c r="B49" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
+      <c r="C49" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D49" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E49" s="46">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -51982,18 +51976,10 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B50" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C50" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D50" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A50" s="35"/>
+      <c r="B50" s="35"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52006,18 +51992,16 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
-      <c r="B51" s="34">
-        <v>15.0</v>
+      <c r="B51" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C51" s="15">
-        <v>10.0</v>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D51" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52029,20 +52013,18 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B52" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C52" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D52" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E52" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52053,10 +52035,18 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="35"/>
-      <c r="B53" s="35"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
+      <c r="A53" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C53" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D53" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52068,11 +52058,21 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="34"/>
-      <c r="B54" s="35"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="A54" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B54" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C54" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D54" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E54" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52098,8 +52098,8 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
+      <c r="A56" s="34"/>
+      <c r="B56" s="35"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
@@ -52113,8 +52113,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4"/>
+      <c r="A57" s="35"/>
+      <c r="B57" s="35"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -66167,6 +66167,36 @@
       <c r="L993" s="4"/>
       <c r="M993" s="4"/>
     </row>
+    <row r="994">
+      <c r="A994" s="4"/>
+      <c r="B994" s="4"/>
+      <c r="C994" s="4"/>
+      <c r="D994" s="4"/>
+      <c r="E994" s="4"/>
+      <c r="F994" s="4"/>
+      <c r="G994" s="4"/>
+      <c r="H994" s="4"/>
+      <c r="I994" s="4"/>
+      <c r="J994" s="4"/>
+      <c r="K994" s="4"/>
+      <c r="L994" s="4"/>
+      <c r="M994" s="4"/>
+    </row>
+    <row r="995">
+      <c r="A995" s="4"/>
+      <c r="B995" s="4"/>
+      <c r="C995" s="4"/>
+      <c r="D995" s="4"/>
+      <c r="E995" s="4"/>
+      <c r="F995" s="4"/>
+      <c r="G995" s="4"/>
+      <c r="H995" s="4"/>
+      <c r="I995" s="4"/>
+      <c r="J995" s="4"/>
+      <c r="K995" s="4"/>
+      <c r="L995" s="4"/>
+      <c r="M995" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:13:53.218Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51420,13 +51420,11 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="27"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="24"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51437,21 +51435,11 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D25" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E25" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="A25" s="7"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51462,19 +51450,11 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="41">
-        <v>30.0</v>
-      </c>
-      <c r="C26" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D26" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="27"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="24"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51485,11 +51465,13 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="16"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="24"/>
+      <c r="A27" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="27"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51500,13 +51482,21 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="s">
-        <v>11</v>
+      <c r="A28" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D28" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51517,21 +51507,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>6</v>
+      <c r="A29" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B29" s="8">
-        <v>9.0</v>
+      <c r="B29" s="41">
+        <v>30.0</v>
       </c>
-      <c r="C29" s="8">
-        <v>20.0</v>
+      <c r="C29" s="41">
+        <v>15.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="41">
         <v>1.0</v>
       </c>
-      <c r="E29" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51542,21 +51530,11 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C30" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D30" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E30" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="A30" s="16"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51567,24 +51545,14 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>6</v>
+      <c r="A31" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B31" s="8">
-        <v>10.0</v>
-      </c>
-      <c r="C31" s="8">
-        <v>250.0</v>
-      </c>
-      <c r="D31" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E31" s="25">
-        <v>46038.439073761576</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
@@ -51594,13 +51562,21 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="42" t="s">
-        <v>27</v>
+      <c r="A32" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="24"/>
+      <c r="B32" s="8">
+        <v>9.0</v>
+      </c>
+      <c r="C32" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D32" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E32" s="25">
+        <v>46006.95620635417</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51612,19 +51588,19 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
-      <c r="B33" s="36">
-        <v>2.0</v>
+      <c r="B33" s="8">
+        <v>55.0</v>
       </c>
-      <c r="C33" s="36">
-        <v>100.0</v>
+      <c r="C33" s="8">
+        <v>20.0</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="8">
         <v>1.0</v>
       </c>
       <c r="E33" s="25">
-        <v>45900.48749</v>
+        <v>46006.95627618056</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51639,19 +51615,21 @@
       <c r="A34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="36">
-        <v>2.0</v>
+      <c r="B34" s="8">
+        <v>10.0</v>
       </c>
-      <c r="C34" s="36">
-        <v>85.0</v>
+      <c r="C34" s="8">
+        <v>250.0</v>
       </c>
-      <c r="D34" s="36">
+      <c r="D34" s="8">
         <v>1.0</v>
       </c>
       <c r="E34" s="25">
-        <v>45900.48745738426</v>
+        <v>46038.439073761576</v>
       </c>
-      <c r="F34" s="4"/>
+      <c r="F34" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
@@ -51661,21 +51639,13 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="s">
-        <v>7</v>
+      <c r="A35" s="42" t="s">
+        <v>27</v>
       </c>
-      <c r="B35" s="36">
-        <v>70.0</v>
-      </c>
-      <c r="C35" s="36">
-        <v>10.0</v>
-      </c>
-      <c r="D35" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E35" s="25">
-        <v>45900.48752491898</v>
-      </c>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="24"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51686,11 +51656,21 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="24"/>
+      <c r="A36" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B36" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C36" s="36">
+        <v>100.0</v>
+      </c>
+      <c r="D36" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E36" s="25">
+        <v>45900.48749</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51702,15 +51682,19 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
-      <c r="B37" s="8" t="s">
-        <v>30</v>
+      <c r="B37" s="36">
+        <v>2.0</v>
       </c>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
+      <c r="C37" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D37" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E37" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51722,16 +51706,20 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7">
-        <v>50.0</v>
+      <c r="A38" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B38" s="8">
-        <v>100.0</v>
+      <c r="B38" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
+      <c r="C38" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D38" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E38" s="25">
-        <v>45946.87887299768</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51743,13 +51731,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="43" t="s">
-        <v>31</v>
-      </c>
-      <c r="B39" s="44"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="45"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51760,20 +51746,16 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="34" t="s">
-        <v>32</v>
+      <c r="A40" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B40" s="34">
-        <v>100.0</v>
+      <c r="B40" s="8" t="s">
+        <v>30</v>
       </c>
-      <c r="C40" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D40" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E40" s="46">
-        <v>46009.783484375</v>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="25">
+        <v>45946.87875708334</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51785,11 +51767,17 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="35"/>
-      <c r="B41" s="35"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="A41" s="7">
+        <v>50.0</v>
+      </c>
+      <c r="B41" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51800,13 +51788,13 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="34" t="s">
-        <v>33</v>
+      <c r="A42" s="43" t="s">
+        <v>31</v>
       </c>
-      <c r="B42" s="35"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="B42" s="44"/>
+      <c r="C42" s="44"/>
+      <c r="D42" s="44"/>
+      <c r="E42" s="45"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51817,20 +51805,20 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>7</v>
+      <c r="A43" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="B43" s="34">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="C43" s="15">
-        <v>20.0</v>
+        <v>1.0</v>
       </c>
       <c r="D43" s="15">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E43" s="46">
-        <v>46038.9559609375</v>
+        <v>46009.783484375</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -51842,19 +51830,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B44" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C44" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="A44" s="35"/>
+      <c r="B44" s="35"/>
+      <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="46">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51865,7 +51845,9 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="35"/>
+      <c r="A45" s="34" t="s">
+        <v>33</v>
+      </c>
       <c r="B45" s="35"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -51880,16 +51862,20 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="34" t="s">
-        <v>35</v>
+      <c r="A46" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B46" s="34" t="s">
-        <v>12</v>
+      <c r="B46" s="34">
+        <v>50.0</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
+      <c r="C46" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D46" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E46" s="46">
-        <v>46044.0116671875</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51902,19 +51888,17 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B47" s="34">
-        <v>5.0</v>
+        <v>15.0</v>
       </c>
       <c r="C47" s="15">
-        <v>80.0</v>
+        <v>16.0</v>
       </c>
-      <c r="D47" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="D47" s="4"/>
       <c r="E47" s="46">
-        <v>46044.01310700232</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -51926,21 +51910,11 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B48" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C48" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D48" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E48" s="46">
-        <v>46044.013194907406</v>
-      </c>
+      <c r="A48" s="35"/>
+      <c r="B48" s="35"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51952,19 +51926,15 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
-      <c r="B49" s="34">
-        <v>30.0</v>
+      <c r="B49" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C49" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D49" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
       <c r="E49" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -51976,11 +51946,21 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="35"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
+      <c r="A50" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B50" s="34">
+        <v>5.0</v>
+      </c>
+      <c r="C50" s="15">
+        <v>80.0</v>
+      </c>
+      <c r="D50" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E50" s="46">
+        <v>46044.01310700232</v>
+      </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -51992,15 +51972,19 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
-      <c r="B51" s="34" t="s">
-        <v>27</v>
+      <c r="B51" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
+      <c r="C51" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D51" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E51" s="46">
-        <v>46044.0136399537</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -52013,18 +51997,20 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="B52" s="34">
-        <v>5.0</v>
+        <v>30.0</v>
       </c>
       <c r="C52" s="15">
-        <v>80.0</v>
+        <v>10.0</v>
       </c>
       <c r="D52" s="15">
         <v>1.0</v>
       </c>
-      <c r="E52" s="4"/>
+      <c r="E52" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52035,18 +52021,10 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C53" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D53" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52059,19 +52037,15 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
-      <c r="B54" s="34">
-        <v>20.0</v>
+      <c r="B54" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C54" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D54" s="15">
-        <v>6.0</v>
-      </c>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
       <c r="E54" s="46">
-        <v>46044.014003055556</v>
+        <v>46044.0136399537</v>
       </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52083,10 +52057,18 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="35"/>
-      <c r="B55" s="35"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
+      <c r="A55" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B55" s="34">
+        <v>5.0</v>
+      </c>
+      <c r="C55" s="15">
+        <v>80.0</v>
+      </c>
+      <c r="D55" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52098,10 +52080,18 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="34"/>
-      <c r="B56" s="35"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
+      <c r="A56" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B56" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C56" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D56" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52113,11 +52103,21 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="35"/>
-      <c r="B57" s="35"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="A57" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C57" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D57" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E57" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52128,8 +52128,8 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
+      <c r="A58" s="35"/>
+      <c r="B58" s="35"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52143,8 +52143,8 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
+      <c r="A59" s="34"/>
+      <c r="B59" s="35"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
@@ -52158,8 +52158,8 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
+      <c r="A60" s="35"/>
+      <c r="B60" s="35"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
@@ -66197,6 +66197,51 @@
       <c r="L995" s="4"/>
       <c r="M995" s="4"/>
     </row>
+    <row r="996">
+      <c r="A996" s="4"/>
+      <c r="B996" s="4"/>
+      <c r="C996" s="4"/>
+      <c r="D996" s="4"/>
+      <c r="E996" s="4"/>
+      <c r="F996" s="4"/>
+      <c r="G996" s="4"/>
+      <c r="H996" s="4"/>
+      <c r="I996" s="4"/>
+      <c r="J996" s="4"/>
+      <c r="K996" s="4"/>
+      <c r="L996" s="4"/>
+      <c r="M996" s="4"/>
+    </row>
+    <row r="997">
+      <c r="A997" s="4"/>
+      <c r="B997" s="4"/>
+      <c r="C997" s="4"/>
+      <c r="D997" s="4"/>
+      <c r="E997" s="4"/>
+      <c r="F997" s="4"/>
+      <c r="G997" s="4"/>
+      <c r="H997" s="4"/>
+      <c r="I997" s="4"/>
+      <c r="J997" s="4"/>
+      <c r="K997" s="4"/>
+      <c r="L997" s="4"/>
+      <c r="M997" s="4"/>
+    </row>
+    <row r="998">
+      <c r="A998" s="4"/>
+      <c r="B998" s="4"/>
+      <c r="C998" s="4"/>
+      <c r="D998" s="4"/>
+      <c r="E998" s="4"/>
+      <c r="F998" s="4"/>
+      <c r="G998" s="4"/>
+      <c r="H998" s="4"/>
+      <c r="I998" s="4"/>
+      <c r="J998" s="4"/>
+      <c r="K998" s="4"/>
+      <c r="L998" s="4"/>
+      <c r="M998" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:13:56.624Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -51390,8 +51390,12 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7"/>
-      <c r="B22" s="17"/>
+      <c r="A22" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="40" t="s">
+        <v>24</v>
+      </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
       <c r="E22" s="24"/>
@@ -51405,10 +51409,18 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
+      <c r="A23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="C23" s="36">
+        <v>50.0</v>
+      </c>
+      <c r="D23" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -51420,10 +51432,18 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
+      <c r="A24" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" s="36">
+        <v>8.0</v>
+      </c>
+      <c r="C24" s="36">
+        <v>30.0</v>
+      </c>
+      <c r="D24" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E24" s="24"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -51435,10 +51455,18 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
+      <c r="A25" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="36">
+        <v>17.0</v>
+      </c>
+      <c r="C25" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D25" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:14:07.629Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51412,16 +51412,14 @@
       <c r="A23" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C23" s="36">
-        <v>50.0</v>
-      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
       <c r="D23" s="8">
         <v>1.0</v>
       </c>
-      <c r="E23" s="24"/>
+      <c r="E23" s="25">
+        <v>46155.884781307876</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51435,12 +51433,8 @@
       <c r="A24" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="36">
-        <v>8.0</v>
-      </c>
-      <c r="C24" s="36">
-        <v>30.0</v>
-      </c>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
@@ -51458,12 +51452,8 @@
       <c r="A25" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="36">
-        <v>17.0</v>
-      </c>
-      <c r="C25" s="36">
-        <v>15.0</v>
-      </c>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
       <c r="D25" s="8">
         <v>1.0</v>
       </c>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:14:19.614Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51452,12 +51452,18 @@
       <c r="A25" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="36"/>
+      <c r="B25" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="C25" s="36">
+        <v>10.0</v>
+      </c>
       <c r="D25" s="8">
         <v>1.0</v>
       </c>
-      <c r="E25" s="24"/>
+      <c r="E25" s="25">
+        <v>46155.88493537037</v>
+      </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:14:27.979Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51453,7 +51453,7 @@
         <v>7</v>
       </c>
       <c r="B25" s="36">
-        <v>20.0</v>
+        <v>17.0</v>
       </c>
       <c r="C25" s="36">
         <v>10.0</v>
@@ -51462,7 +51462,7 @@
         <v>1.0</v>
       </c>
       <c r="E25" s="25">
-        <v>46155.88495121528</v>
+        <v>46155.88500635416</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:23:13.538Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51456,13 +51456,13 @@
         <v>18.0</v>
       </c>
       <c r="C25" s="36">
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="D25" s="8">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E25" s="25">
-        <v>46155.88500635416</v>
+        <v>46155.89110758102</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-13T13:23:59.836Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51412,13 +51412,17 @@
       <c r="A23" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="36"/>
+      <c r="B23" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="C23" s="36">
+        <v>50.0</v>
+      </c>
       <c r="D23" s="8">
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46155.884781307876</v>
+        <v>46155.89164559028</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -51433,8 +51437,12 @@
       <c r="A24" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
+      <c r="B24" s="36">
+        <v>8.0</v>
+      </c>
+      <c r="C24" s="36">
+        <v>30.0</v>
+      </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:18:31.992Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51350,21 +51350,11 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="36">
-        <v>17.0</v>
-      </c>
-      <c r="C20" s="36">
-        <v>15.0</v>
-      </c>
-      <c r="D20" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E20" s="25">
-        <v>46155.877253784725</v>
-      </c>
+      <c r="A20" s="7"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51375,11 +51365,21 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="24"/>
+      <c r="A21" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="36">
+        <v>17.0</v>
+      </c>
+      <c r="C21" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D21" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E21" s="25">
+        <v>46155.877253784725</v>
+      </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51390,12 +51390,8 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" s="40" t="s">
-        <v>24</v>
-      </c>
+      <c r="A22" s="7"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
       <c r="E22" s="24"/>
@@ -51409,21 +51405,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>18</v>
+      <c r="A23" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B23" s="36">
-        <v>6.0</v>
+      <c r="B23" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C23" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D23" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E23" s="25">
-        <v>46155.89164559028</v>
-      </c>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51435,18 +51425,20 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B24" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C24" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="24"/>
+      <c r="E24" s="25">
+        <v>46155.89164559028</v>
+      </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51458,20 +51450,18 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" s="36">
-        <v>18.0</v>
+        <v>8.0</v>
       </c>
       <c r="C25" s="36">
-        <v>14.0</v>
+        <v>30.0</v>
       </c>
       <c r="D25" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E25" s="25">
-        <v>46155.89113405092</v>
-      </c>
+      <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51482,11 +51472,21 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="24"/>
+      <c r="A26" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C26" s="36">
+        <v>14.0</v>
+      </c>
+      <c r="D26" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="E26" s="25">
+        <v>46155.89113405092</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51497,13 +51497,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="27"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51514,21 +51512,13 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="s">
-        <v>6</v>
+      <c r="A28" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D28" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E28" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="27"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51540,10 +51530,10 @@
     </row>
     <row r="29">
       <c r="A29" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B29" s="41">
-        <v>30.0</v>
+      <c r="B29" s="41" t="s">
+        <v>25</v>
       </c>
       <c r="C29" s="41">
         <v>15.0</v>
@@ -51551,7 +51541,9 @@
       <c r="D29" s="41">
         <v>1.0</v>
       </c>
-      <c r="E29" s="27"/>
+      <c r="E29" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51562,11 +51554,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="16"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="24"/>
+      <c r="A30" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C30" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D30" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51577,9 +51577,7 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A31" s="16"/>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -51594,21 +51592,13 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>6</v>
+      <c r="A32" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B32" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C32" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D32" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E32" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="24"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51620,10 +51610,10 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C33" s="8">
         <v>20.0</v>
@@ -51632,7 +51622,7 @@
         <v>1.0</v>
       </c>
       <c r="E33" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51645,23 +51635,21 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B34" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C34" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D34" s="8">
         <v>1.0</v>
       </c>
       <c r="E34" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F34" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
@@ -51671,14 +51659,24 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="42" t="s">
-        <v>27</v>
+      <c r="A35" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="4"/>
+      <c r="B35" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C35" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D35" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E35" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
@@ -51688,21 +51686,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="s">
-        <v>28</v>
+      <c r="A36" s="42" t="s">
+        <v>27</v>
       </c>
-      <c r="B36" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C36" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D36" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E36" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51714,19 +51704,19 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B37" s="36">
         <v>2.0</v>
       </c>
       <c r="C37" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D37" s="36">
         <v>1.0</v>
       </c>
       <c r="E37" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51739,19 +51729,19 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C38" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D38" s="36">
         <v>1.0</v>
       </c>
       <c r="E38" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51763,11 +51753,21 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="7"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="24"/>
+      <c r="A39" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C39" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D39" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E39" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51778,17 +51778,11 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="A40" s="7"/>
+      <c r="B40" s="8"/>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
-      <c r="E40" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E40" s="24"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51799,16 +51793,16 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7">
-        <v>50.0</v>
+      <c r="A41" s="7" t="s">
+        <v>29</v>
       </c>
-      <c r="B41" s="8">
-        <v>100.0</v>
+      <c r="B41" s="8" t="s">
+        <v>30</v>
       </c>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
       <c r="E41" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51820,13 +51814,17 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="43" t="s">
-        <v>31</v>
+      <c r="A42" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B42" s="44"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="45"/>
+      <c r="B42" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51837,21 +51835,13 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="34" t="s">
-        <v>32</v>
+      <c r="A43" s="43" t="s">
+        <v>31</v>
       </c>
-      <c r="B43" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C43" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D43" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E43" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B43" s="44"/>
+      <c r="C43" s="44"/>
+      <c r="D43" s="44"/>
+      <c r="E43" s="45"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51862,11 +51852,21 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="35"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="A44" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C44" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D44" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E44" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51877,9 +51877,7 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="34" t="s">
-        <v>33</v>
-      </c>
+      <c r="A45" s="35"/>
       <c r="B45" s="35"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -51894,21 +51892,13 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>7</v>
+      <c r="A46" s="34" t="s">
+        <v>33</v>
       </c>
-      <c r="B46" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C46" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D46" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E46" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B46" s="35"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51919,18 +51909,20 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="34" t="s">
-        <v>34</v>
+      <c r="A47" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B47" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C47" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D47" s="4"/>
+      <c r="D47" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E47" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -51942,11 +51934,19 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="35"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="4"/>
+      <c r="A48" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B48" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C48" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="E48" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51957,17 +51957,11 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B49" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A49" s="35"/>
+      <c r="B49" s="35"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -51979,19 +51973,15 @@
     </row>
     <row r="50">
       <c r="A50" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B50" s="34">
-        <v>5.0</v>
+      <c r="B50" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C50" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D50" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
       <c r="E50" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52004,19 +51994,19 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B51" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C51" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D51" s="15">
         <v>1.0</v>
       </c>
       <c r="E51" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -52029,10 +52019,10 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B52" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C52" s="15">
         <v>10.0</v>
@@ -52041,7 +52031,7 @@
         <v>1.0</v>
       </c>
       <c r="E52" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52053,11 +52043,21 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="35"/>
-      <c r="B53" s="35"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
+      <c r="A53" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C53" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D53" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E53" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52068,17 +52068,11 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B54" s="34" t="s">
-        <v>27</v>
-      </c>
+      <c r="A54" s="35"/>
+      <c r="B54" s="35"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52090,18 +52084,16 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B55" s="34">
-        <v>5.0</v>
+      <c r="B55" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C55" s="15">
-        <v>80.0</v>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D55" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52113,13 +52105,13 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B56" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C56" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D56" s="15">
         <v>1.0</v>
@@ -52136,20 +52128,18 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B57" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C57" s="15">
         <v>10.0</v>
       </c>
       <c r="D57" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E57" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52160,11 +52150,21 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="35"/>
-      <c r="B58" s="35"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
+      <c r="A58" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C58" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D58" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E58" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52175,7 +52175,7 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="34"/>
+      <c r="A59" s="35"/>
       <c r="B59" s="35"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
@@ -52190,7 +52190,7 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="35"/>
+      <c r="A60" s="34"/>
       <c r="B60" s="35"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
@@ -52205,8 +52205,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
+      <c r="A61" s="35"/>
+      <c r="B61" s="35"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -66274,6 +66274,21 @@
       <c r="L998" s="4"/>
       <c r="M998" s="4"/>
     </row>
+    <row r="999">
+      <c r="A999" s="4"/>
+      <c r="B999" s="4"/>
+      <c r="C999" s="4"/>
+      <c r="D999" s="4"/>
+      <c r="E999" s="4"/>
+      <c r="F999" s="4"/>
+      <c r="G999" s="4"/>
+      <c r="H999" s="4"/>
+      <c r="I999" s="4"/>
+      <c r="J999" s="4"/>
+      <c r="K999" s="4"/>
+      <c r="L999" s="4"/>
+      <c r="M999" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:19:15.860Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="38">
   <si>
     <t>項目</t>
   </si>
@@ -51350,7 +51350,9 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7"/>
+      <c r="A20" s="7" t="s">
+        <v>16</v>
+      </c>
       <c r="B20" s="36"/>
       <c r="C20" s="36"/>
       <c r="D20" s="8"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:19:21.584Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51353,10 +51353,16 @@
       <c r="A20" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
+      <c r="B20" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="C20" s="36">
+        <v>30.0</v>
+      </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="25"/>
+      <c r="E20" s="25">
+        <v>46156.84675237269</v>
+      </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:19:23.855Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51359,9 +51359,11 @@
       <c r="C20" s="36">
         <v>30.0</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="8">
+        <v>4.0</v>
+      </c>
       <c r="E20" s="25">
-        <v>46156.84675237269</v>
+        <v>46156.84678416667</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:19:32.929Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="39">
   <si>
     <t>項目</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t>PS</t>
+  </si>
+  <si>
+    <t>Detail</t>
   </si>
   <si>
     <t>６</t>
@@ -51365,7 +51368,9 @@
       <c r="E20" s="25">
         <v>46156.84678416667</v>
       </c>
-      <c r="F20" s="4"/>
+      <c r="F20" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -51543,7 +51548,7 @@
         <v>6</v>
       </c>
       <c r="B29" s="41" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C29" s="41">
         <v>15.0</v>
@@ -51685,7 +51690,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51697,7 +51702,7 @@
     </row>
     <row r="36">
       <c r="A36" s="42" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
@@ -51714,7 +51719,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B37" s="36">
         <v>2.0</v>
@@ -51804,10 +51809,10 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -51846,7 +51851,7 @@
     </row>
     <row r="43">
       <c r="A43" s="43" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B43" s="44"/>
       <c r="C43" s="44"/>
@@ -51863,7 +51868,7 @@
     </row>
     <row r="44">
       <c r="A44" s="34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B44" s="34">
         <v>100.0</v>
@@ -51903,7 +51908,7 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B46" s="35"/>
       <c r="C46" s="4"/>
@@ -51945,7 +51950,7 @@
     </row>
     <row r="48">
       <c r="A48" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B48" s="34">
         <v>15.0</v>
@@ -51983,7 +51988,7 @@
     </row>
     <row r="50">
       <c r="A50" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B50" s="34" t="s">
         <v>12</v>
@@ -52004,7 +52009,7 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B51" s="34">
         <v>5.0</v>
@@ -52029,7 +52034,7 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B52" s="34">
         <v>15.0</v>
@@ -52094,10 +52099,10 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B55" s="34" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
@@ -52115,7 +52120,7 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B56" s="34">
         <v>5.0</v>
@@ -52138,7 +52143,7 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B57" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:05.756Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51038,12 +51038,10 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
       <c r="E5" s="24"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -51055,21 +51053,11 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="8">
-        <v>10.0</v>
-      </c>
-      <c r="C6" s="8">
-        <v>45.0</v>
-      </c>
-      <c r="D6" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E6" s="25">
-        <v>46106.73232292824</v>
-      </c>
+      <c r="A6" s="5"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -51080,21 +51068,13 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>16</v>
+      <c r="A7" s="5" t="s">
+        <v>23</v>
       </c>
-      <c r="B7" s="8">
-        <v>11.0</v>
-      </c>
-      <c r="C7" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E7" s="25">
-        <v>46106.732369062505</v>
-      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="24"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51104,12 +51084,22 @@
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="38"/>
+    <row r="8">
+      <c r="A8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C8" s="8">
+        <v>45.0</v>
+      </c>
+      <c r="D8" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E8" s="25">
+        <v>46106.73232292824</v>
+      </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51120,15 +51110,21 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="39" t="s">
-        <v>23</v>
+      <c r="A9" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B9" s="40" t="s">
-        <v>24</v>
+      <c r="B9" s="8">
+        <v>11.0</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="25"/>
+      <c r="C9" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D9" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E9" s="25">
+        <v>46106.732369062505</v>
+      </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51138,20 +51134,12 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="C10" s="8">
-        <v>30.0</v>
-      </c>
-      <c r="D10" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E10" s="25"/>
+    <row r="10" ht="16.5" customHeight="1">
+      <c r="A10" s="5"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="38"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51162,18 +51150,14 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>16</v>
+      <c r="A11" s="39" t="s">
+        <v>23</v>
       </c>
-      <c r="B11" s="8">
-        <v>10.0</v>
+      <c r="B11" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C11" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="25"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -51185,11 +51169,19 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="38"/>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="C12" s="8">
+        <v>30.0</v>
+      </c>
+      <c r="D12" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E12" s="25"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51200,13 +51192,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>8</v>
+      <c r="A13" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C13" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D13" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E13" s="25"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51217,21 +51215,11 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C14" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D14" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E14" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="A14" s="5"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="38"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51242,21 +51230,13 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>7</v>
+      <c r="A15" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B15" s="36">
-        <v>18.0</v>
-      </c>
-      <c r="C15" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D15" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="25">
-        <v>46155.874796793985</v>
-      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51267,11 +51247,21 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="24"/>
+      <c r="A16" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="C16" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E16" s="25">
+        <v>46118.87534236111</v>
+      </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51282,16 +51272,20 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="39" t="s">
-        <v>8</v>
+      <c r="A17" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="40" t="s">
-        <v>24</v>
+      <c r="B17" s="36">
+        <v>18.0</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
+      <c r="C17" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D17" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E17" s="25">
-        <v>46155.850816817125</v>
+        <v>46155.874796793985</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -51303,21 +51297,11 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C18" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D18" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="25">
-        <v>46155.86764509259</v>
-      </c>
+      <c r="A18" s="7"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51328,20 +51312,16 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="39" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="36">
-        <v>8.0</v>
+      <c r="B19" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C19" s="36">
-        <v>30.0</v>
-      </c>
-      <c r="D19" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
       <c r="E19" s="25">
-        <v>46155.86212506944</v>
+        <v>46155.850816817125</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51354,23 +51334,21 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B20" s="36">
-        <v>10.0</v>
+        <v>6.0</v>
       </c>
       <c r="C20" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D20" s="8">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="E20" s="25">
-        <v>46156.84678416667</v>
+        <v>46155.86764509259</v>
       </c>
-      <c r="F20" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -51381,19 +51359,19 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B21" s="36">
-        <v>17.0</v>
+        <v>8.0</v>
       </c>
       <c r="C21" s="36">
-        <v>15.0</v>
+        <v>30.0</v>
       </c>
       <c r="D21" s="8">
         <v>1.0</v>
       </c>
       <c r="E21" s="25">
-        <v>46155.877253784725</v>
+        <v>46155.86212506944</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -51405,12 +51383,24 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="4"/>
+      <c r="A22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="C22" s="36">
+        <v>30.0</v>
+      </c>
+      <c r="D22" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="E22" s="25">
+        <v>46156.84678416667</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -51420,15 +51410,21 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="39" t="s">
-        <v>10</v>
+      <c r="A23" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B23" s="40" t="s">
-        <v>24</v>
+      <c r="B23" s="36">
+        <v>17.0</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="24"/>
+      <c r="C23" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D23" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E23" s="25">
+        <v>46155.877253784725</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51439,21 +51435,11 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C24" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D24" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E24" s="25">
-        <v>46155.89164559028</v>
-      </c>
+      <c r="A24" s="7"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="24"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51464,18 +51450,14 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>6</v>
+      <c r="A25" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B25" s="36">
-        <v>8.0</v>
+      <c r="B25" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C25" s="36">
-        <v>30.0</v>
-      </c>
-      <c r="D25" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
       <c r="E25" s="24"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -51488,19 +51470,19 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B26" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C26" s="36">
-        <v>14.0</v>
+        <v>50.0</v>
       </c>
       <c r="D26" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="E26" s="25">
-        <v>46155.89113405092</v>
+        <v>46155.89164559028</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -51512,10 +51494,18 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
+      <c r="A27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" s="36">
+        <v>8.0</v>
+      </c>
+      <c r="C27" s="36">
+        <v>30.0</v>
+      </c>
+      <c r="D27" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E27" s="24"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51527,13 +51517,21 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>10</v>
+      <c r="A28" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="27"/>
+      <c r="B28" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C28" s="36">
+        <v>14.0</v>
+      </c>
+      <c r="D28" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="E28" s="25">
+        <v>46155.89113405092</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51544,21 +51542,11 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D29" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E29" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="A29" s="7"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51569,18 +51557,12 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>7</v>
+      <c r="A30" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B30" s="41">
-        <v>30.0</v>
-      </c>
-      <c r="C30" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D30" s="41">
-        <v>1.0</v>
-      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
       <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -51592,11 +51574,21 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="16"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="24"/>
+      <c r="A31" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D31" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E31" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51607,13 +51599,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="s">
-        <v>11</v>
+      <c r="A32" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="24"/>
+      <c r="B32" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C32" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D32" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E32" s="27"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51624,21 +51622,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B33" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C33" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D33" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E33" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="A33" s="16"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="24"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51649,21 +51637,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="s">
-        <v>7</v>
+      <c r="A34" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B34" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C34" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D34" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E34" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="24"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51678,20 +51658,18 @@
         <v>6</v>
       </c>
       <c r="B35" s="8">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C35" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D35" s="8">
         <v>1.0</v>
       </c>
       <c r="E35" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95620635417</v>
       </c>
-      <c r="F35" s="15" t="s">
-        <v>27</v>
-      </c>
+      <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
@@ -51701,13 +51679,21 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="42" t="s">
-        <v>28</v>
+      <c r="A36" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="24"/>
+      <c r="B36" s="8">
+        <v>55.0</v>
+      </c>
+      <c r="C36" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D36" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E36" s="25">
+        <v>46006.95627618056</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51719,21 +51705,23 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
-      <c r="B37" s="36">
-        <v>2.0</v>
+      <c r="B37" s="8">
+        <v>10.0</v>
       </c>
-      <c r="C37" s="36">
-        <v>100.0</v>
+      <c r="C37" s="8">
+        <v>250.0</v>
       </c>
-      <c r="D37" s="36">
+      <c r="D37" s="8">
         <v>1.0</v>
       </c>
       <c r="E37" s="25">
-        <v>45900.48749</v>
+        <v>46038.439073761576</v>
       </c>
-      <c r="F37" s="4"/>
+      <c r="F37" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
@@ -51743,21 +51731,13 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>6</v>
+      <c r="A38" s="42" t="s">
+        <v>28</v>
       </c>
-      <c r="B38" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C38" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D38" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E38" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="24"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51769,19 +51749,19 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B39" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C39" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D39" s="36">
         <v>1.0</v>
       </c>
       <c r="E39" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51793,11 +51773,21 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="24"/>
+      <c r="A40" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C40" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D40" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E40" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51809,15 +51799,19 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
-        <v>30</v>
+        <v>7</v>
       </c>
-      <c r="B41" s="8" t="s">
-        <v>31</v>
+      <c r="B41" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
+      <c r="C41" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D41" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E41" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51829,17 +51823,11 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B42" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A42" s="7"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="24"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51850,13 +51838,17 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="43" t="s">
-        <v>32</v>
+      <c r="A43" s="7" t="s">
+        <v>30</v>
       </c>
-      <c r="B43" s="44"/>
-      <c r="C43" s="44"/>
-      <c r="D43" s="44"/>
-      <c r="E43" s="45"/>
+      <c r="B43" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51867,20 +51859,16 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="s">
-        <v>33</v>
+      <c r="A44" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B44" s="34">
+      <c r="B44" s="8">
         <v>100.0</v>
       </c>
-      <c r="C44" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D44" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E44" s="46">
-        <v>46009.783484375</v>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51892,11 +51880,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="35"/>
-      <c r="B45" s="35"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
+      <c r="A45" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B45" s="44"/>
+      <c r="C45" s="44"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="45"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51908,12 +51898,20 @@
     </row>
     <row r="46">
       <c r="A46" s="34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
-      <c r="B46" s="35"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="B46" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C46" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D46" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E46" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51924,21 +51922,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B47" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C47" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D47" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E47" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A47" s="35"/>
+      <c r="B47" s="35"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51950,18 +51938,12 @@
     </row>
     <row r="48">
       <c r="A48" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
-      <c r="B48" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C48" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B48" s="35"/>
+      <c r="C48" s="4"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="46">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51972,11 +51954,21 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="35"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="A49" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C49" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D49" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E49" s="46">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -51988,15 +51980,17 @@
     </row>
     <row r="50">
       <c r="A50" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B50" s="34" t="s">
-        <v>12</v>
+      <c r="B50" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C50" s="4"/>
+      <c r="C50" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D50" s="4"/>
       <c r="E50" s="46">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52008,21 +52002,11 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B51" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C51" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D51" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E51" s="46">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A51" s="35"/>
+      <c r="B51" s="35"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52034,19 +52018,15 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
-      <c r="B52" s="34">
-        <v>15.0</v>
+      <c r="B52" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C52" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D52" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
       <c r="E52" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52059,19 +52039,19 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B53" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C53" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D53" s="15">
         <v>1.0</v>
       </c>
       <c r="E53" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52083,11 +52063,21 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="35"/>
-      <c r="B54" s="35"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="A54" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C54" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D54" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E54" s="46">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52099,15 +52089,19 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
-      <c r="B55" s="34" t="s">
-        <v>28</v>
+      <c r="B55" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
+      <c r="C55" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D55" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E55" s="46">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52119,18 +52113,10 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B56" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C56" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D56" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A56" s="35"/>
+      <c r="B56" s="35"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52143,18 +52129,16 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
-      <c r="B57" s="34">
-        <v>15.0</v>
+      <c r="B57" s="34" t="s">
+        <v>28</v>
       </c>
-      <c r="C57" s="15">
-        <v>10.0</v>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D57" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52166,20 +52150,18 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B58" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C58" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D58" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E58" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52190,10 +52172,18 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="35"/>
-      <c r="B59" s="35"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
+      <c r="A59" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B59" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C59" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D59" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52205,11 +52195,21 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="34"/>
-      <c r="B60" s="35"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="A60" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B60" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C60" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D60" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E60" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52235,8 +52235,8 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4"/>
+      <c r="A62" s="34"/>
+      <c r="B62" s="35"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
@@ -52250,8 +52250,8 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="35"/>
+      <c r="B63" s="35"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
@@ -66304,6 +66304,36 @@
       <c r="L999" s="4"/>
       <c r="M999" s="4"/>
     </row>
+    <row r="1000">
+      <c r="A1000" s="4"/>
+      <c r="B1000" s="4"/>
+      <c r="C1000" s="4"/>
+      <c r="D1000" s="4"/>
+      <c r="E1000" s="4"/>
+      <c r="F1000" s="4"/>
+      <c r="G1000" s="4"/>
+      <c r="H1000" s="4"/>
+      <c r="I1000" s="4"/>
+      <c r="J1000" s="4"/>
+      <c r="K1000" s="4"/>
+      <c r="L1000" s="4"/>
+      <c r="M1000" s="4"/>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="4"/>
+      <c r="B1001" s="4"/>
+      <c r="C1001" s="4"/>
+      <c r="D1001" s="4"/>
+      <c r="E1001" s="4"/>
+      <c r="F1001" s="4"/>
+      <c r="G1001" s="4"/>
+      <c r="H1001" s="4"/>
+      <c r="I1001" s="4"/>
+      <c r="J1001" s="4"/>
+      <c r="K1001" s="4"/>
+      <c r="L1001" s="4"/>
+      <c r="M1001" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:11.228Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51068,12 +51068,10 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
       <c r="E7" s="24"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -51085,21 +51083,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="s">
-        <v>6</v>
+      <c r="A8" s="5" t="s">
+        <v>23</v>
       </c>
-      <c r="B8" s="8">
-        <v>10.0</v>
-      </c>
-      <c r="C8" s="8">
-        <v>45.0</v>
-      </c>
-      <c r="D8" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E8" s="25">
-        <v>46106.73232292824</v>
-      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="24"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51111,19 +51101,19 @@
     </row>
     <row r="9">
       <c r="A9" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B9" s="8">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
       <c r="C9" s="8">
-        <v>20.0</v>
+        <v>45.0</v>
       </c>
       <c r="D9" s="8">
         <v>1.0</v>
       </c>
       <c r="E9" s="25">
-        <v>46106.732369062505</v>
+        <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -51134,12 +51124,22 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
+    <row r="10">
+      <c r="A10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="8">
+        <v>11.0</v>
+      </c>
+      <c r="C10" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D10" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E10" s="25">
+        <v>46106.732369062505</v>
+      </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -51149,16 +51149,12 @@
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
-    <row r="11">
-      <c r="A11" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="25"/>
+    <row r="11" ht="16.5" customHeight="1">
+      <c r="A11" s="5"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="38"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51169,18 +51165,14 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="39" t="s">
+        <v>23</v>
       </c>
-      <c r="B12" s="8">
-        <v>5.0</v>
+      <c r="B12" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C12" s="8">
-        <v>30.0</v>
-      </c>
-      <c r="D12" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
       <c r="E12" s="25"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -51193,13 +51185,13 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B13" s="8">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="C13" s="8">
-        <v>20.0</v>
+        <v>30.0</v>
       </c>
       <c r="D13" s="8">
         <v>1.0</v>
@@ -51215,11 +51207,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="38"/>
+      <c r="A14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C14" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E14" s="25"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51230,13 +51230,11 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="24"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="38"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51247,21 +51245,13 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>6</v>
+      <c r="A16" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B16" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C16" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D16" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E16" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="24"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51273,10 +51263,10 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B17" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C17" s="36">
         <v>20.0</v>
@@ -51285,7 +51275,7 @@
         <v>1.0</v>
       </c>
       <c r="E17" s="25">
-        <v>46155.874796793985</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -51297,11 +51287,21 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="24"/>
+      <c r="A18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C18" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D18" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E18" s="25">
+        <v>46155.874796793985</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51312,17 +51312,11 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" s="40" t="s">
-        <v>24</v>
-      </c>
+      <c r="A19" s="7"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="25">
-        <v>46155.850816817125</v>
-      </c>
+      <c r="E19" s="24"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51333,20 +51327,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>18</v>
+      <c r="A20" s="39" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="36">
-        <v>6.0</v>
+      <c r="B20" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C20" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D20" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
       <c r="E20" s="25">
-        <v>46155.86764509259</v>
+        <v>46155.850816817125</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -51359,19 +51349,19 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B21" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C21" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D21" s="8">
         <v>1.0</v>
       </c>
       <c r="E21" s="25">
-        <v>46155.86212506944</v>
+        <v>46155.86764509259</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -51384,23 +51374,21 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B22" s="36">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="C22" s="36">
         <v>30.0</v>
       </c>
       <c r="D22" s="8">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="E22" s="25">
-        <v>46156.84678416667</v>
+        <v>46155.86212506944</v>
       </c>
-      <c r="F22" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -51414,18 +51402,20 @@
         <v>16</v>
       </c>
       <c r="B23" s="36">
-        <v>17.0</v>
+        <v>10.0</v>
       </c>
       <c r="C23" s="36">
-        <v>15.0</v>
+        <v>30.0</v>
       </c>
       <c r="D23" s="8">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46155.877253784725</v>
+        <v>46156.84678416667</v>
       </c>
-      <c r="F23" s="4"/>
+      <c r="F23" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -51435,11 +51425,21 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="24"/>
+      <c r="A24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="36">
+        <v>17.0</v>
+      </c>
+      <c r="C24" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D24" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="25">
+        <v>46155.877253784725</v>
+      </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -51450,12 +51450,8 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" s="40" t="s">
-        <v>24</v>
-      </c>
+      <c r="A25" s="7"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="24"/>
@@ -51469,21 +51465,15 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>18</v>
+      <c r="A26" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B26" s="36">
-        <v>6.0</v>
+      <c r="B26" s="40" t="s">
+        <v>24</v>
       </c>
-      <c r="C26" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D26" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="25">
-        <v>46155.89164559028</v>
-      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="24"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51495,18 +51485,20 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B27" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C27" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D27" s="8">
         <v>1.0</v>
       </c>
-      <c r="E27" s="24"/>
+      <c r="E27" s="25">
+        <v>46155.89164559028</v>
+      </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51518,20 +51510,18 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B28" s="36">
-        <v>18.0</v>
+        <v>8.0</v>
       </c>
       <c r="C28" s="36">
-        <v>14.0</v>
+        <v>30.0</v>
       </c>
       <c r="D28" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E28" s="25">
-        <v>46155.89113405092</v>
-      </c>
+      <c r="E28" s="24"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51542,11 +51532,21 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="24"/>
+      <c r="A29" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C29" s="36">
+        <v>14.0</v>
+      </c>
+      <c r="D29" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="E29" s="25">
+        <v>46155.89113405092</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51557,13 +51557,11 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="27"/>
+      <c r="A30" s="7"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51574,21 +51572,13 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="s">
-        <v>6</v>
+      <c r="A31" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B31" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D31" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E31" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="27"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51600,10 +51590,10 @@
     </row>
     <row r="32">
       <c r="A32" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B32" s="41">
-        <v>30.0</v>
+      <c r="B32" s="41" t="s">
+        <v>26</v>
       </c>
       <c r="C32" s="41">
         <v>15.0</v>
@@ -51611,7 +51601,9 @@
       <c r="D32" s="41">
         <v>1.0</v>
       </c>
-      <c r="E32" s="27"/>
+      <c r="E32" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51622,11 +51614,19 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="16"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="24"/>
+      <c r="A33" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C33" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D33" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51637,9 +51637,7 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A34" s="16"/>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -51654,21 +51652,13 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="s">
-        <v>6</v>
+      <c r="A35" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B35" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C35" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D35" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E35" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="24"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51680,10 +51670,10 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C36" s="8">
         <v>20.0</v>
@@ -51692,7 +51682,7 @@
         <v>1.0</v>
       </c>
       <c r="E36" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -51705,23 +51695,21 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B37" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C37" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D37" s="8">
         <v>1.0</v>
       </c>
       <c r="E37" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F37" s="15" t="s">
-        <v>27</v>
-      </c>
+      <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
@@ -51731,14 +51719,24 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="42" t="s">
-        <v>28</v>
+      <c r="A38" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="4"/>
+      <c r="B38" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C38" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D38" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E38" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
@@ -51748,21 +51746,13 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="s">
-        <v>29</v>
+      <c r="A39" s="42" t="s">
+        <v>28</v>
       </c>
-      <c r="B39" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C39" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D39" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E39" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51774,19 +51764,19 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="B40" s="36">
         <v>2.0</v>
       </c>
       <c r="C40" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D40" s="36">
         <v>1.0</v>
       </c>
       <c r="E40" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51799,19 +51789,19 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C41" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D41" s="36">
         <v>1.0</v>
       </c>
       <c r="E41" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51823,11 +51813,21 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="24"/>
+      <c r="A42" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C42" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D42" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E42" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51838,17 +51838,11 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="A43" s="7"/>
+      <c r="B43" s="8"/>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
-      <c r="E43" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E43" s="24"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51859,16 +51853,16 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7">
-        <v>50.0</v>
+      <c r="A44" s="7" t="s">
+        <v>30</v>
       </c>
-      <c r="B44" s="8">
-        <v>100.0</v>
+      <c r="B44" s="8" t="s">
+        <v>31</v>
       </c>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
       <c r="E44" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51880,13 +51874,17 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="43" t="s">
-        <v>32</v>
+      <c r="A45" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B45" s="44"/>
-      <c r="C45" s="44"/>
-      <c r="D45" s="44"/>
-      <c r="E45" s="45"/>
+      <c r="B45" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51897,21 +51895,13 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="34" t="s">
-        <v>33</v>
+      <c r="A46" s="43" t="s">
+        <v>32</v>
       </c>
-      <c r="B46" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C46" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D46" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E46" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B46" s="44"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="45"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51922,11 +51912,21 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="35"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="A47" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C47" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D47" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E47" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51937,9 +51937,7 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="34" t="s">
-        <v>34</v>
-      </c>
+      <c r="A48" s="35"/>
       <c r="B48" s="35"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
@@ -51954,21 +51952,13 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
-        <v>7</v>
+      <c r="A49" s="34" t="s">
+        <v>34</v>
       </c>
-      <c r="B49" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C49" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D49" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E49" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B49" s="35"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -51979,18 +51969,20 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="34" t="s">
-        <v>35</v>
+      <c r="A50" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B50" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C50" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D50" s="4"/>
+      <c r="D50" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E50" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52002,11 +51994,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="35"/>
-      <c r="B51" s="35"/>
-      <c r="C51" s="4"/>
+      <c r="A51" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B51" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C51" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="E51" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52017,17 +52017,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B52" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A52" s="35"/>
+      <c r="B52" s="35"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
-      <c r="E52" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52039,19 +52033,15 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
-      <c r="B53" s="34">
-        <v>5.0</v>
+      <c r="B53" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C53" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D53" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
       <c r="E53" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52064,19 +52054,19 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B54" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C54" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D54" s="15">
         <v>1.0</v>
       </c>
       <c r="E54" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52089,10 +52079,10 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B55" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C55" s="15">
         <v>10.0</v>
@@ -52101,7 +52091,7 @@
         <v>1.0</v>
       </c>
       <c r="E55" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52113,11 +52103,21 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="35"/>
-      <c r="B56" s="35"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
+      <c r="A56" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B56" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C56" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D56" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E56" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -52128,17 +52128,11 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B57" s="34" t="s">
-        <v>28</v>
-      </c>
+      <c r="A57" s="35"/>
+      <c r="B57" s="35"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52150,18 +52144,16 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
-      <c r="B58" s="34">
-        <v>5.0</v>
+      <c r="B58" s="34" t="s">
+        <v>28</v>
       </c>
-      <c r="C58" s="15">
-        <v>80.0</v>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D58" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52173,13 +52165,13 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B59" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C59" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D59" s="15">
         <v>1.0</v>
@@ -52196,20 +52188,18 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B60" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C60" s="15">
         <v>10.0</v>
       </c>
       <c r="D60" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E60" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52220,11 +52210,21 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="35"/>
-      <c r="B61" s="35"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
+      <c r="A61" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B61" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C61" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D61" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E61" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52235,7 +52235,7 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="34"/>
+      <c r="A62" s="35"/>
       <c r="B62" s="35"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52250,7 +52250,7 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="35"/>
+      <c r="A63" s="34"/>
       <c r="B63" s="35"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
@@ -52265,8 +52265,8 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
+      <c r="A64" s="35"/>
+      <c r="B64" s="35"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -66334,6 +66334,21 @@
       <c r="L1001" s="4"/>
       <c r="M1001" s="4"/>
     </row>
+    <row r="1002">
+      <c r="A1002" s="4"/>
+      <c r="B1002" s="4"/>
+      <c r="C1002" s="4"/>
+      <c r="D1002" s="4"/>
+      <c r="E1002" s="4"/>
+      <c r="F1002" s="4"/>
+      <c r="G1002" s="4"/>
+      <c r="H1002" s="4"/>
+      <c r="I1002" s="4"/>
+      <c r="J1002" s="4"/>
+      <c r="K1002" s="4"/>
+      <c r="L1002" s="4"/>
+      <c r="M1002" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:18.324Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51022,7 +51022,7 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
-    <row r="4">
+    <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -51037,7 +51037,7 @@
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
     </row>
-    <row r="5">
+    <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -51052,7 +51052,7 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
     </row>
-    <row r="6">
+    <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -51067,7 +51067,7 @@
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
     </row>
-    <row r="7">
+    <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:28.392Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="40">
   <si>
     <t>項目</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>刀壓</t>
+  </si>
+  <si>
+    <t>Cut紙</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -51038,7 +51041,9 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5"/>
+      <c r="A5" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -51084,7 +51089,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -51166,10 +51171,10 @@
     </row>
     <row r="12">
       <c r="A12" s="39" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -51331,7 +51336,7 @@
         <v>8</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -51414,7 +51419,7 @@
         <v>46156.84678416667</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51469,7 +51474,7 @@
         <v>10</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -51593,7 +51598,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C32" s="41">
         <v>15.0</v>
@@ -51735,7 +51740,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51747,7 +51752,7 @@
     </row>
     <row r="39">
       <c r="A39" s="42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -51764,7 +51769,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B40" s="36">
         <v>2.0</v>
@@ -51854,10 +51859,10 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -51896,7 +51901,7 @@
     </row>
     <row r="46">
       <c r="A46" s="43" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B46" s="44"/>
       <c r="C46" s="44"/>
@@ -51913,7 +51918,7 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B47" s="34">
         <v>100.0</v>
@@ -51953,7 +51958,7 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
@@ -51995,7 +52000,7 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B51" s="34">
         <v>15.0</v>
@@ -52033,7 +52038,7 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B53" s="34" t="s">
         <v>12</v>
@@ -52054,7 +52059,7 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B54" s="34">
         <v>5.0</v>
@@ -52079,7 +52084,7 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B55" s="34">
         <v>15.0</v>
@@ -52144,10 +52149,10 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B58" s="34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
@@ -52165,7 +52170,7 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B59" s="34">
         <v>5.0</v>
@@ -52188,7 +52193,7 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B60" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:36.296Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>Cut紙</t>
+  </si>
+  <si>
+    <t>03mm</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -51058,7 +51061,9 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5"/>
+      <c r="A6" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
@@ -51089,7 +51094,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -51171,10 +51176,10 @@
     </row>
     <row r="12">
       <c r="A12" s="39" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -51336,7 +51341,7 @@
         <v>8</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -51419,7 +51424,7 @@
         <v>46156.84678416667</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51474,7 +51479,7 @@
         <v>10</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -51598,7 +51603,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C32" s="41">
         <v>15.0</v>
@@ -51740,7 +51745,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51752,7 +51757,7 @@
     </row>
     <row r="39">
       <c r="A39" s="42" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -51769,7 +51774,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B40" s="36">
         <v>2.0</v>
@@ -51859,10 +51864,10 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -51901,7 +51906,7 @@
     </row>
     <row r="46">
       <c r="A46" s="43" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B46" s="44"/>
       <c r="C46" s="44"/>
@@ -51918,7 +51923,7 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B47" s="34">
         <v>100.0</v>
@@ -51958,7 +51963,7 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
@@ -52000,7 +52005,7 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B51" s="34">
         <v>15.0</v>
@@ -52038,7 +52043,7 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B53" s="34" t="s">
         <v>12</v>
@@ -52059,7 +52064,7 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B54" s="34">
         <v>5.0</v>
@@ -52084,7 +52089,7 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B55" s="34">
         <v>15.0</v>
@@ -52149,10 +52154,10 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B58" s="34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
@@ -52170,7 +52175,7 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B59" s="34">
         <v>5.0</v>
@@ -52193,7 +52198,7 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B60" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:40.741Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51047,10 +51047,14 @@
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="17"/>
+      <c r="B5" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
-      <c r="E5" s="24"/>
+      <c r="E5" s="25">
+        <v>46156.86017103009</v>
+      </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51061,9 +51065,6 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:44.742Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -302,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -411,6 +411,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -51065,6 +51068,9 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="37" t="s">
+        <v>16</v>
+      </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
@@ -51162,10 +51168,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="39"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51176,10 +51182,10 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="41" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="8"/>
@@ -51242,10 +51248,10 @@
     </row>
     <row r="15">
       <c r="A15" s="5"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="38"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51338,10 +51344,10 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="41" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="17"/>
@@ -51476,10 +51482,10 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="39" t="s">
+      <c r="A26" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="41" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="17"/>
@@ -51603,13 +51609,13 @@
       <c r="A32" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="41" t="s">
+      <c r="B32" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="41">
+      <c r="C32" s="42">
         <v>15.0</v>
       </c>
-      <c r="D32" s="41">
+      <c r="D32" s="42">
         <v>1.0</v>
       </c>
       <c r="E32" s="26">
@@ -51628,13 +51634,13 @@
       <c r="A33" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="41">
+      <c r="B33" s="42">
         <v>30.0</v>
       </c>
-      <c r="C33" s="41">
+      <c r="C33" s="42">
         <v>15.0</v>
       </c>
-      <c r="D33" s="41">
+      <c r="D33" s="42">
         <v>1.0</v>
       </c>
       <c r="E33" s="27"/>
@@ -51757,7 +51763,7 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="42" t="s">
+      <c r="A39" s="43" t="s">
         <v>30</v>
       </c>
       <c r="B39" s="17"/>
@@ -51906,13 +51912,13 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="44"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="44"/>
-      <c r="E46" s="45"/>
+      <c r="B46" s="45"/>
+      <c r="C46" s="45"/>
+      <c r="D46" s="45"/>
+      <c r="E46" s="46"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51935,7 +51941,7 @@
       <c r="D47" s="15">
         <v>2.0</v>
       </c>
-      <c r="E47" s="46">
+      <c r="E47" s="47">
         <v>46009.783484375</v>
       </c>
       <c r="F47" s="4"/>
@@ -51992,7 +51998,7 @@
       <c r="D50" s="15">
         <v>1.0</v>
       </c>
-      <c r="E50" s="46">
+      <c r="E50" s="47">
         <v>46038.9559609375</v>
       </c>
       <c r="F50" s="4"/>
@@ -52015,7 +52021,7 @@
         <v>16.0</v>
       </c>
       <c r="D51" s="4"/>
-      <c r="E51" s="46">
+      <c r="E51" s="47">
         <v>46136.01284993056</v>
       </c>
       <c r="F51" s="4"/>
@@ -52051,7 +52057,7 @@
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="46">
+      <c r="E53" s="47">
         <v>46044.0116671875</v>
       </c>
       <c r="F53" s="4"/>
@@ -52076,7 +52082,7 @@
       <c r="D54" s="15">
         <v>1.0</v>
       </c>
-      <c r="E54" s="46">
+      <c r="E54" s="47">
         <v>46044.01310700232</v>
       </c>
       <c r="F54" s="4"/>
@@ -52101,7 +52107,7 @@
       <c r="D55" s="15">
         <v>1.0</v>
       </c>
-      <c r="E55" s="46">
+      <c r="E55" s="47">
         <v>46044.013194907406</v>
       </c>
       <c r="F55" s="4"/>
@@ -52126,7 +52132,7 @@
       <c r="D56" s="15">
         <v>1.0</v>
       </c>
-      <c r="E56" s="46">
+      <c r="E56" s="47">
         <v>46056.701985011576</v>
       </c>
       <c r="F56" s="4"/>
@@ -52162,7 +52168,7 @@
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="46">
+      <c r="E58" s="47">
         <v>46044.0136399537</v>
       </c>
       <c r="F58" s="4"/>
@@ -52233,7 +52239,7 @@
       <c r="D61" s="15">
         <v>6.0</v>
       </c>
-      <c r="E61" s="46">
+      <c r="E61" s="47">
         <v>46044.014003055556</v>
       </c>
       <c r="F61" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:49.039Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -302,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -411,9 +411,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -51055,9 +51052,7 @@
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
-      <c r="E5" s="25">
-        <v>46156.86017103009</v>
-      </c>
+      <c r="E5" s="25"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51068,12 +51063,18 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
+      <c r="B6" s="8">
+        <v>11.0</v>
+      </c>
+      <c r="C6" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D6" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E6" s="24"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -51168,10 +51169,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="38"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51182,10 +51183,10 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="40" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="8"/>
@@ -51248,10 +51249,10 @@
     </row>
     <row r="15">
       <c r="A15" s="5"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="39"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="38"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51344,10 +51345,10 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="40" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="17"/>
@@ -51482,10 +51483,10 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="17"/>
@@ -51609,13 +51610,13 @@
       <c r="A32" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="42" t="s">
+      <c r="B32" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="42">
+      <c r="C32" s="41">
         <v>15.0</v>
       </c>
-      <c r="D32" s="42">
+      <c r="D32" s="41">
         <v>1.0</v>
       </c>
       <c r="E32" s="26">
@@ -51634,13 +51635,13 @@
       <c r="A33" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="42">
+      <c r="B33" s="41">
         <v>30.0</v>
       </c>
-      <c r="C33" s="42">
+      <c r="C33" s="41">
         <v>15.0</v>
       </c>
-      <c r="D33" s="42">
+      <c r="D33" s="41">
         <v>1.0</v>
       </c>
       <c r="E33" s="27"/>
@@ -51763,7 +51764,7 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="43" t="s">
+      <c r="A39" s="42" t="s">
         <v>30</v>
       </c>
       <c r="B39" s="17"/>
@@ -51912,13 +51913,13 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="44" t="s">
+      <c r="A46" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="45"/>
-      <c r="C46" s="45"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="46"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="45"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51941,7 +51942,7 @@
       <c r="D47" s="15">
         <v>2.0</v>
       </c>
-      <c r="E47" s="47">
+      <c r="E47" s="46">
         <v>46009.783484375</v>
       </c>
       <c r="F47" s="4"/>
@@ -51998,7 +51999,7 @@
       <c r="D50" s="15">
         <v>1.0</v>
       </c>
-      <c r="E50" s="47">
+      <c r="E50" s="46">
         <v>46038.9559609375</v>
       </c>
       <c r="F50" s="4"/>
@@ -52021,7 +52022,7 @@
         <v>16.0</v>
       </c>
       <c r="D51" s="4"/>
-      <c r="E51" s="47">
+      <c r="E51" s="46">
         <v>46136.01284993056</v>
       </c>
       <c r="F51" s="4"/>
@@ -52057,7 +52058,7 @@
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="47">
+      <c r="E53" s="46">
         <v>46044.0116671875</v>
       </c>
       <c r="F53" s="4"/>
@@ -52082,7 +52083,7 @@
       <c r="D54" s="15">
         <v>1.0</v>
       </c>
-      <c r="E54" s="47">
+      <c r="E54" s="46">
         <v>46044.01310700232</v>
       </c>
       <c r="F54" s="4"/>
@@ -52107,7 +52108,7 @@
       <c r="D55" s="15">
         <v>1.0</v>
       </c>
-      <c r="E55" s="47">
+      <c r="E55" s="46">
         <v>46044.013194907406</v>
       </c>
       <c r="F55" s="4"/>
@@ -52132,7 +52133,7 @@
       <c r="D56" s="15">
         <v>1.0</v>
       </c>
-      <c r="E56" s="47">
+      <c r="E56" s="46">
         <v>46056.701985011576</v>
       </c>
       <c r="F56" s="4"/>
@@ -52168,7 +52169,7 @@
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="47">
+      <c r="E58" s="46">
         <v>46044.0136399537</v>
       </c>
       <c r="F58" s="4"/>
@@ -52239,7 +52240,7 @@
       <c r="D61" s="15">
         <v>6.0</v>
       </c>
-      <c r="E61" s="47">
+      <c r="E61" s="46">
         <v>46044.014003055556</v>
       </c>
       <c r="F61" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:38:55.884Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51067,15 +51067,17 @@
         <v>16</v>
       </c>
       <c r="B6" s="8">
-        <v>11.0</v>
+        <v>6.0</v>
       </c>
       <c r="C6" s="8">
-        <v>20.0</v>
+        <v>60.0</v>
       </c>
       <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="24"/>
+      <c r="E6" s="25">
+        <v>46156.860351111114</v>
+      </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:46:39.564Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="40">
   <si>
     <t>項目</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>刀壓</t>
-  </si>
-  <si>
-    <t>Cut紙</t>
   </si>
   <si>
     <t>03mm</t>
@@ -51045,10 +51042,10 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -51104,7 +51101,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -51186,10 +51183,10 @@
     </row>
     <row r="12">
       <c r="A12" s="39" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -51351,7 +51348,7 @@
         <v>8</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -51434,7 +51431,7 @@
         <v>46156.84678416667</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -51489,7 +51486,7 @@
         <v>10</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -51613,7 +51610,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C32" s="41">
         <v>15.0</v>
@@ -51755,7 +51752,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51767,7 +51764,7 @@
     </row>
     <row r="39">
       <c r="A39" s="42" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -51784,7 +51781,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40" s="36">
         <v>2.0</v>
@@ -51874,10 +51871,10 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -51916,7 +51913,7 @@
     </row>
     <row r="46">
       <c r="A46" s="43" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B46" s="44"/>
       <c r="C46" s="44"/>
@@ -51933,7 +51930,7 @@
     </row>
     <row r="47">
       <c r="A47" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B47" s="34">
         <v>100.0</v>
@@ -51973,7 +51970,7 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
@@ -52015,7 +52012,7 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B51" s="34">
         <v>15.0</v>
@@ -52053,7 +52050,7 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B53" s="34" t="s">
         <v>12</v>
@@ -52074,7 +52071,7 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B54" s="34">
         <v>5.0</v>
@@ -52099,7 +52096,7 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B55" s="34">
         <v>15.0</v>
@@ -52164,10 +52161,10 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B58" s="34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
@@ -52185,7 +52182,7 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B59" s="34">
         <v>5.0</v>
@@ -52208,7 +52205,7 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B60" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T12:46:56.199Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="40">
   <si>
     <t>項目</t>
   </si>
@@ -17866,10 +17866,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
+      <c r="A36" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17883,10 +17887,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
+      <c r="A37" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="C37" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="D37" s="17"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17900,10 +17910,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
+      <c r="A38" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="C38" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="D38" s="17"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T15:22:19.932Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51217,18 +51217,10 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="C13" s="8">
-        <v>30.0</v>
-      </c>
-      <c r="D13" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="25"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -51241,13 +51233,13 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B14" s="8">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="C14" s="8">
-        <v>20.0</v>
+        <v>30.0</v>
       </c>
       <c r="D14" s="8">
         <v>1.0</v>
@@ -51263,11 +51255,19 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="38"/>
+      <c r="A15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C15" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D15" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E15" s="25"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51278,13 +51278,11 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="24"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="38"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51295,21 +51293,13 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>6</v>
+      <c r="A17" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B17" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C17" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D17" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E17" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51321,10 +51311,10 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B18" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C18" s="36">
         <v>20.0</v>
@@ -51333,7 +51323,7 @@
         <v>1.0</v>
       </c>
       <c r="E18" s="25">
-        <v>46155.874796793985</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -51345,11 +51335,21 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="24"/>
+      <c r="A19" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C19" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D19" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E19" s="25">
+        <v>46155.874796793985</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51360,17 +51360,11 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="40" t="s">
-        <v>25</v>
-      </c>
+      <c r="A20" s="7"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="25">
-        <v>46155.850816817125</v>
-      </c>
+      <c r="E20" s="24"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51381,20 +51375,16 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>18</v>
+      <c r="A21" s="39" t="s">
+        <v>8</v>
       </c>
-      <c r="B21" s="36">
-        <v>6.0</v>
+      <c r="B21" s="40" t="s">
+        <v>25</v>
       </c>
-      <c r="C21" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D21" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
       <c r="E21" s="25">
-        <v>46155.86764509259</v>
+        <v>46155.850816817125</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -51407,19 +51397,19 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B22" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C22" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D22" s="8">
         <v>1.0</v>
       </c>
       <c r="E22" s="25">
-        <v>46155.86212506944</v>
+        <v>46155.86764509259</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51432,23 +51422,21 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B23" s="36">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="C23" s="36">
         <v>30.0</v>
       </c>
       <c r="D23" s="8">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46156.84678416667</v>
+        <v>46155.86212506944</v>
       </c>
-      <c r="F23" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -51462,18 +51450,20 @@
         <v>16</v>
       </c>
       <c r="B24" s="36">
-        <v>17.0</v>
+        <v>10.0</v>
       </c>
       <c r="C24" s="36">
-        <v>15.0</v>
+        <v>30.0</v>
       </c>
       <c r="D24" s="8">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="E24" s="25">
-        <v>46155.877253784725</v>
+        <v>46156.84678416667</v>
       </c>
-      <c r="F24" s="4"/>
+      <c r="F24" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -51483,11 +51473,21 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="24"/>
+      <c r="A25" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="36">
+        <v>17.0</v>
+      </c>
+      <c r="C25" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D25" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="25">
+        <v>46155.877253784725</v>
+      </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51498,12 +51498,8 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="40" t="s">
-        <v>25</v>
-      </c>
+      <c r="A26" s="7"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
       <c r="E26" s="24"/>
@@ -51517,21 +51513,15 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>18</v>
+      <c r="A27" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="36">
-        <v>6.0</v>
+      <c r="B27" s="40" t="s">
+        <v>25</v>
       </c>
-      <c r="C27" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D27" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E27" s="25">
-        <v>46155.89164559028</v>
-      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51543,18 +51533,20 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B28" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C28" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D28" s="8">
         <v>1.0</v>
       </c>
-      <c r="E28" s="24"/>
+      <c r="E28" s="25">
+        <v>46155.89164559028</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51566,20 +51558,18 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B29" s="36">
-        <v>18.0</v>
+        <v>8.0</v>
       </c>
       <c r="C29" s="36">
-        <v>14.0</v>
+        <v>30.0</v>
       </c>
       <c r="D29" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E29" s="25">
-        <v>46155.89113405092</v>
-      </c>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51590,11 +51580,21 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="24"/>
+      <c r="A30" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C30" s="36">
+        <v>14.0</v>
+      </c>
+      <c r="D30" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="E30" s="25">
+        <v>46155.89113405092</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51605,13 +51605,11 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="27"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="24"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51622,21 +51620,13 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="s">
-        <v>6</v>
+      <c r="A32" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B32" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C32" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D32" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E32" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="27"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51648,10 +51638,10 @@
     </row>
     <row r="33">
       <c r="A33" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B33" s="41">
-        <v>30.0</v>
+      <c r="B33" s="41" t="s">
+        <v>27</v>
       </c>
       <c r="C33" s="41">
         <v>15.0</v>
@@ -51659,7 +51649,9 @@
       <c r="D33" s="41">
         <v>1.0</v>
       </c>
-      <c r="E33" s="27"/>
+      <c r="E33" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51670,11 +51662,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="16"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="24"/>
+      <c r="A34" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C34" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D34" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E34" s="27"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51685,9 +51685,7 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A35" s="16"/>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -51702,21 +51700,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="s">
-        <v>6</v>
+      <c r="A36" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B36" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C36" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D36" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E36" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51728,10 +51718,10 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C37" s="8">
         <v>20.0</v>
@@ -51740,7 +51730,7 @@
         <v>1.0</v>
       </c>
       <c r="E37" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51753,23 +51743,21 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B38" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C38" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D38" s="8">
         <v>1.0</v>
       </c>
       <c r="E38" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F38" s="15" t="s">
-        <v>28</v>
-      </c>
+      <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
@@ -51779,14 +51767,24 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="42" t="s">
-        <v>29</v>
+      <c r="A39" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="4"/>
+      <c r="B39" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C39" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D39" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E39" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
@@ -51796,21 +51794,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>30</v>
+      <c r="A40" s="42" t="s">
+        <v>29</v>
       </c>
-      <c r="B40" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C40" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D40" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E40" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="24"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51822,19 +51812,19 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B41" s="36">
         <v>2.0</v>
       </c>
       <c r="C41" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D41" s="36">
         <v>1.0</v>
       </c>
       <c r="E41" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51847,19 +51837,19 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C42" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D42" s="36">
         <v>1.0</v>
       </c>
       <c r="E42" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -51871,11 +51861,21 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="24"/>
+      <c r="A43" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C43" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D43" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E43" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51886,17 +51886,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>32</v>
-      </c>
+      <c r="A44" s="7"/>
+      <c r="B44" s="8"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
-      <c r="E44" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E44" s="24"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51907,16 +51901,16 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7">
-        <v>50.0</v>
+      <c r="A45" s="7" t="s">
+        <v>31</v>
       </c>
-      <c r="B45" s="8">
-        <v>100.0</v>
+      <c r="B45" s="8" t="s">
+        <v>32</v>
       </c>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
       <c r="E45" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51928,13 +51922,17 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="43" t="s">
-        <v>33</v>
+      <c r="A46" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B46" s="44"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="44"/>
-      <c r="E46" s="45"/>
+      <c r="B46" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51945,21 +51943,13 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="34" t="s">
-        <v>34</v>
+      <c r="A47" s="43" t="s">
+        <v>33</v>
       </c>
-      <c r="B47" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C47" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D47" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E47" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B47" s="44"/>
+      <c r="C47" s="44"/>
+      <c r="D47" s="44"/>
+      <c r="E47" s="45"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51970,11 +51960,21 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="35"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="A48" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B48" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C48" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D48" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E48" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51985,9 +51985,7 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="34" t="s">
-        <v>35</v>
-      </c>
+      <c r="A49" s="35"/>
       <c r="B49" s="35"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -52002,21 +52000,13 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="s">
-        <v>7</v>
+      <c r="A50" s="34" t="s">
+        <v>35</v>
       </c>
-      <c r="B50" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C50" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D50" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E50" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B50" s="35"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52027,18 +52017,20 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="34" t="s">
-        <v>36</v>
+      <c r="A51" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B51" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C51" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D51" s="4"/>
+      <c r="D51" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E51" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -52050,11 +52042,19 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="35"/>
-      <c r="B52" s="35"/>
-      <c r="C52" s="4"/>
+      <c r="A52" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C52" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
+      <c r="E52" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52065,17 +52065,11 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52087,19 +52081,15 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B54" s="34">
-        <v>5.0</v>
+      <c r="B54" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C54" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D54" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
       <c r="E54" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52112,19 +52102,19 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B55" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C55" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D55" s="15">
         <v>1.0</v>
       </c>
       <c r="E55" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52137,10 +52127,10 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B56" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C56" s="15">
         <v>10.0</v>
@@ -52149,7 +52139,7 @@
         <v>1.0</v>
       </c>
       <c r="E56" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52161,11 +52151,21 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="35"/>
-      <c r="B57" s="35"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="A57" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C57" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D57" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E57" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52176,17 +52176,11 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B58" s="34" t="s">
-        <v>29</v>
-      </c>
+      <c r="A58" s="35"/>
+      <c r="B58" s="35"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52198,18 +52192,16 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B59" s="34">
-        <v>5.0</v>
+      <c r="B59" s="34" t="s">
+        <v>29</v>
       </c>
-      <c r="C59" s="15">
-        <v>80.0</v>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D59" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52221,13 +52213,13 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B60" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C60" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D60" s="15">
         <v>1.0</v>
@@ -52244,20 +52236,18 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B61" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C61" s="15">
         <v>10.0</v>
       </c>
       <c r="D61" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E61" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52268,11 +52258,21 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="35"/>
-      <c r="B62" s="35"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="A62" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B62" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C62" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D62" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E62" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52283,7 +52283,7 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="34"/>
+      <c r="A63" s="35"/>
       <c r="B63" s="35"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
@@ -52298,7 +52298,7 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="35"/>
+      <c r="A64" s="34"/>
       <c r="B64" s="35"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
@@ -52313,8 +52313,8 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
+      <c r="A65" s="35"/>
+      <c r="B65" s="35"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
@@ -66382,6 +66382,21 @@
       <c r="L1002" s="4"/>
       <c r="M1002" s="4"/>
     </row>
+    <row r="1003">
+      <c r="A1003" s="4"/>
+      <c r="B1003" s="4"/>
+      <c r="C1003" s="4"/>
+      <c r="D1003" s="4"/>
+      <c r="E1003" s="4"/>
+      <c r="F1003" s="4"/>
+      <c r="G1003" s="4"/>
+      <c r="H1003" s="4"/>
+      <c r="I1003" s="4"/>
+      <c r="J1003" s="4"/>
+      <c r="K1003" s="4"/>
+      <c r="L1003" s="4"/>
+      <c r="M1003" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-14T15:22:45.175Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="40">
   <si>
     <t>項目</t>
   </si>
@@ -51217,9 +51217,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
+      <c r="A13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="C13" s="8">
+        <v>50.0</v>
+      </c>
       <c r="D13" s="8"/>
       <c r="E13" s="25"/>
       <c r="F13" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-16T12:09:42.959Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51227,7 +51227,9 @@
         <v>50.0</v>
       </c>
       <c r="D13" s="8"/>
-      <c r="E13" s="25"/>
+      <c r="E13" s="25">
+        <v>46156.98310679398</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51265,7 +51267,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="8">
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="C15" s="8">
         <v>20.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-16T13:10:36.216Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51275,7 +51275,9 @@
       <c r="D15" s="8">
         <v>1.0</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="25">
+        <v>46158.840069502316</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51592,7 +51594,7 @@
         <v>7</v>
       </c>
       <c r="B30" s="36">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
       <c r="C30" s="36">
         <v>14.0</v>
@@ -51601,7 +51603,7 @@
         <v>2.0</v>
       </c>
       <c r="E30" s="25">
-        <v>46155.89113405092</v>
+        <v>46158.8823238426</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-16T13:11:05.906Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51597,13 +51597,13 @@
         <v>15.0</v>
       </c>
       <c r="C30" s="36">
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="D30" s="8">
         <v>2.0</v>
       </c>
       <c r="E30" s="25">
-        <v>46158.8823238426</v>
+        <v>46158.88268241898</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:25:14.354Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51263,21 +51263,11 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="C15" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D15" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="25">
-        <v>46158.840069502316</v>
-      </c>
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="25"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51288,11 +51278,21 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="38"/>
+      <c r="A16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="8">
+        <v>12.0</v>
+      </c>
+      <c r="C16" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E16" s="25">
+        <v>46158.840069502316</v>
+      </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51303,13 +51303,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="38"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51320,21 +51318,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="C18" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="D18" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="25">
-        <v>46118.87534236111</v>
-      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51346,10 +51336,10 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" s="36">
-        <v>18.0</v>
+        <v>6.0</v>
       </c>
       <c r="C19" s="36">
         <v>20.0</v>
@@ -51358,7 +51348,7 @@
         <v>1.0</v>
       </c>
       <c r="E19" s="25">
-        <v>46155.874796793985</v>
+        <v>46118.87534236111</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51370,11 +51360,21 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="24"/>
+      <c r="A20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="36">
+        <v>18.0</v>
+      </c>
+      <c r="C20" s="36">
+        <v>20.0</v>
+      </c>
+      <c r="D20" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E20" s="25">
+        <v>46155.874796793985</v>
+      </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -51385,17 +51385,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" s="40" t="s">
-        <v>25</v>
-      </c>
+      <c r="A21" s="7"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="25">
-        <v>46155.850816817125</v>
-      </c>
+      <c r="E21" s="24"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51406,20 +51400,16 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>18</v>
+      <c r="A22" s="39" t="s">
+        <v>8</v>
       </c>
-      <c r="B22" s="36">
-        <v>6.0</v>
+      <c r="B22" s="40" t="s">
+        <v>25</v>
       </c>
-      <c r="C22" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D22" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
       <c r="E22" s="25">
-        <v>46155.86764509259</v>
+        <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51432,19 +51422,19 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B23" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C23" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D23" s="8">
         <v>1.0</v>
       </c>
       <c r="E23" s="25">
-        <v>46155.86212506944</v>
+        <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -51457,23 +51447,21 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B24" s="36">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="C24" s="36">
         <v>30.0</v>
       </c>
       <c r="D24" s="8">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="E24" s="25">
-        <v>46156.84678416667</v>
+        <v>46155.86212506944</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -51487,18 +51475,20 @@
         <v>16</v>
       </c>
       <c r="B25" s="36">
-        <v>17.0</v>
+        <v>10.0</v>
       </c>
       <c r="C25" s="36">
-        <v>15.0</v>
+        <v>30.0</v>
       </c>
       <c r="D25" s="8">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="E25" s="25">
-        <v>46155.877253784725</v>
+        <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="4"/>
+      <c r="F25" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -51508,11 +51498,21 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="24"/>
+      <c r="A26" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="36">
+        <v>17.0</v>
+      </c>
+      <c r="C26" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="D26" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E26" s="25">
+        <v>46155.877253784725</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51523,12 +51523,8 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" s="40" t="s">
-        <v>25</v>
-      </c>
+      <c r="A27" s="7"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="24"/>
@@ -51542,21 +51538,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>18</v>
+      <c r="A28" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="36">
-        <v>6.0</v>
+      <c r="B28" s="40" t="s">
+        <v>25</v>
       </c>
-      <c r="C28" s="36">
-        <v>50.0</v>
-      </c>
-      <c r="D28" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E28" s="25">
-        <v>46155.89164559028</v>
-      </c>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="24"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51568,18 +51558,20 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B29" s="36">
-        <v>8.0</v>
+        <v>6.0</v>
       </c>
       <c r="C29" s="36">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="D29" s="8">
         <v>1.0</v>
       </c>
-      <c r="E29" s="24"/>
+      <c r="E29" s="25">
+        <v>46155.89164559028</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51591,20 +51583,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" s="36">
-        <v>15.0</v>
+        <v>8.0</v>
       </c>
       <c r="C30" s="36">
-        <v>10.0</v>
+        <v>30.0</v>
       </c>
       <c r="D30" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E30" s="25">
-        <v>46158.88268241898</v>
-      </c>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51615,11 +51605,21 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="24"/>
+      <c r="A31" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="36">
+        <v>15.0</v>
+      </c>
+      <c r="C31" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D31" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="E31" s="25">
+        <v>46158.88268241898</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51630,13 +51630,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="27"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="24"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51647,21 +51645,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="s">
-        <v>6</v>
+      <c r="A33" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B33" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C33" s="41">
-        <v>15.0</v>
-      </c>
-      <c r="D33" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="E33" s="26">
-        <v>46117.900830185186</v>
-      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51673,10 +51663,10 @@
     </row>
     <row r="34">
       <c r="A34" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B34" s="41">
-        <v>30.0</v>
+      <c r="B34" s="41" t="s">
+        <v>27</v>
       </c>
       <c r="C34" s="41">
         <v>15.0</v>
@@ -51684,7 +51674,9 @@
       <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="27"/>
+      <c r="E34" s="26">
+        <v>46117.900830185186</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51695,11 +51687,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="16"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="24"/>
+      <c r="A35" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="41">
+        <v>30.0</v>
+      </c>
+      <c r="C35" s="41">
+        <v>15.0</v>
+      </c>
+      <c r="D35" s="41">
+        <v>1.0</v>
+      </c>
+      <c r="E35" s="27"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51710,9 +51710,7 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A36" s="16"/>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -51727,21 +51725,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="s">
-        <v>6</v>
+      <c r="A37" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B37" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C37" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D37" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E37" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="24"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51753,10 +51743,10 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C38" s="8">
         <v>20.0</v>
@@ -51765,7 +51755,7 @@
         <v>1.0</v>
       </c>
       <c r="E38" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51778,23 +51768,21 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B39" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C39" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D39" s="8">
         <v>1.0</v>
       </c>
       <c r="E39" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F39" s="15" t="s">
-        <v>28</v>
-      </c>
+      <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
@@ -51804,14 +51792,24 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="42" t="s">
-        <v>29</v>
+      <c r="A40" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="4"/>
+      <c r="B40" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C40" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D40" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E40" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
@@ -51821,21 +51819,13 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>30</v>
+      <c r="A41" s="42" t="s">
+        <v>29</v>
       </c>
-      <c r="B41" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C41" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D41" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E41" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="24"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51847,19 +51837,19 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B42" s="36">
         <v>2.0</v>
       </c>
       <c r="C42" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D42" s="36">
         <v>1.0</v>
       </c>
       <c r="E42" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -51872,19 +51862,19 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C43" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D43" s="36">
         <v>1.0</v>
       </c>
       <c r="E43" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -51896,11 +51886,21 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="24"/>
+      <c r="A44" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C44" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D44" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E44" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51911,17 +51911,11 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>32</v>
-      </c>
+      <c r="A45" s="7"/>
+      <c r="B45" s="8"/>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
-      <c r="E45" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E45" s="24"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51932,16 +51926,16 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7">
-        <v>50.0</v>
+      <c r="A46" s="7" t="s">
+        <v>31</v>
       </c>
-      <c r="B46" s="8">
-        <v>100.0</v>
+      <c r="B46" s="8" t="s">
+        <v>32</v>
       </c>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
       <c r="E46" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51953,13 +51947,17 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="43" t="s">
-        <v>33</v>
+      <c r="A47" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B47" s="44"/>
-      <c r="C47" s="44"/>
-      <c r="D47" s="44"/>
-      <c r="E47" s="45"/>
+      <c r="B47" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51970,21 +51968,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="34" t="s">
-        <v>34</v>
+      <c r="A48" s="43" t="s">
+        <v>33</v>
       </c>
-      <c r="B48" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C48" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D48" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E48" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B48" s="44"/>
+      <c r="C48" s="44"/>
+      <c r="D48" s="44"/>
+      <c r="E48" s="45"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -51995,11 +51985,21 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="35"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="A49" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C49" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D49" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E49" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52010,9 +52010,7 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="34" t="s">
-        <v>35</v>
-      </c>
+      <c r="A50" s="35"/>
       <c r="B50" s="35"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
@@ -52027,21 +52025,13 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>7</v>
+      <c r="A51" s="34" t="s">
+        <v>35</v>
       </c>
-      <c r="B51" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C51" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D51" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E51" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B51" s="35"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52052,18 +52042,20 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="34" t="s">
-        <v>36</v>
+      <c r="A52" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B52" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C52" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D52" s="4"/>
+      <c r="D52" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E52" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52075,11 +52067,19 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="35"/>
-      <c r="B53" s="35"/>
-      <c r="C53" s="4"/>
+      <c r="A53" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B53" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C53" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
+      <c r="E53" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52090,17 +52090,11 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B54" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A54" s="35"/>
+      <c r="B54" s="35"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52112,19 +52106,15 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B55" s="34">
-        <v>5.0</v>
+      <c r="B55" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C55" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D55" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
       <c r="E55" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52137,19 +52127,19 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B56" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C56" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D56" s="15">
         <v>1.0</v>
       </c>
       <c r="E56" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52162,10 +52152,10 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B57" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C57" s="15">
         <v>10.0</v>
@@ -52174,7 +52164,7 @@
         <v>1.0</v>
       </c>
       <c r="E57" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -52186,11 +52176,21 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="35"/>
-      <c r="B58" s="35"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
+      <c r="A58" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C58" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D58" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E58" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52201,17 +52201,11 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B59" s="34" t="s">
-        <v>29</v>
-      </c>
+      <c r="A59" s="35"/>
+      <c r="B59" s="35"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
-      <c r="E59" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52223,18 +52217,16 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B60" s="34">
-        <v>5.0</v>
+      <c r="B60" s="34" t="s">
+        <v>29</v>
       </c>
-      <c r="C60" s="15">
-        <v>80.0</v>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D60" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52246,13 +52238,13 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B61" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C61" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D61" s="15">
         <v>1.0</v>
@@ -52269,20 +52261,18 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B62" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C62" s="15">
         <v>10.0</v>
       </c>
       <c r="D62" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E62" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52293,11 +52283,21 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="35"/>
-      <c r="B63" s="35"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="A63" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B63" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C63" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D63" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E63" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52308,7 +52308,7 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="34"/>
+      <c r="A64" s="35"/>
       <c r="B64" s="35"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
@@ -52323,7 +52323,7 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="35"/>
+      <c r="A65" s="34"/>
       <c r="B65" s="35"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
@@ -52338,8 +52338,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="4"/>
-      <c r="B66" s="4"/>
+      <c r="A66" s="35"/>
+      <c r="B66" s="35"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -66407,6 +66407,21 @@
       <c r="L1003" s="4"/>
       <c r="M1003" s="4"/>
     </row>
+    <row r="1004">
+      <c r="A1004" s="4"/>
+      <c r="B1004" s="4"/>
+      <c r="C1004" s="4"/>
+      <c r="D1004" s="4"/>
+      <c r="E1004" s="4"/>
+      <c r="F1004" s="4"/>
+      <c r="G1004" s="4"/>
+      <c r="H1004" s="4"/>
+      <c r="I1004" s="4"/>
+      <c r="J1004" s="4"/>
+      <c r="K1004" s="4"/>
+      <c r="L1004" s="4"/>
+      <c r="M1004" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:25:18.906Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>PS</t>
+  </si>
+  <si>
+    <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
@@ -51263,12 +51266,16 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7"/>
+      <c r="A15" s="7" t="s">
+        <v>26</v>
+      </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="25"/>
-      <c r="F15" s="4"/>
+      <c r="F15" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -51487,7 +51494,7 @@
         <v>46156.84678416667</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51666,7 +51673,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="41" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C34" s="41">
         <v>15.0</v>
@@ -51808,7 +51815,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51820,7 +51827,7 @@
     </row>
     <row r="41">
       <c r="A41" s="42" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
@@ -51837,7 +51844,7 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B42" s="36">
         <v>2.0</v>
@@ -51927,10 +51934,10 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
@@ -51969,7 +51976,7 @@
     </row>
     <row r="48">
       <c r="A48" s="43" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B48" s="44"/>
       <c r="C48" s="44"/>
@@ -51986,7 +51993,7 @@
     </row>
     <row r="49">
       <c r="A49" s="34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B49" s="34">
         <v>100.0</v>
@@ -52026,7 +52033,7 @@
     </row>
     <row r="51">
       <c r="A51" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B51" s="35"/>
       <c r="C51" s="4"/>
@@ -52068,7 +52075,7 @@
     </row>
     <row r="53">
       <c r="A53" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B53" s="34">
         <v>15.0</v>
@@ -52106,7 +52113,7 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B55" s="34" t="s">
         <v>12</v>
@@ -52127,7 +52134,7 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B56" s="34">
         <v>5.0</v>
@@ -52152,7 +52159,7 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B57" s="34">
         <v>15.0</v>
@@ -52217,10 +52224,10 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B60" s="34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
@@ -52238,7 +52245,7 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B61" s="34">
         <v>5.0</v>
@@ -52261,7 +52268,7 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B62" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:25:23.157Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51269,10 +51269,14 @@
       <c r="A15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="8"/>
+      <c r="B15" s="8">
+        <v>10.0</v>
+      </c>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
-      <c r="E15" s="25"/>
+      <c r="E15" s="25">
+        <v>46160.850943067126</v>
+      </c>
       <c r="F15" s="15" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:25:26.283Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51272,10 +51272,14 @@
       <c r="B15" s="8">
         <v>10.0</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+      <c r="C15" s="8">
+        <v>30.0</v>
+      </c>
+      <c r="D15" s="8">
+        <v>2.0</v>
+      </c>
       <c r="E15" s="25">
-        <v>46160.850943067126</v>
+        <v>46160.85097443287</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:29:30.499Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51270,16 +51270,16 @@
         <v>26</v>
       </c>
       <c r="B15" s="8">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="C15" s="8">
         <v>30.0</v>
       </c>
       <c r="D15" s="8">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="E15" s="25">
-        <v>46160.85097443287</v>
+        <v>46160.85380729167</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T12:33:18.843Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51227,11 +51227,11 @@
         <v>5.0</v>
       </c>
       <c r="C13" s="8">
-        <v>50.0</v>
+        <v>60.0</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="25">
-        <v>46156.98310679398</v>
+        <v>46160.85645340278</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-18T13:08:52.378Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51229,7 +51229,9 @@
       <c r="C13" s="8">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8"/>
+      <c r="D13" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E13" s="25">
         <v>46160.85645340278</v>
       </c>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-05-27T14:37:44.945Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51233,7 +51233,7 @@
         <v>1.0</v>
       </c>
       <c r="E13" s="25">
-        <v>46160.85645340278</v>
+        <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -51632,10 +51632,10 @@
         <v>10.0</v>
       </c>
       <c r="D31" s="8">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="E31" s="25">
-        <v>46158.88268241898</v>
+        <v>46169.942858842594</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-03T14:59:13.433Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51632,10 +51632,10 @@
         <v>10.0</v>
       </c>
       <c r="D31" s="8">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E31" s="25">
-        <v>46169.942858842594</v>
+        <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-09T09:07:54.219Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34669,15 +34669,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34689,23 +34685,17 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>6</v>
+      <c r="A7" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B7" s="11">
-        <v>4.0</v>
+      <c r="B7" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="C7" s="11">
-        <v>10.0</v>
-      </c>
-      <c r="D7" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="E7" s="14">
-        <v>45957.92965825232</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -34716,10 +34706,10 @@
     </row>
     <row r="8">
       <c r="A8" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="11">
-        <v>20.0</v>
+        <v>4.0</v>
       </c>
       <c r="C8" s="11">
         <v>10.0</v>
@@ -34728,7 +34718,7 @@
         <v>1.0</v>
       </c>
       <c r="E8" s="14">
-        <v>46116.685309016204</v>
+        <v>45957.92965825232</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
@@ -34741,13 +34731,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="16"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
+      <c r="A9" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="11">
+        <v>20.0</v>
+      </c>
+      <c r="C9" s="11">
+        <v>10.0</v>
+      </c>
+      <c r="D9" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="E9" s="14">
+        <v>46116.685309016204</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34757,12 +34757,10 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="17"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="8"/>
       <c r="C10" s="17"/>
-      <c r="D10" s="8"/>
+      <c r="D10" s="17"/>
       <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -34775,23 +34773,15 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
+      <c r="A11" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="B11" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="C11" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E11" s="9">
-        <v>46042.0</v>
-      </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -34808,14 +34798,16 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="8">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="D12" s="8">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="E12" s="9">
+        <v>46042.0</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
@@ -34826,13 +34818,13 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" s="8">
-        <v>32.0</v>
+        <v>5.0</v>
       </c>
       <c r="C13" s="8">
-        <v>5.0</v>
+        <v>15.0</v>
       </c>
       <c r="D13" s="8">
         <v>1.0</v>
@@ -34849,10 +34841,18 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="16"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="A14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="8">
+        <v>32.0</v>
+      </c>
+      <c r="C14" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -34865,13 +34865,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="12"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34883,18 +34881,12 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>6</v>
+      <c r="A16" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B16" s="11">
-        <v>5.0</v>
-      </c>
-      <c r="C16" s="11">
-        <v>5.0</v>
-      </c>
-      <c r="D16" s="11">
-        <v>1.0</v>
-      </c>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34908,10 +34900,10 @@
     </row>
     <row r="17">
       <c r="A17" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B17" s="11">
-        <v>50.0</v>
+        <v>5.0</v>
       </c>
       <c r="C17" s="11">
         <v>5.0</v>
@@ -34931,11 +34923,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="6"/>
+      <c r="A18" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="11">
+        <v>50.0</v>
+      </c>
+      <c r="C18" s="11">
+        <v>5.0</v>
+      </c>
+      <c r="D18" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="E18" s="12"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34947,9 +34947,7 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>12</v>
-      </c>
+      <c r="A19" s="16"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
@@ -34965,18 +34963,12 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>6</v>
+      <c r="A20" s="5" t="s">
+        <v>12</v>
       </c>
-      <c r="B20" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="C20" s="8">
-        <v>5.0</v>
-      </c>
-      <c r="D20" s="8">
-        <v>1.0</v>
-      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
       <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -34990,11 +34982,17 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
+      <c r="B21" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="C21" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="D21" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35007,7 +35005,9 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="16"/>
+      <c r="A22" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
@@ -35023,13 +35023,11 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="12"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="6"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35041,18 +35039,12 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>6</v>
+      <c r="A24" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B24" s="11">
-        <v>5.0</v>
-      </c>
-      <c r="C24" s="11">
-        <v>5.0</v>
-      </c>
-      <c r="D24" s="11">
-        <v>1.0</v>
-      </c>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
       <c r="E24" s="12"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -35065,17 +35057,19 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="s">
-        <v>7</v>
+      <c r="A25" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B25" s="20">
-        <v>55.0</v>
+      <c r="B25" s="11">
+        <v>5.0</v>
       </c>
-      <c r="C25" s="20">
-        <v>2.0</v>
+      <c r="C25" s="11">
+        <v>5.0</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="E25" s="12"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35087,11 +35081,17 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
+      <c r="A26" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="20">
+        <v>55.0</v>
+      </c>
+      <c r="C26" s="20">
+        <v>2.0</v>
+      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="22"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35103,17 +35103,11 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>15</v>
-      </c>
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
-      <c r="E27" s="23">
-        <v>46051.96156388889</v>
-      </c>
+      <c r="E27" s="17"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35126,17 +35120,15 @@
     </row>
     <row r="28">
       <c r="A28" s="8" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
-      <c r="B28" s="8">
-        <v>2.0</v>
+      <c r="B28" s="8" t="s">
+        <v>15</v>
       </c>
-      <c r="C28" s="8">
-        <v>100.0</v>
-      </c>
+      <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="23">
-        <v>46100.83597384259</v>
+        <v>46051.96156388889</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35150,17 +35142,17 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B29" s="8">
-        <v>20.0</v>
+        <v>2.0</v>
       </c>
       <c r="C29" s="8">
         <v>100.0</v>
       </c>
       <c r="D29" s="17"/>
       <c r="E29" s="23">
-        <v>46100.83604224537</v>
+        <v>46100.83597384259</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35173,11 +35165,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
+      <c r="A30" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="C30" s="8">
+        <v>100.0</v>
+      </c>
       <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
+      <c r="E30" s="23">
+        <v>46100.83604224537</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35205,11 +35205,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -50963,6 +50963,22 @@
       <c r="L1016" s="4"/>
       <c r="M1016" s="4"/>
       <c r="N1016" s="4"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="4"/>
+      <c r="B1017" s="4"/>
+      <c r="C1017" s="4"/>
+      <c r="D1017" s="4"/>
+      <c r="E1017" s="4"/>
+      <c r="F1017" s="4"/>
+      <c r="G1017" s="4"/>
+      <c r="H1017" s="4"/>
+      <c r="I1017" s="4"/>
+      <c r="J1017" s="4"/>
+      <c r="K1017" s="4"/>
+      <c r="L1017" s="4"/>
+      <c r="M1017" s="4"/>
+      <c r="N1017" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-09T09:08:00.481Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -79,6 +79,9 @@
     <t>反轉cut, 鏡射</t>
   </si>
   <si>
+    <t>FILL</t>
+  </si>
+  <si>
     <t>遮蓋膠紙</t>
   </si>
   <si>
@@ -107,9 +110,6 @@
   </si>
   <si>
     <t>5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
   </si>
   <si>
     <t>雕刻%</t>
@@ -34653,7 +34653,9 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
+      <c r="A5" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -50997,10 +50999,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51080,7 +51082,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -51136,7 +51138,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -51218,10 +51220,10 @@
     </row>
     <row r="12">
       <c r="A12" s="39" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -51285,7 +51287,7 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="8">
         <v>5.0</v>
@@ -51300,7 +51302,7 @@
         <v>46160.85381630787</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51437,7 +51439,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
@@ -51520,7 +51522,7 @@
         <v>46156.84678416667</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51575,7 +51577,7 @@
         <v>10</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
@@ -51699,7 +51701,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C34" s="41">
         <v>15.0</v>
@@ -51841,7 +51843,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51853,7 +51855,7 @@
     </row>
     <row r="41">
       <c r="A41" s="42" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
@@ -51870,7 +51872,7 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B42" s="36">
         <v>2.0</v>
@@ -52253,7 +52255,7 @@
         <v>38</v>
       </c>
       <c r="B60" s="34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-09T09:08:06.755Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34656,10 +34656,14 @@
       <c r="A5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="8">
+        <v>2.0</v>
+      </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="6"/>
+      <c r="E5" s="9">
+        <v>46182.713951122685</v>
+      </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-09T09:08:09.064Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34659,10 +34659,14 @@
       <c r="B5" s="8">
         <v>2.0</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="C5" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E5" s="9">
-        <v>46182.713951122685</v>
+        <v>46182.71397640047</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:10:28.495Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -34666,7 +34666,7 @@
         <v>1.0</v>
       </c>
       <c r="E5" s="9">
-        <v>46182.71397640047</v>
+        <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -51862,9 +51862,7 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="42" t="s">
-        <v>31</v>
-      </c>
+      <c r="A41" s="42"/>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -51879,21 +51877,13 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>21</v>
+      <c r="A42" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="B42" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C42" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D42" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E42" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="24"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -51905,19 +51895,19 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B43" s="36">
         <v>2.0</v>
       </c>
       <c r="C43" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D43" s="36">
         <v>1.0</v>
       </c>
       <c r="E43" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -51930,19 +51920,19 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C44" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D44" s="36">
         <v>1.0</v>
       </c>
       <c r="E44" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -51954,11 +51944,21 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="24"/>
+      <c r="A45" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C45" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D45" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E45" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51969,17 +51969,11 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>33</v>
-      </c>
+      <c r="A46" s="7"/>
+      <c r="B46" s="8"/>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
-      <c r="E46" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E46" s="24"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51990,16 +51984,16 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="7">
-        <v>50.0</v>
+      <c r="A47" s="7" t="s">
+        <v>32</v>
       </c>
-      <c r="B47" s="8">
-        <v>100.0</v>
+      <c r="B47" s="8" t="s">
+        <v>33</v>
       </c>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
       <c r="E47" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52011,13 +52005,17 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="43" t="s">
-        <v>34</v>
+      <c r="A48" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B48" s="44"/>
-      <c r="C48" s="44"/>
-      <c r="D48" s="44"/>
-      <c r="E48" s="45"/>
+      <c r="B48" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52028,21 +52026,13 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="34" t="s">
-        <v>35</v>
+      <c r="A49" s="43" t="s">
+        <v>34</v>
       </c>
-      <c r="B49" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C49" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D49" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E49" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B49" s="44"/>
+      <c r="C49" s="44"/>
+      <c r="D49" s="44"/>
+      <c r="E49" s="45"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52053,11 +52043,21 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="35"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
+      <c r="A50" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B50" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C50" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D50" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E50" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52068,9 +52068,7 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="34" t="s">
-        <v>36</v>
-      </c>
+      <c r="A51" s="35"/>
       <c r="B51" s="35"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
@@ -52085,21 +52083,13 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="s">
-        <v>7</v>
+      <c r="A52" s="34" t="s">
+        <v>36</v>
       </c>
-      <c r="B52" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C52" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D52" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E52" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B52" s="35"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52110,18 +52100,20 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="34" t="s">
-        <v>37</v>
+      <c r="A53" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B53" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C53" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D53" s="4"/>
+      <c r="D53" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E53" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52133,11 +52125,19 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="35"/>
-      <c r="B54" s="35"/>
-      <c r="C54" s="4"/>
+      <c r="A54" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C54" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="E54" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52148,17 +52148,11 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B55" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A55" s="35"/>
+      <c r="B55" s="35"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52170,19 +52164,15 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B56" s="34">
-        <v>5.0</v>
+      <c r="B56" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C56" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D56" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
       <c r="E56" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52195,19 +52185,19 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B57" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C57" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D57" s="15">
         <v>1.0</v>
       </c>
       <c r="E57" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -52220,10 +52210,10 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B58" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C58" s="15">
         <v>10.0</v>
@@ -52232,7 +52222,7 @@
         <v>1.0</v>
       </c>
       <c r="E58" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -52244,11 +52234,21 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="35"/>
-      <c r="B59" s="35"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
+      <c r="A59" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B59" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C59" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D59" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E59" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52259,17 +52259,11 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B60" s="34" t="s">
-        <v>31</v>
-      </c>
+      <c r="A60" s="35"/>
+      <c r="B60" s="35"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52281,18 +52275,16 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B61" s="34">
-        <v>5.0</v>
+      <c r="B61" s="34" t="s">
+        <v>31</v>
       </c>
-      <c r="C61" s="15">
-        <v>80.0</v>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D61" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52304,13 +52296,13 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B62" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C62" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D62" s="15">
         <v>1.0</v>
@@ -52327,20 +52319,18 @@
     </row>
     <row r="63">
       <c r="A63" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B63" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C63" s="15">
         <v>10.0</v>
       </c>
       <c r="D63" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E63" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52351,11 +52341,21 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="35"/>
-      <c r="B64" s="35"/>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
+      <c r="A64" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B64" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C64" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D64" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E64" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -52366,7 +52366,7 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="34"/>
+      <c r="A65" s="35"/>
       <c r="B65" s="35"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
@@ -52381,7 +52381,7 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="35"/>
+      <c r="A66" s="34"/>
       <c r="B66" s="35"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
@@ -52396,8 +52396,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="4"/>
-      <c r="B67" s="4"/>
+      <c r="A67" s="35"/>
+      <c r="B67" s="35"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -66465,6 +66465,21 @@
       <c r="L1004" s="4"/>
       <c r="M1004" s="4"/>
     </row>
+    <row r="1005">
+      <c r="A1005" s="4"/>
+      <c r="B1005" s="4"/>
+      <c r="C1005" s="4"/>
+      <c r="D1005" s="4"/>
+      <c r="E1005" s="4"/>
+      <c r="F1005" s="4"/>
+      <c r="G1005" s="4"/>
+      <c r="H1005" s="4"/>
+      <c r="I1005" s="4"/>
+      <c r="J1005" s="4"/>
+      <c r="K1005" s="4"/>
+      <c r="L1005" s="4"/>
+      <c r="M1005" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:10:32.520Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51877,9 +51877,7 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="42" t="s">
-        <v>31</v>
-      </c>
+      <c r="A42" s="42"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
       <c r="D42" s="17"/>
@@ -51894,21 +51892,11 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B43" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C43" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D43" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E43" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="A43" s="42"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="24"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51919,21 +51907,13 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="s">
-        <v>6</v>
+      <c r="A44" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="B44" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C44" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D44" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E44" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="24"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51945,19 +51925,19 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B45" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C45" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D45" s="36">
         <v>1.0</v>
       </c>
       <c r="E45" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -51969,11 +51949,21 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="24"/>
+      <c r="A46" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C46" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D46" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E46" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51985,15 +51975,19 @@
     </row>
     <row r="47">
       <c r="A47" s="7" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
-      <c r="B47" s="8" t="s">
-        <v>33</v>
+      <c r="B47" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
+      <c r="C47" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D47" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E47" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52005,17 +51999,11 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B48" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A48" s="7"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="24"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52026,13 +52014,17 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="43" t="s">
-        <v>34</v>
+      <c r="A49" s="7" t="s">
+        <v>32</v>
       </c>
-      <c r="B49" s="44"/>
-      <c r="C49" s="44"/>
-      <c r="D49" s="44"/>
-      <c r="E49" s="45"/>
+      <c r="B49" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52043,20 +52035,16 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="34" t="s">
-        <v>35</v>
+      <c r="A50" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B50" s="34">
+      <c r="B50" s="8">
         <v>100.0</v>
       </c>
-      <c r="C50" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D50" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E50" s="46">
-        <v>46009.783484375</v>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52068,11 +52056,13 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="35"/>
-      <c r="B51" s="35"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="A51" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" s="44"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="45"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52084,12 +52074,20 @@
     </row>
     <row r="52">
       <c r="A52" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B52" s="35"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
+      <c r="B52" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C52" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D52" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E52" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52100,21 +52098,11 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B53" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C53" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D53" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E53" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52126,18 +52114,12 @@
     </row>
     <row r="54">
       <c r="A54" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
-      <c r="B54" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C54" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B54" s="35"/>
+      <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="46">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52148,11 +52130,21 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="35"/>
-      <c r="B55" s="35"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
+      <c r="A55" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C55" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D55" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E55" s="46">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52164,15 +52156,17 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B56" s="34" t="s">
-        <v>12</v>
+      <c r="B56" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C56" s="4"/>
+      <c r="C56" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D56" s="4"/>
       <c r="E56" s="46">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52184,21 +52178,11 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="B57" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C57" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D57" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E57" s="46">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A57" s="35"/>
+      <c r="B57" s="35"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52210,19 +52194,15 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
-      <c r="B58" s="34">
-        <v>15.0</v>
+      <c r="B58" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C58" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D58" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
       <c r="E58" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -52235,19 +52215,19 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B59" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C59" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D59" s="15">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52259,11 +52239,21 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="35"/>
-      <c r="B60" s="35"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="A60" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B60" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C60" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D60" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E60" s="46">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52275,15 +52265,19 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
-      <c r="B61" s="34" t="s">
-        <v>31</v>
+      <c r="B61" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
+      <c r="C61" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D61" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E61" s="46">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
@@ -52295,18 +52289,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="B62" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C62" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D62" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A62" s="35"/>
+      <c r="B62" s="35"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
@@ -52319,18 +52305,16 @@
     </row>
     <row r="63">
       <c r="A63" s="34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
-      <c r="B63" s="34">
-        <v>15.0</v>
+      <c r="B63" s="34" t="s">
+        <v>31</v>
       </c>
-      <c r="C63" s="15">
-        <v>10.0</v>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D63" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52342,20 +52326,18 @@
     </row>
     <row r="64">
       <c r="A64" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B64" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C64" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D64" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E64" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E64" s="4"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -52366,10 +52348,18 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="35"/>
-      <c r="B65" s="35"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="4"/>
+      <c r="A65" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B65" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C65" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D65" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -52381,11 +52371,21 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="34"/>
-      <c r="B66" s="35"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="A66" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B66" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C66" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D66" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E66" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52411,8 +52411,8 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
+      <c r="A68" s="34"/>
+      <c r="B68" s="35"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
@@ -52426,8 +52426,8 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
+      <c r="A69" s="35"/>
+      <c r="B69" s="35"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
@@ -66480,6 +66480,36 @@
       <c r="L1005" s="4"/>
       <c r="M1005" s="4"/>
     </row>
+    <row r="1006">
+      <c r="A1006" s="4"/>
+      <c r="B1006" s="4"/>
+      <c r="C1006" s="4"/>
+      <c r="D1006" s="4"/>
+      <c r="E1006" s="4"/>
+      <c r="F1006" s="4"/>
+      <c r="G1006" s="4"/>
+      <c r="H1006" s="4"/>
+      <c r="I1006" s="4"/>
+      <c r="J1006" s="4"/>
+      <c r="K1006" s="4"/>
+      <c r="L1006" s="4"/>
+      <c r="M1006" s="4"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="4"/>
+      <c r="B1007" s="4"/>
+      <c r="C1007" s="4"/>
+      <c r="D1007" s="4"/>
+      <c r="E1007" s="4"/>
+      <c r="F1007" s="4"/>
+      <c r="G1007" s="4"/>
+      <c r="H1007" s="4"/>
+      <c r="I1007" s="4"/>
+      <c r="J1007" s="4"/>
+      <c r="K1007" s="4"/>
+      <c r="L1007" s="4"/>
+      <c r="M1007" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:10:35.594Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51907,9 +51907,7 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42" t="s">
-        <v>31</v>
-      </c>
+      <c r="A44" s="42"/>
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
       <c r="D44" s="17"/>
@@ -51924,21 +51922,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="s">
-        <v>21</v>
+      <c r="A45" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="B45" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C45" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D45" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E45" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="24"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51950,19 +51940,19 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B46" s="36">
         <v>2.0</v>
       </c>
       <c r="C46" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D46" s="36">
         <v>1.0</v>
       </c>
       <c r="E46" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -51975,19 +51965,19 @@
     </row>
     <row r="47">
       <c r="A47" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B47" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C47" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D47" s="36">
         <v>1.0</v>
       </c>
       <c r="E47" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -51999,11 +51989,21 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="7"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="24"/>
+      <c r="A48" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C48" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D48" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E48" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52014,17 +52014,11 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>33</v>
-      </c>
+      <c r="A49" s="7"/>
+      <c r="B49" s="8"/>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>
-      <c r="E49" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E49" s="24"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52035,16 +52029,16 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7">
-        <v>50.0</v>
+      <c r="A50" s="7" t="s">
+        <v>32</v>
       </c>
-      <c r="B50" s="8">
-        <v>100.0</v>
+      <c r="B50" s="8" t="s">
+        <v>33</v>
       </c>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
       <c r="E50" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52056,13 +52050,17 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="43" t="s">
-        <v>34</v>
+      <c r="A51" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B51" s="44"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="45"/>
+      <c r="B51" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52073,21 +52071,13 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="34" t="s">
-        <v>35</v>
+      <c r="A52" s="43" t="s">
+        <v>34</v>
       </c>
-      <c r="B52" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C52" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D52" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E52" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B52" s="44"/>
+      <c r="C52" s="44"/>
+      <c r="D52" s="44"/>
+      <c r="E52" s="45"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52098,11 +52088,21 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="35"/>
-      <c r="B53" s="35"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
+      <c r="A53" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B53" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C53" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D53" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E53" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52113,9 +52113,7 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="34" t="s">
-        <v>36</v>
-      </c>
+      <c r="A54" s="35"/>
       <c r="B54" s="35"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
@@ -52130,21 +52128,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="s">
-        <v>7</v>
+      <c r="A55" s="34" t="s">
+        <v>36</v>
       </c>
-      <c r="B55" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C55" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D55" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E55" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B55" s="35"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52155,18 +52145,20 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="34" t="s">
-        <v>37</v>
+      <c r="A56" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B56" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C56" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D56" s="4"/>
+      <c r="D56" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E56" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52178,11 +52170,19 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="35"/>
-      <c r="B57" s="35"/>
-      <c r="C57" s="4"/>
+      <c r="A57" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B57" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C57" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="E57" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52193,17 +52193,11 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A58" s="35"/>
+      <c r="B58" s="35"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52215,19 +52209,15 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B59" s="34">
-        <v>5.0</v>
+      <c r="B59" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C59" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D59" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
       <c r="E59" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52240,19 +52230,19 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B60" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C60" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D60" s="15">
         <v>1.0</v>
       </c>
       <c r="E60" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
@@ -52265,10 +52255,10 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B61" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C61" s="15">
         <v>10.0</v>
@@ -52277,7 +52267,7 @@
         <v>1.0</v>
       </c>
       <c r="E61" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
@@ -52289,11 +52279,21 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="35"/>
-      <c r="B62" s="35"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="A62" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B62" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C62" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D62" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E62" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52304,17 +52304,11 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B63" s="34" t="s">
-        <v>31</v>
-      </c>
+      <c r="A63" s="35"/>
+      <c r="B63" s="35"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52326,18 +52320,16 @@
     </row>
     <row r="64">
       <c r="A64" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B64" s="34">
-        <v>5.0</v>
+      <c r="B64" s="34" t="s">
+        <v>31</v>
       </c>
-      <c r="C64" s="15">
-        <v>80.0</v>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D64" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E64" s="4"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -52349,13 +52341,13 @@
     </row>
     <row r="65">
       <c r="A65" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B65" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C65" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D65" s="15">
         <v>1.0</v>
@@ -52372,20 +52364,18 @@
     </row>
     <row r="66">
       <c r="A66" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B66" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C66" s="15">
         <v>10.0</v>
       </c>
       <c r="D66" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E66" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52396,11 +52386,21 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="35"/>
-      <c r="B67" s="35"/>
-      <c r="C67" s="4"/>
-      <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="A67" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B67" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C67" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D67" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E67" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52411,7 +52411,7 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="34"/>
+      <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52426,7 +52426,7 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="35"/>
+      <c r="A69" s="34"/>
       <c r="B69" s="35"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -52441,8 +52441,8 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="4"/>
-      <c r="B70" s="4"/>
+      <c r="A70" s="35"/>
+      <c r="B70" s="35"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
@@ -66510,6 +66510,21 @@
       <c r="L1007" s="4"/>
       <c r="M1007" s="4"/>
     </row>
+    <row r="1008">
+      <c r="A1008" s="4"/>
+      <c r="B1008" s="4"/>
+      <c r="C1008" s="4"/>
+      <c r="D1008" s="4"/>
+      <c r="E1008" s="4"/>
+      <c r="F1008" s="4"/>
+      <c r="G1008" s="4"/>
+      <c r="H1008" s="4"/>
+      <c r="I1008" s="4"/>
+      <c r="J1008" s="4"/>
+      <c r="K1008" s="4"/>
+      <c r="L1008" s="4"/>
+      <c r="M1008" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:10:41.008Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -51877,7 +51877,9 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="42"/>
+      <c r="A42" s="42" t="s">
+        <v>13</v>
+      </c>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
       <c r="D42" s="17"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:10:54.890Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="41">
   <si>
     <t>項目</t>
   </si>
@@ -51894,7 +51894,9 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="42"/>
+      <c r="A43" s="42" t="s">
+        <v>7</v>
+      </c>
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:11:00.743Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51897,10 +51897,16 @@
       <c r="A43" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
+      <c r="B43" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="C43" s="8">
+        <v>10.0</v>
+      </c>
       <c r="D43" s="17"/>
-      <c r="E43" s="24"/>
+      <c r="E43" s="25">
+        <v>46203.632628148145</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:11:03.861Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51903,9 +51903,11 @@
       <c r="C43" s="8">
         <v>10.0</v>
       </c>
-      <c r="D43" s="17"/>
+      <c r="D43" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E43" s="25">
-        <v>46203.632628148145</v>
+        <v>46203.63265940972</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:12:35.484Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51768,9 +51768,7 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A37" s="5"/>
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -51785,21 +51783,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B38" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C38" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D38" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E38" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="A38" s="5"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="24"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51810,21 +51798,13 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="s">
-        <v>7</v>
+      <c r="A39" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B39" s="8">
-        <v>55.0</v>
-      </c>
-      <c r="C39" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D39" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E39" s="25">
-        <v>46006.95627618056</v>
-      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51839,20 +51819,18 @@
         <v>6</v>
       </c>
       <c r="B40" s="8">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C40" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D40" s="8">
         <v>1.0</v>
       </c>
       <c r="E40" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95620635417</v>
       </c>
-      <c r="F40" s="15" t="s">
-        <v>30</v>
-      </c>
+      <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
@@ -51862,11 +51840,21 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="42"/>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="24"/>
+      <c r="A41" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="8">
+        <v>55.0</v>
+      </c>
+      <c r="C41" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D41" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E41" s="25">
+        <v>46006.95627618056</v>
+      </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51877,14 +51865,24 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="42" t="s">
-        <v>13</v>
+      <c r="A42" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="4"/>
+      <c r="B42" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C42" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D42" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E42" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
@@ -51894,21 +51892,11 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B43" s="8">
-        <v>60.0</v>
-      </c>
-      <c r="C43" s="8">
-        <v>10.0</v>
-      </c>
-      <c r="D43" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E43" s="25">
-        <v>46203.63265940972</v>
-      </c>
+      <c r="A43" s="42"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="24"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51919,7 +51907,9 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
+      <c r="A44" s="42" t="s">
+        <v>13</v>
+      </c>
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
       <c r="D44" s="17"/>
@@ -51934,13 +51924,21 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>31</v>
+      <c r="A45" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="24"/>
+      <c r="B45" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="C45" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="D45" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E45" s="25">
+        <v>46203.63265940972</v>
+      </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51951,21 +51949,11 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B46" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C46" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D46" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E46" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="A46" s="42"/>
+      <c r="B46" s="17"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="24"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51976,21 +51964,13 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="s">
-        <v>6</v>
+      <c r="A47" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="B47" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C47" s="36">
-        <v>85.0</v>
-      </c>
-      <c r="D47" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E47" s="25">
-        <v>45900.48745738426</v>
-      </c>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="24"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52002,19 +51982,19 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B48" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C48" s="36">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D48" s="36">
         <v>1.0</v>
       </c>
       <c r="E48" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48749</v>
       </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
@@ -52026,11 +52006,21 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="24"/>
+      <c r="A49" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="C49" s="36">
+        <v>85.0</v>
+      </c>
+      <c r="D49" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E49" s="25">
+        <v>45900.48745738426</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52042,15 +52032,19 @@
     </row>
     <row r="50">
       <c r="A50" s="7" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
-      <c r="B50" s="8" t="s">
-        <v>33</v>
+      <c r="B50" s="36">
+        <v>70.0</v>
       </c>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
+      <c r="C50" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D50" s="36">
+        <v>1.0</v>
+      </c>
       <c r="E50" s="25">
-        <v>45946.87875708334</v>
+        <v>45900.48752491898</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52062,17 +52056,11 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7">
-        <v>50.0</v>
-      </c>
-      <c r="B51" s="8">
-        <v>100.0</v>
-      </c>
-      <c r="C51" s="17"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="25">
-        <v>45946.87887299768</v>
-      </c>
+      <c r="A51" s="7"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="24"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52083,13 +52071,17 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="43" t="s">
-        <v>34</v>
+      <c r="A52" s="7" t="s">
+        <v>32</v>
       </c>
-      <c r="B52" s="44"/>
-      <c r="C52" s="44"/>
-      <c r="D52" s="44"/>
-      <c r="E52" s="45"/>
+      <c r="B52" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="25">
+        <v>45946.87875708334</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52100,20 +52092,16 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="34" t="s">
-        <v>35</v>
+      <c r="A53" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B53" s="34">
+      <c r="B53" s="8">
         <v>100.0</v>
       </c>
-      <c r="C53" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D53" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E53" s="46">
-        <v>46009.783484375</v>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="25">
+        <v>45946.87887299768</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52125,11 +52113,13 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="35"/>
-      <c r="B54" s="35"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="A54" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" s="44"/>
+      <c r="C54" s="44"/>
+      <c r="D54" s="44"/>
+      <c r="E54" s="45"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52141,12 +52131,20 @@
     </row>
     <row r="55">
       <c r="A55" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
-      <c r="B55" s="35"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
+      <c r="B55" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C55" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D55" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E55" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52157,21 +52155,11 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B56" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C56" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D56" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E56" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="A56" s="35"/>
+      <c r="B56" s="35"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -52183,18 +52171,12 @@
     </row>
     <row r="57">
       <c r="A57" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
-      <c r="B57" s="34">
-        <v>15.0</v>
-      </c>
-      <c r="C57" s="15">
-        <v>16.0</v>
-      </c>
+      <c r="B57" s="35"/>
+      <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="46">
-        <v>46136.01284993056</v>
-      </c>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52205,11 +52187,21 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="35"/>
-      <c r="B58" s="35"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
+      <c r="A58" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" s="34">
+        <v>50.0</v>
+      </c>
+      <c r="C58" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="D58" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E58" s="46">
+        <v>46038.9559609375</v>
+      </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52221,15 +52213,17 @@
     </row>
     <row r="59">
       <c r="A59" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B59" s="34" t="s">
-        <v>12</v>
+      <c r="B59" s="34">
+        <v>15.0</v>
       </c>
-      <c r="C59" s="4"/>
+      <c r="C59" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D59" s="4"/>
       <c r="E59" s="46">
-        <v>46044.0116671875</v>
+        <v>46136.01284993056</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52241,21 +52235,11 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="B60" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C60" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D60" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E60" s="46">
-        <v>46044.01310700232</v>
-      </c>
+      <c r="A60" s="35"/>
+      <c r="B60" s="35"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52267,19 +52251,15 @@
     </row>
     <row r="61">
       <c r="A61" s="34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
-      <c r="B61" s="34">
-        <v>15.0</v>
+      <c r="B61" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C61" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="D61" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
       <c r="E61" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
@@ -52292,19 +52272,19 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B62" s="34">
-        <v>30.0</v>
+        <v>5.0</v>
       </c>
       <c r="C62" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D62" s="15">
         <v>1.0</v>
       </c>
       <c r="E62" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
@@ -52316,11 +52296,21 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="35"/>
-      <c r="B63" s="35"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="A63" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B63" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C63" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D63" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E63" s="46">
+        <v>46044.013194907406</v>
+      </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52332,15 +52322,19 @@
     </row>
     <row r="64">
       <c r="A64" s="34" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
-      <c r="B64" s="34" t="s">
-        <v>31</v>
+      <c r="B64" s="34">
+        <v>30.0</v>
       </c>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
+      <c r="C64" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D64" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E64" s="46">
-        <v>46044.0136399537</v>
+        <v>46056.701985011576</v>
       </c>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
@@ -52352,18 +52346,10 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="B65" s="34">
-        <v>5.0</v>
-      </c>
-      <c r="C65" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D65" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="A65" s="35"/>
+      <c r="B65" s="35"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -52376,18 +52362,16 @@
     </row>
     <row r="66">
       <c r="A66" s="34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
-      <c r="B66" s="34">
-        <v>15.0</v>
+      <c r="B66" s="34" t="s">
+        <v>31</v>
       </c>
-      <c r="C66" s="15">
-        <v>10.0</v>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D66" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52399,20 +52383,18 @@
     </row>
     <row r="67">
       <c r="A67" s="34" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B67" s="34">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="C67" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D67" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E67" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52423,10 +52405,18 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="35"/>
-      <c r="B68" s="35"/>
-      <c r="C68" s="4"/>
-      <c r="D68" s="4"/>
+      <c r="A68" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B68" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C68" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D68" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
@@ -52438,11 +52428,21 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="34"/>
-      <c r="B69" s="35"/>
-      <c r="C69" s="4"/>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
+      <c r="A69" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B69" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C69" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D69" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E69" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -52468,8 +52468,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="4"/>
-      <c r="B71" s="4"/>
+      <c r="A71" s="34"/>
+      <c r="B71" s="35"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52483,8 +52483,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="4"/>
-      <c r="B72" s="4"/>
+      <c r="A72" s="35"/>
+      <c r="B72" s="35"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -66537,6 +66537,36 @@
       <c r="L1008" s="4"/>
       <c r="M1008" s="4"/>
     </row>
+    <row r="1009">
+      <c r="A1009" s="4"/>
+      <c r="B1009" s="4"/>
+      <c r="C1009" s="4"/>
+      <c r="D1009" s="4"/>
+      <c r="E1009" s="4"/>
+      <c r="F1009" s="4"/>
+      <c r="G1009" s="4"/>
+      <c r="H1009" s="4"/>
+      <c r="I1009" s="4"/>
+      <c r="J1009" s="4"/>
+      <c r="K1009" s="4"/>
+      <c r="L1009" s="4"/>
+      <c r="M1009" s="4"/>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="4"/>
+      <c r="B1010" s="4"/>
+      <c r="C1010" s="4"/>
+      <c r="D1010" s="4"/>
+      <c r="E1010" s="4"/>
+      <c r="F1010" s="4"/>
+      <c r="G1010" s="4"/>
+      <c r="H1010" s="4"/>
+      <c r="I1010" s="4"/>
+      <c r="J1010" s="4"/>
+      <c r="K1010" s="4"/>
+      <c r="L1010" s="4"/>
+      <c r="M1010" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:12:40.815Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51798,9 +51798,7 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A39" s="5"/>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
@@ -51815,21 +51813,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>6</v>
+      <c r="A40" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B40" s="8">
-        <v>9.0</v>
-      </c>
-      <c r="C40" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="D40" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E40" s="25">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="24"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51841,10 +51831,10 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41" s="8">
-        <v>55.0</v>
+        <v>9.0</v>
       </c>
       <c r="C41" s="8">
         <v>20.0</v>
@@ -51853,7 +51843,7 @@
         <v>1.0</v>
       </c>
       <c r="E41" s="25">
-        <v>46006.95627618056</v>
+        <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51866,23 +51856,21 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B42" s="8">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C42" s="8">
-        <v>250.0</v>
+        <v>20.0</v>
       </c>
       <c r="D42" s="8">
         <v>1.0</v>
       </c>
       <c r="E42" s="25">
-        <v>46038.439073761576</v>
+        <v>46006.95627618056</v>
       </c>
-      <c r="F42" s="15" t="s">
-        <v>30</v>
-      </c>
+      <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
@@ -51892,12 +51880,24 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="42"/>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="4"/>
+      <c r="A43" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C43" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D43" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E43" s="25">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F43" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
@@ -51907,9 +51907,7 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42" t="s">
-        <v>13</v>
-      </c>
+      <c r="A44" s="42"/>
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
       <c r="D44" s="17"/>
@@ -51924,21 +51922,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="s">
-        <v>7</v>
+      <c r="A45" s="42" t="s">
+        <v>13</v>
       </c>
-      <c r="B45" s="8">
-        <v>60.0</v>
-      </c>
-      <c r="C45" s="8">
-        <v>10.0</v>
-      </c>
-      <c r="D45" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="E45" s="25">
-        <v>46203.63265940972</v>
-      </c>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="24"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51949,11 +51939,21 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="42"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="24"/>
+      <c r="A46" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="C46" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="D46" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E46" s="25">
+        <v>46203.63265940972</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -51964,9 +51964,7 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42" t="s">
-        <v>31</v>
-      </c>
+      <c r="A47" s="42"/>
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -51981,21 +51979,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="s">
-        <v>21</v>
+      <c r="A48" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="B48" s="36">
-        <v>2.0</v>
-      </c>
-      <c r="C48" s="36">
-        <v>100.0</v>
-      </c>
-      <c r="D48" s="36">
-        <v>1.0</v>
-      </c>
-      <c r="E48" s="25">
-        <v>45900.48749</v>
-      </c>
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="24"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52007,19 +51997,19 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B49" s="36">
         <v>2.0</v>
       </c>
       <c r="C49" s="36">
-        <v>85.0</v>
+        <v>100.0</v>
       </c>
       <c r="D49" s="36">
         <v>1.0</v>
       </c>
       <c r="E49" s="25">
-        <v>45900.48745738426</v>
+        <v>45900.48749</v>
       </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -52032,19 +52022,19 @@
     </row>
     <row r="50">
       <c r="A50" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B50" s="36">
-        <v>70.0</v>
+        <v>2.0</v>
       </c>
       <c r="C50" s="36">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="D50" s="36">
         <v>1.0</v>
       </c>
       <c r="E50" s="25">
-        <v>45900.48752491898</v>
+        <v>45900.48745738426</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52056,11 +52046,21 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7"/>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="24"/>
+      <c r="A51" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" s="36">
+        <v>70.0</v>
+      </c>
+      <c r="C51" s="36">
+        <v>10.0</v>
+      </c>
+      <c r="D51" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E51" s="25">
+        <v>45900.48752491898</v>
+      </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52071,17 +52071,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B52" s="8" t="s">
-        <v>33</v>
-      </c>
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
       <c r="C52" s="8"/>
       <c r="D52" s="8"/>
-      <c r="E52" s="25">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E52" s="24"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52092,16 +52086,16 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7">
-        <v>50.0</v>
+      <c r="A53" s="7" t="s">
+        <v>32</v>
       </c>
-      <c r="B53" s="8">
-        <v>100.0</v>
+      <c r="B53" s="8" t="s">
+        <v>33</v>
       </c>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
       <c r="E53" s="25">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52113,13 +52107,17 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="43" t="s">
-        <v>34</v>
+      <c r="A54" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B54" s="44"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="44"/>
-      <c r="E54" s="45"/>
+      <c r="B54" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="25">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52130,21 +52128,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="34" t="s">
-        <v>35</v>
+      <c r="A55" s="43" t="s">
+        <v>34</v>
       </c>
-      <c r="B55" s="34">
-        <v>100.0</v>
-      </c>
-      <c r="C55" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D55" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E55" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52155,11 +52145,21 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="35"/>
-      <c r="B56" s="35"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
+      <c r="A56" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" s="34">
+        <v>100.0</v>
+      </c>
+      <c r="C56" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D56" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E56" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -52170,9 +52170,7 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="34" t="s">
-        <v>36</v>
-      </c>
+      <c r="A57" s="35"/>
       <c r="B57" s="35"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
@@ -52187,21 +52185,13 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="s">
-        <v>7</v>
+      <c r="A58" s="34" t="s">
+        <v>36</v>
       </c>
-      <c r="B58" s="34">
-        <v>50.0</v>
-      </c>
-      <c r="C58" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D58" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E58" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B58" s="35"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52212,18 +52202,20 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="34" t="s">
-        <v>37</v>
+      <c r="A59" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B59" s="34">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
       <c r="C59" s="15">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
-      <c r="D59" s="4"/>
+      <c r="D59" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E59" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52235,11 +52227,19 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="35"/>
-      <c r="B60" s="35"/>
-      <c r="C60" s="4"/>
+      <c r="A60" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B60" s="34">
+        <v>15.0</v>
+      </c>
+      <c r="C60" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="E60" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52250,17 +52250,11 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="34" t="s">
-        <v>12</v>
-      </c>
+      <c r="A61" s="35"/>
+      <c r="B61" s="35"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52272,19 +52266,15 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B62" s="34">
-        <v>5.0</v>
+      <c r="B62" s="34" t="s">
+        <v>12</v>
       </c>
-      <c r="C62" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D62" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
       <c r="E62" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
@@ -52297,19 +52287,19 @@
     </row>
     <row r="63">
       <c r="A63" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B63" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C63" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D63" s="15">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
@@ -52322,10 +52312,10 @@
     </row>
     <row r="64">
       <c r="A64" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B64" s="34">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
       <c r="C64" s="15">
         <v>10.0</v>
@@ -52334,7 +52324,7 @@
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
@@ -52346,11 +52336,21 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="35"/>
-      <c r="B65" s="35"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
+      <c r="A65" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B65" s="34">
+        <v>30.0</v>
+      </c>
+      <c r="C65" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D65" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E65" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -52361,17 +52361,11 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B66" s="34" t="s">
-        <v>31</v>
-      </c>
+      <c r="A66" s="35"/>
+      <c r="B66" s="35"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52383,18 +52377,16 @@
     </row>
     <row r="67">
       <c r="A67" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
-      <c r="B67" s="34">
-        <v>5.0</v>
+      <c r="B67" s="34" t="s">
+        <v>31</v>
       </c>
-      <c r="C67" s="15">
-        <v>80.0</v>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D67" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52406,13 +52398,13 @@
     </row>
     <row r="68">
       <c r="A68" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B68" s="34">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
       <c r="C68" s="15">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="D68" s="15">
         <v>1.0</v>
@@ -52429,20 +52421,18 @@
     </row>
     <row r="69">
       <c r="A69" s="34" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B69" s="34">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
       <c r="C69" s="15">
         <v>10.0</v>
       </c>
       <c r="D69" s="15">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
-      <c r="E69" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E69" s="4"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -52453,11 +52443,21 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="35"/>
-      <c r="B70" s="35"/>
-      <c r="C70" s="4"/>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
+      <c r="A70" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B70" s="34">
+        <v>20.0</v>
+      </c>
+      <c r="C70" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D70" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E70" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -52468,7 +52468,7 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="34"/>
+      <c r="A71" s="35"/>
       <c r="B71" s="35"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
@@ -52483,7 +52483,7 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="35"/>
+      <c r="A72" s="34"/>
       <c r="B72" s="35"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
@@ -52498,8 +52498,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
+      <c r="A73" s="35"/>
+      <c r="B73" s="35"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -66567,6 +66567,21 @@
       <c r="L1010" s="4"/>
       <c r="M1010" s="4"/>
     </row>
+    <row r="1011">
+      <c r="A1011" s="4"/>
+      <c r="B1011" s="4"/>
+      <c r="C1011" s="4"/>
+      <c r="D1011" s="4"/>
+      <c r="E1011" s="4"/>
+      <c r="F1011" s="4"/>
+      <c r="G1011" s="4"/>
+      <c r="H1011" s="4"/>
+      <c r="I1011" s="4"/>
+      <c r="J1011" s="4"/>
+      <c r="K1011" s="4"/>
+      <c r="L1011" s="4"/>
+      <c r="M1011" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:12:47.814Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="42">
   <si>
     <t>項目</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>６</t>
+  </si>
+  <si>
+    <t>1.5mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -51768,7 +51771,9 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5"/>
+      <c r="A37" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -51896,7 +51901,7 @@
         <v>46038.439073761576</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51980,7 +51985,7 @@
     </row>
     <row r="48">
       <c r="A48" s="42" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B48" s="17"/>
       <c r="C48" s="17"/>
@@ -52087,10 +52092,10 @@
     </row>
     <row r="53">
       <c r="A53" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C53" s="8"/>
       <c r="D53" s="8"/>
@@ -52129,7 +52134,7 @@
     </row>
     <row r="55">
       <c r="A55" s="43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B55" s="44"/>
       <c r="C55" s="44"/>
@@ -52146,7 +52151,7 @@
     </row>
     <row r="56">
       <c r="A56" s="34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B56" s="34">
         <v>100.0</v>
@@ -52186,7 +52191,7 @@
     </row>
     <row r="58">
       <c r="A58" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B58" s="35"/>
       <c r="C58" s="4"/>
@@ -52228,7 +52233,7 @@
     </row>
     <row r="60">
       <c r="A60" s="34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B60" s="34">
         <v>15.0</v>
@@ -52266,7 +52271,7 @@
     </row>
     <row r="62">
       <c r="A62" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B62" s="34" t="s">
         <v>12</v>
@@ -52287,7 +52292,7 @@
     </row>
     <row r="63">
       <c r="A63" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B63" s="34">
         <v>5.0</v>
@@ -52312,7 +52317,7 @@
     </row>
     <row r="64">
       <c r="A64" s="34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B64" s="34">
         <v>15.0</v>
@@ -52377,10 +52382,10 @@
     </row>
     <row r="67">
       <c r="A67" s="34" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B67" s="34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
@@ -52398,7 +52403,7 @@
     </row>
     <row r="68">
       <c r="A68" s="34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B68" s="34">
         <v>5.0</v>
@@ -52421,7 +52426,7 @@
     </row>
     <row r="69">
       <c r="A69" s="34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B69" s="34">
         <v>15.0</v>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:13:02.894Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="42">
   <si>
     <t>項目</t>
   </si>
@@ -51788,7 +51788,9 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5"/>
+      <c r="A38" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="B38" s="17"/>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:13:13.463Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51791,10 +51791,14 @@
       <c r="A38" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B38" s="17"/>
+      <c r="B38" s="8">
+        <v>40.0</v>
+      </c>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
-      <c r="E38" s="24"/>
+      <c r="E38" s="25">
+        <v>46203.634171261576</v>
+      </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:13:21.506Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51794,10 +51794,12 @@
       <c r="B38" s="8">
         <v>40.0</v>
       </c>
-      <c r="C38" s="17"/>
+      <c r="C38" s="8">
+        <v>15.0</v>
+      </c>
       <c r="D38" s="17"/>
       <c r="E38" s="25">
-        <v>46203.634171261576</v>
+        <v>46203.63426040509</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-06-30T07:46:21.922Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51388,13 +51388,13 @@
         <v>6.0</v>
       </c>
       <c r="C19" s="36">
-        <v>20.0</v>
+        <v>45.0</v>
       </c>
       <c r="D19" s="8">
         <v>1.0</v>
       </c>
       <c r="E19" s="25">
-        <v>46118.87534236111</v>
+        <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51797,9 +51797,11 @@
       <c r="C38" s="8">
         <v>15.0</v>
       </c>
-      <c r="D38" s="17"/>
+      <c r="D38" s="8">
+        <v>1.0</v>
+      </c>
       <c r="E38" s="25">
-        <v>46203.63426040509</v>
+        <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-04T09:20:44.360Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -52065,7 +52065,7 @@
         <v>7</v>
       </c>
       <c r="B51" s="36">
-        <v>70.0</v>
+        <v>60.0</v>
       </c>
       <c r="C51" s="36">
         <v>10.0</v>
@@ -52074,7 +52074,7 @@
         <v>1.0</v>
       </c>
       <c r="E51" s="25">
-        <v>45900.48752491898</v>
+        <v>46207.72272293981</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-04T09:25:03.550Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -52065,7 +52065,7 @@
         <v>7</v>
       </c>
       <c r="B51" s="36">
-        <v>60.0</v>
+        <v>70.0</v>
       </c>
       <c r="C51" s="36">
         <v>10.0</v>
@@ -52074,7 +52074,7 @@
         <v>1.0</v>
       </c>
       <c r="E51" s="25">
-        <v>46207.72272293981</v>
+        <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-10T10:01:29.812Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -17304,13 +17304,13 @@
         <v>4.0</v>
       </c>
       <c r="C10" s="11">
-        <v>6.0</v>
+        <v>25.0</v>
       </c>
       <c r="D10" s="11">
         <v>1.0</v>
       </c>
       <c r="E10" s="26">
-        <v>45900.4876925</v>
+        <v>46213.751012962966</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-10T10:01:42.135Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -51715,13 +51715,13 @@
         <v>29</v>
       </c>
       <c r="C34" s="41">
-        <v>15.0</v>
+        <v>40.0</v>
       </c>
       <c r="D34" s="41">
         <v>1.0</v>
       </c>
       <c r="E34" s="26">
-        <v>46117.900830185186</v>
+        <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-20T07:32:33.978Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,7 +19,13 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -31,22 +37,52 @@
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>Line</t>
   </si>
   <si>
-    <t>Line</t>
+    <t>0.3mm</t>
   </si>
   <si>
     <t>Cut-1/2</t>
   </si>
   <si>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>03mm</t>
+  </si>
+  <si>
+    <t>Cut</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
     <t>0.5mm</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
   </si>
   <si>
     <t>(PS -3)</t>
   </si>
   <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
     <t>1mm</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>2mm</t>
@@ -58,49 +94,7 @@
     <t>4mm</t>
   </si>
   <si>
-    <t>A4紙</t>
-  </si>
-  <si>
     <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>Cut</t>
-  </si>
-  <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
-    <t>刀壓</t>
-  </si>
-  <si>
-    <t>03mm</t>
-  </si>
-  <si>
-    <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>Keep Detail</t>
   </si>
   <si>
     <t>６</t>
@@ -112,7 +106,13 @@
     <t>吉翁號刻線參數</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>5mm</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>雕刻%</t>
@@ -172,12 +172,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -186,6 +180,12 @@
     <font>
       <b/>
       <sz val="14.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -206,14 +206,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,20 +321,32 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -342,26 +354,45 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -375,63 +406,32 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="6"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>8</v>
+      <c r="A6" s="14" t="s">
+        <v>15</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>9</v>
+      <c r="B6" s="15" t="s">
+        <v>17</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>6</v>
+      <c r="A7" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>7</v>
+      <c r="A8" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="21">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="16"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>10</v>
+      <c r="A10" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
+      <c r="A11" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>7</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="16"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="6"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="8"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>11</v>
+      <c r="A15" s="14" t="s">
+        <v>23</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="12"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>6</v>
+      <c r="A16" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>7</v>
+      <c r="A17" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="6"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>12</v>
+      <c r="A19" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>6</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>7</v>
+      <c r="A21" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="6"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>13</v>
+      <c r="A23" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="12"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>6</v>
+      <c r="A24" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="s">
-        <v>7</v>
+      <c r="A25" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>14</v>
+      <c r="A27" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>15</v>
+      <c r="B27" s="9" t="s">
+        <v>26</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="23">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>6</v>
+      <c r="A28" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="23">
+      <c r="D28" s="13"/>
+      <c r="E28" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>16</v>
+      <c r="A29" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="23">
+      <c r="D29" s="13"/>
+      <c r="E29" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="24"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="24"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>17</v>
+      <c r="A5" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="24"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>6</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="24"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>7</v>
+      <c r="A7" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,11 +17261,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="25"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
-        <v>8</v>
+      <c r="A9" s="14" t="s">
+        <v>15</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="26"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,20 +17297,20 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>6</v>
+      <c r="A10" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="11">
-        <v>25.0</v>
+      <c r="C10" s="15">
+        <v>15.0</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="26">
-        <v>46213.751012962966</v>
+      <c r="E10" s="25">
+        <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="s">
-        <v>7</v>
+      <c r="A11" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="25">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="s">
-        <v>18</v>
+      <c r="A12" s="19" t="s">
+        <v>19</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="25">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,12 +17378,12 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="s">
-        <v>17</v>
+      <c r="A13" s="19" t="s">
+        <v>14</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
       <c r="E13" s="27"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -17397,16 +17397,16 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="s">
-        <v>6</v>
+      <c r="A14" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
       <c r="E14" s="27"/>
@@ -17422,16 +17422,16 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>7</v>
+      <c r="A15" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
       <c r="E15" s="27"/>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="16">
       <c r="A16" s="28"/>
-      <c r="E16" s="24"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>10</v>
+      <c r="A17" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="24"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="24"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>7</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="24"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="24"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,12 +17549,12 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>11</v>
+      <c r="A21" s="14" t="s">
+        <v>23</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
       <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -17568,16 +17568,16 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>6</v>
+      <c r="A22" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
       <c r="E22" s="27"/>
@@ -17593,16 +17593,16 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>7</v>
+      <c r="A23" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
       <c r="E23" s="27"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="24"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>12</v>
+      <c r="A25" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="24"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="24"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>7</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="25">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="24"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,12 +17723,12 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>13</v>
+      <c r="A29" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
       <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -17742,16 +17742,16 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>6</v>
+      <c r="A30" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
       <c r="E30" s="27"/>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="s">
-        <v>7</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="30"/>
+      <c r="E31" s="37"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="31" t="s">
-        <v>19</v>
+      <c r="A33" s="38" t="s">
+        <v>30</v>
       </c>
-      <c r="B33" s="32">
+      <c r="B33" s="39">
         <v>5.0</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="39">
         <v>10.0</v>
       </c>
-      <c r="D33" s="32">
+      <c r="D33" s="39">
         <v>2.0</v>
       </c>
-      <c r="E33" s="33">
+      <c r="E33" s="40">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="34" t="s">
-        <v>20</v>
+      <c r="F33" s="41" t="s">
+        <v>32</v>
       </c>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35"/>
-      <c r="K33" s="35"/>
-      <c r="L33" s="35"/>
-      <c r="M33" s="35"/>
-      <c r="N33" s="35"/>
-      <c r="O33" s="35"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>14</v>
+      <c r="A36" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>15</v>
+      <c r="B36" s="9" t="s">
+        <v>26</v>
       </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>6</v>
+      <c r="A37" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="17"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>16</v>
+      <c r="A38" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="17"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>20.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>21</v>
+      <c r="A5" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>2.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="8"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,15 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>8</v>
+      <c r="A7" s="14" t="s">
+        <v>15</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>9</v>
+      <c r="B7" s="15" t="s">
+        <v>17</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34718,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>6</v>
+      <c r="A8" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="15">
         <v>4.0</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="15">
         <v>10.0</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34744,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>7</v>
+      <c r="A9" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="15">
         <v>20.0</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="21">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,11 +34770,11 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="16"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="9"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34786,13 +34786,13 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>10</v>
+      <c r="A11" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34804,23 +34804,23 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="9">
         <v>5.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
@@ -34830,19 +34830,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>6</v>
+      <c r="A13" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>15.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34854,19 +34854,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>7</v>
+      <c r="A14" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>32.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>5.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="6"/>
+      <c r="E14" s="8"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34878,11 +34878,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="16"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="6"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="8"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34894,13 +34894,13 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>11</v>
+      <c r="A16" s="14" t="s">
+        <v>23</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="12"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34912,19 +34912,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>6</v>
+      <c r="A17" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="15">
         <v>5.0</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34936,19 +34936,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="s">
-        <v>7</v>
+      <c r="A18" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="15">
         <v>50.0</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="15">
         <v>5.0</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="15">
         <v>1.0</v>
       </c>
-      <c r="E18" s="12"/>
+      <c r="E18" s="17"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34960,11 +34960,11 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="6"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,13 +34976,13 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>12</v>
+      <c r="A20" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="6"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34994,19 +34994,19 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>6</v>
+      <c r="A21" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="9">
         <v>5.0</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="9">
         <v>5.0</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="6"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35018,13 +35018,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>7</v>
+      <c r="A22" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="6"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35036,11 +35036,11 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="6"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="8"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35052,13 +35052,13 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="s">
-        <v>13</v>
+      <c r="A24" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="12"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35070,19 +35070,19 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="s">
-        <v>6</v>
+      <c r="A25" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="15">
         <v>5.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="15">
         <v>5.0</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="15">
         <v>1.0</v>
       </c>
-      <c r="E25" s="12"/>
+      <c r="E25" s="17"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35094,17 +35094,17 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="s">
-        <v>7</v>
+      <c r="A26" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="31">
         <v>55.0</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="31">
         <v>2.0</v>
       </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="22"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35116,11 +35116,11 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="17"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35132,15 +35132,15 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>14</v>
+      <c r="A28" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>15</v>
+      <c r="B28" s="9" t="s">
+        <v>26</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="23">
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F28" s="4"/>
@@ -35154,17 +35154,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>6</v>
+      <c r="A29" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>2.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="23">
+      <c r="D29" s="13"/>
+      <c r="E29" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F29" s="4"/>
@@ -35178,17 +35178,17 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>16</v>
+      <c r="A30" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="9">
         <v>20.0</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="9">
         <v>100.0</v>
       </c>
-      <c r="D30" s="17"/>
-      <c r="E30" s="23">
+      <c r="D30" s="13"/>
+      <c r="E30" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F30" s="4"/>
@@ -35202,11 +35202,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35218,11 +35218,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51010,19 +51010,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51034,13 +51034,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>6</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51051,19 +51051,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
+      <c r="A3" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="36">
+      <c r="B3" s="7">
         <v>60.0</v>
       </c>
-      <c r="C3" s="36">
+      <c r="C3" s="7">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="24"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51074,11 +51074,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="24"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51089,15 +51089,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" s="6" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>24</v>
+      <c r="B5" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="25"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51108,19 +51108,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>16</v>
+      <c r="A6" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>60.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="12">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51133,11 +51133,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="24"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51148,13 +51148,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>25</v>
+      <c r="A8" s="6" t="s">
+        <v>16</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="24"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51165,19 +51165,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>6</v>
+      <c r="A9" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <v>10.0</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <v>45.0</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <v>1.0</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51190,19 +51190,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>16</v>
+      <c r="A10" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <v>11.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="9">
         <v>20.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51215,11 +51215,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="20"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51230,15 +51230,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="s">
-        <v>25</v>
+      <c r="A12" s="22" t="s">
+        <v>16</v>
       </c>
-      <c r="B12" s="40" t="s">
-        <v>26</v>
+      <c r="B12" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="25"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51249,19 +51249,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>18</v>
+      <c r="A13" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51274,19 +51274,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>6</v>
+      <c r="A14" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>30.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51297,23 +51297,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>27</v>
+      <c r="A15" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="9">
         <v>4.0</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>28</v>
+      <c r="F15" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51324,19 +51324,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>16</v>
+      <c r="A16" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="9">
         <v>12.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="9">
         <v>20.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="9">
         <v>1.0</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51349,11 +51349,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="38"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="20"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51364,13 +51364,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>8</v>
+      <c r="A18" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51381,19 +51381,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="36">
+      <c r="B19" s="7">
         <v>6.0</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="7">
         <v>45.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51406,19 +51406,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
+      <c r="A20" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="36">
+      <c r="B20" s="7">
         <v>18.0</v>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="7">
         <v>20.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51431,11 +51431,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="24"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51446,15 +51446,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="39" t="s">
-        <v>8</v>
+      <c r="A22" s="22" t="s">
+        <v>15</v>
       </c>
-      <c r="B22" s="40" t="s">
-        <v>26</v>
+      <c r="B22" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="25">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51467,19 +51467,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>18</v>
+      <c r="A23" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B23" s="36">
+      <c r="B23" s="7">
         <v>6.0</v>
       </c>
-      <c r="C23" s="36">
+      <c r="C23" s="7">
         <v>50.0</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="9">
         <v>1.0</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51492,19 +51492,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>6</v>
+      <c r="A24" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="36">
+      <c r="B24" s="7">
         <v>8.0</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C24" s="7">
         <v>30.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="25">
+      <c r="E24" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51517,23 +51517,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>16</v>
+      <c r="A25" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B25" s="36">
+      <c r="B25" s="7">
         <v>10.0</v>
       </c>
-      <c r="C25" s="36">
+      <c r="C25" s="7">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="9">
         <v>4.0</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>28</v>
+      <c r="F25" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51544,19 +51544,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>16</v>
+      <c r="A26" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B26" s="36">
+      <c r="B26" s="7">
         <v>17.0</v>
       </c>
-      <c r="C26" s="36">
+      <c r="C26" s="7">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51569,11 +51569,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="24"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51584,15 +51584,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="39" t="s">
-        <v>10</v>
+      <c r="A28" s="22" t="s">
+        <v>20</v>
       </c>
-      <c r="B28" s="40" t="s">
-        <v>26</v>
+      <c r="B28" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="24"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51603,19 +51603,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>18</v>
+      <c r="A29" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B29" s="36">
+      <c r="B29" s="7">
         <v>6.0</v>
       </c>
-      <c r="C29" s="36">
+      <c r="C29" s="7">
         <v>50.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="9">
         <v>1.0</v>
       </c>
-      <c r="E29" s="25">
+      <c r="E29" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51628,19 +51628,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>6</v>
+      <c r="A30" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="7">
         <v>8.0</v>
       </c>
-      <c r="C30" s="36">
+      <c r="C30" s="7">
         <v>30.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="24"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51651,19 +51651,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>7</v>
+      <c r="A31" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="36">
+      <c r="B31" s="7">
         <v>15.0</v>
       </c>
-      <c r="C31" s="36">
+      <c r="C31" s="7">
         <v>10.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="9">
         <v>2.0</v>
       </c>
-      <c r="E31" s="25">
+      <c r="E31" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51676,11 +51676,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="24"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="10"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51691,12 +51691,12 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>10</v>
+      <c r="A33" s="14" t="s">
+        <v>20</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
       <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51708,19 +51708,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="s">
-        <v>6</v>
+      <c r="A34" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>29</v>
+      <c r="B34" s="34" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="34">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="34">
         <v>1.0</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="25">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51733,16 +51733,16 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="s">
-        <v>7</v>
+      <c r="A35" s="19" t="s">
+        <v>9</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="34">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="34">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="34">
         <v>1.0</v>
       </c>
       <c r="E35" s="27"/>
@@ -51756,11 +51756,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="16"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="24"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="10"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51771,13 +51771,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>30</v>
+      <c r="A37" s="6" t="s">
+        <v>28</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="24"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="10"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51788,19 +51788,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>7</v>
+      <c r="A38" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>40.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="9">
         <v>15.0</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="9">
         <v>1.0</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51813,11 +51813,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="24"/>
+      <c r="A39" s="6"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51828,13 +51828,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>11</v>
+      <c r="A40" s="6" t="s">
+        <v>23</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="24"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="10"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51845,19 +51845,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>6</v>
+      <c r="A41" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="9">
         <v>9.0</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="9">
         <v>20.0</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="9">
         <v>1.0</v>
       </c>
-      <c r="E41" s="25">
+      <c r="E41" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51870,19 +51870,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>7</v>
+      <c r="A42" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="9">
         <v>55.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="9">
         <v>20.0</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="9">
         <v>1.0</v>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -51895,23 +51895,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>6</v>
+      <c r="A43" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>10.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="9">
         <v>250.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="25">
+      <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="15" t="s">
-        <v>31</v>
+      <c r="F43" s="16" t="s">
+        <v>29</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51922,11 +51922,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="24"/>
+      <c r="A44" s="36"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="10"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51937,13 +51937,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>13</v>
+      <c r="A45" s="36" t="s">
+        <v>25</v>
       </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="24"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="10"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51954,19 +51954,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>7</v>
+      <c r="A46" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="9">
         <v>60.0</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="9">
         <v>10.0</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="9">
         <v>1.0</v>
       </c>
-      <c r="E46" s="25">
+      <c r="E46" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -51979,11 +51979,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="24"/>
+      <c r="A47" s="36"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51994,13 +51994,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
-        <v>32</v>
+      <c r="A48" s="36" t="s">
+        <v>31</v>
       </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="24"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="10"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52011,19 +52011,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
-        <v>21</v>
+      <c r="A49" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B49" s="36">
+      <c r="B49" s="7">
         <v>2.0</v>
       </c>
-      <c r="C49" s="36">
+      <c r="C49" s="7">
         <v>100.0</v>
       </c>
-      <c r="D49" s="36">
+      <c r="D49" s="7">
         <v>1.0</v>
       </c>
-      <c r="E49" s="25">
+      <c r="E49" s="12">
         <v>45900.48749</v>
       </c>
       <c r="F49" s="4"/>
@@ -52036,19 +52036,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="s">
-        <v>6</v>
+      <c r="A50" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B50" s="36">
+      <c r="B50" s="7">
         <v>2.0</v>
       </c>
-      <c r="C50" s="36">
+      <c r="C50" s="7">
         <v>85.0</v>
       </c>
-      <c r="D50" s="36">
+      <c r="D50" s="7">
         <v>1.0</v>
       </c>
-      <c r="E50" s="25">
+      <c r="E50" s="12">
         <v>45900.48745738426</v>
       </c>
       <c r="F50" s="4"/>
@@ -52061,19 +52061,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>7</v>
+      <c r="A51" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B51" s="36">
+      <c r="B51" s="7">
         <v>70.0</v>
       </c>
-      <c r="C51" s="36">
+      <c r="C51" s="7">
         <v>10.0</v>
       </c>
-      <c r="D51" s="36">
+      <c r="D51" s="7">
         <v>1.0</v>
       </c>
-      <c r="E51" s="25">
+      <c r="E51" s="12">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52086,11 +52086,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="24"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="10"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52101,15 +52101,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="25">
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52122,15 +52122,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="7">
+      <c r="A54" s="5">
         <v>50.0</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="9">
         <v>100.0</v>
       </c>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="25">
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52160,16 +52160,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="34" t="s">
+      <c r="A56" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="34">
+      <c r="B56" s="41">
         <v>100.0</v>
       </c>
-      <c r="C56" s="15">
+      <c r="C56" s="16">
         <v>1.0</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="16">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52185,8 +52185,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="35"/>
-      <c r="B57" s="35"/>
+      <c r="A57" s="42"/>
+      <c r="B57" s="42"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52200,10 +52200,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="34" t="s">
+      <c r="A58" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="35"/>
+      <c r="B58" s="42"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52217,16 +52217,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="s">
-        <v>7</v>
+      <c r="A59" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B59" s="34">
+      <c r="B59" s="41">
         <v>50.0</v>
       </c>
-      <c r="C59" s="15">
+      <c r="C59" s="16">
         <v>20.0</v>
       </c>
-      <c r="D59" s="15">
+      <c r="D59" s="16">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52242,13 +52242,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="34" t="s">
+      <c r="A60" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="34">
+      <c r="B60" s="41">
         <v>15.0</v>
       </c>
-      <c r="C60" s="15">
+      <c r="C60" s="16">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52265,8 +52265,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="35"/>
-      <c r="B61" s="35"/>
+      <c r="A61" s="42"/>
+      <c r="B61" s="42"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52280,11 +52280,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="34" t="s">
+      <c r="A62" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="34" t="s">
-        <v>12</v>
+      <c r="B62" s="41" t="s">
+        <v>24</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52301,16 +52301,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="34" t="s">
+      <c r="A63" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="34">
+      <c r="B63" s="41">
         <v>5.0</v>
       </c>
-      <c r="C63" s="15">
+      <c r="C63" s="16">
         <v>80.0</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="16">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52326,16 +52326,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="34" t="s">
+      <c r="A64" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="34">
+      <c r="B64" s="41">
         <v>15.0</v>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="16">
         <v>10.0</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="16">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52351,16 +52351,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="34" t="s">
-        <v>16</v>
+      <c r="A65" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B65" s="34">
+      <c r="B65" s="41">
         <v>30.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="16">
         <v>10.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="16">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52376,8 +52376,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="35"/>
-      <c r="B66" s="35"/>
+      <c r="A66" s="42"/>
+      <c r="B66" s="42"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52391,11 +52391,11 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="34" t="s">
+      <c r="A67" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="34" t="s">
-        <v>32</v>
+      <c r="B67" s="41" t="s">
+        <v>31</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
@@ -52412,16 +52412,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="34" t="s">
+      <c r="A68" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="34">
+      <c r="B68" s="41">
         <v>5.0</v>
       </c>
-      <c r="C68" s="15">
+      <c r="C68" s="16">
         <v>80.0</v>
       </c>
-      <c r="D68" s="15">
+      <c r="D68" s="16">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52435,16 +52435,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="34" t="s">
+      <c r="A69" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="34">
+      <c r="B69" s="41">
         <v>15.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="16">
         <v>10.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="16">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52458,16 +52458,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="34" t="s">
-        <v>16</v>
+      <c r="A70" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B70" s="34">
+      <c r="B70" s="41">
         <v>20.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="16">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="16">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52483,8 +52483,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="35"/>
-      <c r="B71" s="35"/>
+      <c r="A71" s="42"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52498,8 +52498,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="34"/>
-      <c r="B72" s="35"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="42"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52513,8 +52513,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="35"/>
-      <c r="B73" s="35"/>
+      <c r="A73" s="42"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-20T11:25:07.635Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -16,10 +16,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="42">
   <si>
-    <t>遮蓋膠紙</t>
+    <t>項目</t>
   </si>
   <si>
-    <t>項目</t>
+    <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>刀壓</t>
@@ -37,10 +37,10 @@
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>Line</t>
+    <t>0.3mm</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>Line</t>
   </si>
   <si>
     <t>Cut-1/2</t>
@@ -49,25 +49,28 @@
     <t>A4紙</t>
   </si>
   <si>
+    <t>(PS)</t>
+  </si>
+  <si>
     <t>03mm</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>0.5mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>(PS -3)</t>
+    <t>1mm</t>
   </si>
   <si>
     <t>PS</t>
@@ -79,9 +82,6 @@
     <t>cut</t>
   </si>
   <si>
-    <t>1mm</t>
-  </si>
-  <si>
     <t>Keep Detail</t>
   </si>
   <si>
@@ -91,28 +91,28 @@
     <t>3mm</t>
   </si>
   <si>
-    <t>６</t>
+    <t>4mm</t>
   </si>
   <si>
-    <t>4mm</t>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>雕刻%</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,23 +321,23 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -348,10 +348,10 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -363,38 +363,35 @@
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -412,26 +409,29 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -679,7 +679,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,16 +719,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -745,16 +745,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="12"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="10"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,11 +785,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -806,7 +806,7 @@
     </row>
     <row r="7">
       <c r="A7" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="16">
         <v>4.0</v>
@@ -817,11 +817,11 @@
       <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -843,11 +843,11 @@
       <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,8 +857,8 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="25"/>
-      <c r="B9" s="7"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="12"/>
@@ -873,12 +873,12 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>21</v>
+      <c r="A10" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="7"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
+      <c r="A11" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
       <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="10"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
+      <c r="A14" s="21"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="10"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,12 +981,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
       <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1000,7 +1000,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B16" s="16">
         <v>5.0</v>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="25"/>
+      <c r="A18" s="21"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>7</v>
+      <c r="A20" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="10"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="10"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,12 +1139,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
-        <v>26</v>
+      <c r="A23" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
       <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B24" s="16">
         <v>5.0</v>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="33"/>
-      <c r="E25" s="34"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>28</v>
+      <c r="B27" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="35">
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>7</v>
+      <c r="A28" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B28" s="7">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="35">
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>13</v>
+      <c r="A29" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="35">
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17098,7 +17098,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,16 +17140,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
+      <c r="A5" s="6" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
       <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,10 +17261,10 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="8"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="20"/>
+      <c r="E9" s="24"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17298,7 +17298,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="16">
         <v>4.0</v>
@@ -17309,7 +17309,7 @@
       <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="24">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17336,7 +17336,7 @@
       <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="24">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17352,7 +17352,7 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" s="16">
         <v>4.0</v>
@@ -17363,7 +17363,7 @@
       <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="24">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17379,7 +17379,7 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -17398,7 +17398,7 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B14" s="16">
         <v>2.0</v>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
-      <c r="E16" s="9"/>
+      <c r="A16" s="28"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>21</v>
+      <c r="A17" s="5" t="s">
+        <v>18</v>
       </c>
-      <c r="B17" s="28" t="s">
-        <v>12</v>
+      <c r="B17" s="29" t="s">
+        <v>11</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="9"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,12 +17549,12 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
       <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -17569,7 +17569,7 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B22" s="16">
         <v>8.0</v>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
+      <c r="A24" s="21"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="9"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,16 +17679,16 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="7">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
       <c r="E27" s="11">
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
+      <c r="A28" s="21"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,12 +17723,12 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
-        <v>26</v>
+      <c r="A29" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
       <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -17743,7 +17743,7 @@
     </row>
     <row r="30">
       <c r="A30" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B30" s="16">
         <v>18.0</v>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="s">
+      <c r="A31" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="32">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="37"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="38" t="s">
-        <v>31</v>
+      <c r="A33" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="39">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="39">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="39">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="40">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="41" t="s">
-        <v>32</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,11 +17872,11 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>28</v>
+      <c r="B36" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -17893,13 +17893,13 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="s">
-        <v>7</v>
+      <c r="A37" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="7">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
       <c r="D37" s="13"/>
@@ -17916,13 +17916,13 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>13</v>
+      <c r="A38" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
       <c r="D38" s="13"/>
@@ -34564,7 +34564,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,16 +34604,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -34630,16 +34630,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="10">
         <v>20.0</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="12">
@@ -34656,16 +34656,16 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" s="6" t="s">
+        <v>13</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="10">
         <v>2.0</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
       <c r="E5" s="12">
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="10"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="9"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,11 +34698,11 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
@@ -34719,7 +34719,7 @@
     </row>
     <row r="8">
       <c r="A8" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="16">
         <v>4.0</v>
@@ -34730,11 +34730,11 @@
       <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34756,11 +34756,11 @@
       <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,8 +34770,8 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="25"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="12"/>
@@ -34786,12 +34786,12 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>21</v>
+      <c r="A11" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
-      <c r="D11" s="7"/>
+      <c r="D11" s="10"/>
       <c r="E11" s="12"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34804,23 +34804,23 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="10">
         <v>5.0</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
       <c r="E12" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
@@ -34830,19 +34830,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>7</v>
+      <c r="A13" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="10">
         <v>15.0</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34854,19 +34854,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="10">
         <v>32.0</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="10">
         <v>5.0</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="10"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34878,11 +34878,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="25"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="10"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34894,12 +34894,12 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
       <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34913,7 +34913,7 @@
     </row>
     <row r="17">
       <c r="A17" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B17" s="16">
         <v>5.0</v>
@@ -34960,11 +34960,11 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="25"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,13 +34976,13 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34994,19 +34994,19 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
-        <v>7</v>
+      <c r="A21" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="10">
         <v>5.0</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="10">
         <v>5.0</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="10">
         <v>1.0</v>
       </c>
-      <c r="E21" s="10"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35018,13 +35018,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="10"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35036,11 +35036,11 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="25"/>
+      <c r="A23" s="21"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="10"/>
+      <c r="E23" s="9"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35052,12 +35052,12 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="s">
-        <v>26</v>
+      <c r="A24" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
       <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -35071,7 +35071,7 @@
     </row>
     <row r="25">
       <c r="A25" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B25" s="16">
         <v>5.0</v>
@@ -35094,17 +35094,17 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="32">
+      <c r="B26" s="31">
         <v>55.0</v>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="31">
         <v>2.0</v>
       </c>
-      <c r="D26" s="33"/>
-      <c r="E26" s="34"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35132,15 +35132,15 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>28</v>
+      <c r="B28" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="35">
+      <c r="E28" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F28" s="4"/>
@@ -35154,17 +35154,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>7</v>
+      <c r="A29" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="10">
         <v>2.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="35">
+      <c r="E29" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F29" s="4"/>
@@ -35178,17 +35178,17 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>13</v>
+      <c r="A30" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="10">
         <v>20.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="10">
         <v>100.0</v>
       </c>
       <c r="D30" s="13"/>
-      <c r="E30" s="35">
+      <c r="E30" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F30" s="4"/>
@@ -51010,7 +51010,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>2</v>
@@ -51034,13 +51034,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51051,19 +51051,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="8">
         <v>60.0</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51074,11 +51074,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="8"/>
+      <c r="A4" s="5"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="9"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51089,11 +51089,11 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>11</v>
+      <c r="B5" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -51108,16 +51108,16 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>13</v>
+      <c r="A6" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
       <c r="E6" s="11">
@@ -51133,11 +51133,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="8"/>
+      <c r="A7" s="5"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="9"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51148,13 +51148,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>16</v>
+      <c r="A8" s="5" t="s">
+        <v>17</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51165,16 +51165,16 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
       <c r="E9" s="11">
@@ -51190,16 +51190,16 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>13</v>
+      <c r="A10" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
       <c r="E10" s="11">
@@ -51215,11 +51215,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="8"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="21"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="22"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51231,13 +51231,13 @@
     </row>
     <row r="12">
       <c r="A12" s="23" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>18</v>
+      <c r="B12" s="25" t="s">
+        <v>19</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -51249,16 +51249,16 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>19</v>
+      <c r="A13" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="11">
@@ -51274,16 +51274,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="11"/>
@@ -51297,22 +51297,22 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>20</v>
+      <c r="A15" s="6" t="s">
+        <v>21</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
       <c r="E15" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G15" s="4"/>
@@ -51324,16 +51324,16 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>13</v>
+      <c r="A16" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
       <c r="E16" s="11">
@@ -51349,11 +51349,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="21"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51364,13 +51364,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51381,16 +51381,16 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>7</v>
+      <c r="A19" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="8">
         <v>6.0</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="8">
         <v>45.0</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
       <c r="E19" s="11">
@@ -51406,16 +51406,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="8">
         <v>18.0</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="8">
         <v>20.0</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="11">
@@ -51431,11 +51431,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
+      <c r="A21" s="6"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51449,8 +51449,8 @@
       <c r="A22" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>18</v>
+      <c r="B22" s="25" t="s">
+        <v>19</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -51467,16 +51467,16 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>19</v>
+      <c r="A23" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B23" s="6">
+      <c r="B23" s="8">
         <v>6.0</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="8">
         <v>50.0</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
       <c r="E23" s="11">
@@ -51492,16 +51492,16 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
+      <c r="A24" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="6">
+      <c r="B24" s="8">
         <v>8.0</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="8">
         <v>30.0</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
       <c r="E24" s="11">
@@ -51517,22 +51517,22 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>13</v>
+      <c r="A25" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B25" s="6">
+      <c r="B25" s="8">
         <v>10.0</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="8">
         <v>30.0</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
       <c r="E25" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G25" s="4"/>
@@ -51544,16 +51544,16 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>13</v>
+      <c r="A26" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B26" s="6">
+      <c r="B26" s="8">
         <v>17.0</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
       <c r="E26" s="11">
@@ -51569,11 +51569,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
+      <c r="A27" s="6"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51585,14 +51585,14 @@
     </row>
     <row r="28">
       <c r="A28" s="23" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
-      <c r="B28" s="24" t="s">
-        <v>18</v>
+      <c r="B28" s="25" t="s">
+        <v>19</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51603,16 +51603,16 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>19</v>
+      <c r="A29" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="8">
         <v>6.0</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="8">
         <v>50.0</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
       <c r="E29" s="11">
@@ -51628,19 +51628,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>7</v>
+      <c r="A30" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="8">
         <v>8.0</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="8">
         <v>30.0</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51651,16 +51651,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="6">
+      <c r="B31" s="8">
         <v>15.0</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="8">
         <v>10.0</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
       <c r="E31" s="11">
@@ -51676,11 +51676,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
+      <c r="A32" s="6"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="9"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51691,8 +51691,8 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="s">
-        <v>21</v>
+      <c r="A33" s="14" t="s">
+        <v>18</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
@@ -51709,18 +51709,18 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B34" s="30" t="s">
-        <v>25</v>
+      <c r="B34" s="35" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C34" s="35">
         <v>40.0</v>
       </c>
-      <c r="D34" s="30">
+      <c r="D34" s="35">
         <v>1.0</v>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="24">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51736,13 +51736,13 @@
       <c r="A35" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="30">
+      <c r="B35" s="35">
         <v>30.0</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="35">
         <v>15.0</v>
       </c>
-      <c r="D35" s="30">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
       <c r="E35" s="26"/>
@@ -51756,11 +51756,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="25"/>
+      <c r="A36" s="21"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="9"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51771,13 +51771,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>27</v>
+      <c r="A37" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="9"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51788,16 +51788,16 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
       <c r="E38" s="11">
@@ -51813,11 +51813,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="8"/>
+      <c r="A39" s="5"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="9"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51828,13 +51828,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="9"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51845,16 +51845,16 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>7</v>
+      <c r="A41" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B41" s="7">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="7">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="7">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
       <c r="E41" s="11">
@@ -51870,16 +51870,16 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="7">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="7">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="7">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
       <c r="E42" s="11">
@@ -51895,23 +51895,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>7</v>
+      <c r="A43" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B43" s="7">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="7">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="7">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
       <c r="E43" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="14" t="s">
-        <v>29</v>
+      <c r="F43" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51922,11 +51922,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="36"/>
+      <c r="A44" s="42"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="9"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51937,13 +51937,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="36" t="s">
-        <v>26</v>
+      <c r="A45" s="42" t="s">
+        <v>25</v>
       </c>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="9"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51954,16 +51954,16 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="7">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="7">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="7">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
       <c r="E46" s="11">
@@ -51979,11 +51979,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="36"/>
+      <c r="A47" s="42"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="9"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -51994,13 +51994,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="36" t="s">
-        <v>30</v>
+      <c r="A48" s="42" t="s">
+        <v>32</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="9"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52011,16 +52011,16 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>14</v>
+      <c r="A49" s="6" t="s">
+        <v>13</v>
       </c>
-      <c r="B49" s="6">
+      <c r="B49" s="8">
         <v>70.0</v>
       </c>
-      <c r="C49" s="6">
+      <c r="C49" s="8">
         <v>300.0</v>
       </c>
-      <c r="D49" s="6">
+      <c r="D49" s="8">
         <v>1.0</v>
       </c>
       <c r="E49" s="11">
@@ -52036,20 +52036,20 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>7</v>
+      <c r="A50" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B50" s="6">
+      <c r="B50" s="8">
         <v>10.0</v>
       </c>
-      <c r="C50" s="6">
-        <v>85.0</v>
+      <c r="C50" s="8">
+        <v>20.0</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D50" s="8">
         <v>1.0</v>
       </c>
       <c r="E50" s="11">
-        <v>45900.48745738426</v>
+        <v>46223.80908288194</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52061,16 +52061,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="6">
+      <c r="B51" s="8">
         <v>70.0</v>
       </c>
-      <c r="C51" s="6">
+      <c r="C51" s="8">
         <v>10.0</v>
       </c>
-      <c r="D51" s="6">
+      <c r="D51" s="8">
         <v>1.0</v>
       </c>
       <c r="E51" s="11">
@@ -52086,11 +52086,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="9"/>
+      <c r="A52" s="6"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="7"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52101,14 +52101,14 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B53" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
       <c r="E53" s="11">
         <v>45946.87875708334</v>
       </c>
@@ -52122,10 +52122,10 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="5">
+      <c r="A54" s="6">
         <v>50.0</v>
       </c>
-      <c r="B54" s="7">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
       <c r="C54" s="13"/>
@@ -52160,16 +52160,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="s">
+      <c r="A56" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="41">
+      <c r="B56" s="40">
         <v>100.0</v>
       </c>
-      <c r="C56" s="14">
+      <c r="C56" s="15">
         <v>1.0</v>
       </c>
-      <c r="D56" s="14">
+      <c r="D56" s="15">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52185,8 +52185,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="42"/>
-      <c r="B57" s="42"/>
+      <c r="A57" s="41"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52200,10 +52200,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52217,16 +52217,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="41">
+      <c r="B59" s="40">
         <v>50.0</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="15">
         <v>20.0</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59" s="15">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52242,13 +52242,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="41" t="s">
+      <c r="A60" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="41">
+      <c r="B60" s="40">
         <v>15.0</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="15">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52265,8 +52265,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="42"/>
-      <c r="B61" s="42"/>
+      <c r="A61" s="41"/>
+      <c r="B61" s="41"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52280,10 +52280,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="41" t="s">
+      <c r="B62" s="40" t="s">
         <v>24</v>
       </c>
       <c r="C62" s="4"/>
@@ -52301,16 +52301,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="41">
+      <c r="B63" s="40">
         <v>5.0</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="15">
         <v>80.0</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="15">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52326,16 +52326,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="41">
+      <c r="B64" s="40">
         <v>15.0</v>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="15">
         <v>10.0</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64" s="15">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52351,16 +52351,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="41" t="s">
-        <v>13</v>
+      <c r="A65" s="40" t="s">
+        <v>14</v>
       </c>
-      <c r="B65" s="41">
+      <c r="B65" s="40">
         <v>30.0</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="15">
         <v>10.0</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52376,8 +52376,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="42"/>
-      <c r="B66" s="42"/>
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52391,11 +52391,11 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="41" t="s">
-        <v>30</v>
+      <c r="B67" s="40" t="s">
+        <v>32</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
@@ -52412,16 +52412,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="40">
         <v>5.0</v>
       </c>
-      <c r="C68" s="14">
+      <c r="C68" s="15">
         <v>80.0</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="15">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52435,16 +52435,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="40">
         <v>15.0</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="15">
         <v>10.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52458,16 +52458,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="41" t="s">
-        <v>13</v>
+      <c r="A70" s="40" t="s">
+        <v>14</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="40">
         <v>20.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="15">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52483,8 +52483,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="42"/>
-      <c r="B71" s="42"/>
+      <c r="A71" s="41"/>
+      <c r="B71" s="41"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52498,8 +52498,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="42"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52513,8 +52513,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="42"/>
-      <c r="B73" s="42"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:05.742Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -52,6 +52,9 @@
     <t>03mm</t>
   </si>
   <si>
+    <t>FILL</t>
+  </si>
+  <si>
     <t>(PS)</t>
   </si>
   <si>
@@ -61,16 +64,10 @@
     <t>0.5mm</t>
   </si>
   <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>1mm</t>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>PS</t>
@@ -79,13 +76,16 @@
     <t>Fill</t>
   </si>
   <si>
+    <t>1mm</t>
+  </si>
+  <si>
     <t>cut</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>Keep Detail</t>
   </si>
   <si>
-    <t>Keep Detail</t>
+    <t>2mm</t>
   </si>
   <si>
     <t>3mm</t>
@@ -94,10 +94,10 @@
     <t>4mm</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
+    <t>６</t>
   </si>
   <si>
-    <t>６</t>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -109,12 +109,6 @@
     <t>5mm</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
     <t>雕刻%</t>
   </si>
   <si>
@@ -124,7 +118,13 @@
     <t>20mm</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>Cut1-2</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>柔光板</t>
@@ -333,11 +333,11 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -351,14 +351,14 @@
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -366,28 +366,28 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -406,10 +406,10 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -418,11 +418,20 @@
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -431,15 +440,6 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -722,13 +722,13 @@
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -748,13 +748,13 @@
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="11"/>
@@ -770,9 +770,9 @@
     </row>
     <row r="5">
       <c r="A5" s="6"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
       <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -786,14 +786,14 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="B6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,20 +808,20 @@
       <c r="A7" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
       <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,20 +834,20 @@
       <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
       <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,8 +857,8 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="11"/>
@@ -874,11 +874,11 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="9"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -894,20 +894,20 @@
       <c r="A11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
       <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,13 +920,13 @@
       <c r="A12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
       <c r="E12" s="8"/>
@@ -944,13 +944,13 @@
       <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="8"/>
@@ -965,7 +965,7 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
+      <c r="A14" s="23"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -982,12 +982,12 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,16 +1002,16 @@
       <c r="A16" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,16 +1026,16 @@
       <c r="A17" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,7 +1047,7 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
+      <c r="A18" s="23"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
@@ -1084,13 +1084,13 @@
       <c r="A20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="8"/>
@@ -1123,7 +1123,7 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
+      <c r="A22" s="23"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -1142,10 +1142,10 @@
       <c r="A23" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,16 +1160,16 @@
       <c r="A24" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>26</v>
+      <c r="B27" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="34">
+      <c r="E27" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="34">
+      <c r="E28" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>13</v>
+      <c r="A29" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="34">
+      <c r="E29" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17127,7 +17127,7 @@
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,13 +17143,13 @@
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -17170,16 +17170,16 @@
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17193,12 +17193,12 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,19 +17214,19 @@
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,19 +17239,19 @@
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17262,9 +17262,9 @@
     </row>
     <row r="8">
       <c r="A8" s="6"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17279,12 +17279,12 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="23"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,16 +17300,16 @@
       <c r="A10" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="25">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,16 +17327,16 @@
       <c r="A11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="25">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17352,18 +17352,18 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="25">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17379,12 +17379,12 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="27"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,16 +17400,16 @@
       <c r="A14" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,16 +17425,16 @@
       <c r="A15" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="16">
       <c r="A16" s="28"/>
-      <c r="E16" s="10"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17462,14 +17462,14 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,16 +17485,16 @@
       <c r="A18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,16 +17510,16 @@
       <c r="A19" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17550,12 +17550,12 @@
     </row>
     <row r="21">
       <c r="A21" s="14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,16 +17571,16 @@
       <c r="A22" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,16 +17596,16 @@
       <c r="A23" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="10"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17641,7 +17641,7 @@
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,16 +17657,16 @@
       <c r="A26" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,13 +17682,13 @@
       <c r="A27" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
       <c r="E27" s="12">
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
+      <c r="A28" s="23"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,10 +17726,10 @@
       <c r="A29" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,16 +17745,16 @@
       <c r="A30" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="38" t="s">
-        <v>31</v>
+      <c r="A33" s="39" t="s">
+        <v>34</v>
       </c>
-      <c r="B33" s="39">
+      <c r="B33" s="41">
         <v>5.0</v>
       </c>
-      <c r="C33" s="39">
+      <c r="C33" s="41">
         <v>10.0</v>
       </c>
-      <c r="D33" s="39">
+      <c r="D33" s="41">
         <v>2.0</v>
       </c>
-      <c r="E33" s="40">
+      <c r="E33" s="43">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="41" t="s">
-        <v>32</v>
+      <c r="F33" s="44" t="s">
+        <v>36</v>
       </c>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="G33" s="45"/>
+      <c r="H33" s="45"/>
+      <c r="I33" s="45"/>
+      <c r="J33" s="45"/>
+      <c r="K33" s="45"/>
+      <c r="L33" s="45"/>
+      <c r="M33" s="45"/>
+      <c r="N33" s="45"/>
+      <c r="O33" s="45"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,11 +17872,11 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>26</v>
+      <c r="B36" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -17893,13 +17893,13 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
       <c r="D37" s="13"/>
@@ -17916,13 +17916,13 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
-        <v>13</v>
+      <c r="A38" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
       <c r="D38" s="13"/>
@@ -34607,13 +34607,13 @@
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -34633,13 +34633,13 @@
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>20.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="11">
@@ -34657,15 +34657,15 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>2.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
       <c r="E5" s="11">
@@ -34683,9 +34683,9 @@
     </row>
     <row r="6">
       <c r="A6" s="6"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="8"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -34699,14 +34699,14 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="B7" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34721,20 +34721,20 @@
       <c r="A8" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>4.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>10.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
       <c r="E8" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34747,20 +34747,20 @@
       <c r="A9" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <v>20.0</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
       <c r="E9" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,8 +34770,8 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="20"/>
-      <c r="B10" s="9"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="11"/>
@@ -34786,8 +34786,8 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="9"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="11"/>
@@ -34802,12 +34802,10 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="13"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="13"/>
-      <c r="D12" s="9"/>
+      <c r="D12" s="13"/>
       <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -34820,23 +34818,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="9">
-        <v>5.0</v>
-      </c>
-      <c r="C13" s="9">
-        <v>5.0</v>
-      </c>
-      <c r="D13" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E13" s="11">
-        <v>46042.0</v>
-      </c>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
+      <c r="A13" s="23"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
@@ -34846,19 +34834,13 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="6" t="s">
+        <v>20</v>
       </c>
-      <c r="B14" s="9">
-        <v>5.0</v>
-      </c>
-      <c r="C14" s="9">
-        <v>15.0</v>
-      </c>
-      <c r="D14" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E14" s="8"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34871,20 +34853,22 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B15" s="9">
-        <v>32.0</v>
-      </c>
-      <c r="C15" s="9">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="C15" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="D15" s="10">
         <v>1.0</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
+      <c r="E15" s="11">
+        <v>46042.0</v>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
@@ -34894,10 +34878,18 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="20"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
+      <c r="A16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="C16" s="10">
+        <v>15.0</v>
+      </c>
+      <c r="D16" s="10">
+        <v>1.0</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34910,13 +34902,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="s">
-        <v>22</v>
+      <c r="A17" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="16"/>
+      <c r="B17" s="10">
+        <v>32.0</v>
+      </c>
+      <c r="C17" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="D17" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E17" s="8"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34928,19 +34926,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="C18" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="D18" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="16"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34952,19 +34942,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="s">
-        <v>9</v>
+      <c r="A19" s="14" t="s">
+        <v>23</v>
       </c>
-      <c r="B19" s="15">
-        <v>50.0</v>
-      </c>
-      <c r="C19" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="D19" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E19" s="16"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="17"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,11 +34960,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="C20" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="D20" s="16">
+        <v>1.0</v>
+      </c>
+      <c r="E20" s="17"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34992,13 +34984,19 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
-        <v>24</v>
+      <c r="A21" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="8"/>
+      <c r="B21" s="16">
+        <v>50.0</v>
+      </c>
+      <c r="C21" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="D21" s="16">
+        <v>1.0</v>
+      </c>
+      <c r="E21" s="17"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35010,18 +35008,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" s="9">
-        <v>5.0</v>
-      </c>
-      <c r="C22" s="9">
-        <v>5.0</v>
-      </c>
-      <c r="D22" s="9">
-        <v>1.0</v>
-      </c>
+      <c r="A22" s="23"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -35034,8 +35024,8 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>9</v>
+      <c r="A23" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -35052,10 +35042,18 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="A24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="C24" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="D24" s="10">
+        <v>1.0</v>
+      </c>
       <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -35068,13 +35066,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="s">
-        <v>25</v>
+      <c r="A25" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="16"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35086,19 +35084,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="C26" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="D26" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="16"/>
+      <c r="A26" s="23"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35110,17 +35100,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="30" t="s">
-        <v>9</v>
+      <c r="A27" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B27" s="31">
-        <v>55.0</v>
-      </c>
-      <c r="C27" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="D27" s="32"/>
-      <c r="E27" s="33"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="17"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35132,11 +35118,19 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
+      <c r="A28" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="C28" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="D28" s="16">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="17"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35148,17 +35142,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>10</v>
+      <c r="A29" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B29" s="9" t="s">
-        <v>26</v>
+      <c r="B29" s="31">
+        <v>55.0</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="34">
-        <v>46051.96156388889</v>
+      <c r="C29" s="31">
+        <v>2.0</v>
       </c>
+      <c r="D29" s="32"/>
+      <c r="E29" s="33"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35170,19 +35164,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="9">
-        <v>2.0</v>
-      </c>
-      <c r="C30" s="9">
-        <v>100.0</v>
-      </c>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
       <c r="D30" s="13"/>
-      <c r="E30" s="34">
-        <v>46100.83597384259</v>
-      </c>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35194,18 +35180,16 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="s">
-        <v>13</v>
+      <c r="A31" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B31" s="9">
-        <v>20.0</v>
+      <c r="B31" s="10" t="s">
+        <v>27</v>
       </c>
-      <c r="C31" s="9">
-        <v>100.0</v>
-      </c>
+      <c r="C31" s="13"/>
       <c r="D31" s="13"/>
-      <c r="E31" s="34">
-        <v>46100.83604224537</v>
+      <c r="E31" s="35">
+        <v>46051.96156388889</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -35218,11 +35202,19 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
+      <c r="A32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="C32" s="10">
+        <v>100.0</v>
+      </c>
       <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="E32" s="35">
+        <v>46100.83597384259</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35234,11 +35226,19 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
+      <c r="A33" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="10">
+        <v>20.0</v>
+      </c>
+      <c r="C33" s="10">
+        <v>100.0</v>
+      </c>
       <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="E33" s="35">
+        <v>46100.83604224537</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35250,11 +35250,11 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -35266,11 +35266,11 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51008,6 +51008,38 @@
       <c r="L1018" s="4"/>
       <c r="M1018" s="4"/>
       <c r="N1018" s="4"/>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="4"/>
+      <c r="B1019" s="4"/>
+      <c r="C1019" s="4"/>
+      <c r="D1019" s="4"/>
+      <c r="E1019" s="4"/>
+      <c r="F1019" s="4"/>
+      <c r="G1019" s="4"/>
+      <c r="H1019" s="4"/>
+      <c r="I1019" s="4"/>
+      <c r="J1019" s="4"/>
+      <c r="K1019" s="4"/>
+      <c r="L1019" s="4"/>
+      <c r="M1019" s="4"/>
+      <c r="N1019" s="4"/>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="4"/>
+      <c r="B1020" s="4"/>
+      <c r="C1020" s="4"/>
+      <c r="D1020" s="4"/>
+      <c r="E1020" s="4"/>
+      <c r="F1020" s="4"/>
+      <c r="G1020" s="4"/>
+      <c r="H1020" s="4"/>
+      <c r="I1020" s="4"/>
+      <c r="J1020" s="4"/>
+      <c r="K1020" s="4"/>
+      <c r="L1020" s="4"/>
+      <c r="M1020" s="4"/>
+      <c r="N1020" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -51055,8 +51087,8 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51076,10 +51108,10 @@
       <c r="C3" s="7">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="9"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51094,7 +51126,7 @@
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="10"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51125,15 +51157,15 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
       <c r="E6" s="12">
@@ -51153,7 +51185,7 @@
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="10"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51165,12 +51197,12 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="9"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51184,13 +51216,13 @@
       <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
       <c r="E9" s="12">
@@ -51207,15 +51239,15 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
       <c r="E10" s="12">
@@ -51232,10 +51264,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="6"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="22"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="21"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51246,14 +51278,14 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="s">
-        <v>17</v>
+      <c r="A12" s="22" t="s">
+        <v>16</v>
       </c>
-      <c r="B12" s="25" t="s">
-        <v>19</v>
+      <c r="B12" s="24" t="s">
+        <v>18</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -51266,15 +51298,15 @@
     </row>
     <row r="13" ht="20.25" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="12">
@@ -51293,13 +51325,13 @@
       <c r="A14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="12"/>
@@ -51316,20 +51348,20 @@
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
       <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="17" t="s">
-        <v>23</v>
+      <c r="F15" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51341,15 +51373,15 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
       <c r="E16" s="12">
@@ -51366,10 +51398,10 @@
     </row>
     <row r="17">
       <c r="A17" s="6"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51381,12 +51413,12 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51406,7 +51438,7 @@
       <c r="C19" s="7">
         <v>45.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
       <c r="E19" s="12">
@@ -51431,7 +51463,7 @@
       <c r="C20" s="7">
         <v>20.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="12">
@@ -51451,7 +51483,7 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="10"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51462,11 +51494,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="s">
-        <v>14</v>
+      <c r="A22" s="22" t="s">
+        <v>15</v>
       </c>
-      <c r="B22" s="25" t="s">
-        <v>19</v>
+      <c r="B22" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -51484,7 +51516,7 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" s="7">
         <v>6.0</v>
@@ -51492,7 +51524,7 @@
       <c r="C23" s="7">
         <v>50.0</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
       <c r="E23" s="12">
@@ -51517,7 +51549,7 @@
       <c r="C24" s="7">
         <v>30.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
       <c r="E24" s="12">
@@ -51534,7 +51566,7 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B25" s="7">
         <v>10.0</v>
@@ -51542,14 +51574,14 @@
       <c r="C25" s="7">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
       <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="17" t="s">
-        <v>23</v>
+      <c r="F25" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51561,7 +51593,7 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" s="7">
         <v>17.0</v>
@@ -51569,7 +51601,7 @@
       <c r="C26" s="7">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
       <c r="E26" s="12">
@@ -51589,7 +51621,7 @@
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="10"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51600,15 +51632,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="24" t="s">
         <v>18</v>
-      </c>
-      <c r="B28" s="25" t="s">
-        <v>19</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51620,7 +51652,7 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B29" s="7">
         <v>6.0</v>
@@ -51628,7 +51660,7 @@
       <c r="C29" s="7">
         <v>50.0</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
       <c r="E29" s="12">
@@ -51653,10 +51685,10 @@
       <c r="C30" s="7">
         <v>30.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="10"/>
+      <c r="E30" s="9"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51676,7 +51708,7 @@
       <c r="C31" s="7">
         <v>10.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
       <c r="E31" s="12">
@@ -51696,7 +51728,7 @@
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="10"/>
+      <c r="E32" s="9"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51708,12 +51740,12 @@
     </row>
     <row r="33">
       <c r="A33" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="27"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51727,16 +51759,16 @@
       <c r="A34" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B34" s="35" t="s">
-        <v>27</v>
+      <c r="B34" s="34" t="s">
+        <v>26</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="34">
         <v>40.0</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="34">
         <v>1.0</v>
       </c>
-      <c r="E34" s="23">
+      <c r="E34" s="25">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51752,16 +51784,16 @@
       <c r="A35" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="35">
+      <c r="B35" s="34">
         <v>30.0</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="34">
         <v>15.0</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="34">
         <v>1.0</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51772,11 +51804,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="20"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="10"/>
+      <c r="E36" s="9"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51793,7 +51825,7 @@
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="10"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51807,13 +51839,13 @@
       <c r="A38" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
       <c r="E38" s="12">
@@ -51833,7 +51865,7 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="10"/>
+      <c r="E39" s="9"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51845,12 +51877,12 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="10"/>
+      <c r="E40" s="9"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51864,13 +51896,13 @@
       <c r="A41" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
       <c r="E41" s="12">
@@ -51889,13 +51921,13 @@
       <c r="A42" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
       <c r="E42" s="12">
@@ -51914,19 +51946,19 @@
       <c r="A43" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
       <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="17" t="s">
+      <c r="F43" s="15" t="s">
         <v>29</v>
       </c>
       <c r="G43" s="4"/>
@@ -51942,7 +51974,7 @@
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="10"/>
+      <c r="E44" s="9"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51959,7 +51991,7 @@
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="10"/>
+      <c r="E45" s="9"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -51973,13 +52005,13 @@
       <c r="A46" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
       <c r="E46" s="12">
@@ -51999,7 +52031,7 @@
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="10"/>
+      <c r="E47" s="9"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52016,7 +52048,7 @@
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="10"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52028,7 +52060,7 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B49" s="7">
         <v>70.0</v>
@@ -52103,10 +52135,10 @@
     </row>
     <row r="52">
       <c r="A52" s="5"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="10"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="9"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52118,13 +52150,13 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
-      <c r="B53" s="9" t="s">
-        <v>34</v>
+      <c r="B53" s="10" t="s">
+        <v>32</v>
       </c>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
       <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
@@ -52141,7 +52173,7 @@
       <c r="A54" s="5">
         <v>50.0</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
       <c r="C54" s="13"/>
@@ -52159,13 +52191,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="43" t="s">
-        <v>35</v>
+      <c r="A55" s="38" t="s">
+        <v>33</v>
       </c>
-      <c r="B55" s="44"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="40"/>
+      <c r="C55" s="40"/>
+      <c r="D55" s="40"/>
+      <c r="E55" s="42"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52176,16 +52208,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="s">
-        <v>36</v>
+      <c r="A56" s="44" t="s">
+        <v>35</v>
       </c>
-      <c r="B56" s="41">
+      <c r="B56" s="44">
         <v>100.0</v>
       </c>
-      <c r="C56" s="17">
+      <c r="C56" s="15">
         <v>1.0</v>
       </c>
-      <c r="D56" s="17">
+      <c r="D56" s="15">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52201,8 +52233,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="42"/>
-      <c r="B57" s="42"/>
+      <c r="A57" s="45"/>
+      <c r="B57" s="45"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52216,10 +52248,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="45"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52236,13 +52268,13 @@
       <c r="A59" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="41">
+      <c r="B59" s="44">
         <v>50.0</v>
       </c>
-      <c r="C59" s="17">
+      <c r="C59" s="15">
         <v>20.0</v>
       </c>
-      <c r="D59" s="17">
+      <c r="D59" s="15">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52258,13 +52290,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="41" t="s">
+      <c r="A60" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="41">
+      <c r="B60" s="44">
         <v>15.0</v>
       </c>
-      <c r="C60" s="17">
+      <c r="C60" s="15">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52281,8 +52313,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="42"/>
-      <c r="B61" s="42"/>
+      <c r="A61" s="45"/>
+      <c r="B61" s="45"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52296,10 +52328,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="41" t="s">
+      <c r="B62" s="44" t="s">
         <v>24</v>
       </c>
       <c r="C62" s="4"/>
@@ -52317,16 +52349,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="41">
+      <c r="B63" s="44">
         <v>5.0</v>
       </c>
-      <c r="C63" s="17">
+      <c r="C63" s="15">
         <v>80.0</v>
       </c>
-      <c r="D63" s="17">
+      <c r="D63" s="15">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52342,16 +52374,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="41">
+      <c r="B64" s="44">
         <v>15.0</v>
       </c>
-      <c r="C64" s="17">
+      <c r="C64" s="15">
         <v>10.0</v>
       </c>
-      <c r="D64" s="17">
+      <c r="D64" s="15">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52367,16 +52399,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="41" t="s">
-        <v>13</v>
+      <c r="A65" s="44" t="s">
+        <v>14</v>
       </c>
-      <c r="B65" s="41">
+      <c r="B65" s="44">
         <v>30.0</v>
       </c>
-      <c r="C65" s="17">
+      <c r="C65" s="15">
         <v>10.0</v>
       </c>
-      <c r="D65" s="17">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52392,8 +52424,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="42"/>
-      <c r="B66" s="42"/>
+      <c r="A66" s="45"/>
+      <c r="B66" s="45"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52407,10 +52439,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="41" t="s">
+      <c r="B67" s="44" t="s">
         <v>30</v>
       </c>
       <c r="C67" s="4"/>
@@ -52428,16 +52460,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="44">
         <v>5.0</v>
       </c>
-      <c r="C68" s="17">
+      <c r="C68" s="15">
         <v>80.0</v>
       </c>
-      <c r="D68" s="17">
+      <c r="D68" s="15">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52451,16 +52483,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="44">
         <v>15.0</v>
       </c>
-      <c r="C69" s="17">
+      <c r="C69" s="15">
         <v>10.0</v>
       </c>
-      <c r="D69" s="17">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52474,16 +52506,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="41" t="s">
-        <v>13</v>
+      <c r="A70" s="44" t="s">
+        <v>14</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="44">
         <v>20.0</v>
       </c>
-      <c r="C70" s="17">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="17">
+      <c r="D70" s="15">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52499,8 +52531,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="42"/>
-      <c r="B71" s="42"/>
+      <c r="A71" s="45"/>
+      <c r="B71" s="45"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52514,8 +52546,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="42"/>
+      <c r="A72" s="44"/>
+      <c r="B72" s="45"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52529,8 +52561,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="42"/>
-      <c r="B73" s="42"/>
+      <c r="A73" s="45"/>
+      <c r="B73" s="45"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:08.063Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,13 +19,10 @@
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
   </si>
   <si>
-    <t>刀壓</t>
+    <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>速度</t>
@@ -34,70 +31,79 @@
     <t>次數</t>
   </si>
   <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>最後更新日期</t>
+  </si>
+  <si>
+    <t>0.3mm</t>
   </si>
   <si>
     <t>Line</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut-1/2</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>A4紙</t>
   </si>
   <si>
-    <t>03mm</t>
+    <t>0.5mm</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>03mm</t>
   </si>
   <si>
     <t>(PS)</t>
   </si>
   <si>
-    <t>Cut</t>
+    <t>(PS -3)</t>
   </si>
   <si>
-    <t>0.5mm</t>
+    <t>Cut</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>(PS -3)</t>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>2mm</t>
+  </si>
+  <si>
+    <t>Fill</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
-    <t>Fill</t>
+    <t>cut</t>
   </si>
   <si>
-    <t>1mm</t>
-  </si>
-  <si>
-    <t>cut</t>
+    <t>3mm</t>
   </si>
   <si>
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
-    <t>3mm</t>
-  </si>
-  <si>
     <t>4mm</t>
   </si>
   <si>
-    <t>６</t>
+    <t>(0.9 Power)</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
+    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -118,13 +124,7 @@
     <t>20mm</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
     <t>Cut1-2</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>柔光板</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,13 +321,7 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -335,6 +329,12 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -351,19 +351,25 @@
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -372,22 +378,16 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -406,40 +406,40 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -682,13 +682,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,8 +719,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="10">
         <v>2.0</v>
@@ -745,7 +745,7 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="10">
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6"/>
+      <c r="A5" s="5"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
-      <c r="E5" s="8"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -786,14 +786,14 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -806,22 +806,22 @@
     </row>
     <row r="7">
       <c r="A7" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
       <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,20 +834,20 @@
       <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
       <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,7 +857,7 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="23"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
@@ -873,8 +873,8 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>20</v>
+      <c r="A10" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -891,8 +891,8 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
+      <c r="A11" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B11" s="10">
         <v>5.0</v>
@@ -906,8 +906,8 @@
       <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,8 +917,8 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B12" s="10">
         <v>5.0</v>
@@ -929,7 +929,7 @@
       <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,7 +941,7 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="10">
@@ -953,7 +953,7 @@
       <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="23"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="8"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -982,12 +982,12 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1000,18 +1000,18 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,16 +1026,16 @@
       <c r="A17" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="23"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="8"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>24</v>
+      <c r="A19" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,8 +1081,8 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>7</v>
+      <c r="A20" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B20" s="10">
         <v>5.0</v>
@@ -1093,7 +1093,7 @@
       <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="8"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="23"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,10 +1142,10 @@
       <c r="A23" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1158,18 +1158,18 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1220,14 +1220,14 @@
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="35">
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B28" s="10">
         <v>2.0</v>
@@ -1251,7 +1251,7 @@
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="35">
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B29" s="10">
         <v>20.0</v>
@@ -1275,7 +1275,7 @@
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="35">
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17101,13 +17101,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,8 +17140,8 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="10">
         <v>3.0</v>
@@ -17167,7 +17167,7 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="10">
@@ -17179,7 +17179,7 @@
       <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>13</v>
+      <c r="A5" s="8" t="s">
+        <v>14</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,8 +17211,8 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="10">
         <v>2.0</v>
@@ -17223,10 +17223,10 @@
       <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,7 +17236,7 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="10">
@@ -17249,9 +17249,9 @@
         <v>1.0</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,7 +17261,7 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
+      <c r="A8" s="5"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -17279,12 +17279,12 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="25"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17298,18 +17298,18 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,16 +17327,16 @@
       <c r="A11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17352,18 +17352,18 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17379,12 +17379,12 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="27"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17398,18 +17398,18 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,16 +17425,16 @@
       <c r="A15" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="16">
       <c r="A16" s="28"/>
-      <c r="E16" s="9"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>20</v>
+      <c r="A17" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
-      <c r="E17" s="9"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,8 +17482,8 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B18" s="10">
         <v>5.0</v>
@@ -17494,7 +17494,7 @@
       <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,7 +17507,7 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="10">
@@ -17519,7 +17519,7 @@
       <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="23"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17550,12 +17550,12 @@
     </row>
     <row r="21">
       <c r="A21" s="14" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17569,18 +17569,18 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,16 +17596,16 @@
       <c r="A23" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="23"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>24</v>
+      <c r="A25" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,8 +17654,8 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B26" s="10">
         <v>10.0</v>
@@ -17666,7 +17666,7 @@
       <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="9"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,7 +17679,7 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="10">
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="23"/>
+      <c r="A28" s="20"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,10 +17726,10 @@
       <c r="A29" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17743,18 +17743,18 @@
     </row>
     <row r="30">
       <c r="A30" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17779,7 +17779,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="37"/>
+      <c r="E31" s="35"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="39" t="s">
-        <v>34</v>
+      <c r="A33" s="36" t="s">
+        <v>27</v>
       </c>
-      <c r="B33" s="41">
+      <c r="B33" s="37">
         <v>5.0</v>
       </c>
-      <c r="C33" s="41">
+      <c r="C33" s="37">
         <v>10.0</v>
       </c>
-      <c r="D33" s="41">
+      <c r="D33" s="37">
         <v>2.0</v>
       </c>
-      <c r="E33" s="43">
+      <c r="E33" s="38">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="44" t="s">
-        <v>36</v>
+      <c r="F33" s="39" t="s">
+        <v>28</v>
       </c>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
-      <c r="I33" s="45"/>
-      <c r="J33" s="45"/>
-      <c r="K33" s="45"/>
-      <c r="L33" s="45"/>
-      <c r="M33" s="45"/>
-      <c r="N33" s="45"/>
-      <c r="O33" s="45"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17873,10 +17873,10 @@
     </row>
     <row r="36">
       <c r="A36" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -17894,7 +17894,7 @@
     </row>
     <row r="37">
       <c r="A37" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B37" s="10">
         <v>2.0</v>
@@ -17917,7 +17917,7 @@
     </row>
     <row r="38">
       <c r="A38" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B38" s="10">
         <v>20.0</v>
@@ -34567,13 +34567,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,8 +34604,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="10">
         <v>2.0</v>
@@ -34630,7 +34630,7 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="10">
@@ -34656,8 +34656,8 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
+      <c r="A5" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="B5" s="10">
         <v>2.0</v>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6"/>
+      <c r="A6" s="5"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="8"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34699,14 +34699,14 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="17"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="16"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34719,22 +34719,22 @@
     </row>
     <row r="8">
       <c r="A8" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>4.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>10.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
       <c r="E8" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34747,20 +34747,20 @@
       <c r="A9" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>20.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
       <c r="E9" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,7 +34770,7 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="23"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="10"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -34786,7 +34786,7 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="23"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="10"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -34802,7 +34802,7 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="23"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="10"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -34818,7 +34818,7 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="23"/>
+      <c r="A13" s="20"/>
       <c r="B13" s="10"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
@@ -34834,12 +34834,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="13"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="13"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="13"/>
       <c r="E14" s="11"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -34852,23 +34850,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="C15" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="D15" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="11">
-        <v>46042.0</v>
-      </c>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
@@ -34879,18 +34867,12 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
-      <c r="B16" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="C16" s="10">
-        <v>15.0</v>
-      </c>
-      <c r="D16" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E16" s="8"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34902,11 +34884,11 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>9</v>
+      <c r="A17" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B17" s="10">
-        <v>32.0</v>
+        <v>5.0</v>
       </c>
       <c r="C17" s="10">
         <v>5.0</v>
@@ -34914,9 +34896,11 @@
       <c r="D17" s="10">
         <v>1.0</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="E17" s="11">
+        <v>46042.0</v>
+      </c>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34926,11 +34910,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="23"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="8"/>
+      <c r="A18" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="C18" s="10">
+        <v>15.0</v>
+      </c>
+      <c r="D18" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34942,13 +34934,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="s">
-        <v>23</v>
+      <c r="A19" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="17"/>
+      <c r="B19" s="10">
+        <v>32.0</v>
+      </c>
+      <c r="C19" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="D19" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34960,19 +34958,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="C20" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="D20" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E20" s="17"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34984,19 +34974,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="s">
-        <v>9</v>
+      <c r="A21" s="14" t="s">
+        <v>19</v>
       </c>
-      <c r="B21" s="16">
-        <v>50.0</v>
-      </c>
-      <c r="C21" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="D21" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E21" s="17"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35008,11 +34992,19 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="23"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="8"/>
+      <c r="A22" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="15">
+        <v>5.0</v>
+      </c>
+      <c r="C22" s="15">
+        <v>5.0</v>
+      </c>
+      <c r="D22" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E22" s="16"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35024,13 +35016,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="s">
-        <v>24</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="8"/>
+      <c r="B23" s="15">
+        <v>50.0</v>
+      </c>
+      <c r="C23" s="15">
+        <v>5.0</v>
+      </c>
+      <c r="D23" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35042,19 +35040,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="C24" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="D24" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E24" s="8"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35067,12 +35057,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="8"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35084,11 +35074,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="23"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="8"/>
+      <c r="A26" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="C26" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="D26" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35100,13 +35098,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="s">
-        <v>25</v>
+      <c r="A27" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="17"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35118,19 +35116,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="C28" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="D28" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E28" s="17"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35142,17 +35132,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="30" t="s">
-        <v>9</v>
+      <c r="A29" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B29" s="31">
-        <v>55.0</v>
-      </c>
-      <c r="C29" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="D29" s="32"/>
-      <c r="E29" s="33"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="16"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35164,11 +35150,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="15">
+        <v>5.0</v>
+      </c>
+      <c r="C30" s="15">
+        <v>5.0</v>
+      </c>
+      <c r="D30" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35180,17 +35174,17 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="s">
-        <v>10</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="10" t="s">
-        <v>27</v>
+      <c r="B31" s="31">
+        <v>55.0</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="35">
-        <v>46051.96156388889</v>
+      <c r="C31" s="31">
+        <v>2.0</v>
       </c>
+      <c r="D31" s="32"/>
+      <c r="E31" s="33"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35202,19 +35196,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="10">
-        <v>2.0</v>
-      </c>
-      <c r="C32" s="10">
-        <v>100.0</v>
-      </c>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="35">
-        <v>46100.83597384259</v>
-      </c>
+      <c r="E32" s="13"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35227,17 +35213,15 @@
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
-      <c r="B33" s="10">
-        <v>20.0</v>
+      <c r="B33" s="10" t="s">
+        <v>26</v>
       </c>
-      <c r="C33" s="10">
-        <v>100.0</v>
-      </c>
+      <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="35">
-        <v>46100.83604224537</v>
+      <c r="E33" s="34">
+        <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -35250,11 +35234,19 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
+      <c r="A34" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="C34" s="10">
+        <v>100.0</v>
+      </c>
       <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
+      <c r="E34" s="34">
+        <v>46100.83597384259</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -35266,11 +35258,19 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="13"/>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
+      <c r="A35" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="10">
+        <v>20.0</v>
+      </c>
+      <c r="C35" s="10">
+        <v>100.0</v>
+      </c>
       <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
+      <c r="E35" s="34">
+        <v>46100.83604224537</v>
+      </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -35282,11 +35282,11 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35298,11 +35298,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51040,6 +51040,38 @@
       <c r="L1020" s="4"/>
       <c r="M1020" s="4"/>
       <c r="N1020" s="4"/>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="4"/>
+      <c r="B1021" s="4"/>
+      <c r="C1021" s="4"/>
+      <c r="D1021" s="4"/>
+      <c r="E1021" s="4"/>
+      <c r="F1021" s="4"/>
+      <c r="G1021" s="4"/>
+      <c r="H1021" s="4"/>
+      <c r="I1021" s="4"/>
+      <c r="J1021" s="4"/>
+      <c r="K1021" s="4"/>
+      <c r="L1021" s="4"/>
+      <c r="M1021" s="4"/>
+      <c r="N1021" s="4"/>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="4"/>
+      <c r="B1022" s="4"/>
+      <c r="C1022" s="4"/>
+      <c r="D1022" s="4"/>
+      <c r="E1022" s="4"/>
+      <c r="F1022" s="4"/>
+      <c r="G1022" s="4"/>
+      <c r="H1022" s="4"/>
+      <c r="I1022" s="4"/>
+      <c r="J1022" s="4"/>
+      <c r="K1022" s="4"/>
+      <c r="L1022" s="4"/>
+      <c r="M1022" s="4"/>
+      <c r="N1022" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -51058,16 +51090,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -51082,13 +51114,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
       <c r="D2" s="10"/>
-      <c r="E2" s="9"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51099,19 +51131,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="9">
         <v>60.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
       <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51122,11 +51154,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="6"/>
+      <c r="A4" s="5"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="9"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51137,11 +51169,11 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
+      <c r="A5" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -51156,8 +51188,8 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>14</v>
+      <c r="A6" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="B6" s="10">
         <v>6.0</v>
@@ -51181,11 +51213,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="6"/>
+      <c r="A7" s="5"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="9"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51196,13 +51228,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>16</v>
+      <c r="A8" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
-      <c r="E8" s="9"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51213,8 +51245,8 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B9" s="10">
         <v>10.0</v>
@@ -51238,8 +51270,8 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>14</v>
+      <c r="A10" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="B10" s="10">
         <v>11.0</v>
@@ -51263,11 +51295,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51278,11 +51310,11 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="s">
-        <v>16</v>
+      <c r="A12" s="25" t="s">
+        <v>17</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>18</v>
+      <c r="B12" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -51297,8 +51329,8 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>19</v>
+      <c r="A13" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B13" s="10">
         <v>5.0</v>
@@ -51322,8 +51354,8 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B14" s="10">
         <v>5.0</v>
@@ -51345,8 +51377,8 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>21</v>
+      <c r="A15" s="8" t="s">
+        <v>22</v>
       </c>
       <c r="B15" s="10">
         <v>5.0</v>
@@ -51360,8 +51392,8 @@
       <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>22</v>
+      <c r="F15" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51372,8 +51404,8 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>14</v>
+      <c r="A16" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="B16" s="10">
         <v>12.0</v>
@@ -51397,11 +51429,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="21"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51412,13 +51444,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>15</v>
+      <c r="A18" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51429,13 +51461,13 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>7</v>
+      <c r="A19" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="9">
         <v>6.0</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="9">
         <v>45.0</v>
       </c>
       <c r="D19" s="10">
@@ -51454,13 +51486,13 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="9">
         <v>18.0</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="9">
         <v>20.0</v>
       </c>
       <c r="D20" s="10">
@@ -51479,11 +51511,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
+      <c r="A21" s="8"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51494,11 +51526,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="s">
-        <v>15</v>
+      <c r="A22" s="25" t="s">
+        <v>12</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>18</v>
+      <c r="B22" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -51515,13 +51547,13 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>19</v>
+      <c r="A23" s="8" t="s">
+        <v>20</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="9">
         <v>6.0</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="9">
         <v>50.0</v>
       </c>
       <c r="D23" s="10">
@@ -51540,13 +51572,13 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
+      <c r="A24" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="9">
         <v>8.0</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="9">
         <v>30.0</v>
       </c>
       <c r="D24" s="10">
@@ -51565,13 +51597,13 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>14</v>
+      <c r="A25" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="9">
         <v>10.0</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="9">
         <v>30.0</v>
       </c>
       <c r="D25" s="10">
@@ -51580,8 +51612,8 @@
       <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>22</v>
+      <c r="F25" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51592,13 +51624,13 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>14</v>
+      <c r="A26" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="9">
         <v>17.0</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
       <c r="D26" s="10">
@@ -51617,11 +51649,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
+      <c r="A27" s="8"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51632,15 +51664,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="s">
-        <v>20</v>
+      <c r="A28" s="25" t="s">
+        <v>18</v>
       </c>
-      <c r="B28" s="24" t="s">
-        <v>18</v>
+      <c r="B28" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51651,13 +51683,13 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>19</v>
+      <c r="A29" s="8" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="9">
         <v>6.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="9">
         <v>50.0</v>
       </c>
       <c r="D29" s="10">
@@ -51676,19 +51708,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>7</v>
+      <c r="A30" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="9">
         <v>8.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="9">
         <v>30.0</v>
       </c>
       <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51699,13 +51731,13 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="9">
         <v>15.0</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="9">
         <v>10.0</v>
       </c>
       <c r="D31" s="10">
@@ -51724,11 +51756,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
+      <c r="A32" s="8"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="9"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51740,12 +51772,12 @@
     </row>
     <row r="33">
       <c r="A33" s="14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="26"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51757,18 +51789,18 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="B34" s="34" t="s">
-        <v>26</v>
+      <c r="B34" s="41" t="s">
+        <v>29</v>
       </c>
-      <c r="C34" s="34">
+      <c r="C34" s="41">
         <v>40.0</v>
       </c>
-      <c r="D34" s="34">
+      <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51784,16 +51816,16 @@
       <c r="A35" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="34">
+      <c r="B35" s="41">
         <v>30.0</v>
       </c>
-      <c r="C35" s="34">
+      <c r="C35" s="41">
         <v>15.0</v>
       </c>
-      <c r="D35" s="34">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="27"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51804,11 +51836,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="23"/>
+      <c r="A36" s="20"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="9"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51819,13 +51851,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="s">
-        <v>28</v>
+      <c r="A37" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="9"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51836,7 +51868,7 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B38" s="10">
@@ -51861,11 +51893,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="6"/>
+      <c r="A39" s="5"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="9"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51876,13 +51908,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="s">
-        <v>23</v>
+      <c r="A40" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="9"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51893,8 +51925,8 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>7</v>
+      <c r="A41" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B41" s="10">
         <v>9.0</v>
@@ -51918,7 +51950,7 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B42" s="10">
@@ -51943,8 +51975,8 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>7</v>
+      <c r="A43" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="B43" s="10">
         <v>10.0</v>
@@ -51958,8 +51990,8 @@
       <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="15" t="s">
-        <v>29</v>
+      <c r="F43" s="17" t="s">
+        <v>31</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -51970,11 +52002,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="36"/>
+      <c r="A44" s="42"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="9"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -51985,13 +52017,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="36" t="s">
+      <c r="A45" s="42" t="s">
         <v>25</v>
       </c>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="9"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52002,7 +52034,7 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B46" s="10">
@@ -52027,11 +52059,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="36"/>
+      <c r="A47" s="42"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="9"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52042,13 +52074,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="36" t="s">
-        <v>30</v>
+      <c r="A48" s="42" t="s">
+        <v>32</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="9"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52059,16 +52091,16 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>12</v>
+      <c r="A49" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B49" s="7">
+      <c r="B49" s="9">
         <v>70.0</v>
       </c>
-      <c r="C49" s="7">
+      <c r="C49" s="9">
         <v>300.0</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="9">
         <v>1.0</v>
       </c>
       <c r="E49" s="12">
@@ -52084,16 +52116,16 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>7</v>
+      <c r="A50" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B50" s="9">
         <v>10.0</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C50" s="9">
         <v>20.0</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="9">
         <v>1.0</v>
       </c>
       <c r="E50" s="12">
@@ -52109,16 +52141,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="7">
+      <c r="B51" s="9">
         <v>70.0</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51" s="9">
         <v>10.0</v>
       </c>
-      <c r="D51" s="7">
+      <c r="D51" s="9">
         <v>1.0</v>
       </c>
       <c r="E51" s="12">
@@ -52134,11 +52166,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
+      <c r="A52" s="8"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
-      <c r="E52" s="9"/>
+      <c r="E52" s="7"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52149,11 +52181,11 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
-        <v>31</v>
+      <c r="A53" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="10"/>
@@ -52170,7 +52202,7 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="5">
+      <c r="A54" s="8">
         <v>50.0</v>
       </c>
       <c r="B54" s="10">
@@ -52191,13 +52223,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="38" t="s">
-        <v>33</v>
+      <c r="A55" s="43" t="s">
+        <v>35</v>
       </c>
-      <c r="B55" s="40"/>
-      <c r="C55" s="40"/>
-      <c r="D55" s="40"/>
-      <c r="E55" s="42"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52208,16 +52240,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="44" t="s">
-        <v>35</v>
+      <c r="A56" s="39" t="s">
+        <v>36</v>
       </c>
-      <c r="B56" s="44">
+      <c r="B56" s="39">
         <v>100.0</v>
       </c>
-      <c r="C56" s="15">
+      <c r="C56" s="17">
         <v>1.0</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="17">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52233,8 +52265,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="45"/>
-      <c r="B57" s="45"/>
+      <c r="A57" s="40"/>
+      <c r="B57" s="40"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52248,10 +52280,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="44" t="s">
+      <c r="A58" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="45"/>
+      <c r="B58" s="40"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52265,16 +52297,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="44">
+      <c r="B59" s="39">
         <v>50.0</v>
       </c>
-      <c r="C59" s="15">
+      <c r="C59" s="17">
         <v>20.0</v>
       </c>
-      <c r="D59" s="15">
+      <c r="D59" s="17">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52290,13 +52322,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="44" t="s">
+      <c r="A60" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="44">
+      <c r="B60" s="39">
         <v>15.0</v>
       </c>
-      <c r="C60" s="15">
+      <c r="C60" s="17">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52313,8 +52345,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="45"/>
-      <c r="B61" s="45"/>
+      <c r="A61" s="40"/>
+      <c r="B61" s="40"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52328,11 +52360,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="44" t="s">
+      <c r="A62" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="44" t="s">
-        <v>24</v>
+      <c r="B62" s="39" t="s">
+        <v>23</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52349,16 +52381,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="44" t="s">
+      <c r="A63" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="44">
+      <c r="B63" s="39">
         <v>5.0</v>
       </c>
-      <c r="C63" s="15">
+      <c r="C63" s="17">
         <v>80.0</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="17">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52374,16 +52406,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="44" t="s">
+      <c r="A64" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="44">
+      <c r="B64" s="39">
         <v>15.0</v>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="17">
         <v>10.0</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="17">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52399,16 +52431,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="44" t="s">
-        <v>14</v>
+      <c r="A65" s="39" t="s">
+        <v>16</v>
       </c>
-      <c r="B65" s="44">
+      <c r="B65" s="39">
         <v>30.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="17">
         <v>10.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="17">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52424,8 +52456,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="45"/>
-      <c r="B66" s="45"/>
+      <c r="A66" s="40"/>
+      <c r="B66" s="40"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52439,11 +52471,11 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="44" t="s">
+      <c r="A67" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="44" t="s">
-        <v>30</v>
+      <c r="B67" s="39" t="s">
+        <v>32</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
@@ -52460,16 +52492,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="44" t="s">
+      <c r="A68" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="44">
+      <c r="B68" s="39">
         <v>5.0</v>
       </c>
-      <c r="C68" s="15">
+      <c r="C68" s="17">
         <v>80.0</v>
       </c>
-      <c r="D68" s="15">
+      <c r="D68" s="17">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52483,16 +52515,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="44" t="s">
+      <c r="A69" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="44">
+      <c r="B69" s="39">
         <v>15.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="17">
         <v>10.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="17">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52506,16 +52538,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="44" t="s">
-        <v>14</v>
+      <c r="A70" s="39" t="s">
+        <v>16</v>
       </c>
-      <c r="B70" s="44">
+      <c r="B70" s="39">
         <v>20.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="17">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="17">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52531,8 +52563,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="45"/>
-      <c r="B71" s="45"/>
+      <c r="A71" s="40"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52546,8 +52578,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="44"/>
-      <c r="B72" s="45"/>
+      <c r="A72" s="39"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52561,8 +52593,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="45"/>
-      <c r="B73" s="45"/>
+      <c r="A73" s="40"/>
+      <c r="B73" s="40"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:13.918Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,15 +14,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="42">
   <si>
     <t>項目</t>
+  </si>
+  <si>
+    <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>功率</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
+    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -31,28 +34,19 @@
     <t>次數</t>
   </si>
   <si>
-    <t>刀壓</t>
+    <t>最後更新日期</t>
   </si>
   <si>
-    <t>最後更新日期</t>
+    <t>Line</t>
   </si>
   <si>
     <t>0.3mm</t>
   </si>
   <si>
-    <t>Line</t>
-  </si>
-  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
     <t>A4紙</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
   </si>
   <si>
     <t>03mm</t>
@@ -61,13 +55,31 @@
     <t>(PS)</t>
   </si>
   <si>
+    <t>Cut</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
     <t>(PS -3)</t>
   </si>
   <si>
-    <t>Cut</t>
+    <t>PS</t>
   </si>
   <si>
-    <t>0.3 mm</t>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>1mm</t>
@@ -76,43 +88,25 @@
     <t>2mm</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>cut</t>
+    <t>６</t>
   </si>
   <si>
     <t>3mm</t>
   </si>
   <si>
-    <t>Keep Detail</t>
+    <t>1.5mm</t>
   </si>
   <si>
     <t>4mm</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>６</t>
-  </si>
-  <si>
-    <t>1.5mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>雕刻%</t>
@@ -130,7 +124,13 @@
     <t>柔光板</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>生日牌</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,32 +321,35 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -354,13 +357,25 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -369,29 +384,20 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -409,30 +415,6 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -442,7 +424,25 @@
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -682,13 +682,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>8</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="6"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>12</v>
+      <c r="A6" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>15</v>
+      <c r="B6" s="16" t="s">
+        <v>17</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="19"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
-        <v>8</v>
+      <c r="A7" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="24">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="24">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="9"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>18</v>
+      <c r="A10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>8</v>
+      <c r="A11" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>8</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
+      <c r="A14" s="25"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="6"/>
+      <c r="E14" s="8"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
-        <v>19</v>
+      <c r="A15" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
-        <v>8</v>
+      <c r="A16" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
+      <c r="A18" s="25"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="6"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>23</v>
+      <c r="A19" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="6"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>8</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="6"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
+      <c r="A22" s="25"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="6"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
-        <v>25</v>
+      <c r="A23" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="19"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
-        <v>8</v>
+      <c r="A24" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="19"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="33">
         <v>55.0</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="33">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="35"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>11</v>
+      <c r="A27" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>26</v>
+      <c r="B27" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="34">
+      <c r="E27" s="36">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>8</v>
+      <c r="A28" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="34">
+      <c r="E28" s="36">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>16</v>
+      <c r="A29" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="34">
+      <c r="E29" s="36">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17101,13 +17101,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>8</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>14</v>
+      <c r="A5" s="5" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>8</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,11 +17261,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="12"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>12</v>
+      <c r="A9" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17297,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
-        <v>8</v>
+      <c r="A10" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="20">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="20">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>20</v>
+      <c r="A12" s="22" t="s">
+        <v>19</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>14</v>
+      <c r="A13" s="22" t="s">
+        <v>12</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="27"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17397,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
-        <v>8</v>
+      <c r="A14" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17422,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="7"/>
+      <c r="A16" s="27"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>18</v>
+      <c r="A17" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="7"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>8</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="7"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
+      <c r="A20" s="25"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="7"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
-        <v>19</v>
+      <c r="A21" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="27"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17568,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
-        <v>8</v>
+      <c r="A22" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17593,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
+      <c r="A24" s="25"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="7"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>23</v>
+      <c r="A25" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="7"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>8</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="7"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
+      <c r="A28" s="25"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
-        <v>25</v>
+      <c r="A29" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="27"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17742,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
-        <v>8</v>
+      <c r="A30" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="33">
         <v>70.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="33">
         <v>5.0</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="33">
         <v>1.0</v>
       </c>
-      <c r="E31" s="35"/>
+      <c r="E31" s="40"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="36" t="s">
-        <v>27</v>
+      <c r="A33" s="44" t="s">
+        <v>36</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B33" s="45">
         <v>5.0</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="45">
         <v>10.0</v>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="45">
         <v>2.0</v>
       </c>
-      <c r="E33" s="38">
+      <c r="E33" s="46">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="39" t="s">
-        <v>28</v>
+      <c r="F33" s="41" t="s">
+        <v>38</v>
       </c>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="43"/>
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="43"/>
+      <c r="M33" s="43"/>
+      <c r="N33" s="43"/>
+      <c r="O33" s="43"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,11 +17872,11 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>11</v>
+      <c r="A36" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>26</v>
+      <c r="B36" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -17893,13 +17893,13 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>8</v>
+      <c r="A37" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
       <c r="D37" s="13"/>
@@ -17916,13 +17916,13 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>16</v>
+      <c r="A38" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
       <c r="D38" s="13"/>
@@ -34567,13 +34567,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>8</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>20.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
+      <c r="A5" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>2.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="8"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,15 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="s">
-        <v>12</v>
+      <c r="A7" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>15</v>
+      <c r="B7" s="16" t="s">
+        <v>17</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="19"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34718,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
-        <v>8</v>
+      <c r="A8" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>4.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>10.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="24">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34744,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <v>20.0</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="24">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,11 +34770,11 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="20"/>
-      <c r="B10" s="10"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="9"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="11"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34786,11 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="11"/>
+      <c r="A11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="8"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34802,11 +34801,21 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="20"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="11"/>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="C12" s="9">
+        <v>15.0</v>
+      </c>
+      <c r="D12" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="E12" s="12">
+        <v>46106.732072326384</v>
+      </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34818,11 +34827,21 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="20"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="11"/>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
+        <v>20.0</v>
+      </c>
+      <c r="C13" s="9">
+        <v>20.0</v>
+      </c>
+      <c r="D13" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="E13" s="12">
+        <v>46147.893450902775</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34834,11 +34853,21 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="11"/>
+      <c r="A14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="C14" s="9">
+        <v>20.0</v>
+      </c>
+      <c r="D14" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>46182.71399388889</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34850,11 +34879,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="20"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="9"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="11"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34866,13 +34895,13 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>18</v>
+      <c r="A16" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="11"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34884,23 +34913,23 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>8</v>
+      <c r="A17" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>5.0</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="9">
         <v>5.0</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34910,19 +34939,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>8</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>15.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34934,19 +34963,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>32.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34958,11 +34987,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
+      <c r="A20" s="25"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="6"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34974,13 +35003,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
-        <v>19</v>
+      <c r="A21" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="16"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -34992,19 +35021,19 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
-        <v>8</v>
+      <c r="A22" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>5.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>5.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="16"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35016,19 +35045,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>50.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="16"/>
+      <c r="E23" s="19"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35040,11 +35069,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
+      <c r="A24" s="25"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="6"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35056,13 +35085,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>23</v>
+      <c r="A25" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="6"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35074,19 +35103,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>8</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>5.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>5.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35098,13 +35127,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="6"/>
+      <c r="E27" s="8"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35116,11 +35145,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
+      <c r="A28" s="25"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="6"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35132,13 +35161,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
-        <v>25</v>
+      <c r="A29" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="16"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="19"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35150,19 +35179,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
-        <v>8</v>
+      <c r="A30" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>5.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="16"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35174,17 +35203,17 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="33">
         <v>55.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="33">
         <v>2.0</v>
       </c>
-      <c r="D31" s="32"/>
-      <c r="E31" s="33"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="35"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35212,15 +35241,15 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>11</v>
+      <c r="A33" s="9" t="s">
+        <v>10</v>
       </c>
-      <c r="B33" s="10" t="s">
-        <v>26</v>
+      <c r="B33" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="34">
+      <c r="E33" s="36">
         <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
@@ -35234,17 +35263,17 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>8</v>
+      <c r="A34" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="9">
         <v>2.0</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="9">
         <v>100.0</v>
       </c>
       <c r="D34" s="13"/>
-      <c r="E34" s="34">
+      <c r="E34" s="36">
         <v>46100.83597384259</v>
       </c>
       <c r="F34" s="4"/>
@@ -35258,17 +35287,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>16</v>
+      <c r="A35" s="9" t="s">
+        <v>13</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="9">
         <v>20.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
       <c r="D35" s="13"/>
-      <c r="E35" s="34">
+      <c r="E35" s="36">
         <v>46100.83604224537</v>
       </c>
       <c r="F35" s="4"/>
@@ -51090,16 +51119,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>6</v>
@@ -51114,13 +51143,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51131,19 +51160,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="7">
         <v>60.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="7">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51154,11 +51183,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="5"/>
+      <c r="A4" s="6"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="7"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51169,15 +51198,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="12"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51188,19 +51217,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>16</v>
+      <c r="A6" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>60.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51213,11 +51242,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="5"/>
+      <c r="A7" s="6"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="7"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51228,13 +51257,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>17</v>
+      <c r="A8" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51245,19 +51274,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>8</v>
+      <c r="A9" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="9">
         <v>10.0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="9">
         <v>45.0</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="9">
         <v>1.0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="11">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51270,19 +51299,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>16</v>
+      <c r="A10" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>11.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>20.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="11">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51295,11 +51324,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51310,15 +51339,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="s">
-        <v>17</v>
+      <c r="A12" s="21" t="s">
+        <v>15</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>21</v>
+      <c r="B12" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51329,19 +51358,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>20</v>
+      <c r="A13" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>5.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>60.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="11">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51354,19 +51383,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>8</v>
+      <c r="A14" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>30.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51377,23 +51406,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>22</v>
+      <c r="A15" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>4.0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="17" t="s">
-        <v>24</v>
+      <c r="F15" s="14" t="s">
+        <v>21</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51404,19 +51433,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>16</v>
+      <c r="A16" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>12.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <v>20.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="11">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51429,11 +51458,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="18"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51444,13 +51473,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>12</v>
+      <c r="A18" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="7"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51461,19 +51490,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>8</v>
+      <c r="A19" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="7">
         <v>6.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="7">
         <v>45.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="11">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51486,19 +51515,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="7">
         <v>18.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="7">
         <v>20.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51511,11 +51540,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8"/>
+      <c r="A21" s="5"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="7"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51526,15 +51555,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="s">
-        <v>12</v>
+      <c r="A22" s="21" t="s">
+        <v>16</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>21</v>
+      <c r="B22" s="23" t="s">
+        <v>18</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="12">
+      <c r="E22" s="11">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51547,19 +51576,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>20</v>
+      <c r="A23" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="7">
         <v>6.0</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="7">
         <v>50.0</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="9">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="11">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51572,19 +51601,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>8</v>
+      <c r="A24" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="7">
         <v>8.0</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="7">
         <v>30.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="11">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51597,23 +51626,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>16</v>
+      <c r="A25" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="7">
         <v>10.0</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="7">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <v>4.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="17" t="s">
-        <v>24</v>
+      <c r="F25" s="14" t="s">
+        <v>21</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51624,19 +51653,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>16</v>
+      <c r="A26" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="7">
         <v>17.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="7">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="11">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51649,11 +51678,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8"/>
+      <c r="A27" s="5"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="7"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51664,15 +51693,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="23" t="s">
         <v>18</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>21</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51683,19 +51712,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>20</v>
+      <c r="A29" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="7">
         <v>6.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="7">
         <v>50.0</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="9">
         <v>1.0</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="11">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51708,19 +51737,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>8</v>
+      <c r="A30" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="7">
         <v>8.0</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="7">
         <v>30.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="7"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51731,19 +51760,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="7">
         <v>15.0</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="7">
         <v>10.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="9">
         <v>2.0</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="11">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51756,11 +51785,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8"/>
+      <c r="A32" s="5"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="7"/>
+      <c r="E32" s="10"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51771,13 +51800,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="s">
-        <v>18</v>
+      <c r="A33" s="15" t="s">
+        <v>22</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="27"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51788,19 +51817,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="s">
-        <v>8</v>
+      <c r="A34" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>29</v>
+      <c r="B34" s="30" t="s">
+        <v>24</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="30">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="30">
         <v>1.0</v>
       </c>
-      <c r="E34" s="21">
+      <c r="E34" s="20">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51813,19 +51842,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="30">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="30">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="30">
         <v>1.0</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51836,11 +51865,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="20"/>
+      <c r="A36" s="25"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="7"/>
+      <c r="E36" s="10"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51851,13 +51880,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>30</v>
+      <c r="A37" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="7"/>
+      <c r="E37" s="10"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51868,19 +51897,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>40.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>15.0</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="9">
         <v>1.0</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="11">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51893,11 +51922,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
+      <c r="A39" s="6"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="7"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51908,13 +51937,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>19</v>
+      <c r="A40" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="7"/>
+      <c r="E40" s="10"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51925,19 +51954,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="s">
-        <v>8</v>
+      <c r="A41" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="9">
         <v>9.0</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="9">
         <v>20.0</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="9">
         <v>1.0</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="11">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51950,19 +51979,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="9">
         <v>55.0</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="9">
         <v>20.0</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="9">
         <v>1.0</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="11">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -51975,23 +52004,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
-        <v>8</v>
+      <c r="A43" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="9">
         <v>10.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="9">
         <v>250.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="17" t="s">
-        <v>31</v>
+      <c r="F43" s="14" t="s">
+        <v>28</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52002,11 +52031,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
+      <c r="A44" s="31"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="7"/>
+      <c r="E44" s="10"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52017,13 +52046,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>25</v>
+      <c r="A45" s="31" t="s">
+        <v>27</v>
       </c>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="7"/>
+      <c r="E45" s="10"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52034,19 +52063,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="s">
+      <c r="A46" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="9">
         <v>60.0</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="9">
         <v>10.0</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="9">
         <v>1.0</v>
       </c>
-      <c r="E46" s="12">
+      <c r="E46" s="11">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52059,11 +52088,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
+      <c r="A47" s="31"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="7"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52074,13 +52103,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
-        <v>32</v>
+      <c r="A48" s="31" t="s">
+        <v>29</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="7"/>
+      <c r="E48" s="10"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52091,19 +52120,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="s">
-        <v>10</v>
+      <c r="A49" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="7">
         <v>70.0</v>
       </c>
-      <c r="C49" s="9">
+      <c r="C49" s="7">
         <v>300.0</v>
       </c>
-      <c r="D49" s="9">
+      <c r="D49" s="7">
         <v>1.0</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="11">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52116,19 +52145,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="s">
-        <v>8</v>
+      <c r="A50" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="7">
         <v>10.0</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="7">
         <v>20.0</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="7">
         <v>1.0</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="11">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52141,19 +52170,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="7">
         <v>70.0</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="7">
         <v>10.0</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="7">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="11">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52166,11 +52195,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="8"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="7"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="10"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52181,15 +52210,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="s">
-        <v>33</v>
+      <c r="A53" s="5" t="s">
+        <v>31</v>
       </c>
-      <c r="B53" s="10" t="s">
-        <v>34</v>
+      <c r="B53" s="9" t="s">
+        <v>32</v>
       </c>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="12">
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="11">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52202,15 +52231,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="8">
+      <c r="A54" s="5">
         <v>50.0</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="9">
         <v>100.0</v>
       </c>
       <c r="C54" s="13"/>
       <c r="D54" s="13"/>
-      <c r="E54" s="12">
+      <c r="E54" s="11">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52223,13 +52252,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="43" t="s">
-        <v>35</v>
+      <c r="A55" s="37" t="s">
+        <v>33</v>
       </c>
-      <c r="B55" s="44"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="38"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="39"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52240,19 +52269,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="39" t="s">
-        <v>36</v>
+      <c r="A56" s="41" t="s">
+        <v>34</v>
       </c>
-      <c r="B56" s="39">
+      <c r="B56" s="41">
         <v>100.0</v>
       </c>
-      <c r="C56" s="17">
+      <c r="C56" s="14">
         <v>1.0</v>
       </c>
-      <c r="D56" s="17">
+      <c r="D56" s="14">
         <v>2.0</v>
       </c>
-      <c r="E56" s="46">
+      <c r="E56" s="42">
         <v>46009.783484375</v>
       </c>
       <c r="F56" s="4"/>
@@ -52265,8 +52294,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="40"/>
-      <c r="B57" s="40"/>
+      <c r="A57" s="43"/>
+      <c r="B57" s="43"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52280,10 +52309,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="39" t="s">
-        <v>37</v>
+      <c r="A58" s="41" t="s">
+        <v>35</v>
       </c>
-      <c r="B58" s="40"/>
+      <c r="B58" s="43"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52297,19 +52326,19 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="39">
+      <c r="B59" s="41">
         <v>50.0</v>
       </c>
-      <c r="C59" s="17">
+      <c r="C59" s="14">
         <v>20.0</v>
       </c>
-      <c r="D59" s="17">
+      <c r="D59" s="14">
         <v>1.0</v>
       </c>
-      <c r="E59" s="46">
+      <c r="E59" s="42">
         <v>46038.9559609375</v>
       </c>
       <c r="F59" s="4"/>
@@ -52322,17 +52351,17 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="39" t="s">
-        <v>38</v>
+      <c r="A60" s="41" t="s">
+        <v>37</v>
       </c>
-      <c r="B60" s="39">
+      <c r="B60" s="41">
         <v>15.0</v>
       </c>
-      <c r="C60" s="17">
+      <c r="C60" s="14">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="46">
+      <c r="E60" s="42">
         <v>46136.01284993056</v>
       </c>
       <c r="F60" s="4"/>
@@ -52345,8 +52374,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="40"/>
-      <c r="B61" s="40"/>
+      <c r="A61" s="43"/>
+      <c r="B61" s="43"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52360,15 +52389,15 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="s">
+      <c r="A62" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="39" t="s">
-        <v>23</v>
+      <c r="B62" s="41" t="s">
+        <v>25</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="46">
+      <c r="E62" s="42">
         <v>46044.0116671875</v>
       </c>
       <c r="F62" s="4"/>
@@ -52381,19 +52410,19 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="s">
+      <c r="A63" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="39">
+      <c r="B63" s="41">
         <v>5.0</v>
       </c>
-      <c r="C63" s="17">
+      <c r="C63" s="14">
         <v>80.0</v>
       </c>
-      <c r="D63" s="17">
+      <c r="D63" s="14">
         <v>1.0</v>
       </c>
-      <c r="E63" s="46">
+      <c r="E63" s="42">
         <v>46044.01310700232</v>
       </c>
       <c r="F63" s="4"/>
@@ -52406,19 +52435,19 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="39" t="s">
+      <c r="A64" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="39">
+      <c r="B64" s="41">
         <v>15.0</v>
       </c>
-      <c r="C64" s="17">
+      <c r="C64" s="14">
         <v>10.0</v>
       </c>
-      <c r="D64" s="17">
+      <c r="D64" s="14">
         <v>1.0</v>
       </c>
-      <c r="E64" s="46">
+      <c r="E64" s="42">
         <v>46044.013194907406</v>
       </c>
       <c r="F64" s="4"/>
@@ -52431,19 +52460,19 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="39" t="s">
-        <v>16</v>
+      <c r="A65" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B65" s="39">
+      <c r="B65" s="41">
         <v>30.0</v>
       </c>
-      <c r="C65" s="17">
+      <c r="C65" s="14">
         <v>10.0</v>
       </c>
-      <c r="D65" s="17">
+      <c r="D65" s="14">
         <v>1.0</v>
       </c>
-      <c r="E65" s="46">
+      <c r="E65" s="42">
         <v>46056.701985011576</v>
       </c>
       <c r="F65" s="4"/>
@@ -52456,8 +52485,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="40"/>
-      <c r="B66" s="40"/>
+      <c r="A66" s="43"/>
+      <c r="B66" s="43"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52471,15 +52500,15 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="39" t="s">
+      <c r="A67" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="39" t="s">
-        <v>32</v>
+      <c r="B67" s="41" t="s">
+        <v>29</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="46">
+      <c r="E67" s="42">
         <v>46044.0136399537</v>
       </c>
       <c r="F67" s="4"/>
@@ -52492,16 +52521,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="s">
+      <c r="A68" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="39">
+      <c r="B68" s="41">
         <v>5.0</v>
       </c>
-      <c r="C68" s="17">
+      <c r="C68" s="14">
         <v>80.0</v>
       </c>
-      <c r="D68" s="17">
+      <c r="D68" s="14">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52515,16 +52544,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="s">
+      <c r="A69" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="39">
+      <c r="B69" s="41">
         <v>15.0</v>
       </c>
-      <c r="C69" s="17">
+      <c r="C69" s="14">
         <v>10.0</v>
       </c>
-      <c r="D69" s="17">
+      <c r="D69" s="14">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52538,19 +52567,19 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="s">
-        <v>16</v>
+      <c r="A70" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B70" s="39">
+      <c r="B70" s="41">
         <v>20.0</v>
       </c>
-      <c r="C70" s="17">
+      <c r="C70" s="14">
         <v>10.0</v>
       </c>
-      <c r="D70" s="17">
+      <c r="D70" s="14">
         <v>6.0</v>
       </c>
-      <c r="E70" s="46">
+      <c r="E70" s="42">
         <v>46044.014003055556</v>
       </c>
       <c r="F70" s="4"/>
@@ -52563,8 +52592,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="40"/>
-      <c r="B71" s="40"/>
+      <c r="A71" s="43"/>
+      <c r="B71" s="43"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52578,8 +52607,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="39"/>
-      <c r="B72" s="40"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="43"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52593,8 +52622,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="40"/>
-      <c r="B73" s="40"/>
+      <c r="A73" s="43"/>
+      <c r="B73" s="43"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:17.816Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -37,43 +37,46 @@
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>Line</t>
+    <t>0.3mm</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>Line</t>
   </si>
   <si>
     <t>Cut-1/2</t>
   </si>
   <si>
+    <t>(PS)</t>
+  </si>
+  <si>
     <t>A4紙</t>
+  </si>
+  <si>
+    <t>FILL</t>
   </si>
   <si>
     <t>03mm</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>0.5mm</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
+    <t>Fill</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
-    <t>Fill</t>
+    <t>1mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -82,31 +85,34 @@
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>1mm</t>
+    <t>2mm</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>4mm</t>
+  </si>
+  <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
   </si>
   <si>
-    <t>3mm</t>
-  </si>
-  <si>
     <t>1.5mm</t>
-  </si>
-  <si>
-    <t>4mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>雕刻%</t>
@@ -124,13 +130,7 @@
     <t>柔光板</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
     <t>紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>生日牌</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,23 +321,23 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -357,54 +357,66 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -413,6 +425,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -424,25 +442,7 @@
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,16 +719,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -745,16 +745,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="12"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -786,14 +786,14 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
-      <c r="E6" s="19"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,8 +805,8 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="s">
-        <v>7</v>
+      <c r="A7" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B7" s="16">
         <v>4.0</v>
@@ -817,7 +817,7 @@
       <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="20">
         <v>45957.92965825232</v>
       </c>
       <c r="F7" s="14"/>
@@ -831,7 +831,7 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="16">
@@ -843,7 +843,7 @@
       <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="20">
         <v>45954.915123425926</v>
       </c>
       <c r="F8" s="14"/>
@@ -857,8 +857,8 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="25"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="12"/>
@@ -873,12 +873,12 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>22</v>
+      <c r="A10" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="9"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -891,16 +891,16 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
+      <c r="A11" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
       <c r="E11" s="12">
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
+      <c r="A14" s="24"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="8"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,10 +984,10 @@
       <c r="A15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="19"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,8 +999,8 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="s">
-        <v>7</v>
+      <c r="A16" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B16" s="16">
         <v>5.0</v>
@@ -1011,7 +1011,7 @@
       <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="19"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,7 +1023,7 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="16">
@@ -1035,7 +1035,7 @@
       <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="19"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="25"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="8"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>25</v>
+      <c r="A19" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>7</v>
+      <c r="A20" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="8"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1140,12 +1140,12 @@
     </row>
     <row r="23">
       <c r="A23" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="19"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,8 +1157,8 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="s">
-        <v>7</v>
+      <c r="A24" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B24" s="16">
         <v>5.0</v>
@@ -1169,7 +1169,7 @@
       <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="19"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="33">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="33">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="34"/>
-      <c r="E25" s="35"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="39"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>10</v>
+      <c r="A27" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>30</v>
+      <c r="B27" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="36">
+      <c r="E27" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
-        <v>7</v>
+      <c r="A28" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="36">
+      <c r="E28" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>13</v>
+      <c r="A29" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
-      <c r="E29" s="36">
+      <c r="E29" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,16 +17140,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
+      <c r="A5" s="6" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,19 +17211,19 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
+      <c r="E6" s="9"/>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
@@ -17236,16 +17236,16 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
       <c r="E7" s="11"/>
@@ -17261,10 +17261,10 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17279,12 +17279,12 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="20"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,8 +17297,8 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="s">
-        <v>7</v>
+      <c r="A10" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B10" s="16">
         <v>4.0</v>
@@ -17309,7 +17309,7 @@
       <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="18">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,7 +17324,7 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="16">
@@ -17336,7 +17336,7 @@
       <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="18">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,8 +17351,8 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="s">
-        <v>19</v>
+      <c r="A12" s="19" t="s">
+        <v>18</v>
       </c>
       <c r="B12" s="16">
         <v>4.0</v>
@@ -17363,7 +17363,7 @@
       <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="18">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="s">
-        <v>12</v>
+      <c r="A13" s="19" t="s">
+        <v>10</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="26"/>
+      <c r="E13" s="21"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,8 +17397,8 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="s">
-        <v>7</v>
+      <c r="A14" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B14" s="16">
         <v>2.0</v>
@@ -17409,7 +17409,7 @@
       <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="21"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,7 +17422,7 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="16">
@@ -17434,7 +17434,7 @@
       <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="21"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="16">
       <c r="A16" s="27"/>
-      <c r="E16" s="10"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>22</v>
+      <c r="A17" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>12</v>
+      <c r="B17" s="28" t="s">
+        <v>10</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,10 +17552,10 @@
       <c r="A21" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="21"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,8 +17568,8 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="s">
-        <v>7</v>
+      <c r="A22" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B22" s="16">
         <v>8.0</v>
@@ -17580,7 +17580,7 @@
       <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,7 +17593,7 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="16">
@@ -17605,7 +17605,7 @@
       <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="21"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
+      <c r="A24" s="24"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="10"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>25</v>
+      <c r="A25" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,16 +17679,16 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
       <c r="E27" s="11">
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17724,12 +17724,12 @@
     </row>
     <row r="29">
       <c r="A29" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="21"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,8 +17742,8 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="s">
-        <v>7</v>
+      <c r="A30" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B30" s="16">
         <v>18.0</v>
@@ -17754,7 +17754,7 @@
       <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="21"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="40"/>
+      <c r="E31" s="32"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="44" t="s">
-        <v>36</v>
+      <c r="A33" s="33" t="s">
+        <v>26</v>
       </c>
-      <c r="B33" s="45">
+      <c r="B33" s="34">
         <v>5.0</v>
       </c>
-      <c r="C33" s="45">
+      <c r="C33" s="34">
         <v>10.0</v>
       </c>
-      <c r="D33" s="45">
+      <c r="D33" s="34">
         <v>2.0</v>
       </c>
-      <c r="E33" s="46">
+      <c r="E33" s="35">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="41" t="s">
-        <v>38</v>
+      <c r="F33" s="36" t="s">
+        <v>27</v>
       </c>
-      <c r="G33" s="43"/>
-      <c r="H33" s="43"/>
-      <c r="I33" s="43"/>
-      <c r="J33" s="43"/>
-      <c r="K33" s="43"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="43"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="37"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="37"/>
+      <c r="M33" s="37"/>
+      <c r="N33" s="37"/>
+      <c r="O33" s="37"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,11 +17872,11 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>10</v>
+      <c r="A36" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>30</v>
+      <c r="B36" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -17893,13 +17893,13 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
-        <v>7</v>
+      <c r="A37" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
       <c r="D37" s="13"/>
@@ -17916,13 +17916,13 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
-        <v>13</v>
+      <c r="A38" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
       <c r="D38" s="13"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,16 +34604,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -34630,16 +34630,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>20.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="12">
@@ -34656,16 +34656,16 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>2.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
       <c r="E5" s="12">
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="8"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="7"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34699,14 +34699,14 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
-      <c r="E7" s="19"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,8 +34718,8 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="s">
-        <v>7</v>
+      <c r="A8" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B8" s="16">
         <v>4.0</v>
@@ -34730,7 +34730,7 @@
       <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="20">
         <v>45957.92965825232</v>
       </c>
       <c r="F8" s="14"/>
@@ -34744,7 +34744,7 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="16">
@@ -34756,7 +34756,7 @@
       <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="20">
         <v>46116.685309016204</v>
       </c>
       <c r="F9" s="14"/>
@@ -34770,8 +34770,8 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="25"/>
-      <c r="B10" s="9"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="12"/>
@@ -34786,10 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>8</v>
+      <c r="A11" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="7"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34801,16 +34801,16 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>2.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
       <c r="E12" s="12">
@@ -34827,16 +34827,16 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>20.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>20.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="12">
@@ -34853,16 +34853,16 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>14</v>
+      <c r="A14" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>2.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>20.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="12">
@@ -34879,8 +34879,8 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="25"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="10"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="12"/>
@@ -34895,12 +34895,12 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>22</v>
+      <c r="A16" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="9"/>
+      <c r="D16" s="10"/>
       <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34913,16 +34913,16 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>7</v>
+      <c r="A17" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="10">
         <v>5.0</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <v>5.0</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="10">
         <v>1.0</v>
       </c>
       <c r="E17" s="12">
@@ -34939,19 +34939,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>15.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34963,19 +34963,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>32.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34987,11 +34987,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="8"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35006,10 +35006,10 @@
       <c r="A21" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="19"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35021,8 +35021,8 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="s">
-        <v>7</v>
+      <c r="A22" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B22" s="16">
         <v>5.0</v>
@@ -35033,7 +35033,7 @@
       <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="19"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35045,7 +35045,7 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="16">
@@ -35057,7 +35057,7 @@
       <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="19"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35069,11 +35069,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
+      <c r="A24" s="24"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="8"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35085,13 +35085,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>25</v>
+      <c r="A25" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="8"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35103,19 +35103,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>5.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>5.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35127,13 +35127,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="8"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35145,11 +35145,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35162,12 +35162,12 @@
     </row>
     <row r="29">
       <c r="A29" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="19"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="17"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35179,8 +35179,8 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="s">
-        <v>7</v>
+      <c r="A30" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="B30" s="16">
         <v>5.0</v>
@@ -35191,7 +35191,7 @@
       <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="19"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35203,17 +35203,17 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="31">
         <v>55.0</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="31">
         <v>2.0</v>
       </c>
-      <c r="D31" s="34"/>
-      <c r="E31" s="35"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="39"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35241,15 +35241,15 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="s">
-        <v>10</v>
+      <c r="A33" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>30</v>
+      <c r="B33" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="36">
+      <c r="E33" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
@@ -35263,17 +35263,17 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>7</v>
+      <c r="A34" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="10">
         <v>2.0</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="10">
         <v>100.0</v>
       </c>
       <c r="D34" s="13"/>
-      <c r="E34" s="36">
+      <c r="E34" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F34" s="4"/>
@@ -35287,17 +35287,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
-        <v>13</v>
+      <c r="A35" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="10">
         <v>20.0</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
       <c r="D35" s="13"/>
-      <c r="E35" s="36">
+      <c r="E35" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F35" s="4"/>
@@ -51143,13 +51143,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="10"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51160,19 +51160,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>60.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="9"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51183,11 +51183,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="6"/>
+      <c r="A4" s="5"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="10"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51198,11 +51198,11 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
+      <c r="A5" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -51217,16 +51217,16 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>13</v>
+      <c r="A6" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
       <c r="E6" s="11">
@@ -51242,11 +51242,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="6"/>
+      <c r="A7" s="5"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="10"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51257,13 +51257,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>15</v>
+      <c r="A8" s="5" t="s">
+        <v>17</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="9"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51274,16 +51274,16 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
       <c r="E9" s="11">
@@ -51299,16 +51299,16 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>13</v>
+      <c r="A10" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
       <c r="E10" s="11">
@@ -51324,11 +51324,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51339,14 +51339,14 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="s">
-        <v>15</v>
+      <c r="A12" s="25" t="s">
+        <v>17</v>
       </c>
-      <c r="B12" s="23" t="s">
-        <v>18</v>
+      <c r="B12" s="26" t="s">
+        <v>19</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -51358,16 +51358,16 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>19</v>
+      <c r="A13" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="11">
@@ -51383,16 +51383,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="11"/>
@@ -51406,23 +51406,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>20</v>
+      <c r="A15" s="6" t="s">
+        <v>21</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
       <c r="E15" s="11">
         <v>46160.85381630787</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51433,16 +51433,16 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>13</v>
+      <c r="A16" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
       <c r="E16" s="11">
@@ -51458,11 +51458,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="18"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51473,13 +51473,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>16</v>
+      <c r="A18" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51490,16 +51490,16 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>7</v>
+      <c r="A19" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="8">
         <v>6.0</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="8">
         <v>45.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
       <c r="E19" s="11">
@@ -51515,16 +51515,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="8">
         <v>18.0</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="8">
         <v>20.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="11">
@@ -51540,11 +51540,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
+      <c r="A21" s="6"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="10"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51555,11 +51555,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="s">
-        <v>16</v>
+      <c r="A22" s="25" t="s">
+        <v>14</v>
       </c>
-      <c r="B22" s="23" t="s">
-        <v>18</v>
+      <c r="B22" s="26" t="s">
+        <v>19</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -51576,16 +51576,16 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>19</v>
+      <c r="A23" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="8">
         <v>6.0</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>50.0</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
       <c r="E23" s="11">
@@ -51601,16 +51601,16 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
+      <c r="A24" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="8">
         <v>8.0</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>30.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
       <c r="E24" s="11">
@@ -51626,23 +51626,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>13</v>
+      <c r="A25" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="8">
         <v>10.0</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="8">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
       <c r="E25" s="11">
         <v>46156.84678416667</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51653,16 +51653,16 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>13</v>
+      <c r="A26" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="8">
         <v>17.0</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
       <c r="E26" s="11">
@@ -51678,11 +51678,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
+      <c r="A27" s="6"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="10"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51693,15 +51693,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="s">
-        <v>22</v>
+      <c r="A28" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="B28" s="23" t="s">
-        <v>18</v>
+      <c r="B28" s="26" t="s">
+        <v>19</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51712,16 +51712,16 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>19</v>
+      <c r="A29" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="8">
         <v>6.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="8">
         <v>50.0</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
       <c r="E29" s="11">
@@ -51737,19 +51737,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>7</v>
+      <c r="A30" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="8">
         <v>8.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="8">
         <v>30.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="10"/>
+      <c r="E30" s="9"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51760,16 +51760,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="8">
         <v>15.0</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="8">
         <v>10.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
       <c r="E31" s="11">
@@ -51785,11 +51785,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
+      <c r="A32" s="6"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="10"/>
+      <c r="E32" s="9"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51801,12 +51801,12 @@
     </row>
     <row r="33">
       <c r="A33" s="15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
-      <c r="E33" s="26"/>
+      <c r="E33" s="21"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51817,19 +51817,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="s">
-        <v>7</v>
+      <c r="A34" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B34" s="30" t="s">
-        <v>24</v>
+      <c r="B34" s="41" t="s">
+        <v>29</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C34" s="41">
         <v>40.0</v>
       </c>
-      <c r="D34" s="30">
+      <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="18">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51842,19 +51842,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="30">
+      <c r="B35" s="41">
         <v>30.0</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="41">
         <v>15.0</v>
       </c>
-      <c r="D35" s="30">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="21"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51865,11 +51865,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="25"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="10"/>
+      <c r="E36" s="9"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51880,13 +51880,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="s">
-        <v>26</v>
+      <c r="A37" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="10"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51897,16 +51897,16 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
       <c r="E38" s="11">
@@ -51922,11 +51922,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="6"/>
+      <c r="A39" s="5"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="10"/>
+      <c r="E39" s="9"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51937,13 +51937,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="10"/>
+      <c r="E40" s="9"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51954,16 +51954,16 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>7</v>
+      <c r="A41" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
       <c r="E41" s="11">
@@ -51979,16 +51979,16 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
       <c r="E42" s="11">
@@ -52004,23 +52004,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>7</v>
+      <c r="A43" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
       <c r="E43" s="11">
         <v>46038.439073761576</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52031,11 +52031,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="31"/>
+      <c r="A44" s="42"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="10"/>
+      <c r="E44" s="9"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52046,13 +52046,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="31" t="s">
-        <v>27</v>
+      <c r="A45" s="42" t="s">
+        <v>25</v>
       </c>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="10"/>
+      <c r="E45" s="9"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52063,16 +52063,16 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
       <c r="E46" s="11">
@@ -52088,11 +52088,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="31"/>
+      <c r="A47" s="42"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="10"/>
+      <c r="E47" s="9"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52103,13 +52103,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="31" t="s">
-        <v>29</v>
+      <c r="A48" s="42" t="s">
+        <v>32</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="10"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52120,16 +52120,16 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>14</v>
+      <c r="A49" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B49" s="7">
+      <c r="B49" s="8">
         <v>70.0</v>
       </c>
-      <c r="C49" s="7">
+      <c r="C49" s="8">
         <v>300.0</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="8">
         <v>1.0</v>
       </c>
       <c r="E49" s="11">
@@ -52145,16 +52145,16 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>7</v>
+      <c r="A50" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B50" s="8">
         <v>10.0</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C50" s="8">
         <v>20.0</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="8">
         <v>1.0</v>
       </c>
       <c r="E50" s="11">
@@ -52170,16 +52170,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="7">
+      <c r="B51" s="8">
         <v>70.0</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51" s="8">
         <v>10.0</v>
       </c>
-      <c r="D51" s="7">
+      <c r="D51" s="8">
         <v>1.0</v>
       </c>
       <c r="E51" s="11">
@@ -52195,11 +52195,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="10"/>
+      <c r="A52" s="6"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="9"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52210,14 +52210,14 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
-        <v>31</v>
+      <c r="A53" s="6" t="s">
+        <v>33</v>
       </c>
-      <c r="B53" s="9" t="s">
-        <v>32</v>
+      <c r="B53" s="10" t="s">
+        <v>34</v>
       </c>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
       <c r="E53" s="11">
         <v>45946.87875708334</v>
       </c>
@@ -52231,10 +52231,10 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="5">
+      <c r="A54" s="6">
         <v>50.0</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
       <c r="C54" s="13"/>
@@ -52252,13 +52252,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="37" t="s">
-        <v>33</v>
+      <c r="A55" s="43" t="s">
+        <v>35</v>
       </c>
-      <c r="B55" s="38"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52269,10 +52269,10 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="s">
-        <v>34</v>
+      <c r="A56" s="36" t="s">
+        <v>36</v>
       </c>
-      <c r="B56" s="41">
+      <c r="B56" s="36">
         <v>100.0</v>
       </c>
       <c r="C56" s="14">
@@ -52281,7 +52281,7 @@
       <c r="D56" s="14">
         <v>2.0</v>
       </c>
-      <c r="E56" s="42">
+      <c r="E56" s="46">
         <v>46009.783484375</v>
       </c>
       <c r="F56" s="4"/>
@@ -52294,8 +52294,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="43"/>
-      <c r="B57" s="43"/>
+      <c r="A57" s="37"/>
+      <c r="B57" s="37"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52309,10 +52309,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="41" t="s">
-        <v>35</v>
+      <c r="A58" s="36" t="s">
+        <v>37</v>
       </c>
-      <c r="B58" s="43"/>
+      <c r="B58" s="37"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52326,10 +52326,10 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="41">
+      <c r="B59" s="36">
         <v>50.0</v>
       </c>
       <c r="C59" s="14">
@@ -52338,7 +52338,7 @@
       <c r="D59" s="14">
         <v>1.0</v>
       </c>
-      <c r="E59" s="42">
+      <c r="E59" s="46">
         <v>46038.9559609375</v>
       </c>
       <c r="F59" s="4"/>
@@ -52351,17 +52351,17 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="41" t="s">
-        <v>37</v>
+      <c r="A60" s="36" t="s">
+        <v>38</v>
       </c>
-      <c r="B60" s="41">
+      <c r="B60" s="36">
         <v>15.0</v>
       </c>
       <c r="C60" s="14">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="42">
+      <c r="E60" s="46">
         <v>46136.01284993056</v>
       </c>
       <c r="F60" s="4"/>
@@ -52374,8 +52374,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="43"/>
-      <c r="B61" s="43"/>
+      <c r="A61" s="37"/>
+      <c r="B61" s="37"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52389,15 +52389,15 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="41" t="s">
-        <v>25</v>
+      <c r="B62" s="36" t="s">
+        <v>24</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="42">
+      <c r="E62" s="46">
         <v>46044.0116671875</v>
       </c>
       <c r="F62" s="4"/>
@@ -52410,10 +52410,10 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="41">
+      <c r="B63" s="36">
         <v>5.0</v>
       </c>
       <c r="C63" s="14">
@@ -52422,7 +52422,7 @@
       <c r="D63" s="14">
         <v>1.0</v>
       </c>
-      <c r="E63" s="42">
+      <c r="E63" s="46">
         <v>46044.01310700232</v>
       </c>
       <c r="F63" s="4"/>
@@ -52435,10 +52435,10 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="41">
+      <c r="B64" s="36">
         <v>15.0</v>
       </c>
       <c r="C64" s="14">
@@ -52447,7 +52447,7 @@
       <c r="D64" s="14">
         <v>1.0</v>
       </c>
-      <c r="E64" s="42">
+      <c r="E64" s="46">
         <v>46044.013194907406</v>
       </c>
       <c r="F64" s="4"/>
@@ -52460,10 +52460,10 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="41" t="s">
-        <v>13</v>
+      <c r="A65" s="36" t="s">
+        <v>15</v>
       </c>
-      <c r="B65" s="41">
+      <c r="B65" s="36">
         <v>30.0</v>
       </c>
       <c r="C65" s="14">
@@ -52472,7 +52472,7 @@
       <c r="D65" s="14">
         <v>1.0</v>
       </c>
-      <c r="E65" s="42">
+      <c r="E65" s="46">
         <v>46056.701985011576</v>
       </c>
       <c r="F65" s="4"/>
@@ -52485,8 +52485,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="43"/>
-      <c r="B66" s="43"/>
+      <c r="A66" s="37"/>
+      <c r="B66" s="37"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52500,15 +52500,15 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="41" t="s">
-        <v>29</v>
+      <c r="B67" s="36" t="s">
+        <v>32</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="42">
+      <c r="E67" s="46">
         <v>46044.0136399537</v>
       </c>
       <c r="F67" s="4"/>
@@ -52521,10 +52521,10 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="36">
         <v>5.0</v>
       </c>
       <c r="C68" s="14">
@@ -52544,10 +52544,10 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="36">
         <v>15.0</v>
       </c>
       <c r="C69" s="14">
@@ -52567,10 +52567,10 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="41" t="s">
-        <v>13</v>
+      <c r="A70" s="36" t="s">
+        <v>15</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="36">
         <v>20.0</v>
       </c>
       <c r="C70" s="14">
@@ -52579,7 +52579,7 @@
       <c r="D70" s="14">
         <v>6.0</v>
       </c>
-      <c r="E70" s="42">
+      <c r="E70" s="46">
         <v>46044.014003055556</v>
       </c>
       <c r="F70" s="4"/>
@@ -52592,8 +52592,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="43"/>
-      <c r="B71" s="43"/>
+      <c r="A71" s="37"/>
+      <c r="B71" s="37"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52607,8 +52607,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="43"/>
+      <c r="A72" s="36"/>
+      <c r="B72" s="37"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52622,8 +52622,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="43"/>
-      <c r="B73" s="43"/>
+      <c r="A73" s="37"/>
+      <c r="B73" s="37"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:20.685Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,13 +19,7 @@
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -46,43 +40,13 @@
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>A4紙</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>03mm</t>
-  </si>
-  <si>
     <t>0.5mm</t>
-  </si>
-  <si>
-    <t>Cut</t>
   </si>
   <si>
     <t>(PS -3)</t>
   </si>
   <si>
-    <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
     <t>1mm</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>Keep Detail</t>
   </si>
   <si>
     <t>2mm</t>
@@ -94,19 +58,55 @@
     <t>4mm</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
+    <t>A4紙</t>
   </si>
   <si>
     <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>Cut</t>
+  </si>
+  <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
+    <t>刀壓</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>03mm</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
+  </si>
+  <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -324,31 +324,16 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -360,36 +345,20 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -398,6 +367,49 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -417,18 +429,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -705,9 +705,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>8</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -770,10 +770,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>14</v>
+      <c r="A6" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>16</v>
+      <c r="B6" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="s">
-        <v>8</v>
+      <c r="A7" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="11">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="11">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="11">
         <v>1.0</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="14">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="s">
-        <v>9</v>
+      <c r="A8" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="11">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="11">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="11">
         <v>1.0</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="14">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="24"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="12"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="9"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -874,12 +874,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="12"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>8</v>
+      <c r="A11" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>8</v>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
-      <c r="E12" s="7"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="7"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="24"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="7"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>23</v>
+      <c r="A15" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="s">
-        <v>8</v>
+      <c r="A16" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="11">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="11">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="11">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="s">
-        <v>9</v>
+      <c r="A17" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="11">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="11">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="11">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="12"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="24"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="7"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1064,12 +1064,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>8</v>
+      <c r="A20" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="7"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
-        <v>9</v>
+      <c r="A21" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="7"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="24"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="7"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
-        <v>25</v>
+      <c r="A23" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="12"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="s">
-        <v>8</v>
+      <c r="A24" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="11">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="11">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="11">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="12"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="s">
-        <v>9</v>
+      <c r="A25" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="20">
         <v>55.0</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="20">
         <v>2.0</v>
       </c>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>11</v>
+      <c r="A27" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>28</v>
+      <c r="B27" s="8" t="s">
+        <v>15</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="40">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="23">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>8</v>
+      <c r="A28" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="40">
+      <c r="D28" s="17"/>
+      <c r="E28" s="23">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>15</v>
+      <c r="A29" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="40">
+      <c r="D29" s="17"/>
+      <c r="E29" s="23">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="17"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="17"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17125,9 +17125,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="25"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>8</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="26">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="25"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
+      <c r="A5" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="25"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>8</v>
+      <c r="A6" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>9</v>
+      <c r="A7" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17262,10 +17262,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="26"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
-        <v>14</v>
+      <c r="A9" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="29"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17297,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="s">
-        <v>8</v>
+      <c r="A10" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="11">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="11">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="11">
         <v>1.0</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="29">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="s">
-        <v>9</v>
+      <c r="A11" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="11">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="11">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="11">
         <v>1.0</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="29">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="s">
-        <v>18</v>
+      <c r="A12" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="11">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="11">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="11">
         <v>1.0</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="29">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="s">
-        <v>10</v>
+      <c r="A13" s="13" t="s">
+        <v>21</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="21"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="32"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17397,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="s">
-        <v>8</v>
+      <c r="A14" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="11">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="11">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="11">
         <v>1.0</v>
       </c>
-      <c r="E14" s="21"/>
+      <c r="E14" s="32"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17422,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="s">
-        <v>9</v>
+      <c r="A15" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="11">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="11">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="11">
         <v>1.0</v>
       </c>
-      <c r="E15" s="21"/>
+      <c r="E15" s="32"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
-      <c r="E16" s="9"/>
+      <c r="A16" s="33"/>
+      <c r="E16" s="25"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17462,14 +17462,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="9"/>
+      <c r="B17" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="25"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>8</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
+      <c r="E18" s="25"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="25"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="24"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>23</v>
+      <c r="A21" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="21"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="32"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17568,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="s">
-        <v>8</v>
+      <c r="A22" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="11">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="11">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="11">
         <v>1.0</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="32"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17593,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="s">
-        <v>9</v>
+      <c r="A23" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="11">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="11">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="11">
         <v>2.0</v>
       </c>
-      <c r="E23" s="21"/>
+      <c r="E23" s="32"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="24"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="25"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17636,12 +17636,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
-        <v>8</v>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="9"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="8">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="26">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="24"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
-        <v>25</v>
+      <c r="A29" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="21"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="32"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17742,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="s">
-        <v>8</v>
+      <c r="A30" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="11">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="11">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="11">
         <v>1.0</v>
       </c>
-      <c r="E30" s="21"/>
+      <c r="E30" s="32"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
-        <v>9</v>
+      <c r="A31" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="20">
         <v>70.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="20">
         <v>5.0</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="20">
         <v>1.0</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="33" t="s">
-        <v>26</v>
+      <c r="A33" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="34">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="34">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="34">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="35">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="36" t="s">
-        <v>27</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="37"/>
-      <c r="K33" s="37"/>
-      <c r="L33" s="37"/>
-      <c r="M33" s="37"/>
-      <c r="N33" s="37"/>
-      <c r="O33" s="37"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>11</v>
+      <c r="A36" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>28</v>
+      <c r="B36" s="8" t="s">
+        <v>15</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>8</v>
+      <c r="A37" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="8">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="17"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>15</v>
+      <c r="A38" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="17"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34590,9 +34590,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>8</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>20.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="9">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>12</v>
+      <c r="A5" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="8">
         <v>2.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <v>1.0</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="9">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34683,10 +34683,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,15 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="s">
-        <v>14</v>
+      <c r="A7" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>16</v>
+      <c r="B7" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="17"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34718,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="s">
-        <v>8</v>
+      <c r="A8" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="11">
         <v>4.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="11">
         <v>10.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="11">
         <v>1.0</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="14">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34744,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="s">
-        <v>9</v>
+      <c r="A9" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="11">
         <v>20.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="11">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="11">
         <v>1.0</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="14">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,11 +34770,11 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="24"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="12"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34787,9 +34787,9 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
-      <c r="E11" s="7"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34801,21 +34801,13 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>8</v>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B12" s="10">
-        <v>2.0</v>
-      </c>
-      <c r="C12" s="10">
-        <v>15.0</v>
-      </c>
-      <c r="D12" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E12" s="12">
-        <v>46106.732072326384</v>
-      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34827,19 +34819,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>20.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>20.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="9">
         <v>46147.893450902775</v>
       </c>
       <c r="F13" s="4"/>
@@ -34853,19 +34845,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>12</v>
+      <c r="A14" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>2.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>20.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="9">
         <v>46182.71399388889</v>
       </c>
       <c r="F14" s="4"/>
@@ -34879,11 +34871,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="24"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="12"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34896,12 +34888,12 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="12"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34913,23 +34905,23 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>8</v>
+      <c r="A17" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="8">
         <v>5.0</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <v>5.0</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="8">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34939,19 +34931,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>8</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>15.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="7"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34963,19 +34955,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>32.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34987,11 +34979,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="24"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="7"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35003,13 +34995,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>23</v>
+      <c r="A21" s="10" t="s">
+        <v>11</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="17"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="12"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35021,19 +35013,19 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="s">
-        <v>8</v>
+      <c r="A22" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="11">
         <v>5.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="11">
         <v>5.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="11">
         <v>1.0</v>
       </c>
-      <c r="E22" s="17"/>
+      <c r="E22" s="12"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35045,19 +35037,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="s">
-        <v>9</v>
+      <c r="A23" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="11">
         <v>50.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="11">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="11">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="12"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35069,11 +35061,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="24"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="7"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35086,12 +35078,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="7"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35103,19 +35095,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
-        <v>8</v>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>5.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>5.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="7"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35127,13 +35119,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="7"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35145,11 +35137,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="24"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35161,13 +35153,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
-        <v>25</v>
+      <c r="A29" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="17"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="12"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35179,19 +35171,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="s">
-        <v>8</v>
+      <c r="A30" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="11">
         <v>5.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="11">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="11">
         <v>1.0</v>
       </c>
-      <c r="E30" s="17"/>
+      <c r="E30" s="12"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35203,17 +35195,17 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
-        <v>9</v>
+      <c r="A31" s="19" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="20">
         <v>55.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="20">
         <v>2.0</v>
       </c>
-      <c r="D31" s="38"/>
-      <c r="E31" s="39"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="22"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35225,11 +35217,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35241,15 +35233,15 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>11</v>
+      <c r="A33" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B33" s="10" t="s">
-        <v>28</v>
+      <c r="B33" s="8" t="s">
+        <v>15</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="40">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="23">
         <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
@@ -35263,17 +35255,17 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>8</v>
+      <c r="A34" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="8">
         <v>2.0</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="8">
         <v>100.0</v>
       </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="40">
+      <c r="D34" s="17"/>
+      <c r="E34" s="23">
         <v>46100.83597384259</v>
       </c>
       <c r="F34" s="4"/>
@@ -35287,17 +35279,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>15</v>
+      <c r="A35" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="8">
         <v>20.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="40">
+      <c r="D35" s="17"/>
+      <c r="E35" s="23">
         <v>46100.83604224537</v>
       </c>
       <c r="F35" s="4"/>
@@ -35311,11 +35303,11 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="A36" s="17"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35327,11 +35319,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="17"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51119,19 +51111,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51143,13 +51135,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="25"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51160,19 +51152,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>9</v>
+      <c r="A3" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="24">
         <v>60.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="24">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="25"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51184,10 +51176,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="9"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="25"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51199,14 +51191,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="26"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51217,19 +51209,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>15</v>
+      <c r="A6" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>60.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="26">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51243,10 +51235,10 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="9"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="25"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51258,12 +51250,12 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="9"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="25"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51274,19 +51266,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>8</v>
+      <c r="A9" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="8">
         <v>10.0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <v>45.0</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="8">
         <v>1.0</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="26">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51299,19 +51291,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>15</v>
+      <c r="A10" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="8">
         <v>11.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <v>20.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="26">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51325,10 +51317,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="28"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51339,15 +51331,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="s">
-        <v>17</v>
+      <c r="A12" s="30" t="s">
+        <v>22</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>19</v>
+      <c r="B12" s="31" t="s">
+        <v>23</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="26"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51358,19 +51350,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>18</v>
+      <c r="A13" s="7" t="s">
+        <v>24</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>5.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>60.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="26">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51383,19 +51375,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>8</v>
+      <c r="A14" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>30.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51406,23 +51398,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>21</v>
+      <c r="A15" s="7" t="s">
+        <v>25</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="8">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="8">
         <v>4.0</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="26">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>22</v>
+      <c r="F15" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51433,19 +51425,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>15</v>
+      <c r="A16" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="8">
         <v>12.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>20.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="8">
         <v>1.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="26">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51459,10 +51451,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="28"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51474,12 +51466,12 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="25"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51490,19 +51482,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>8</v>
+      <c r="A19" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="24">
         <v>6.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="24">
         <v>45.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="26">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51515,19 +51507,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>9</v>
+      <c r="A20" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="24">
         <v>18.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="24">
         <v>20.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="26">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51540,11 +51532,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="6"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51555,15 +51547,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="s">
-        <v>14</v>
+      <c r="A22" s="30" t="s">
+        <v>8</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>19</v>
+      <c r="B22" s="31" t="s">
+        <v>23</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="11">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="26">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51576,19 +51568,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="s">
-        <v>18</v>
+      <c r="A23" s="7" t="s">
+        <v>24</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="24">
         <v>6.0</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="24">
         <v>50.0</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="8">
         <v>1.0</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="26">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51601,19 +51593,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="s">
-        <v>8</v>
+      <c r="A24" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="24">
         <v>8.0</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="24">
         <v>30.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="26">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51626,23 +51618,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>15</v>
+      <c r="A25" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="24">
         <v>10.0</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="24">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="8">
         <v>4.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="26">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>22</v>
+      <c r="F25" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51653,19 +51645,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
-        <v>15</v>
+      <c r="A26" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="24">
         <v>17.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="24">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="26">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51678,11 +51670,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51693,15 +51685,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="s">
-        <v>20</v>
+      <c r="A28" s="30" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="26" t="s">
-        <v>19</v>
+      <c r="B28" s="31" t="s">
+        <v>23</v>
       </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51712,19 +51704,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="s">
-        <v>18</v>
+      <c r="A29" s="7" t="s">
+        <v>24</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="24">
         <v>6.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="24">
         <v>50.0</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="8">
         <v>1.0</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="26">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51737,19 +51729,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="s">
-        <v>8</v>
+      <c r="A30" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="24">
         <v>8.0</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="24">
         <v>30.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51760,19 +51752,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="s">
-        <v>9</v>
+      <c r="A31" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="24">
         <v>15.0</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="24">
         <v>10.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="8">
         <v>2.0</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="26">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51785,11 +51777,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="6"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="9"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="25"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51800,13 +51792,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="s">
-        <v>20</v>
+      <c r="A33" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="21"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="32"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51817,19 +51809,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="s">
-        <v>8</v>
+      <c r="A34" s="13" t="s">
+        <v>6</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>29</v>
+      <c r="B34" s="35" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="35">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="35">
         <v>1.0</v>
       </c>
-      <c r="E34" s="18">
+      <c r="E34" s="29">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51842,19 +51834,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="s">
-        <v>9</v>
+      <c r="A35" s="13" t="s">
+        <v>7</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="35">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="35">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="21"/>
+      <c r="E35" s="32"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51865,11 +51857,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="24"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="9"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51881,12 +51873,12 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="9"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51897,19 +51889,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="s">
-        <v>9</v>
+      <c r="A38" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>40.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>15.0</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="8">
         <v>1.0</v>
       </c>
-      <c r="E38" s="11">
+      <c r="E38" s="26">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51923,10 +51915,10 @@
     </row>
     <row r="39">
       <c r="A39" s="5"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="9"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="25"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51938,12 +51930,12 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="9"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="25"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51954,19 +51946,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="s">
-        <v>8</v>
+      <c r="A41" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="8">
         <v>9.0</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="8">
         <v>20.0</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="8">
         <v>1.0</v>
       </c>
-      <c r="E41" s="11">
+      <c r="E41" s="26">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51979,19 +51971,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="s">
-        <v>9</v>
+      <c r="A42" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="8">
         <v>55.0</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="8">
         <v>20.0</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="8">
         <v>1.0</v>
       </c>
-      <c r="E42" s="11">
+      <c r="E42" s="26">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -52004,22 +51996,22 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="s">
-        <v>8</v>
+      <c r="A43" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="8">
         <v>10.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="8">
         <v>250.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="26">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="14" t="s">
+      <c r="F43" s="15" t="s">
         <v>31</v>
       </c>
       <c r="G43" s="4"/>
@@ -52032,10 +52024,10 @@
     </row>
     <row r="44">
       <c r="A44" s="42"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="9"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="25"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52047,12 +52039,12 @@
     </row>
     <row r="45">
       <c r="A45" s="42" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="9"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="25"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52063,19 +52055,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="s">
-        <v>9</v>
+      <c r="A46" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="8">
         <v>60.0</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="8">
         <v>10.0</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="8">
         <v>1.0</v>
       </c>
-      <c r="E46" s="11">
+      <c r="E46" s="26">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52089,10 +52081,10 @@
     </row>
     <row r="47">
       <c r="A47" s="42"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="9"/>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="25"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52106,10 +52098,10 @@
       <c r="A48" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="9"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="25"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52120,19 +52112,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="s">
-        <v>12</v>
+      <c r="A49" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B49" s="8">
+      <c r="B49" s="24">
         <v>70.0</v>
       </c>
-      <c r="C49" s="8">
+      <c r="C49" s="24">
         <v>300.0</v>
       </c>
-      <c r="D49" s="8">
+      <c r="D49" s="24">
         <v>1.0</v>
       </c>
-      <c r="E49" s="11">
+      <c r="E49" s="26">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52145,19 +52137,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="s">
-        <v>8</v>
+      <c r="A50" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B50" s="8">
+      <c r="B50" s="24">
         <v>10.0</v>
       </c>
-      <c r="C50" s="8">
+      <c r="C50" s="24">
         <v>20.0</v>
       </c>
-      <c r="D50" s="8">
+      <c r="D50" s="24">
         <v>1.0</v>
       </c>
-      <c r="E50" s="11">
+      <c r="E50" s="26">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52170,19 +52162,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="s">
-        <v>9</v>
+      <c r="A51" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="24">
         <v>70.0</v>
       </c>
-      <c r="C51" s="8">
+      <c r="C51" s="24">
         <v>10.0</v>
       </c>
-      <c r="D51" s="8">
+      <c r="D51" s="24">
         <v>1.0</v>
       </c>
-      <c r="E51" s="11">
+      <c r="E51" s="26">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52195,11 +52187,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="6"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="9"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="25"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52210,15 +52202,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="11">
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="26">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52231,15 +52223,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="6">
+      <c r="A54" s="7">
         <v>50.0</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="8">
         <v>100.0</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="11">
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="26">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52269,16 +52261,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="36" t="s">
+      <c r="A56" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="36">
+      <c r="B56" s="40">
         <v>100.0</v>
       </c>
-      <c r="C56" s="14">
+      <c r="C56" s="15">
         <v>1.0</v>
       </c>
-      <c r="D56" s="14">
+      <c r="D56" s="15">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52294,8 +52286,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="37"/>
-      <c r="B57" s="37"/>
+      <c r="A57" s="41"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52309,10 +52301,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="36" t="s">
+      <c r="A58" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="37"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52326,16 +52318,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="s">
-        <v>9</v>
+      <c r="A59" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B59" s="36">
+      <c r="B59" s="40">
         <v>50.0</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="15">
         <v>20.0</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59" s="15">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52351,13 +52343,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="36" t="s">
+      <c r="A60" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="36">
+      <c r="B60" s="40">
         <v>15.0</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="15">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52374,8 +52366,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="37"/>
-      <c r="B61" s="37"/>
+      <c r="A61" s="41"/>
+      <c r="B61" s="41"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52389,11 +52381,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="36" t="s">
+      <c r="A62" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="36" t="s">
-        <v>24</v>
+      <c r="B62" s="40" t="s">
+        <v>12</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52410,16 +52402,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="36" t="s">
+      <c r="A63" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="36">
+      <c r="B63" s="40">
         <v>5.0</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="15">
         <v>80.0</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="15">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52435,16 +52427,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="36" t="s">
+      <c r="A64" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="36">
+      <c r="B64" s="40">
         <v>15.0</v>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="15">
         <v>10.0</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64" s="15">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52460,16 +52452,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="36" t="s">
-        <v>15</v>
+      <c r="A65" s="40" t="s">
+        <v>16</v>
       </c>
-      <c r="B65" s="36">
+      <c r="B65" s="40">
         <v>30.0</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="15">
         <v>10.0</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52485,8 +52477,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="37"/>
-      <c r="B66" s="37"/>
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52500,10 +52492,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="36" t="s">
+      <c r="A67" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="36" t="s">
+      <c r="B67" s="40" t="s">
         <v>32</v>
       </c>
       <c r="C67" s="4"/>
@@ -52521,16 +52513,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="36" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="36">
+      <c r="B68" s="40">
         <v>5.0</v>
       </c>
-      <c r="C68" s="14">
+      <c r="C68" s="15">
         <v>80.0</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="15">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52544,16 +52536,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="36" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="36">
+      <c r="B69" s="40">
         <v>15.0</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="15">
         <v>10.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52567,16 +52559,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="36" t="s">
-        <v>15</v>
+      <c r="A70" s="40" t="s">
+        <v>16</v>
       </c>
-      <c r="B70" s="36">
+      <c r="B70" s="40">
         <v>20.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="15">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52592,8 +52584,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="37"/>
-      <c r="B71" s="37"/>
+      <c r="A71" s="41"/>
+      <c r="B71" s="41"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52607,8 +52599,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="36"/>
-      <c r="B72" s="37"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52622,8 +52614,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="37"/>
-      <c r="B73" s="37"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:24.554Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,6 +19,9 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
   </si>
   <si>
@@ -28,61 +31,46 @@
     <t>次數</t>
   </si>
   <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>最後更新日期</t>
+  </si>
+  <si>
+    <t>Line</t>
   </si>
   <si>
     <t>0.3mm</t>
   </si>
   <si>
-    <t>Line</t>
+    <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut-1/2</t>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>03mm</t>
   </si>
   <si>
     <t>0.5mm</t>
   </si>
   <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>1mm</t>
-  </si>
-  <si>
-    <t>2mm</t>
-  </si>
-  <si>
-    <t>3mm</t>
-  </si>
-  <si>
-    <t>4mm</t>
-  </si>
-  <si>
-    <t>A4紙</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
-    <t>刀壓</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>03mm</t>
-  </si>
-  <si>
     <t>(PS)</t>
   </si>
   <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
     <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>1mm</t>
   </si>
   <si>
     <t>PS</t>
@@ -94,7 +82,19 @@
     <t>cut</t>
   </si>
   <si>
+    <t>2mm</t>
+  </si>
+  <si>
     <t>Keep Detail</t>
+  </si>
+  <si>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>4mm</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
@@ -103,13 +103,13 @@
     <t>1.5mm</t>
   </si>
   <si>
+    <t>吉翁號刻線參數</t>
+  </si>
+  <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,20 +321,32 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -357,11 +369,30 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -378,60 +409,29 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="6"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>8</v>
+      <c r="A6" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>9</v>
+      <c r="B6" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>6</v>
+      <c r="A7" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="18">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>7</v>
+      <c r="A8" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="18">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="16"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>10</v>
+      <c r="A10" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
+      <c r="A11" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>7</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="16"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="6"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="8"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>11</v>
+      <c r="A15" s="14" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="12"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>6</v>
+      <c r="A16" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>7</v>
+      <c r="A17" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="6"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>12</v>
+      <c r="A19" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>6</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>7</v>
+      <c r="A21" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="6"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>13</v>
+      <c r="A23" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="12"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>6</v>
+      <c r="A24" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="s">
-        <v>7</v>
+      <c r="A25" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>14</v>
+      <c r="A27" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>15</v>
+      <c r="B27" s="10" t="s">
+        <v>26</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="23">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>6</v>
+      <c r="A28" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="23">
+      <c r="D28" s="13"/>
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>16</v>
+      <c r="A29" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="23">
+      <c r="D29" s="13"/>
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="25"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>21</v>
+      <c r="A5" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="25"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>6</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="25"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>7</v>
+      <c r="A7" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,11 +17261,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="26"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
-        <v>8</v>
+      <c r="A9" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="29"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17297,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>6</v>
+      <c r="A10" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="15">
         <v>15.0</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="25">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="s">
-        <v>7</v>
+      <c r="A11" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="25">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="s">
-        <v>24</v>
+      <c r="A12" s="17" t="s">
+        <v>20</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="25">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="s">
-        <v>21</v>
+      <c r="A13" s="17" t="s">
+        <v>15</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="32"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="27"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17397,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="s">
-        <v>6</v>
+      <c r="A14" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="32"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17422,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>7</v>
+      <c r="A15" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="32"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="33"/>
-      <c r="E16" s="25"/>
+      <c r="A16" s="28"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>10</v>
+      <c r="A17" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B17" s="34" t="s">
-        <v>21</v>
+      <c r="B17" s="29" t="s">
+        <v>15</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="25"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="25"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>7</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="25"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="25"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>11</v>
+      <c r="A21" s="14" t="s">
+        <v>22</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="32"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17568,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>6</v>
+      <c r="A22" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="32"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17593,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>7</v>
+      <c r="A23" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="32"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="25"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>12</v>
+      <c r="A25" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="25"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="25"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>7</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="25"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>13</v>
+      <c r="A29" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="32"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17742,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>6</v>
+      <c r="A30" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="32"/>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,16 +17767,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="s">
-        <v>7</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
       <c r="E31" s="36"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
-        <v>29</v>
+      <c r="A33" s="38" t="s">
+        <v>30</v>
       </c>
-      <c r="B33" s="38">
+      <c r="B33" s="39">
         <v>5.0</v>
       </c>
-      <c r="C33" s="38">
+      <c r="C33" s="39">
         <v>10.0</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="39">
         <v>2.0</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="40">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="40" t="s">
-        <v>30</v>
+      <c r="F33" s="41" t="s">
+        <v>31</v>
       </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>14</v>
+      <c r="A36" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>15</v>
+      <c r="B36" s="10" t="s">
+        <v>26</v>
       </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>6</v>
+      <c r="A37" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
-      <c r="D37" s="17"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>16</v>
+      <c r="A38" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
-      <c r="D38" s="17"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>20.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>19</v>
+      <c r="A5" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="10">
         <v>2.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="8"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,15 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>8</v>
+      <c r="A7" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>9</v>
+      <c r="B7" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="16"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34718,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>6</v>
+      <c r="A8" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="15">
         <v>4.0</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="15">
         <v>10.0</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="18">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34744,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>7</v>
+      <c r="A9" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="15">
         <v>20.0</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="18">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,11 +34770,11 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="16"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="9"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34786,10 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>8</v>
+      <c r="A11" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="E11" s="6"/>
+      <c r="E11" s="8"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34801,13 +34801,13 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34819,20 +34819,20 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>7</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>20.0</v>
       </c>
-      <c r="C13" s="8">
-        <v>20.0</v>
+      <c r="C13" s="10">
+        <v>10.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="9">
-        <v>46147.893450902775</v>
+      <c r="E13" s="11">
+        <v>46228.70790929398</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -34845,19 +34845,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>19</v>
+      <c r="A14" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>2.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="10">
         <v>20.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F14" s="4"/>
@@ -34871,11 +34871,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="16"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="9"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34887,13 +34887,13 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>10</v>
+      <c r="A16" s="6" t="s">
+        <v>18</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34905,23 +34905,23 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>6</v>
+      <c r="A17" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="10">
         <v>5.0</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="10">
         <v>5.0</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="10">
         <v>1.0</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34931,19 +34931,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>15.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34955,19 +34955,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>7</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>32.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34979,11 +34979,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="6"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34995,13 +34995,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>11</v>
+      <c r="A21" s="14" t="s">
+        <v>22</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="12"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35013,19 +35013,19 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>6</v>
+      <c r="A22" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="15">
         <v>5.0</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="15">
         <v>5.0</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="12"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35037,19 +35037,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>7</v>
+      <c r="A23" s="17" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="15">
         <v>50.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="15">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35061,11 +35061,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="6"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35077,13 +35077,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>12</v>
+      <c r="A25" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="6"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35095,19 +35095,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>5.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>5.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35119,13 +35119,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>7</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="6"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="8"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35137,11 +35137,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="6"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35153,13 +35153,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>13</v>
+      <c r="A29" s="14" t="s">
+        <v>25</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="12"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="16"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35171,19 +35171,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>6</v>
+      <c r="A30" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="15">
         <v>5.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="12"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35195,17 +35195,17 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="s">
-        <v>7</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="31">
         <v>55.0</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="31">
         <v>2.0</v>
       </c>
-      <c r="D31" s="21"/>
-      <c r="E31" s="22"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="33"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35217,11 +35217,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35233,15 +35233,15 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>14</v>
+      <c r="A33" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>15</v>
+      <c r="B33" s="10" t="s">
+        <v>26</v>
       </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="23">
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
@@ -35255,17 +35255,17 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>6</v>
+      <c r="A34" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="10">
         <v>2.0</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C34" s="10">
         <v>100.0</v>
       </c>
-      <c r="D34" s="17"/>
-      <c r="E34" s="23">
+      <c r="D34" s="13"/>
+      <c r="E34" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F34" s="4"/>
@@ -35279,17 +35279,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
-        <v>16</v>
+      <c r="A35" s="10" t="s">
+        <v>14</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="10">
         <v>20.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
-      <c r="D35" s="17"/>
-      <c r="E35" s="23">
+      <c r="D35" s="13"/>
+      <c r="E35" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F35" s="4"/>
@@ -35303,11 +35303,11 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35319,11 +35319,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51111,19 +51111,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51135,13 +51135,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>6</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="25"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51152,19 +51152,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
+      <c r="A3" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="7">
         <v>60.0</v>
       </c>
-      <c r="C3" s="24">
+      <c r="C3" s="7">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="9"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51175,11 +51175,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="25"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51190,15 +51190,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" s="6" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>20</v>
+      <c r="B5" s="6" t="s">
+        <v>11</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="26"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51209,19 +51209,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>16</v>
+      <c r="A6" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="12">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51234,11 +51234,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="25"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51249,13 +51249,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>22</v>
+      <c r="A8" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="25"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="9"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51266,19 +51266,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>6</v>
+      <c r="A9" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51291,19 +51291,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>16</v>
+      <c r="A10" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51316,11 +51316,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="28"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="22"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51331,15 +51331,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="s">
-        <v>22</v>
+      <c r="A12" s="23" t="s">
+        <v>17</v>
       </c>
-      <c r="B12" s="31" t="s">
-        <v>23</v>
+      <c r="B12" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="26"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51350,19 +51350,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>24</v>
+      <c r="A13" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51375,19 +51375,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>6</v>
+      <c r="A14" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51398,23 +51398,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>25</v>
+      <c r="A15" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>26</v>
+      <c r="F15" s="19" t="s">
+        <v>23</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51425,19 +51425,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>16</v>
+      <c r="A16" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51450,11 +51450,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="28"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51465,13 +51465,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>8</v>
+      <c r="A18" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="25"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51482,19 +51482,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="7">
         <v>6.0</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="7">
         <v>45.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="26">
+      <c r="E19" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51507,19 +51507,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
+      <c r="A20" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B20" s="7">
         <v>18.0</v>
       </c>
-      <c r="C20" s="24">
+      <c r="C20" s="7">
         <v>20.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E20" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51532,11 +51532,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="25"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51547,15 +51547,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="s">
-        <v>8</v>
+      <c r="A22" s="23" t="s">
+        <v>12</v>
       </c>
-      <c r="B22" s="31" t="s">
-        <v>23</v>
+      <c r="B22" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="26">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51568,19 +51568,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>24</v>
+      <c r="A23" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B23" s="24">
+      <c r="B23" s="7">
         <v>6.0</v>
       </c>
-      <c r="C23" s="24">
+      <c r="C23" s="7">
         <v>50.0</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
-      <c r="E23" s="26">
+      <c r="E23" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51593,19 +51593,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>6</v>
+      <c r="A24" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="24">
+      <c r="B24" s="7">
         <v>8.0</v>
       </c>
-      <c r="C24" s="24">
+      <c r="C24" s="7">
         <v>30.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51618,23 +51618,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>16</v>
+      <c r="A25" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="7">
         <v>10.0</v>
       </c>
-      <c r="C25" s="24">
+      <c r="C25" s="7">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>26</v>
+      <c r="F25" s="19" t="s">
+        <v>23</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51645,19 +51645,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>16</v>
+      <c r="A26" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B26" s="24">
+      <c r="B26" s="7">
         <v>17.0</v>
       </c>
-      <c r="C26" s="24">
+      <c r="C26" s="7">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51670,11 +51670,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="25"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51685,15 +51685,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="s">
-        <v>10</v>
+      <c r="A28" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="B28" s="31" t="s">
-        <v>23</v>
+      <c r="B28" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="25"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51704,19 +51704,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>24</v>
+      <c r="A29" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="24">
+      <c r="B29" s="7">
         <v>6.0</v>
       </c>
-      <c r="C29" s="24">
+      <c r="C29" s="7">
         <v>50.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51729,19 +51729,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>6</v>
+      <c r="A30" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="24">
+      <c r="B30" s="7">
         <v>8.0</v>
       </c>
-      <c r="C30" s="24">
+      <c r="C30" s="7">
         <v>30.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="25"/>
+      <c r="E30" s="9"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51752,19 +51752,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>7</v>
+      <c r="A31" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="24">
+      <c r="B31" s="7">
         <v>15.0</v>
       </c>
-      <c r="C31" s="24">
+      <c r="C31" s="7">
         <v>10.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
-      <c r="E31" s="26">
+      <c r="E31" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51777,11 +51777,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="25"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="9"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51792,13 +51792,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>10</v>
+      <c r="A33" s="14" t="s">
+        <v>18</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="32"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51809,8 +51809,8 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="s">
-        <v>6</v>
+      <c r="A34" s="17" t="s">
+        <v>7</v>
       </c>
       <c r="B34" s="35" t="s">
         <v>27</v>
@@ -51821,7 +51821,7 @@
       <c r="D34" s="35">
         <v>1.0</v>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="25">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51834,8 +51834,8 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="s">
-        <v>7</v>
+      <c r="A35" s="17" t="s">
+        <v>9</v>
       </c>
       <c r="B35" s="35">
         <v>30.0</v>
@@ -51846,7 +51846,7 @@
       <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="32"/>
+      <c r="E35" s="27"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51857,11 +51857,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="16"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="25"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="9"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51872,13 +51872,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="25"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51889,19 +51889,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>7</v>
+      <c r="A38" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51914,11 +51914,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="25"/>
+      <c r="A39" s="6"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="9"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51929,13 +51929,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>11</v>
+      <c r="A40" s="6" t="s">
+        <v>22</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="25"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="9"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51946,19 +51946,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>6</v>
+      <c r="A41" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51971,19 +51971,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>7</v>
+      <c r="A42" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -51996,23 +51996,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>6</v>
+      <c r="A43" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="15" t="s">
-        <v>31</v>
+      <c r="F43" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52023,11 +52023,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="25"/>
+      <c r="A44" s="37"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="9"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52038,13 +52038,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>13</v>
+      <c r="A45" s="37" t="s">
+        <v>25</v>
       </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="25"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="9"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52055,19 +52055,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>7</v>
+      <c r="A46" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52080,11 +52080,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="25"/>
+      <c r="A47" s="37"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="9"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52095,13 +52095,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
+      <c r="A48" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="25"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52112,19 +52112,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
-        <v>19</v>
+      <c r="A49" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B49" s="24">
+      <c r="B49" s="7">
         <v>70.0</v>
       </c>
-      <c r="C49" s="24">
+      <c r="C49" s="7">
         <v>300.0</v>
       </c>
-      <c r="D49" s="24">
+      <c r="D49" s="7">
         <v>1.0</v>
       </c>
-      <c r="E49" s="26">
+      <c r="E49" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52137,19 +52137,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="s">
-        <v>6</v>
+      <c r="A50" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B50" s="24">
+      <c r="B50" s="7">
         <v>10.0</v>
       </c>
-      <c r="C50" s="24">
+      <c r="C50" s="7">
         <v>20.0</v>
       </c>
-      <c r="D50" s="24">
+      <c r="D50" s="7">
         <v>1.0</v>
       </c>
-      <c r="E50" s="26">
+      <c r="E50" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52162,19 +52162,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>7</v>
+      <c r="A51" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B51" s="24">
+      <c r="B51" s="7">
         <v>70.0</v>
       </c>
-      <c r="C51" s="24">
+      <c r="C51" s="7">
         <v>10.0</v>
       </c>
-      <c r="D51" s="24">
+      <c r="D51" s="7">
         <v>1.0</v>
       </c>
-      <c r="E51" s="26">
+      <c r="E51" s="12">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52187,11 +52187,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="25"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="9"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52202,15 +52202,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="26">
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52223,15 +52223,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="7">
+      <c r="A54" s="5">
         <v>50.0</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="26">
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52261,16 +52261,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="40" t="s">
+      <c r="A56" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="40">
+      <c r="B56" s="41">
         <v>100.0</v>
       </c>
-      <c r="C56" s="15">
+      <c r="C56" s="19">
         <v>1.0</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="19">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52286,8 +52286,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="41"/>
-      <c r="B57" s="41"/>
+      <c r="A57" s="42"/>
+      <c r="B57" s="42"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52301,10 +52301,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="40" t="s">
+      <c r="A58" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="41"/>
+      <c r="B58" s="42"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52318,16 +52318,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="s">
-        <v>7</v>
+      <c r="A59" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B59" s="40">
+      <c r="B59" s="41">
         <v>50.0</v>
       </c>
-      <c r="C59" s="15">
+      <c r="C59" s="19">
         <v>20.0</v>
       </c>
-      <c r="D59" s="15">
+      <c r="D59" s="19">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52343,13 +52343,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="s">
+      <c r="A60" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="40">
+      <c r="B60" s="41">
         <v>15.0</v>
       </c>
-      <c r="C60" s="15">
+      <c r="C60" s="19">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52366,8 +52366,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="41"/>
-      <c r="B61" s="41"/>
+      <c r="A61" s="42"/>
+      <c r="B61" s="42"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52381,11 +52381,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
+      <c r="A62" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="40" t="s">
-        <v>12</v>
+      <c r="B62" s="41" t="s">
+        <v>24</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52402,16 +52402,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="s">
+      <c r="A63" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="40">
+      <c r="B63" s="41">
         <v>5.0</v>
       </c>
-      <c r="C63" s="15">
+      <c r="C63" s="19">
         <v>80.0</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="19">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52427,16 +52427,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
+      <c r="A64" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="40">
+      <c r="B64" s="41">
         <v>15.0</v>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="19">
         <v>10.0</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="19">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52452,16 +52452,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="40" t="s">
-        <v>16</v>
+      <c r="A65" s="41" t="s">
+        <v>14</v>
       </c>
-      <c r="B65" s="40">
+      <c r="B65" s="41">
         <v>30.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="19">
         <v>10.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="19">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52477,8 +52477,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="41"/>
-      <c r="B66" s="41"/>
+      <c r="A66" s="42"/>
+      <c r="B66" s="42"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52492,10 +52492,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40" t="s">
+      <c r="A67" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="40" t="s">
+      <c r="B67" s="41" t="s">
         <v>32</v>
       </c>
       <c r="C67" s="4"/>
@@ -52513,16 +52513,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="40">
+      <c r="B68" s="41">
         <v>5.0</v>
       </c>
-      <c r="C68" s="15">
+      <c r="C68" s="19">
         <v>80.0</v>
       </c>
-      <c r="D68" s="15">
+      <c r="D68" s="19">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52536,16 +52536,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
+      <c r="A69" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="40">
+      <c r="B69" s="41">
         <v>15.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="19">
         <v>10.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="19">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52559,16 +52559,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
-        <v>16</v>
+      <c r="A70" s="41" t="s">
+        <v>14</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="41">
         <v>20.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="19">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="19">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52584,8 +52584,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="41"/>
-      <c r="B71" s="41"/>
+      <c r="A71" s="42"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52599,8 +52599,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="41"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="42"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52614,8 +52614,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="41"/>
-      <c r="B73" s="41"/>
+      <c r="A73" s="42"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:27.224Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,9 +19,6 @@
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
   </si>
   <si>
@@ -31,19 +28,34 @@
     <t>次數</t>
   </si>
   <si>
-    <t>刀壓</t>
+    <t>最後更新日期</t>
   </si>
   <si>
-    <t>最後更新日期</t>
+    <t>0.3mm</t>
   </si>
   <si>
     <t>Line</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>Cut-1/2</t>
+  </si>
+  <si>
+    <t>刀壓</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
+    <t>(PS)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -52,19 +64,7 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
     <t>Cut</t>
-  </si>
-  <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -73,10 +73,10 @@
     <t>1mm</t>
   </si>
   <si>
-    <t>PS</t>
+    <t>Fill</t>
   </si>
   <si>
-    <t>Fill</t>
+    <t>PS</t>
   </si>
   <si>
     <t>cut</t>
@@ -100,16 +100,16 @@
     <t>６</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>1.5mm</t>
   </si>
   <si>
-    <t>吉翁號刻線參數</t>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
+    <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -321,20 +321,14 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -342,14 +336,20 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -360,10 +360,13 @@
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -381,13 +384,10 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -415,23 +415,23 @@
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,11 +785,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>12</v>
+      <c r="A6" s="13" t="s">
+        <v>10</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C6" s="15"/>
       <c r="D6" s="15"/>
@@ -806,7 +806,7 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="15">
         <v>4.0</v>
@@ -817,11 +817,11 @@
       <c r="D7" s="15">
         <v>1.0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -832,7 +832,7 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="15">
         <v>25.0</v>
@@ -843,11 +843,11 @@
       <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="9"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
+      <c r="A11" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="8"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,12 +981,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
       <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1000,7 +1000,7 @@
     </row>
     <row r="16">
       <c r="A16" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="15">
         <v>5.0</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B17" s="15">
         <v>50.0</v>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="8"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="8"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>7</v>
+      <c r="A20" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
-        <v>9</v>
+      <c r="A21" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="8"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="8"/>
+      <c r="A22" s="21"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,12 +1139,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
       <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="24">
       <c r="A24" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B24" s="15">
         <v>5.0</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,14 +1219,14 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>10</v>
+      <c r="A27" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
       <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -1241,16 +1241,16 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>7</v>
+      <c r="A28" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
+      <c r="D28" s="14"/>
       <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -1265,16 +1265,16 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>14</v>
+      <c r="A29" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,16 +17140,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>15</v>
+      <c r="A5" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
+      <c r="A7" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,10 +17261,10 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
       <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>12</v>
+      <c r="A9" s="13" t="s">
+        <v>10</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
-      <c r="E9" s="25"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17298,7 +17298,7 @@
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="15">
         <v>4.0</v>
@@ -17309,7 +17309,7 @@
       <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="20">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17325,7 +17325,7 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="15">
         <v>25.0</v>
@@ -17336,7 +17336,7 @@
       <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="20">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17352,7 +17352,7 @@
     </row>
     <row r="12">
       <c r="A12" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="15">
         <v>4.0</v>
@@ -17363,7 +17363,7 @@
       <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="20">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17379,12 +17379,12 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
-      <c r="E13" s="27"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17398,7 +17398,7 @@
     </row>
     <row r="14">
       <c r="A14" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="15">
         <v>2.0</v>
@@ -17409,7 +17409,7 @@
       <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17423,7 +17423,7 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" s="15">
         <v>18.0</v>
@@ -17434,7 +17434,7 @@
       <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="16">
       <c r="A16" s="28"/>
-      <c r="E16" s="9"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="9"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17569,7 +17569,7 @@
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" s="15">
         <v>8.0</v>
@@ -17580,7 +17580,7 @@
       <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17594,7 +17594,7 @@
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" s="15">
         <v>55.0</v>
@@ -17605,7 +17605,7 @@
       <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="9"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,16 +17679,16 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="8">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="8">
         <v>2.0</v>
       </c>
       <c r="E27" s="12">
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17743,7 +17743,7 @@
     </row>
     <row r="30">
       <c r="A30" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" s="15">
         <v>18.0</v>
@@ -17754,7 +17754,7 @@
       <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17768,7 +17768,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="38" t="s">
+      <c r="A33" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="38">
+        <v>5.0</v>
+      </c>
+      <c r="C33" s="38">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="38">
+        <v>2.0</v>
+      </c>
+      <c r="E33" s="39">
+        <v>46043.55545597222</v>
+      </c>
+      <c r="F33" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="39">
-        <v>5.0</v>
-      </c>
-      <c r="C33" s="39">
-        <v>10.0</v>
-      </c>
-      <c r="D33" s="39">
-        <v>2.0</v>
-      </c>
-      <c r="E33" s="40">
-        <v>46043.55545597222</v>
-      </c>
-      <c r="F33" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>10</v>
+      <c r="A36" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>7</v>
+      <c r="A37" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="8">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="14"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>14</v>
+      <c r="A38" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="14"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>20.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="9">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>13</v>
+      <c r="A5" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="8">
         <v>2.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <v>1.0</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="9">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="8"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,11 +34698,11 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="s">
-        <v>12</v>
+      <c r="A7" s="13" t="s">
+        <v>10</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
@@ -34719,7 +34719,7 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="15">
         <v>4.0</v>
@@ -34730,11 +34730,11 @@
       <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34745,7 +34745,7 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="15">
         <v>20.0</v>
@@ -34756,11 +34756,11 @@
       <c r="D9" s="15">
         <v>1.0</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,11 +34770,11 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="20"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="11"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34786,10 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>12</v>
+      <c r="A11" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34801,13 +34801,13 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34819,19 +34819,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>20.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>10.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="9">
         <v>46228.70790929398</v>
       </c>
       <c r="F13" s="4"/>
@@ -34845,21 +34845,13 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>13</v>
+      <c r="A14" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B14" s="10">
-        <v>2.0</v>
-      </c>
-      <c r="C14" s="10">
-        <v>20.0</v>
-      </c>
-      <c r="D14" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E14" s="11">
-        <v>46182.71399388889</v>
-      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34871,11 +34863,11 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="20"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="11"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34887,13 +34879,13 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="11"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34905,23 +34897,23 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>7</v>
+      <c r="A17" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="8">
         <v>5.0</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <v>5.0</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="8">
         <v>1.0</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34931,19 +34923,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>15.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34955,19 +34947,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>32.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34979,11 +34971,11 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34995,12 +34987,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
       <c r="E21" s="16"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35014,7 +35006,7 @@
     </row>
     <row r="22">
       <c r="A22" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" s="15">
         <v>5.0</v>
@@ -35038,7 +35030,7 @@
     </row>
     <row r="23">
       <c r="A23" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" s="15">
         <v>50.0</v>
@@ -35061,11 +35053,11 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35077,13 +35069,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="8"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35095,19 +35087,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>5.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>5.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35119,13 +35111,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="8"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35137,11 +35129,11 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35153,12 +35145,12 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
       <c r="E29" s="16"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35172,7 +35164,7 @@
     </row>
     <row r="30">
       <c r="A30" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" s="15">
         <v>5.0</v>
@@ -35196,7 +35188,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B31" s="31">
         <v>55.0</v>
@@ -35217,11 +35209,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35233,14 +35225,14 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>10</v>
+      <c r="A33" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
       <c r="E33" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -35255,16 +35247,16 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>7</v>
+      <c r="A34" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="8">
         <v>2.0</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="8">
         <v>100.0</v>
       </c>
-      <c r="D34" s="13"/>
+      <c r="D34" s="14"/>
       <c r="E34" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -35279,16 +35271,16 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>14</v>
+      <c r="A35" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="8">
         <v>20.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
+      <c r="D35" s="14"/>
       <c r="E35" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -35303,11 +35295,11 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35319,11 +35311,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51111,19 +51103,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51135,13 +51127,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51152,19 +51144,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="11">
         <v>60.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="11">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51175,11 +51167,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="9"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51190,14 +51182,14 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
+      <c r="A5" s="5" t="s">
+        <v>14</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
+      <c r="B5" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
       <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -51209,16 +51201,16 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>14</v>
+      <c r="A6" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>60.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
       <c r="E6" s="12">
@@ -51234,11 +51226,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="9"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51249,13 +51241,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="9"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51266,16 +51258,16 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="8">
         <v>10.0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <v>45.0</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="8">
         <v>1.0</v>
       </c>
       <c r="E9" s="12">
@@ -51291,16 +51283,16 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>14</v>
+      <c r="A10" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="8">
         <v>11.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <v>20.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="8">
         <v>1.0</v>
       </c>
       <c r="E10" s="12">
@@ -51316,11 +51308,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="22"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51331,14 +51323,14 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>19</v>
+      <c r="B12" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
       <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
@@ -51350,16 +51342,16 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>20</v>
+      <c r="A13" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>5.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>60.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
       <c r="E13" s="12">
@@ -51375,16 +51367,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>30.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
       <c r="E14" s="12"/>
@@ -51398,22 +51390,22 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="8">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="8">
         <v>4.0</v>
       </c>
       <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="4"/>
@@ -51425,16 +51417,16 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>14</v>
+      <c r="A16" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="8">
         <v>12.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>20.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="8">
         <v>1.0</v>
       </c>
       <c r="E16" s="12">
@@ -51450,11 +51442,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51465,13 +51457,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>12</v>
+      <c r="A18" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51482,16 +51474,16 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>7</v>
+      <c r="A19" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="11">
         <v>6.0</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="11">
         <v>45.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
       <c r="E19" s="12">
@@ -51507,16 +51499,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>9</v>
+      <c r="A20" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="11">
         <v>18.0</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="11">
         <v>20.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="12">
@@ -51532,11 +51524,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51547,14 +51539,14 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="s">
-        <v>12</v>
+      <c r="A22" s="24" t="s">
+        <v>10</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>19</v>
+      <c r="B22" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
@@ -51568,16 +51560,16 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>20</v>
+      <c r="A23" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="11">
         <v>6.0</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="11">
         <v>50.0</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="8">
         <v>1.0</v>
       </c>
       <c r="E23" s="12">
@@ -51593,16 +51585,16 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
+      <c r="A24" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="11">
         <v>8.0</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="11">
         <v>30.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="8">
         <v>1.0</v>
       </c>
       <c r="E24" s="12">
@@ -51618,22 +51610,22 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>14</v>
+      <c r="A25" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="11">
         <v>10.0</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="11">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="8">
         <v>4.0</v>
       </c>
       <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="18" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="4"/>
@@ -51645,16 +51637,16 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>14</v>
+      <c r="A26" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="11">
         <v>17.0</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="11">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
       <c r="E26" s="12">
@@ -51670,11 +51662,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51685,15 +51677,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="24" t="s">
-        <v>19</v>
+      <c r="B28" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51704,16 +51696,16 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>20</v>
+      <c r="A29" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="11">
         <v>6.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="11">
         <v>50.0</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="8">
         <v>1.0</v>
       </c>
       <c r="E29" s="12">
@@ -51729,19 +51721,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>7</v>
+      <c r="A30" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="11">
         <v>8.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="11">
         <v>30.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51752,16 +51744,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>9</v>
+      <c r="A31" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="11">
         <v>15.0</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="11">
         <v>10.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="8">
         <v>2.0</v>
       </c>
       <c r="E31" s="12">
@@ -51777,11 +51769,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="9"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="10"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51792,13 +51784,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="13" t="s">
         <v>18</v>
       </c>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
       <c r="D33" s="15"/>
-      <c r="E33" s="27"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51810,7 +51802,7 @@
     </row>
     <row r="34">
       <c r="A34" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B34" s="35" t="s">
         <v>27</v>
@@ -51821,7 +51813,7 @@
       <c r="D34" s="35">
         <v>1.0</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="20">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51835,7 +51827,7 @@
     </row>
     <row r="35">
       <c r="A35" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" s="35">
         <v>30.0</v>
@@ -51846,7 +51838,7 @@
       <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51857,11 +51849,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="20"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="9"/>
+      <c r="A36" s="21"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="10"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51872,13 +51864,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="s">
-        <v>28</v>
+      <c r="A37" s="5" t="s">
+        <v>29</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="9"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="10"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51889,16 +51881,16 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
-        <v>9</v>
+      <c r="A38" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>40.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>15.0</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="8">
         <v>1.0</v>
       </c>
       <c r="E38" s="12">
@@ -51914,11 +51906,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="6"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="9"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51929,13 +51921,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="9"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="10"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51946,16 +51938,16 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>7</v>
+      <c r="A41" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="8">
         <v>9.0</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="8">
         <v>20.0</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="8">
         <v>1.0</v>
       </c>
       <c r="E41" s="12">
@@ -51971,16 +51963,16 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
-        <v>9</v>
+      <c r="A42" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="8">
         <v>55.0</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="8">
         <v>20.0</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="8">
         <v>1.0</v>
       </c>
       <c r="E42" s="12">
@@ -51996,23 +51988,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>7</v>
+      <c r="A43" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="8">
         <v>10.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="8">
         <v>250.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="8">
         <v>1.0</v>
       </c>
       <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="19" t="s">
-        <v>29</v>
+      <c r="F43" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52023,11 +52015,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="37"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="9"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="10"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52038,13 +52030,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="37" t="s">
+      <c r="A45" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="9"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="10"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52055,16 +52047,16 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
-        <v>9</v>
+      <c r="A46" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="8">
         <v>60.0</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="8">
         <v>10.0</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="8">
         <v>1.0</v>
       </c>
       <c r="E46" s="12">
@@ -52080,11 +52072,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="37"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="9"/>
+      <c r="A47" s="42"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52095,13 +52087,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="37" t="s">
+      <c r="A48" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="9"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="10"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52112,16 +52104,16 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>13</v>
+      <c r="A49" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B49" s="7">
+      <c r="B49" s="11">
         <v>70.0</v>
       </c>
-      <c r="C49" s="7">
+      <c r="C49" s="11">
         <v>300.0</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="11">
         <v>1.0</v>
       </c>
       <c r="E49" s="12">
@@ -52137,16 +52129,16 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>7</v>
+      <c r="A50" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B50" s="11">
         <v>10.0</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C50" s="11">
         <v>20.0</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="11">
         <v>1.0</v>
       </c>
       <c r="E50" s="12">
@@ -52162,16 +52154,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
-        <v>9</v>
+      <c r="A51" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B51" s="7">
+      <c r="B51" s="11">
         <v>70.0</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51" s="11">
         <v>10.0</v>
       </c>
-      <c r="D51" s="7">
+      <c r="D51" s="11">
         <v>1.0</v>
       </c>
       <c r="E51" s="12">
@@ -52187,11 +52179,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="9"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="10"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52202,14 +52194,14 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
       <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
@@ -52223,14 +52215,14 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="5">
+      <c r="A54" s="7">
         <v>50.0</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="8">
         <v>100.0</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
       <c r="E54" s="12">
         <v>45946.87887299768</v>
       </c>
@@ -52261,16 +52253,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="s">
+      <c r="A56" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="41">
+      <c r="B56" s="40">
         <v>100.0</v>
       </c>
-      <c r="C56" s="19">
+      <c r="C56" s="18">
         <v>1.0</v>
       </c>
-      <c r="D56" s="19">
+      <c r="D56" s="18">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52286,8 +52278,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="42"/>
-      <c r="B57" s="42"/>
+      <c r="A57" s="41"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52301,10 +52293,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52318,16 +52310,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
-        <v>9</v>
+      <c r="A59" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B59" s="41">
+      <c r="B59" s="40">
         <v>50.0</v>
       </c>
-      <c r="C59" s="19">
+      <c r="C59" s="18">
         <v>20.0</v>
       </c>
-      <c r="D59" s="19">
+      <c r="D59" s="18">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52343,13 +52335,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="41" t="s">
+      <c r="A60" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="41">
+      <c r="B60" s="40">
         <v>15.0</v>
       </c>
-      <c r="C60" s="19">
+      <c r="C60" s="18">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52366,8 +52358,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="42"/>
-      <c r="B61" s="42"/>
+      <c r="A61" s="41"/>
+      <c r="B61" s="41"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52381,10 +52373,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="41" t="s">
+      <c r="B62" s="40" t="s">
         <v>24</v>
       </c>
       <c r="C62" s="4"/>
@@ -52402,16 +52394,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="41">
+      <c r="B63" s="40">
         <v>5.0</v>
       </c>
-      <c r="C63" s="19">
+      <c r="C63" s="18">
         <v>80.0</v>
       </c>
-      <c r="D63" s="19">
+      <c r="D63" s="18">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52427,16 +52419,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="41">
+      <c r="B64" s="40">
         <v>15.0</v>
       </c>
-      <c r="C64" s="19">
+      <c r="C64" s="18">
         <v>10.0</v>
       </c>
-      <c r="D64" s="19">
+      <c r="D64" s="18">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52452,16 +52444,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="41" t="s">
-        <v>14</v>
+      <c r="A65" s="40" t="s">
+        <v>16</v>
       </c>
-      <c r="B65" s="41">
+      <c r="B65" s="40">
         <v>30.0</v>
       </c>
-      <c r="C65" s="19">
+      <c r="C65" s="18">
         <v>10.0</v>
       </c>
-      <c r="D65" s="19">
+      <c r="D65" s="18">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52477,8 +52469,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="42"/>
-      <c r="B66" s="42"/>
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52492,10 +52484,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="41" t="s">
+      <c r="B67" s="40" t="s">
         <v>32</v>
       </c>
       <c r="C67" s="4"/>
@@ -52513,16 +52505,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="40">
         <v>5.0</v>
       </c>
-      <c r="C68" s="19">
+      <c r="C68" s="18">
         <v>80.0</v>
       </c>
-      <c r="D68" s="19">
+      <c r="D68" s="18">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52536,16 +52528,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="40">
         <v>15.0</v>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="18">
         <v>10.0</v>
       </c>
-      <c r="D69" s="19">
+      <c r="D69" s="18">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52559,16 +52551,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="41" t="s">
-        <v>14</v>
+      <c r="A70" s="40" t="s">
+        <v>16</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="40">
         <v>20.0</v>
       </c>
-      <c r="C70" s="19">
+      <c r="C70" s="18">
         <v>10.0</v>
       </c>
-      <c r="D70" s="19">
+      <c r="D70" s="18">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52584,8 +52576,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="42"/>
-      <c r="B71" s="42"/>
+      <c r="A71" s="41"/>
+      <c r="B71" s="41"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52599,8 +52591,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="42"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52614,8 +52606,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="42"/>
-      <c r="B73" s="42"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-25T08:59:28.446Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,6 +19,9 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
   </si>
   <si>
@@ -28,34 +31,25 @@
     <t>次數</t>
   </si>
   <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>最後更新日期</t>
+  </si>
+  <si>
+    <t>Line</t>
   </si>
   <si>
     <t>0.3mm</t>
   </si>
   <si>
-    <t>Line</t>
-  </si>
-  <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>刀壓</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
+    <t>(PS)</t>
   </si>
   <si>
     <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>(PS)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -64,25 +58,31 @@
     <t>03mm</t>
   </si>
   <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
     <t>Cut</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>1mm</t>
+    <t>Fill</t>
   </si>
   <si>
-    <t>Fill</t>
+    <t>1mm</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
-    <t>cut</t>
+    <t>2mm</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
@@ -94,19 +94,19 @@
     <t>4mm</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
     <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
     <t>1.5mm</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -206,14 +206,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,35 +321,38 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -360,16 +363,16 @@
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -378,38 +381,23 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -421,14 +409,26 @@
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>8</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="6"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>10</v>
+      <c r="A6" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>12</v>
+      <c r="B6" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="s">
-        <v>6</v>
+      <c r="A7" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="20">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="s">
-        <v>8</v>
+      <c r="A8" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="20">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -858,10 +858,10 @@
     </row>
     <row r="9">
       <c r="A9" s="21"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="9"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>18</v>
+      <c r="A10" s="6" t="s">
+        <v>19</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
+      <c r="A11" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>8</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -966,10 +966,10 @@
     </row>
     <row r="14">
       <c r="A14" s="21"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="6"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>22</v>
+      <c r="A15" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="s">
-        <v>6</v>
+      <c r="A16" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="s">
-        <v>8</v>
+      <c r="A17" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="18">
       <c r="A18" s="21"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="6"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>6</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>8</v>
+      <c r="A21" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1124,10 +1124,10 @@
     </row>
     <row r="22">
       <c r="A22" s="21"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="6"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="s">
-        <v>6</v>
+      <c r="A24" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1190,8 +1190,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="37"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>14</v>
+      <c r="A27" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>26</v>
+      <c r="B27" s="10" t="s">
+        <v>28</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="34">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>6</v>
+      <c r="A28" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="34">
+      <c r="D28" s="13"/>
+      <c r="E28" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>16</v>
+      <c r="A29" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="34">
+      <c r="D29" s="13"/>
+      <c r="E29" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>8</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>13</v>
+      <c r="A5" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>6</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>8</v>
+      <c r="A7" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,11 +17261,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="12"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>10</v>
+      <c r="A9" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="19"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17297,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
-        <v>6</v>
+      <c r="A10" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="19">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="s">
-        <v>8</v>
+      <c r="A11" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="19">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="s">
-        <v>19</v>
+      <c r="A12" s="18" t="s">
+        <v>18</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="19">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="s">
-        <v>13</v>
+      <c r="A13" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17397,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="s">
-        <v>6</v>
+      <c r="A14" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17422,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="s">
-        <v>8</v>
+      <c r="A15" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="25"/>
+      <c r="E16" s="8"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>18</v>
+      <c r="A17" s="6" t="s">
+        <v>19</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>13</v>
+      <c r="B17" s="26" t="s">
+        <v>10</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="8"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>8</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17533,10 +17533,10 @@
     </row>
     <row r="20">
       <c r="A20" s="21"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="10"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>22</v>
+      <c r="A21" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17568,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="s">
-        <v>6</v>
+      <c r="A22" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17593,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
-        <v>8</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="22"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17619,10 +17619,10 @@
     </row>
     <row r="24">
       <c r="A24" s="21"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="10"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="10"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>8</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17707,10 +17707,10 @@
     </row>
     <row r="28">
       <c r="A28" s="21"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="10"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="22"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17742,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="s">
-        <v>6</v>
+      <c r="A30" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="22"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17768,7 +17768,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17779,7 +17779,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="36"/>
+      <c r="E31" s="32"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
-        <v>28</v>
+      <c r="A33" s="33" t="s">
+        <v>26</v>
       </c>
-      <c r="B33" s="38">
+      <c r="B33" s="34">
         <v>5.0</v>
       </c>
-      <c r="C33" s="38">
+      <c r="C33" s="34">
         <v>10.0</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="34">
         <v>2.0</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="36">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="40" t="s">
-        <v>30</v>
+      <c r="F33" s="38" t="s">
+        <v>27</v>
       </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="39"/>
+      <c r="K33" s="39"/>
+      <c r="L33" s="39"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="39"/>
+      <c r="O33" s="39"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>14</v>
+      <c r="A36" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>26</v>
+      <c r="B36" s="10" t="s">
+        <v>28</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>6</v>
+      <c r="A37" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
-      <c r="D37" s="14"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>16</v>
+      <c r="A38" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
-      <c r="D38" s="14"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,19 +34630,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>8</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>20.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="12">
         <v>46147.893450902775</v>
       </c>
       <c r="F4" s="4"/>
@@ -34656,19 +34656,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="10">
         <v>2.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="12">
         <v>46182.71399388889</v>
       </c>
       <c r="F5" s="4"/>
@@ -34682,11 +34682,11 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="9"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,15 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>10</v>
+      <c r="A7" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>12</v>
+      <c r="B7" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34718,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="s">
-        <v>6</v>
+      <c r="A8" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>4.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>10.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="20">
         <v>45957.92965825232</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34744,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="s">
-        <v>8</v>
+      <c r="A9" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <v>20.0</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="20">
         <v>46116.685309016204</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34771,10 +34771,10 @@
     </row>
     <row r="10">
       <c r="A10" s="21"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -34786,10 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>10</v>
+      <c r="A11" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="E11" s="6"/>
+      <c r="E11" s="9"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34801,13 +34801,13 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34819,19 +34819,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>8</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>20.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>10.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="12">
         <v>46228.70790929398</v>
       </c>
       <c r="F13" s="4"/>
@@ -34845,13 +34845,13 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34864,10 +34864,10 @@
     </row>
     <row r="15">
       <c r="A15" s="21"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34879,13 +34879,13 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>18</v>
+      <c r="A16" s="6" t="s">
+        <v>19</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34897,23 +34897,23 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>6</v>
+      <c r="A17" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="10">
         <v>5.0</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="10">
         <v>5.0</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="10">
         <v>1.0</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34923,19 +34923,19 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>15.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -34947,19 +34947,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>8</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>32.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34972,10 +34972,10 @@
     </row>
     <row r="20">
       <c r="A20" s="21"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="6"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34987,13 +34987,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>22</v>
+      <c r="A21" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="16"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35005,19 +35005,19 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="s">
-        <v>6</v>
+      <c r="A22" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>5.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>5.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="16"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35029,19 +35029,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
-        <v>8</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>50.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="16"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35054,10 +35054,10 @@
     </row>
     <row r="24">
       <c r="A24" s="21"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="6"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35069,13 +35069,13 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="6"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35087,19 +35087,19 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>5.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>5.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35111,13 +35111,13 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>8</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="6"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35130,10 +35130,10 @@
     </row>
     <row r="28">
       <c r="A28" s="21"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="6"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35145,13 +35145,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="16"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="17"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35163,19 +35163,19 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="s">
-        <v>6</v>
+      <c r="A30" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>5.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="16"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35188,7 +35188,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" s="31">
         <v>55.0</v>
@@ -35196,8 +35196,8 @@
       <c r="C31" s="31">
         <v>2.0</v>
       </c>
-      <c r="D31" s="32"/>
-      <c r="E31" s="33"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="37"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35209,11 +35209,11 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="14"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35225,15 +35225,15 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>14</v>
+      <c r="A33" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>26</v>
+      <c r="B33" s="10" t="s">
+        <v>28</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="34">
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F33" s="4"/>
@@ -35247,17 +35247,17 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>6</v>
+      <c r="A34" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="10">
         <v>2.0</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C34" s="10">
         <v>100.0</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="34">
+      <c r="D34" s="13"/>
+      <c r="E34" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F34" s="4"/>
@@ -35271,17 +35271,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
-        <v>16</v>
+      <c r="A35" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="10">
         <v>20.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="34">
+      <c r="D35" s="13"/>
+      <c r="E35" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F35" s="4"/>
@@ -35295,11 +35295,11 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="14"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35311,11 +35311,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51103,19 +51103,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51127,13 +51127,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>6</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="10"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51144,19 +51144,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>8</v>
+      <c r="A3" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="7">
         <v>60.0</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="7">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="8"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51167,11 +51167,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="10"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51182,15 +51182,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>15</v>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51201,19 +51201,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>16</v>
+      <c r="A6" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51226,11 +51226,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="10"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="8"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51241,13 +51241,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="8"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51258,19 +51258,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>6</v>
+      <c r="A9" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="11">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51283,19 +51283,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>16</v>
+      <c r="A10" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="11">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51308,11 +51308,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="24"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51323,15 +51323,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51342,19 +51342,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>19</v>
+      <c r="A13" s="5" t="s">
+        <v>18</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="11">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51367,19 +51367,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>6</v>
+      <c r="A14" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51390,22 +51390,22 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>21</v>
+      <c r="A15" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="4"/>
@@ -51417,19 +51417,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>16</v>
+      <c r="A16" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="11">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51442,11 +51442,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51457,13 +51457,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>10</v>
+      <c r="A18" s="6" t="s">
+        <v>14</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="10"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51474,19 +51474,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="7">
         <v>6.0</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="7">
         <v>45.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="11">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51499,19 +51499,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>8</v>
+      <c r="A20" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="7">
         <v>18.0</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="7">
         <v>20.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51524,11 +51524,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="10"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51539,15 +51539,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="s">
-        <v>10</v>
+      <c r="A22" s="27" t="s">
+        <v>14</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="12">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="11">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51560,19 +51560,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>19</v>
+      <c r="A23" s="5" t="s">
+        <v>18</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="7">
         <v>6.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="7">
         <v>50.0</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="11">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51585,19 +51585,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>6</v>
+      <c r="A24" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="7">
         <v>8.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="7">
         <v>30.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="11">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51610,22 +51610,22 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>16</v>
+      <c r="A25" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="7">
         <v>10.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="7">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="4"/>
@@ -51637,19 +51637,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>16</v>
+      <c r="A26" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="7">
         <v>17.0</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="7">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="11">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51662,11 +51662,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="10"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="8"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51677,15 +51677,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="s">
-        <v>18</v>
+      <c r="A28" s="27" t="s">
+        <v>19</v>
       </c>
-      <c r="B28" s="25" t="s">
+      <c r="B28" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="10"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51696,19 +51696,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>19</v>
+      <c r="A29" s="5" t="s">
+        <v>18</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="7">
         <v>6.0</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="7">
         <v>50.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="11">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51721,19 +51721,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>6</v>
+      <c r="A30" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="7">
         <v>8.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="7">
         <v>30.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="10"/>
+      <c r="E30" s="8"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51744,19 +51744,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>8</v>
+      <c r="A31" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="7">
         <v>15.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="7">
         <v>10.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="11">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51769,11 +51769,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="10"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="8"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51784,13 +51784,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="s">
-        <v>18</v>
+      <c r="A33" s="15" t="s">
+        <v>19</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="26"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="22"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51801,19 +51801,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="s">
-        <v>6</v>
+      <c r="A34" s="18" t="s">
+        <v>7</v>
       </c>
-      <c r="B34" s="35" t="s">
-        <v>27</v>
+      <c r="B34" s="41" t="s">
+        <v>29</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="41">
         <v>40.0</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="19">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51826,19 +51826,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="s">
-        <v>8</v>
+      <c r="A35" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B35" s="35">
+      <c r="B35" s="41">
         <v>30.0</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="41">
         <v>15.0</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="22"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51850,10 +51850,10 @@
     </row>
     <row r="36">
       <c r="A36" s="21"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="10"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="8"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51864,13 +51864,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>29</v>
+      <c r="A37" s="6" t="s">
+        <v>30</v>
       </c>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="10"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="8"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51881,19 +51881,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>8</v>
+      <c r="A38" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="11">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51906,11 +51906,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="10"/>
+      <c r="A39" s="6"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="8"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51921,13 +51921,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>22</v>
+      <c r="A40" s="6" t="s">
+        <v>21</v>
       </c>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="10"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="8"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51938,19 +51938,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>6</v>
+      <c r="A41" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="11">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51963,19 +51963,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>8</v>
+      <c r="A42" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="11">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -51988,22 +51988,22 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>6</v>
+      <c r="A43" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="18" t="s">
+      <c r="F43" s="14" t="s">
         <v>31</v>
       </c>
       <c r="G43" s="4"/>
@@ -52016,10 +52016,10 @@
     </row>
     <row r="44">
       <c r="A44" s="42"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="10"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="8"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52033,10 +52033,10 @@
       <c r="A45" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="10"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="8"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52047,19 +52047,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>8</v>
+      <c r="A46" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
-      <c r="E46" s="12">
+      <c r="E46" s="11">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52073,10 +52073,10 @@
     </row>
     <row r="47">
       <c r="A47" s="42"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="10"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="8"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52090,10 +52090,10 @@
       <c r="A48" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="10"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="8"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52104,19 +52104,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
+      <c r="A49" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="7">
         <v>70.0</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="7">
         <v>300.0</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="7">
         <v>1.0</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="11">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52129,19 +52129,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="s">
-        <v>6</v>
+      <c r="A50" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="7">
         <v>10.0</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="7">
         <v>20.0</v>
       </c>
-      <c r="D50" s="11">
+      <c r="D50" s="7">
         <v>1.0</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="11">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52154,19 +52154,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>8</v>
+      <c r="A51" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="7">
         <v>70.0</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="7">
         <v>10.0</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="7">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="11">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52179,11 +52179,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="10"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="8"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52194,15 +52194,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="12">
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="11">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52215,15 +52215,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="7">
+      <c r="A54" s="5">
         <v>50.0</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="12">
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="11">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52253,16 +52253,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="40" t="s">
+      <c r="A56" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="40">
+      <c r="B56" s="38">
         <v>100.0</v>
       </c>
-      <c r="C56" s="18">
+      <c r="C56" s="14">
         <v>1.0</v>
       </c>
-      <c r="D56" s="18">
+      <c r="D56" s="14">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52278,8 +52278,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="41"/>
-      <c r="B57" s="41"/>
+      <c r="A57" s="39"/>
+      <c r="B57" s="39"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52293,10 +52293,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="40" t="s">
+      <c r="A58" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="41"/>
+      <c r="B58" s="39"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52310,16 +52310,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="s">
-        <v>8</v>
+      <c r="A59" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B59" s="40">
+      <c r="B59" s="38">
         <v>50.0</v>
       </c>
-      <c r="C59" s="18">
+      <c r="C59" s="14">
         <v>20.0</v>
       </c>
-      <c r="D59" s="18">
+      <c r="D59" s="14">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52335,13 +52335,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="s">
+      <c r="A60" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="40">
+      <c r="B60" s="38">
         <v>15.0</v>
       </c>
-      <c r="C60" s="18">
+      <c r="C60" s="14">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52358,8 +52358,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="41"/>
-      <c r="B61" s="41"/>
+      <c r="A61" s="39"/>
+      <c r="B61" s="39"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52373,10 +52373,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
+      <c r="A62" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="B62" s="40" t="s">
+      <c r="B62" s="38" t="s">
         <v>24</v>
       </c>
       <c r="C62" s="4"/>
@@ -52394,16 +52394,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="s">
+      <c r="A63" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="40">
+      <c r="B63" s="38">
         <v>5.0</v>
       </c>
-      <c r="C63" s="18">
+      <c r="C63" s="14">
         <v>80.0</v>
       </c>
-      <c r="D63" s="18">
+      <c r="D63" s="14">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52419,16 +52419,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
+      <c r="A64" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="40">
+      <c r="B64" s="38">
         <v>15.0</v>
       </c>
-      <c r="C64" s="18">
+      <c r="C64" s="14">
         <v>10.0</v>
       </c>
-      <c r="D64" s="18">
+      <c r="D64" s="14">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52444,16 +52444,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="40" t="s">
-        <v>16</v>
+      <c r="A65" s="38" t="s">
+        <v>15</v>
       </c>
-      <c r="B65" s="40">
+      <c r="B65" s="38">
         <v>30.0</v>
       </c>
-      <c r="C65" s="18">
+      <c r="C65" s="14">
         <v>10.0</v>
       </c>
-      <c r="D65" s="18">
+      <c r="D65" s="14">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52469,8 +52469,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="41"/>
-      <c r="B66" s="41"/>
+      <c r="A66" s="39"/>
+      <c r="B66" s="39"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52484,10 +52484,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40" t="s">
+      <c r="A67" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="40" t="s">
+      <c r="B67" s="38" t="s">
         <v>32</v>
       </c>
       <c r="C67" s="4"/>
@@ -52505,16 +52505,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="40">
+      <c r="B68" s="38">
         <v>5.0</v>
       </c>
-      <c r="C68" s="18">
+      <c r="C68" s="14">
         <v>80.0</v>
       </c>
-      <c r="D68" s="18">
+      <c r="D68" s="14">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52528,16 +52528,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
+      <c r="A69" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="40">
+      <c r="B69" s="38">
         <v>15.0</v>
       </c>
-      <c r="C69" s="18">
+      <c r="C69" s="14">
         <v>10.0</v>
       </c>
-      <c r="D69" s="18">
+      <c r="D69" s="14">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52551,16 +52551,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
-        <v>16</v>
+      <c r="A70" s="38" t="s">
+        <v>15</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="38">
         <v>20.0</v>
       </c>
-      <c r="C70" s="18">
+      <c r="C70" s="14">
         <v>10.0</v>
       </c>
-      <c r="D70" s="18">
+      <c r="D70" s="14">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52576,8 +52576,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="41"/>
-      <c r="B71" s="41"/>
+      <c r="A71" s="39"/>
+      <c r="B71" s="39"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52591,8 +52591,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="41"/>
+      <c r="A72" s="38"/>
+      <c r="B72" s="39"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52606,8 +52606,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="41"/>
-      <c r="B73" s="41"/>
+      <c r="A73" s="39"/>
+      <c r="B73" s="39"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-29T13:59:55.537Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,9 +19,6 @@
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
   </si>
   <si>
@@ -31,25 +28,31 @@
     <t>次數</t>
   </si>
   <si>
-    <t>刀壓</t>
+    <t>最後更新日期</t>
   </si>
   <si>
-    <t>最後更新日期</t>
+    <t>0.3mm</t>
   </si>
   <si>
     <t>Line</t>
   </si>
   <si>
-    <t>0.3mm</t>
-  </si>
-  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>FILL</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -58,28 +61,25 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>(PS -3)</t>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>1mm</t>
   </si>
   <si>
     <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>1mm</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
     <t>2mm</t>
+  </si>
+  <si>
+    <t>Fill</t>
   </si>
   <si>
     <t>cut</t>
@@ -92,12 +92,6 @@
   </si>
   <si>
     <t>4mm</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>(0.9 Power)</t>
@@ -141,6 +135,12 @@
   <si>
     <t>刻線</t>
   </si>
+  <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
+  </si>
 </sst>
 </file>
 
@@ -178,14 +178,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -206,14 +206,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,34 +321,28 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -357,22 +351,22 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -381,17 +375,19 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -400,37 +396,23 @@
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -442,7 +424,25 @@
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -682,16 +682,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -704,10 +704,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -719,19 +719,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -745,19 +745,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -769,11 +769,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -785,15 +785,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>14</v>
+      <c r="A6" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>16</v>
+      <c r="B6" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +805,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
-        <v>7</v>
+      <c r="A7" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="14">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="14">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <v>1.0</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="18">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +831,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
-        <v>9</v>
+      <c r="A8" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="14">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="14">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <v>1.0</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="18">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,11 +857,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="21"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="12"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="9"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -873,13 +873,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>19</v>
+      <c r="A10" s="5" t="s">
+        <v>17</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="12"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -891,23 +891,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
+      <c r="A11" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -917,19 +917,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>7</v>
+      <c r="A12" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -941,19 +941,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="9"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -965,11 +965,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="21"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="9"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -981,13 +981,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>21</v>
+      <c r="A15" s="13" t="s">
+        <v>20</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +999,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
-        <v>7</v>
+      <c r="A16" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="14">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="14">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="14">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1023,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="s">
-        <v>9</v>
+      <c r="A17" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="14">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="14">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="14">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,11 +1047,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="21"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1063,13 +1063,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="9"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1081,19 +1081,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>7</v>
+      <c r="A20" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="9"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1105,13 +1105,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
-        <v>9</v>
+      <c r="A21" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1123,11 +1123,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="21"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="9"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1139,13 +1139,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1157,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
-        <v>7</v>
+      <c r="A24" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="14">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="14">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="14">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1181,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="s">
-        <v>9</v>
+      <c r="A25" s="28" t="s">
+        <v>7</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="29">
         <v>55.0</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="29">
         <v>2.0</v>
       </c>
-      <c r="D25" s="35"/>
-      <c r="E25" s="37"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="31"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1203,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1219,15 +1219,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>12</v>
+      <c r="A27" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>28</v>
+      <c r="B27" s="8" t="s">
+        <v>26</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="40">
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="33">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1241,17 +1241,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>7</v>
+      <c r="A28" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="40">
+      <c r="D28" s="15"/>
+      <c r="E28" s="33">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1265,17 +1265,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="40">
+      <c r="D29" s="15"/>
+      <c r="E29" s="33">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1289,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1305,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="15"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17101,16 +17101,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17124,10 +17124,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17140,19 +17140,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17167,19 +17167,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17192,13 +17192,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>10</v>
+      <c r="A5" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17211,22 +17211,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17236,22 +17236,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
+      <c r="A7" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17261,11 +17261,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17278,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
-        <v>14</v>
+      <c r="A9" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="19"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="26"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17297,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
-        <v>7</v>
+      <c r="A10" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="14">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="14">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>1.0</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="26">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17324,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="s">
-        <v>9</v>
+      <c r="A11" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="14">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="14">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="14">
         <v>1.0</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="26">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17351,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>18</v>
+      <c r="A12" s="17" t="s">
+        <v>21</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="14">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="14">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="14">
         <v>1.0</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="26">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17378,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>10</v>
+      <c r="A13" s="17" t="s">
+        <v>16</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="22"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="27"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17397,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
-        <v>7</v>
+      <c r="A14" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="14">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="14">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="14">
         <v>1.0</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17422,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
-        <v>9</v>
+      <c r="A15" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="14">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="14">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="14">
         <v>1.0</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17447,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="25"/>
-      <c r="E16" s="8"/>
+      <c r="A16" s="32"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17461,15 +17461,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>19</v>
+      <c r="A17" s="5" t="s">
+        <v>17</v>
       </c>
-      <c r="B17" s="26" t="s">
-        <v>10</v>
+      <c r="B17" s="34" t="s">
+        <v>16</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17482,19 +17482,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17507,19 +17507,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17532,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="21"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17549,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>21</v>
+      <c r="A21" s="13" t="s">
+        <v>20</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="22"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17568,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
-        <v>7</v>
+      <c r="A22" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="14">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="14">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="14">
         <v>1.0</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17593,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
-        <v>9</v>
+      <c r="A23" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="14">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="14">
         <v>2.0</v>
       </c>
-      <c r="E23" s="22"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17618,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="21"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17635,13 +17635,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="8"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17654,19 +17654,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>7</v>
+      <c r="A26" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17679,19 +17679,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="8">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17706,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="21"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17723,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="22"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17742,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
-        <v>7</v>
+      <c r="A30" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="14">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="14">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="14">
         <v>1.0</v>
       </c>
-      <c r="E30" s="22"/>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,19 +17767,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
-        <v>9</v>
+      <c r="A31" s="28" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="29">
         <v>70.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="29">
         <v>5.0</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="29">
         <v>1.0</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="43"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17809,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="33" t="s">
-        <v>26</v>
+      <c r="A33" s="44" t="s">
+        <v>40</v>
       </c>
-      <c r="B33" s="34">
+      <c r="B33" s="45">
         <v>5.0</v>
       </c>
-      <c r="C33" s="34">
+      <c r="C33" s="45">
         <v>10.0</v>
       </c>
-      <c r="D33" s="34">
+      <c r="D33" s="45">
         <v>2.0</v>
       </c>
-      <c r="E33" s="36">
+      <c r="E33" s="46">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="38" t="s">
-        <v>27</v>
+      <c r="F33" s="40" t="s">
+        <v>41</v>
       </c>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
-      <c r="K33" s="39"/>
-      <c r="L33" s="39"/>
-      <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
-      <c r="O33" s="39"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17872,14 +17872,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>12</v>
+      <c r="A36" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>28</v>
+      <c r="B36" s="8" t="s">
+        <v>26</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17893,16 +17893,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>7</v>
+      <c r="A37" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="8">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="15"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17916,16 +17916,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="15"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,16 +34567,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34589,10 +34589,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
+      <c r="A2" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34604,19 +34604,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34630,21 +34630,11 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="10">
-        <v>20.0</v>
-      </c>
-      <c r="C4" s="10">
-        <v>20.0</v>
-      </c>
-      <c r="D4" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E4" s="12">
-        <v>46147.893450902775</v>
-      </c>
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -34656,20 +34646,20 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>11</v>
+      <c r="A5" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B5" s="10">
-        <v>2.0</v>
-      </c>
-      <c r="C5" s="10">
+      <c r="B5" s="8">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="C5" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D5" s="8">
         <v>1.0</v>
       </c>
-      <c r="E5" s="12">
-        <v>46182.71399388889</v>
+      <c r="E5" s="9">
+        <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -34682,11 +34672,21 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="9"/>
+      <c r="A6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="C6" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D6" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E6" s="9">
+        <v>46182.71399388889</v>
+      </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -34698,15 +34698,11 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="17"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34718,23 +34714,17 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
-        <v>7</v>
+      <c r="A8" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B8" s="16">
-        <v>4.0</v>
+      <c r="B8" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="C8" s="16">
-        <v>10.0</v>
-      </c>
-      <c r="D8" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E8" s="20">
-        <v>45957.92965825232</v>
-      </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -34744,23 +34734,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
-        <v>9</v>
+      <c r="A9" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B9" s="16">
-        <v>20.0</v>
+      <c r="B9" s="14">
+        <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="14">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <v>1.0</v>
       </c>
-      <c r="E9" s="20">
-        <v>46116.685309016204</v>
+      <c r="E9" s="18">
+        <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34770,13 +34760,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="21"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
+      <c r="A10" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="C10" s="14">
+        <v>10.0</v>
+      </c>
+      <c r="D10" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="E10" s="18">
+        <v>46116.685309016204</v>
+      </c>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34786,9 +34786,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="A11" s="20"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
       <c r="E11" s="9"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34802,12 +34803,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="12"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34819,21 +34817,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B13" s="10">
-        <v>20.0</v>
-      </c>
-      <c r="C13" s="10">
-        <v>10.0</v>
-      </c>
-      <c r="D13" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E13" s="12">
-        <v>46228.70790929398</v>
-      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34845,13 +34835,21 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>11</v>
+      <c r="A14" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="12"/>
+      <c r="B14" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="C14" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E14" s="9">
+        <v>46228.70790929398</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -34863,11 +34861,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="21"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="12"/>
+      <c r="A15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34879,13 +34879,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="12"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34898,22 +34896,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
-      <c r="B17" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="C17" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="D17" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E17" s="12">
-        <v>46042.0</v>
-      </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -34923,21 +34913,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
-        <v>15.0</v>
+      <c r="C18" s="8">
+        <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
+      <c r="E18" s="9">
+        <v>46042.0</v>
+      </c>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34947,19 +34939,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B19" s="10">
-        <v>32.0</v>
-      </c>
-      <c r="C19" s="10">
+      <c r="B19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="C19" s="8">
+        <v>15.0</v>
+      </c>
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34971,11 +34963,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="21"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="A20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="8">
+        <v>32.0</v>
+      </c>
+      <c r="C20" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="D20" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -34987,13 +34987,11 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="17"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35005,19 +35003,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
-        <v>7</v>
+      <c r="A22" s="13" t="s">
+        <v>20</v>
       </c>
-      <c r="B22" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="C22" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="D22" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E22" s="17"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35029,19 +35021,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
-        <v>9</v>
+      <c r="A23" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B23" s="16">
-        <v>50.0</v>
-      </c>
-      <c r="C23" s="16">
+      <c r="B23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="C23" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="D23" s="14">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35053,11 +35045,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="21"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="A24" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="14">
+        <v>50.0</v>
+      </c>
+      <c r="C24" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="D24" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35069,13 +35069,11 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35088,18 +35086,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
-      <c r="B26" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="C26" s="10">
-        <v>5.0</v>
-      </c>
-      <c r="D26" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="9"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35111,13 +35103,19 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="B27" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="C27" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="D27" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35129,11 +35127,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="21"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="A28" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35145,13 +35145,11 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="17"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35163,19 +35161,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
-        <v>7</v>
+      <c r="A30" s="13" t="s">
+        <v>25</v>
       </c>
-      <c r="B30" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="C30" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="D30" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E30" s="17"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35187,17 +35179,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
-        <v>9</v>
+      <c r="A31" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B31" s="31">
-        <v>55.0</v>
+      <c r="B31" s="14">
+        <v>5.0</v>
       </c>
-      <c r="C31" s="31">
-        <v>2.0</v>
+      <c r="C31" s="14">
+        <v>5.0</v>
       </c>
-      <c r="D31" s="35"/>
-      <c r="E31" s="37"/>
+      <c r="D31" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="E31" s="16"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35209,11 +35203,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="A32" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="29">
+        <v>55.0</v>
+      </c>
+      <c r="C32" s="29">
+        <v>2.0</v>
+      </c>
+      <c r="D32" s="30"/>
+      <c r="E32" s="31"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35225,17 +35225,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="40">
-        <v>46051.96156388889</v>
-      </c>
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35247,18 +35241,16 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>7</v>
+      <c r="A34" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B34" s="10">
-        <v>2.0</v>
+      <c r="B34" s="8" t="s">
+        <v>26</v>
       </c>
-      <c r="C34" s="10">
-        <v>100.0</v>
-      </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="40">
-        <v>46100.83597384259</v>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="33">
+        <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -35271,18 +35263,18 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>15</v>
+      <c r="A35" s="8" t="s">
+        <v>6</v>
       </c>
-      <c r="B35" s="10">
-        <v>20.0</v>
+      <c r="B35" s="8">
+        <v>2.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="40">
-        <v>46100.83604224537</v>
+      <c r="D35" s="15"/>
+      <c r="E35" s="33">
+        <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -35295,11 +35287,19 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="A36" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="C36" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="33">
+        <v>46100.83604224537</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -35311,11 +35311,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35327,11 +35327,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51085,6 +51085,22 @@
       <c r="L1022" s="4"/>
       <c r="M1022" s="4"/>
       <c r="N1022" s="4"/>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="4"/>
+      <c r="B1023" s="4"/>
+      <c r="C1023" s="4"/>
+      <c r="D1023" s="4"/>
+      <c r="E1023" s="4"/>
+      <c r="F1023" s="4"/>
+      <c r="G1023" s="4"/>
+      <c r="H1023" s="4"/>
+      <c r="I1023" s="4"/>
+      <c r="J1023" s="4"/>
+      <c r="K1023" s="4"/>
+      <c r="L1023" s="4"/>
+      <c r="M1023" s="4"/>
+      <c r="N1023" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -51103,19 +51119,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51127,13 +51143,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="8"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51144,19 +51160,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
+      <c r="A3" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="11">
         <v>60.0</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="11">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51167,11 +51183,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="8"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51182,15 +51198,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="11"/>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51201,19 +51217,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>60.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51226,11 +51242,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="8"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51241,13 +51257,13 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>17</v>
+      <c r="A8" s="5" t="s">
+        <v>18</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51258,19 +51274,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
+      <c r="A9" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="8">
         <v>10.0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <v>45.0</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="8">
         <v>1.0</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51283,19 +51299,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="8">
         <v>11.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <v>20.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51308,11 +51324,11 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="24"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="22"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51323,15 +51339,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="s">
-        <v>17</v>
+      <c r="A12" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="B12" s="28" t="s">
-        <v>20</v>
+      <c r="B12" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51342,19 +51358,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>18</v>
+      <c r="A13" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="8">
         <v>5.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>60.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51367,19 +51383,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>7</v>
+      <c r="A14" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="8">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>30.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51390,22 +51406,22 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="8">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="8">
         <v>4.0</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="19" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="4"/>
@@ -51417,19 +51433,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="8">
         <v>12.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>20.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="8">
         <v>1.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51442,11 +51458,11 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51457,13 +51473,13 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>14</v>
+      <c r="A18" s="5" t="s">
+        <v>11</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="8"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51474,19 +51490,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>7</v>
+      <c r="A19" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="11">
         <v>6.0</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="11">
         <v>45.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51499,19 +51515,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>9</v>
+      <c r="A20" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="11">
         <v>18.0</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="11">
         <v>20.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51524,11 +51540,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="8"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51539,15 +51555,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="s">
-        <v>14</v>
+      <c r="A22" s="23" t="s">
+        <v>11</v>
       </c>
-      <c r="B22" s="28" t="s">
-        <v>20</v>
+      <c r="B22" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="11">
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51560,19 +51576,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>18</v>
+      <c r="A23" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="11">
         <v>6.0</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="11">
         <v>50.0</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="8">
         <v>1.0</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51585,19 +51601,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>7</v>
+      <c r="A24" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="11">
         <v>8.0</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="11">
         <v>30.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51610,22 +51626,22 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="11">
         <v>10.0</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="11">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="8">
         <v>4.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="19" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="4"/>
@@ -51637,19 +51653,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="11">
         <v>17.0</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="11">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51662,11 +51678,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="8"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51677,15 +51693,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51696,19 +51712,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>18</v>
+      <c r="A29" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="11">
         <v>6.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="11">
         <v>50.0</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="8">
         <v>1.0</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51721,19 +51737,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>7</v>
+      <c r="A30" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="11">
         <v>8.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="11">
         <v>30.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="8"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51744,19 +51760,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>9</v>
+      <c r="A31" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="11">
         <v>15.0</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="11">
         <v>10.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="8">
         <v>2.0</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51769,11 +51785,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="8"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="10"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51784,13 +51800,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="s">
-        <v>19</v>
+      <c r="A33" s="13" t="s">
+        <v>17</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="22"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="27"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51801,19 +51817,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="s">
-        <v>7</v>
+      <c r="A34" s="17" t="s">
+        <v>6</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>29</v>
+      <c r="B34" s="35" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="35">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="35">
         <v>1.0</v>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="26">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51826,19 +51842,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="s">
-        <v>9</v>
+      <c r="A35" s="17" t="s">
+        <v>7</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="35">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="35">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="22"/>
+      <c r="E35" s="27"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51849,11 +51865,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="21"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="8"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="10"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51864,13 +51880,13 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="s">
-        <v>30</v>
+      <c r="A37" s="5" t="s">
+        <v>28</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="8"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="10"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51881,19 +51897,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
-        <v>9</v>
+      <c r="A38" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="8">
         <v>40.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <v>15.0</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="8">
         <v>1.0</v>
       </c>
-      <c r="E38" s="11">
+      <c r="E38" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51906,11 +51922,11 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="6"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="8"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51921,13 +51937,13 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="s">
-        <v>21</v>
+      <c r="A40" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="8"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="10"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51938,19 +51954,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>7</v>
+      <c r="A41" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="8">
         <v>9.0</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="8">
         <v>20.0</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="8">
         <v>1.0</v>
       </c>
-      <c r="E41" s="11">
+      <c r="E41" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51963,19 +51979,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
-        <v>9</v>
+      <c r="A42" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="8">
         <v>55.0</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="8">
         <v>20.0</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="8">
         <v>1.0</v>
       </c>
-      <c r="E42" s="11">
+      <c r="E42" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -51988,23 +52004,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>7</v>
+      <c r="A43" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="8">
         <v>10.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="8">
         <v>250.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="14" t="s">
-        <v>31</v>
+      <c r="F43" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52015,11 +52031,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="8"/>
+      <c r="A44" s="36"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="10"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52030,13 +52046,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
+      <c r="A45" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="8"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="10"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52047,19 +52063,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
-        <v>9</v>
+      <c r="A46" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="8">
         <v>60.0</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="8">
         <v>10.0</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="8">
         <v>1.0</v>
       </c>
-      <c r="E46" s="11">
+      <c r="E46" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52072,11 +52088,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="8"/>
+      <c r="A47" s="36"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52087,13 +52103,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
-        <v>32</v>
+      <c r="A48" s="36" t="s">
+        <v>30</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="8"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="10"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52104,19 +52120,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>11</v>
+      <c r="A49" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B49" s="7">
+      <c r="B49" s="11">
         <v>70.0</v>
       </c>
-      <c r="C49" s="7">
+      <c r="C49" s="11">
         <v>300.0</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="11">
         <v>1.0</v>
       </c>
-      <c r="E49" s="11">
+      <c r="E49" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52129,19 +52145,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>7</v>
+      <c r="A50" s="7" t="s">
+        <v>6</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B50" s="11">
         <v>10.0</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C50" s="11">
         <v>20.0</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="11">
         <v>1.0</v>
       </c>
-      <c r="E50" s="11">
+      <c r="E50" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52154,19 +52170,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
-        <v>9</v>
+      <c r="A51" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B51" s="7">
+      <c r="B51" s="11">
         <v>70.0</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51" s="11">
         <v>10.0</v>
       </c>
-      <c r="D51" s="7">
+      <c r="D51" s="11">
         <v>1.0</v>
       </c>
-      <c r="E51" s="11">
+      <c r="E51" s="12">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52179,11 +52195,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="8"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="10"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52194,15 +52210,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
-        <v>33</v>
+      <c r="A53" s="7" t="s">
+        <v>31</v>
       </c>
-      <c r="B53" s="10" t="s">
-        <v>34</v>
+      <c r="B53" s="8" t="s">
+        <v>32</v>
       </c>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="11">
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52215,15 +52231,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="5">
+      <c r="A54" s="7">
         <v>50.0</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="8">
         <v>100.0</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="11">
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52236,13 +52252,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="43" t="s">
-        <v>35</v>
+      <c r="A55" s="37" t="s">
+        <v>33</v>
       </c>
-      <c r="B55" s="44"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="38"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="39"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52253,19 +52269,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="38" t="s">
-        <v>36</v>
+      <c r="A56" s="40" t="s">
+        <v>34</v>
       </c>
-      <c r="B56" s="38">
+      <c r="B56" s="40">
         <v>100.0</v>
       </c>
-      <c r="C56" s="14">
+      <c r="C56" s="19">
         <v>1.0</v>
       </c>
-      <c r="D56" s="14">
+      <c r="D56" s="19">
         <v>2.0</v>
       </c>
-      <c r="E56" s="46">
+      <c r="E56" s="41">
         <v>46009.783484375</v>
       </c>
       <c r="F56" s="4"/>
@@ -52278,8 +52294,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="39"/>
-      <c r="B57" s="39"/>
+      <c r="A57" s="42"/>
+      <c r="B57" s="42"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52293,10 +52309,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="38" t="s">
-        <v>37</v>
+      <c r="A58" s="40" t="s">
+        <v>35</v>
       </c>
-      <c r="B58" s="39"/>
+      <c r="B58" s="42"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52310,19 +52326,19 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
-        <v>9</v>
+      <c r="A59" s="7" t="s">
+        <v>7</v>
       </c>
-      <c r="B59" s="38">
+      <c r="B59" s="40">
         <v>50.0</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="19">
         <v>20.0</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59" s="19">
         <v>1.0</v>
       </c>
-      <c r="E59" s="46">
+      <c r="E59" s="41">
         <v>46038.9559609375</v>
       </c>
       <c r="F59" s="4"/>
@@ -52335,17 +52351,17 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="38" t="s">
-        <v>38</v>
+      <c r="A60" s="40" t="s">
+        <v>36</v>
       </c>
-      <c r="B60" s="38">
+      <c r="B60" s="40">
         <v>15.0</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="19">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="46">
+      <c r="E60" s="41">
         <v>46136.01284993056</v>
       </c>
       <c r="F60" s="4"/>
@@ -52358,8 +52374,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="39"/>
-      <c r="B61" s="39"/>
+      <c r="A61" s="42"/>
+      <c r="B61" s="42"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52373,15 +52389,15 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="38" t="s">
-        <v>39</v>
+      <c r="A62" s="40" t="s">
+        <v>37</v>
       </c>
-      <c r="B62" s="38" t="s">
+      <c r="B62" s="40" t="s">
         <v>24</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="46">
+      <c r="E62" s="41">
         <v>46044.0116671875</v>
       </c>
       <c r="F62" s="4"/>
@@ -52394,19 +52410,19 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="38" t="s">
-        <v>40</v>
+      <c r="A63" s="40" t="s">
+        <v>38</v>
       </c>
-      <c r="B63" s="38">
+      <c r="B63" s="40">
         <v>5.0</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="19">
         <v>80.0</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="19">
         <v>1.0</v>
       </c>
-      <c r="E63" s="46">
+      <c r="E63" s="41">
         <v>46044.01310700232</v>
       </c>
       <c r="F63" s="4"/>
@@ -52419,19 +52435,19 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="38" t="s">
-        <v>41</v>
+      <c r="A64" s="40" t="s">
+        <v>39</v>
       </c>
-      <c r="B64" s="38">
+      <c r="B64" s="40">
         <v>15.0</v>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="19">
         <v>10.0</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64" s="19">
         <v>1.0</v>
       </c>
-      <c r="E64" s="46">
+      <c r="E64" s="41">
         <v>46044.013194907406</v>
       </c>
       <c r="F64" s="4"/>
@@ -52444,19 +52460,19 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="38" t="s">
+      <c r="A65" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B65" s="38">
+      <c r="B65" s="40">
         <v>30.0</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="19">
         <v>10.0</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="19">
         <v>1.0</v>
       </c>
-      <c r="E65" s="46">
+      <c r="E65" s="41">
         <v>46056.701985011576</v>
       </c>
       <c r="F65" s="4"/>
@@ -52469,8 +52485,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="39"/>
-      <c r="B66" s="39"/>
+      <c r="A66" s="42"/>
+      <c r="B66" s="42"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52484,15 +52500,15 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="38" t="s">
-        <v>39</v>
+      <c r="A67" s="40" t="s">
+        <v>37</v>
       </c>
-      <c r="B67" s="38" t="s">
-        <v>32</v>
+      <c r="B67" s="40" t="s">
+        <v>30</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="46">
+      <c r="E67" s="41">
         <v>46044.0136399537</v>
       </c>
       <c r="F67" s="4"/>
@@ -52505,16 +52521,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="38" t="s">
-        <v>40</v>
+      <c r="A68" s="40" t="s">
+        <v>38</v>
       </c>
-      <c r="B68" s="38">
+      <c r="B68" s="40">
         <v>5.0</v>
       </c>
-      <c r="C68" s="14">
+      <c r="C68" s="19">
         <v>80.0</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="19">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52528,16 +52544,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="38" t="s">
-        <v>41</v>
+      <c r="A69" s="40" t="s">
+        <v>39</v>
       </c>
-      <c r="B69" s="38">
+      <c r="B69" s="40">
         <v>15.0</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="19">
         <v>10.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="19">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52551,19 +52567,19 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="38" t="s">
+      <c r="A70" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B70" s="38">
+      <c r="B70" s="40">
         <v>20.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="19">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="19">
         <v>6.0</v>
       </c>
-      <c r="E70" s="46">
+      <c r="E70" s="41">
         <v>46044.014003055556</v>
       </c>
       <c r="F70" s="4"/>
@@ -52576,8 +52592,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="39"/>
-      <c r="B71" s="39"/>
+      <c r="A71" s="42"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52591,8 +52607,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="38"/>
-      <c r="B72" s="39"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="42"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52606,8 +52622,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="39"/>
-      <c r="B73" s="39"/>
+      <c r="A73" s="42"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-29T14:00:02.466Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="43">
   <si>
     <t>項目</t>
   </si>
@@ -40,34 +40,58 @@
     <t>Cut-1/2</t>
   </si>
   <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>2mm</t>
+  </si>
+  <si>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>4mm</t>
+  </si>
+  <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>Cut</t>
+  </si>
+  <si>
     <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>刀壓</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>甲板紙</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>A4紙</t>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>03mm</t>
-  </si>
-  <si>
-    <t>Cut</t>
-  </si>
-  <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>1mm</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -76,25 +100,10 @@
     <t>PS</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
     <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
-  </si>
-  <si>
-    <t>3mm</t>
-  </si>
-  <si>
-    <t>4mm</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
@@ -135,12 +144,6 @@
   <si>
     <t>刻線</t>
   </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
-  </si>
 </sst>
 </file>
 
@@ -178,14 +181,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -206,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -336,23 +339,11 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -369,16 +360,13 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -389,6 +377,10 @@
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -402,17 +394,46 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -424,25 +445,7 @@
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -785,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>11</v>
+      <c r="A6" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>12</v>
+      <c r="B6" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -805,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="11">
         <v>4.0</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="11">
         <v>10.0</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="11">
         <v>1.0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="14">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -831,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="11">
         <v>25.0</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="11">
         <v>5.0</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="11">
         <v>1.0</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="14">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -857,10 +860,10 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
       <c r="E9" s="9"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -874,10 +877,10 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="8"/>
       <c r="E10" s="9"/>
       <c r="F10" s="4"/>
@@ -906,8 +909,8 @@
       <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -965,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -981,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>20</v>
+      <c r="A15" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -999,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="11">
         <v>5.0</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="11">
         <v>5.0</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="11">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1023,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="11">
         <v>50.0</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="11">
         <v>5.0</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="11">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="12"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1047,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1064,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1108,9 +1111,9 @@
       <c r="A21" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1123,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1139,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>25</v>
+      <c r="A23" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="12"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1157,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="11">
         <v>5.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="11">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="11">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="12"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1181,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="26">
         <v>55.0</v>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="26">
         <v>2.0</v>
       </c>
-      <c r="D25" s="30"/>
-      <c r="E25" s="31"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1203,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1220,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="33">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="29">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1250,8 +1253,8 @@
       <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="15"/>
-      <c r="E28" s="33">
+      <c r="D28" s="17"/>
+      <c r="E28" s="29">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1266,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B29" s="8">
         <v>20.0</v>
@@ -1274,8 +1277,8 @@
       <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="15"/>
-      <c r="E29" s="33">
+      <c r="D29" s="17"/>
+      <c r="E29" s="29">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1289,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="15"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
+      <c r="A30" s="17"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1305,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="15"/>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
+      <c r="A31" s="17"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17127,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="18"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17152,7 +17155,7 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="19">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17179,7 +17182,7 @@
       <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="18"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17193,12 +17196,12 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="10"/>
+      <c r="E5" s="18"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17223,10 +17226,10 @@
       <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17248,10 +17251,10 @@
       <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,7 +17268,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
-      <c r="E8" s="12"/>
+      <c r="E8" s="19"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17278,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>11</v>
+      <c r="A9" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="26"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17297,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="11">
         <v>4.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="11">
         <v>15.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <v>1.0</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17324,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="11">
         <v>25.0</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="11">
         <v>10.0</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="11">
         <v>1.0</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17351,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="s">
-        <v>21</v>
+      <c r="A12" s="13" t="s">
+        <v>14</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="11">
         <v>4.0</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="11">
         <v>10.0</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="11">
         <v>1.0</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17378,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="s">
-        <v>16</v>
+      <c r="A13" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="27"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17397,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="11">
         <v>2.0</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="11">
         <v>18.0</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="11">
         <v>1.0</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17422,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="11">
         <v>18.0</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="11">
         <v>4.0</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="11">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17447,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="32"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="23"/>
+      <c r="E16" s="18"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17462,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
-      <c r="B17" s="34" t="s">
-        <v>16</v>
+      <c r="B17" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="10"/>
+      <c r="E17" s="18"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17494,7 +17497,7 @@
       <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="18"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17519,7 +17522,7 @@
       <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="18"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17532,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="10"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="18"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17549,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>20</v>
+      <c r="A21" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="27"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17568,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="11">
         <v>8.0</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="11">
         <v>15.0</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="11">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17593,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="11">
         <v>55.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="11">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="11">
         <v>2.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="22"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17618,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="10"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="18"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17636,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="10"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="18"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17666,7 +17669,7 @@
       <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="18"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17691,7 +17694,7 @@
       <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="19">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17706,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="10"/>
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="18"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17723,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
-        <v>25</v>
+      <c r="A29" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="27"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="22"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17742,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="11">
         <v>18.0</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="11">
         <v>5.0</v>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="11">
         <v>1.0</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="22"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17767,19 +17770,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="29">
+      <c r="B31" s="26">
         <v>70.0</v>
       </c>
-      <c r="C31" s="29">
+      <c r="C31" s="26">
         <v>5.0</v>
       </c>
-      <c r="D31" s="29">
+      <c r="D31" s="26">
         <v>1.0</v>
       </c>
-      <c r="E31" s="43"/>
+      <c r="E31" s="31"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17809,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="44" t="s">
-        <v>40</v>
+      <c r="A33" s="32" t="s">
+        <v>23</v>
       </c>
-      <c r="B33" s="45">
+      <c r="B33" s="33">
         <v>5.0</v>
       </c>
-      <c r="C33" s="45">
+      <c r="C33" s="33">
         <v>10.0</v>
       </c>
-      <c r="D33" s="45">
+      <c r="D33" s="33">
         <v>2.0</v>
       </c>
-      <c r="E33" s="46">
+      <c r="E33" s="34">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="40" t="s">
-        <v>41</v>
+      <c r="F33" s="35" t="s">
+        <v>24</v>
       </c>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="36"/>
+      <c r="J33" s="36"/>
+      <c r="K33" s="36"/>
+      <c r="L33" s="36"/>
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
+      <c r="O33" s="36"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17873,13 +17876,13 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17902,7 +17905,7 @@
       <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="15"/>
+      <c r="D37" s="17"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17917,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B38" s="8">
         <v>20.0</v>
@@ -17925,7 +17928,7 @@
       <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="15"/>
+      <c r="D38" s="17"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34630,7 +34633,9 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7"/>
+      <c r="A4" s="7" t="s">
+        <v>16</v>
+      </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -34673,7 +34678,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B6" s="8">
         <v>2.0</v>
@@ -34714,15 +34719,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>11</v>
+      <c r="A8" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>12</v>
+      <c r="B8" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34734,23 +34739,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="11">
         <v>4.0</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="11">
         <v>10.0</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <v>1.0</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="14">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34760,23 +34765,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="11">
         <v>20.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="11">
         <v>10.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <v>1.0</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="14">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34786,10 +34791,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="8"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
       <c r="E11" s="9"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34803,7 +34808,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34862,7 +34867,7 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -34879,10 +34884,10 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="20"/>
+      <c r="A16" s="16"/>
       <c r="B16" s="8"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
       <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34896,10 +34901,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
       <c r="D17" s="8"/>
       <c r="E17" s="9"/>
       <c r="F17" s="4"/>
@@ -34928,8 +34933,8 @@
       <c r="E18" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34987,10 +34992,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="20"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35003,13 +35008,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>20</v>
+      <c r="A22" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="16"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="12"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35021,19 +35026,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="11">
         <v>5.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="11">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="11">
         <v>1.0</v>
       </c>
-      <c r="E23" s="16"/>
+      <c r="E23" s="12"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35045,19 +35050,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="11">
         <v>50.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="11">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="11">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="12"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35069,10 +35074,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
+      <c r="A25" s="16"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35086,11 +35091,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35130,9 +35135,9 @@
       <c r="A28" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35145,10 +35150,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="20"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35161,13 +35166,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>25</v>
+      <c r="A30" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="16"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="12"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35179,19 +35184,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="11">
         <v>5.0</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="11">
         <v>5.0</v>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="11">
         <v>1.0</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="12"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35203,17 +35208,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="26">
         <v>55.0</v>
       </c>
-      <c r="C32" s="29">
+      <c r="C32" s="26">
         <v>2.0</v>
       </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="31"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="28"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35225,11 +35230,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="15"/>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
+      <c r="A33" s="17"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35242,14 +35247,14 @@
     </row>
     <row r="34">
       <c r="A34" s="8" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="33">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="29">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35272,8 +35277,8 @@
       <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="33">
+      <c r="D35" s="17"/>
+      <c r="E35" s="29">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35288,7 +35293,7 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B36" s="8">
         <v>20.0</v>
@@ -35296,8 +35301,8 @@
       <c r="C36" s="8">
         <v>100.0</v>
       </c>
-      <c r="D36" s="15"/>
-      <c r="E36" s="33">
+      <c r="D36" s="17"/>
+      <c r="E36" s="29">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35311,11 +35316,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="15"/>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
+      <c r="A37" s="17"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35327,11 +35332,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51119,10 +51124,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51146,10 +51151,10 @@
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
       <c r="D2" s="8"/>
-      <c r="E2" s="10"/>
+      <c r="E2" s="18"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51163,16 +51168,16 @@
       <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="30">
         <v>60.0</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="30">
         <v>20.0</v>
       </c>
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51184,10 +51189,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="10"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="18"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51199,14 +51204,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="19"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51218,7 +51223,7 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B6" s="8">
         <v>6.0</v>
@@ -51229,7 +51234,7 @@
       <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="19">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51243,10 +51248,10 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="10"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="18"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51258,12 +51263,12 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
-      <c r="E8" s="10"/>
+      <c r="E8" s="18"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51286,7 +51291,7 @@
       <c r="D9" s="8">
         <v>1.0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="19">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51300,7 +51305,7 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B10" s="8">
         <v>11.0</v>
@@ -51311,7 +51316,7 @@
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="19">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51325,10 +51330,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="22"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="38"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51339,15 +51344,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>18</v>
+      <c r="A12" s="39" t="s">
+        <v>26</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>19</v>
+      <c r="B12" s="40" t="s">
+        <v>27</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
-      <c r="E12" s="12"/>
+      <c r="E12" s="19"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51359,7 +51364,7 @@
     </row>
     <row r="13" ht="20.25" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B13" s="8">
         <v>5.0</v>
@@ -51370,7 +51375,7 @@
       <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="19">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51395,7 +51400,7 @@
       <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51407,7 +51412,7 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B15" s="8">
         <v>5.0</v>
@@ -51418,11 +51423,11 @@
       <c r="D15" s="8">
         <v>4.0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="19">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="19" t="s">
-        <v>23</v>
+      <c r="F15" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51434,7 +51439,7 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B16" s="8">
         <v>12.0</v>
@@ -51445,7 +51450,7 @@
       <c r="D16" s="8">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="19">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51459,10 +51464,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="38"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51474,12 +51479,12 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="10"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="18"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51493,16 +51498,16 @@
       <c r="A19" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="30">
         <v>6.0</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="30">
         <v>45.0</v>
       </c>
       <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="19">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51518,16 +51523,16 @@
       <c r="A20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="30">
         <v>18.0</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="30">
         <v>20.0</v>
       </c>
       <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="19">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51541,10 +51546,10 @@
     </row>
     <row r="21">
       <c r="A21" s="7"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="10"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="18"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51555,15 +51560,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="s">
-        <v>11</v>
+      <c r="A22" s="39" t="s">
+        <v>8</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>19</v>
+      <c r="B22" s="40" t="s">
+        <v>27</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="12">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="19">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51577,18 +51582,18 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="30">
         <v>6.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="30">
         <v>50.0</v>
       </c>
       <c r="D23" s="8">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="19">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51604,16 +51609,16 @@
       <c r="A24" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="30">
         <v>8.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="30">
         <v>30.0</v>
       </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="19">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51627,22 +51632,22 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="30">
         <v>10.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="30">
         <v>30.0</v>
       </c>
       <c r="D25" s="8">
         <v>4.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="19">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="19" t="s">
-        <v>23</v>
+      <c r="F25" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51654,18 +51659,18 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="30">
         <v>17.0</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="30">
         <v>15.0</v>
       </c>
       <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="19">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51679,10 +51684,10 @@
     </row>
     <row r="27">
       <c r="A27" s="7"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="10"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="18"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51693,15 +51698,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="s">
-        <v>17</v>
+      <c r="A28" s="39" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="24" t="s">
-        <v>19</v>
+      <c r="B28" s="40" t="s">
+        <v>27</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="10"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="18"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51713,18 +51718,18 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="30">
         <v>6.0</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="30">
         <v>50.0</v>
       </c>
       <c r="D29" s="8">
         <v>1.0</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="19">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51740,16 +51745,16 @@
       <c r="A30" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="30">
         <v>8.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="30">
         <v>30.0</v>
       </c>
       <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="10"/>
+      <c r="E30" s="18"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51763,16 +51768,16 @@
       <c r="A31" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="30">
         <v>15.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="30">
         <v>10.0</v>
       </c>
       <c r="D31" s="8">
         <v>2.0</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="19">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51786,10 +51791,10 @@
     </row>
     <row r="32">
       <c r="A32" s="7"/>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="10"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51800,13 +51805,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="s">
-        <v>17</v>
+      <c r="A33" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="27"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="22"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51817,19 +51822,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="35" t="s">
-        <v>27</v>
+      <c r="B34" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="41">
         <v>40.0</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51842,19 +51847,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="35">
+      <c r="B35" s="41">
         <v>30.0</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="41">
         <v>15.0</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="22"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51865,11 +51870,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="20"/>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="10"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="18"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51881,12 +51886,12 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="10"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="18"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51909,7 +51914,7 @@
       <c r="D38" s="8">
         <v>1.0</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="19">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51923,10 +51928,10 @@
     </row>
     <row r="39">
       <c r="A39" s="5"/>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="10"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="18"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51938,12 +51943,12 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
-      <c r="B40" s="15"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="10"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="18"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51966,7 +51971,7 @@
       <c r="D41" s="8">
         <v>1.0</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="19">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51991,7 +51996,7 @@
       <c r="D42" s="8">
         <v>1.0</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="19">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -52016,11 +52021,11 @@
       <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="19">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="19" t="s">
-        <v>29</v>
+      <c r="F43" s="15" t="s">
+        <v>32</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52031,11 +52036,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="36"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="10"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="18"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52046,13 +52051,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="36" t="s">
-        <v>25</v>
+      <c r="A45" s="42" t="s">
+        <v>15</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="10"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="18"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52075,7 +52080,7 @@
       <c r="D46" s="8">
         <v>1.0</v>
       </c>
-      <c r="E46" s="12">
+      <c r="E46" s="19">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52088,11 +52093,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="36"/>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="10"/>
+      <c r="A47" s="42"/>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="18"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52103,13 +52108,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="36" t="s">
-        <v>30</v>
+      <c r="A48" s="42" t="s">
+        <v>33</v>
       </c>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="10"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="18"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52121,18 +52126,18 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="30">
         <v>70.0</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="30">
         <v>300.0</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="30">
         <v>1.0</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="19">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52148,16 +52153,16 @@
       <c r="A50" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="30">
         <v>10.0</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="30">
         <v>20.0</v>
       </c>
-      <c r="D50" s="11">
+      <c r="D50" s="30">
         <v>1.0</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="19">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52173,16 +52178,16 @@
       <c r="A51" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="30">
         <v>70.0</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="30">
         <v>10.0</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D51" s="30">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="19">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52199,7 +52204,7 @@
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
       <c r="D52" s="8"/>
-      <c r="E52" s="10"/>
+      <c r="E52" s="18"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52211,14 +52216,14 @@
     </row>
     <row r="53">
       <c r="A53" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C53" s="8"/>
       <c r="D53" s="8"/>
-      <c r="E53" s="12">
+      <c r="E53" s="19">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52237,9 +52242,9 @@
       <c r="B54" s="8">
         <v>100.0</v>
       </c>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="12">
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="19">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52252,13 +52257,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="37" t="s">
-        <v>33</v>
+      <c r="A55" s="43" t="s">
+        <v>36</v>
       </c>
-      <c r="B55" s="38"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52269,19 +52274,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="40" t="s">
-        <v>34</v>
+      <c r="A56" s="35" t="s">
+        <v>37</v>
       </c>
-      <c r="B56" s="40">
+      <c r="B56" s="35">
         <v>100.0</v>
       </c>
-      <c r="C56" s="19">
+      <c r="C56" s="15">
         <v>1.0</v>
       </c>
-      <c r="D56" s="19">
+      <c r="D56" s="15">
         <v>2.0</v>
       </c>
-      <c r="E56" s="41">
+      <c r="E56" s="46">
         <v>46009.783484375</v>
       </c>
       <c r="F56" s="4"/>
@@ -52294,8 +52299,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="42"/>
-      <c r="B57" s="42"/>
+      <c r="A57" s="36"/>
+      <c r="B57" s="36"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52309,10 +52314,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="40" t="s">
-        <v>35</v>
+      <c r="A58" s="35" t="s">
+        <v>38</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="36"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52329,16 +52334,16 @@
       <c r="A59" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B59" s="40">
+      <c r="B59" s="35">
         <v>50.0</v>
       </c>
-      <c r="C59" s="19">
+      <c r="C59" s="15">
         <v>20.0</v>
       </c>
-      <c r="D59" s="19">
+      <c r="D59" s="15">
         <v>1.0</v>
       </c>
-      <c r="E59" s="41">
+      <c r="E59" s="46">
         <v>46038.9559609375</v>
       </c>
       <c r="F59" s="4"/>
@@ -52351,17 +52356,17 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="s">
-        <v>36</v>
+      <c r="A60" s="35" t="s">
+        <v>39</v>
       </c>
-      <c r="B60" s="40">
+      <c r="B60" s="35">
         <v>15.0</v>
       </c>
-      <c r="C60" s="19">
+      <c r="C60" s="15">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="41">
+      <c r="E60" s="46">
         <v>46136.01284993056</v>
       </c>
       <c r="F60" s="4"/>
@@ -52374,8 +52379,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="42"/>
-      <c r="B61" s="42"/>
+      <c r="A61" s="36"/>
+      <c r="B61" s="36"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52389,15 +52394,15 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
-        <v>37</v>
+      <c r="A62" s="35" t="s">
+        <v>40</v>
       </c>
-      <c r="B62" s="40" t="s">
-        <v>24</v>
+      <c r="B62" s="35" t="s">
+        <v>13</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="41">
+      <c r="E62" s="46">
         <v>46044.0116671875</v>
       </c>
       <c r="F62" s="4"/>
@@ -52410,19 +52415,19 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="s">
-        <v>38</v>
+      <c r="A63" s="35" t="s">
+        <v>41</v>
       </c>
-      <c r="B63" s="40">
+      <c r="B63" s="35">
         <v>5.0</v>
       </c>
-      <c r="C63" s="19">
+      <c r="C63" s="15">
         <v>80.0</v>
       </c>
-      <c r="D63" s="19">
+      <c r="D63" s="15">
         <v>1.0</v>
       </c>
-      <c r="E63" s="41">
+      <c r="E63" s="46">
         <v>46044.01310700232</v>
       </c>
       <c r="F63" s="4"/>
@@ -52435,19 +52440,19 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
-        <v>39</v>
+      <c r="A64" s="35" t="s">
+        <v>42</v>
       </c>
-      <c r="B64" s="40">
+      <c r="B64" s="35">
         <v>15.0</v>
       </c>
-      <c r="C64" s="19">
+      <c r="C64" s="15">
         <v>10.0</v>
       </c>
-      <c r="D64" s="19">
+      <c r="D64" s="15">
         <v>1.0</v>
       </c>
-      <c r="E64" s="41">
+      <c r="E64" s="46">
         <v>46044.013194907406</v>
       </c>
       <c r="F64" s="4"/>
@@ -52460,19 +52465,19 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="40" t="s">
-        <v>15</v>
+      <c r="A65" s="35" t="s">
+        <v>20</v>
       </c>
-      <c r="B65" s="40">
+      <c r="B65" s="35">
         <v>30.0</v>
       </c>
-      <c r="C65" s="19">
+      <c r="C65" s="15">
         <v>10.0</v>
       </c>
-      <c r="D65" s="19">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
-      <c r="E65" s="41">
+      <c r="E65" s="46">
         <v>46056.701985011576</v>
       </c>
       <c r="F65" s="4"/>
@@ -52485,8 +52490,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="42"/>
-      <c r="B66" s="42"/>
+      <c r="A66" s="36"/>
+      <c r="B66" s="36"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52500,15 +52505,15 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40" t="s">
-        <v>37</v>
+      <c r="A67" s="35" t="s">
+        <v>40</v>
       </c>
-      <c r="B67" s="40" t="s">
-        <v>30</v>
+      <c r="B67" s="35" t="s">
+        <v>33</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="41">
+      <c r="E67" s="46">
         <v>46044.0136399537</v>
       </c>
       <c r="F67" s="4"/>
@@ -52521,16 +52526,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
-        <v>38</v>
+      <c r="A68" s="35" t="s">
+        <v>41</v>
       </c>
-      <c r="B68" s="40">
+      <c r="B68" s="35">
         <v>5.0</v>
       </c>
-      <c r="C68" s="19">
+      <c r="C68" s="15">
         <v>80.0</v>
       </c>
-      <c r="D68" s="19">
+      <c r="D68" s="15">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52544,16 +52549,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
-        <v>39</v>
+      <c r="A69" s="35" t="s">
+        <v>42</v>
       </c>
-      <c r="B69" s="40">
+      <c r="B69" s="35">
         <v>15.0</v>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="15">
         <v>10.0</v>
       </c>
-      <c r="D69" s="19">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52567,19 +52572,19 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
-        <v>15</v>
+      <c r="A70" s="35" t="s">
+        <v>20</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="35">
         <v>20.0</v>
       </c>
-      <c r="C70" s="19">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="19">
+      <c r="D70" s="15">
         <v>6.0</v>
       </c>
-      <c r="E70" s="41">
+      <c r="E70" s="46">
         <v>46044.014003055556</v>
       </c>
       <c r="F70" s="4"/>
@@ -52592,8 +52597,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="42"/>
-      <c r="B71" s="42"/>
+      <c r="A71" s="36"/>
+      <c r="B71" s="36"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52607,8 +52612,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="42"/>
+      <c r="A72" s="35"/>
+      <c r="B72" s="36"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52622,8 +52627,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="42"/>
-      <c r="B73" s="42"/>
+      <c r="A73" s="36"/>
+      <c r="B73" s="36"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-29T14:00:04.766Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -31,7 +31,13 @@
     <t>最後更新日期</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>0.3mm</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>Line</t>
@@ -40,16 +46,46 @@
     <t>Cut-1/2</t>
   </si>
   <si>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>03mm</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>Cut</t>
+  </si>
+  <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
+  </si>
+  <si>
     <t>0.5mm</t>
+  </si>
+  <si>
+    <t>FILL</t>
   </si>
   <si>
     <t>(PS -3)</t>
   </si>
   <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
     <t>1mm</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>2mm</t>
@@ -58,52 +94,7 @@
     <t>3mm</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
     <t>4mm</t>
-  </si>
-  <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>A4紙</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>Cut</t>
-  </si>
-  <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
-    <t>刀壓</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>03mm</t>
-  </si>
-  <si>
-    <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>Keep Detail</t>
   </si>
   <si>
     <t>６</t>
@@ -112,7 +103,16 @@
     <t>1.5mm</t>
   </si>
   <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
     <t>吉翁號刻線參數</t>
+  </si>
+  <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>5mm</t>
@@ -181,14 +181,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,13 +330,28 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -351,41 +366,44 @@
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -397,44 +415,26 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -708,7 +708,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -722,19 +722,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +748,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>8</v>
+      <c r="A6" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>9</v>
+      <c r="B6" s="16" t="s">
+        <v>18</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
-        <v>6</v>
+      <c r="A7" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>7</v>
+      <c r="A8" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="22">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="16"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>6</v>
+      <c r="A11" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,16 +920,16 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>6</v>
+      <c r="A12" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -944,16 +944,16 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>7</v>
+      <c r="A13" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="16"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>12</v>
+      <c r="A15" s="15" t="s">
+        <v>24</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="12"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>6</v>
+      <c r="A16" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="s">
-        <v>7</v>
+      <c r="A17" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1084,16 +1084,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>6</v>
+      <c r="A20" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1108,12 +1108,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>7</v>
+      <c r="A21" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>15</v>
+      <c r="A23" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="12"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>6</v>
+      <c r="A24" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="s">
-        <v>7</v>
+      <c r="A25" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="26">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="27"/>
-      <c r="E25" s="28"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>18</v>
+      <c r="A27" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>19</v>
+      <c r="B27" s="10" t="s">
+        <v>29</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="29">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>6</v>
+      <c r="A28" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="29">
+      <c r="D28" s="13"/>
+      <c r="E28" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>20</v>
+      <c r="A29" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="29">
+      <c r="D29" s="13"/>
+      <c r="E29" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17128,9 +17128,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
-      <c r="E2" s="18"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,19 +17143,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,19 +17170,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
+      <c r="A4" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="18"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
+      <c r="A5" s="8" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="18"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>6</v>
+      <c r="A6" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>7</v>
+      <c r="A7" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="19"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,12 +17281,12 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
-        <v>8</v>
+      <c r="A9" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
       <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -17300,16 +17300,16 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>6</v>
+      <c r="A10" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
       <c r="E10" s="21">
@@ -17327,16 +17327,16 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="s">
-        <v>7</v>
+      <c r="A11" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
       <c r="E11" s="21">
@@ -17354,16 +17354,16 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="s">
-        <v>14</v>
+      <c r="A12" s="18" t="s">
+        <v>20</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
       <c r="E12" s="21">
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="s">
-        <v>11</v>
+      <c r="A13" s="18" t="s">
+        <v>12</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="22"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="s">
-        <v>6</v>
+      <c r="A14" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>7</v>
+      <c r="A15" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="23"/>
-      <c r="E16" s="18"/>
+      <c r="A16" s="27"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="24" t="s">
-        <v>11</v>
+      <c r="B17" s="29" t="s">
+        <v>12</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="18"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17485,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="18"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17510,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>7</v>
+      <c r="A19" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="18"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>12</v>
+      <c r="A21" s="15" t="s">
+        <v>24</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="22"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>6</v>
+      <c r="A22" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>7</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="22"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="18"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="18"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,19 +17657,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>6</v>
+      <c r="A26" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="18"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,19 +17682,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>7</v>
+      <c r="A27" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="18"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>15</v>
+      <c r="A29" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="22"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>6</v>
+      <c r="A30" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="22"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17770,19 +17770,19 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="s">
-        <v>7</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="26">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="26">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="31"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="32" t="s">
-        <v>23</v>
+      <c r="A33" s="38" t="s">
+        <v>31</v>
       </c>
-      <c r="B33" s="33">
+      <c r="B33" s="39">
         <v>5.0</v>
       </c>
-      <c r="C33" s="33">
+      <c r="C33" s="39">
         <v>10.0</v>
       </c>
-      <c r="D33" s="33">
+      <c r="D33" s="39">
         <v>2.0</v>
       </c>
-      <c r="E33" s="34">
+      <c r="E33" s="40">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="35" t="s">
-        <v>24</v>
+      <c r="F33" s="41" t="s">
+        <v>32</v>
       </c>
-      <c r="G33" s="36"/>
-      <c r="H33" s="36"/>
-      <c r="I33" s="36"/>
-      <c r="J33" s="36"/>
-      <c r="K33" s="36"/>
-      <c r="L33" s="36"/>
-      <c r="M33" s="36"/>
-      <c r="N33" s="36"/>
-      <c r="O33" s="36"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>18</v>
+      <c r="A36" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>19</v>
+      <c r="B36" s="10" t="s">
+        <v>29</v>
       </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>6</v>
+      <c r="A37" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
-      <c r="D37" s="17"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>20</v>
+      <c r="A38" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
-      <c r="D38" s="17"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -34607,19 +34607,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>6</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34633,13 +34633,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>16</v>
+      <c r="A4" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
+      <c r="B4" s="10">
+        <v>10.0</v>
+      </c>
+      <c r="C4" s="10">
+        <v>10.0</v>
+      </c>
+      <c r="D4" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -34651,19 +34657,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>7</v>
+      <c r="A5" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="10">
         <v>20.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34677,19 +34683,19 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>20.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34704,9 +34710,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34719,15 +34725,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
-        <v>8</v>
+      <c r="A8" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>9</v>
+      <c r="B8" s="16" t="s">
+        <v>18</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="12"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34739,23 +34745,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>6</v>
+      <c r="A9" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="16">
         <v>4.0</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34765,23 +34771,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>7</v>
+      <c r="A10" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="16">
         <v>20.0</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="16">
         <v>10.0</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="22">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34791,11 +34797,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="16"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="9"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34808,7 +34814,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34822,13 +34828,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>6</v>
+      <c r="A13" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34840,19 +34846,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>7</v>
+      <c r="A14" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>20.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="10">
         <v>10.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="11">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34866,13 +34872,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34884,11 +34890,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="16"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="9"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34901,12 +34907,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34918,23 +34924,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>6</v>
+      <c r="A18" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34944,16 +34950,16 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="10">
         <v>5.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="10">
         <v>15.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34968,16 +34974,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
+      <c r="A20" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="10">
         <v>32.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -34992,10 +34998,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="16"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35008,13 +35014,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="s">
-        <v>12</v>
+      <c r="A22" s="15" t="s">
+        <v>24</v>
       </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="12"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35026,19 +35032,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>6</v>
+      <c r="A23" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="16">
         <v>5.0</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35050,19 +35056,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="s">
-        <v>7</v>
+      <c r="A24" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="16">
         <v>50.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35074,10 +35080,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35091,11 +35097,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35108,16 +35114,16 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>6</v>
+      <c r="A27" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="10">
         <v>5.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="10">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35132,12 +35138,12 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>7</v>
+      <c r="A28" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35150,10 +35156,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="16"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35166,13 +35172,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="s">
-        <v>15</v>
+      <c r="A30" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="12"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35184,19 +35190,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="s">
-        <v>6</v>
+      <c r="A31" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="16">
         <v>5.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="16">
         <v>5.0</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="16">
         <v>1.0</v>
       </c>
-      <c r="E31" s="12"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35208,17 +35214,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="s">
-        <v>7</v>
+      <c r="A32" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="31">
         <v>55.0</v>
       </c>
-      <c r="C32" s="26">
+      <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="28"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="34"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35230,11 +35236,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="17"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35246,15 +35252,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>18</v>
+      <c r="A34" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>19</v>
+      <c r="B34" s="10" t="s">
+        <v>29</v>
       </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="29">
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35268,17 +35274,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
-        <v>6</v>
+      <c r="A35" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="10">
         <v>2.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
-      <c r="D35" s="17"/>
-      <c r="E35" s="29">
+      <c r="D35" s="13"/>
+      <c r="E35" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35292,17 +35298,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>20</v>
+      <c r="A36" s="10" t="s">
+        <v>13</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="10">
         <v>20.0</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36" s="10">
         <v>100.0</v>
       </c>
-      <c r="D36" s="17"/>
-      <c r="E36" s="29">
+      <c r="D36" s="13"/>
+      <c r="E36" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35316,11 +35322,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35332,11 +35338,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51124,10 +51130,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51148,13 +51154,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>6</v>
+      <c r="A2" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51165,19 +51171,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
+      <c r="A3" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="30">
+      <c r="B3" s="9">
         <v>60.0</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="18"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51189,10 +51195,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51204,14 +51210,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="19"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51222,19 +51228,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>20</v>
+      <c r="A6" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="10">
         <v>60.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="12">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51248,10 +51254,10 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="18"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51263,12 +51269,12 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="18"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51279,19 +51285,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>6</v>
+      <c r="A9" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="10">
         <v>10.0</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="10">
         <v>45.0</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="10">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51304,19 +51310,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>20</v>
+      <c r="A10" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="10">
         <v>20.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51330,10 +51336,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="20"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51344,15 +51350,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="s">
-        <v>26</v>
+      <c r="A12" s="23" t="s">
+        <v>15</v>
       </c>
-      <c r="B12" s="40" t="s">
-        <v>27</v>
+      <c r="B12" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="19"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51363,19 +51369,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>14</v>
+      <c r="A13" s="8" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="10">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51388,19 +51394,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>6</v>
+      <c r="A14" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="10">
         <v>30.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="19"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51411,23 +51417,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>28</v>
+      <c r="A15" s="8" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="10">
         <v>4.0</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>29</v>
+      <c r="F15" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51438,19 +51444,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>20</v>
+      <c r="A16" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="10">
         <v>12.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="10">
         <v>20.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="10">
         <v>1.0</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51464,10 +51470,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="38"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="20"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51479,12 +51485,12 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51495,19 +51501,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>6</v>
+      <c r="A19" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="30">
+      <c r="B19" s="9">
         <v>6.0</v>
       </c>
-      <c r="C19" s="30">
+      <c r="C19" s="9">
         <v>45.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51520,19 +51526,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>7</v>
+      <c r="A20" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="30">
+      <c r="B20" s="9">
         <v>18.0</v>
       </c>
-      <c r="C20" s="30">
+      <c r="C20" s="9">
         <v>20.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51545,11 +51551,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="18"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51560,15 +51566,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="39" t="s">
-        <v>8</v>
+      <c r="A22" s="23" t="s">
+        <v>16</v>
       </c>
-      <c r="B22" s="40" t="s">
-        <v>27</v>
+      <c r="B22" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="19">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51581,19 +51587,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>14</v>
+      <c r="A23" s="8" t="s">
+        <v>20</v>
       </c>
-      <c r="B23" s="30">
+      <c r="B23" s="9">
         <v>6.0</v>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="9">
         <v>50.0</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="10">
         <v>1.0</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51606,19 +51612,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>6</v>
+      <c r="A24" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="9">
         <v>8.0</v>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="9">
         <v>30.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51631,23 +51637,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>20</v>
+      <c r="A25" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B25" s="30">
+      <c r="B25" s="9">
         <v>10.0</v>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="9">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="10">
         <v>4.0</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>29</v>
+      <c r="F25" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51658,19 +51664,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>20</v>
+      <c r="A26" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B26" s="30">
+      <c r="B26" s="9">
         <v>17.0</v>
       </c>
-      <c r="C26" s="30">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51683,11 +51689,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51698,15 +51704,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="39" t="s">
-        <v>10</v>
+      <c r="A28" s="23" t="s">
+        <v>21</v>
       </c>
-      <c r="B28" s="40" t="s">
-        <v>27</v>
+      <c r="B28" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="18"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51717,19 +51723,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>14</v>
+      <c r="A29" s="8" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="30">
+      <c r="B29" s="9">
         <v>6.0</v>
       </c>
-      <c r="C29" s="30">
+      <c r="C29" s="9">
         <v>50.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="10">
         <v>1.0</v>
       </c>
-      <c r="E29" s="19">
+      <c r="E29" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51742,19 +51748,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>6</v>
+      <c r="A30" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="30">
+      <c r="B30" s="9">
         <v>8.0</v>
       </c>
-      <c r="C30" s="30">
+      <c r="C30" s="9">
         <v>30.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="18"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51765,19 +51771,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>7</v>
+      <c r="A31" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="30">
+      <c r="B31" s="9">
         <v>15.0</v>
       </c>
-      <c r="C31" s="30">
+      <c r="C31" s="9">
         <v>10.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="10">
         <v>2.0</v>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51790,11 +51796,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="18"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51805,13 +51811,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>10</v>
+      <c r="A33" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="22"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51822,16 +51828,16 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="s">
-        <v>6</v>
+      <c r="A34" s="18" t="s">
+        <v>8</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>30</v>
+      <c r="B34" s="32" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="32">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="32">
         <v>1.0</v>
       </c>
       <c r="E34" s="21">
@@ -51847,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="s">
-        <v>7</v>
+      <c r="A35" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="32">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="32">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="32">
         <v>1.0</v>
       </c>
-      <c r="E35" s="22"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51870,11 +51876,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="16"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="18"/>
+      <c r="A36" s="25"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51886,12 +51892,12 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="18"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51902,19 +51908,19 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>7</v>
+      <c r="A38" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="10">
         <v>40.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="10">
         <v>15.0</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="10">
         <v>1.0</v>
       </c>
-      <c r="E38" s="19">
+      <c r="E38" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51928,10 +51934,10 @@
     </row>
     <row r="39">
       <c r="A39" s="5"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="18"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51943,12 +51949,12 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="18"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51959,19 +51965,19 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="s">
-        <v>6</v>
+      <c r="A41" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="10">
         <v>9.0</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="10">
         <v>20.0</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="10">
         <v>1.0</v>
       </c>
-      <c r="E41" s="19">
+      <c r="E41" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51984,19 +51990,19 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>7</v>
+      <c r="A42" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="10">
         <v>55.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="10">
         <v>20.0</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="10">
         <v>1.0</v>
       </c>
-      <c r="E42" s="19">
+      <c r="E42" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -52009,23 +52015,23 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>6</v>
+      <c r="A43" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="10">
         <v>10.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="10">
         <v>250.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
-      <c r="E43" s="19">
+      <c r="E43" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="15" t="s">
-        <v>32</v>
+      <c r="F43" s="14" t="s">
+        <v>30</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52036,11 +52042,11 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="18"/>
+      <c r="A44" s="37"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -52051,13 +52057,13 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>15</v>
+      <c r="A45" s="37" t="s">
+        <v>26</v>
       </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="18"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52068,19 +52074,19 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="s">
-        <v>7</v>
+      <c r="A46" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="10">
         <v>60.0</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="10">
         <v>10.0</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="10">
         <v>1.0</v>
       </c>
-      <c r="E46" s="19">
+      <c r="E46" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52093,11 +52099,11 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="18"/>
+      <c r="A47" s="37"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52108,13 +52114,13 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
+      <c r="A48" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="18"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52125,19 +52131,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
+      <c r="A49" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B49" s="30">
+      <c r="B49" s="9">
         <v>70.0</v>
       </c>
-      <c r="C49" s="30">
+      <c r="C49" s="9">
         <v>300.0</v>
       </c>
-      <c r="D49" s="30">
+      <c r="D49" s="9">
         <v>1.0</v>
       </c>
-      <c r="E49" s="19">
+      <c r="E49" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52150,19 +52156,19 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="s">
-        <v>6</v>
+      <c r="A50" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B50" s="30">
+      <c r="B50" s="9">
         <v>10.0</v>
       </c>
-      <c r="C50" s="30">
+      <c r="C50" s="9">
         <v>20.0</v>
       </c>
-      <c r="D50" s="30">
+      <c r="D50" s="9">
         <v>1.0</v>
       </c>
-      <c r="E50" s="19">
+      <c r="E50" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52175,19 +52181,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>7</v>
+      <c r="A51" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B51" s="30">
+      <c r="B51" s="9">
         <v>70.0</v>
       </c>
-      <c r="C51" s="30">
+      <c r="C51" s="9">
         <v>10.0</v>
       </c>
-      <c r="D51" s="30">
+      <c r="D51" s="9">
         <v>1.0</v>
       </c>
-      <c r="E51" s="19">
+      <c r="E51" s="12">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52200,11 +52206,11 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="18"/>
+      <c r="A52" s="8"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="7"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52215,15 +52221,15 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="19">
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52236,15 +52242,15 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="7">
+      <c r="A54" s="8">
         <v>50.0</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="10">
         <v>100.0</v>
       </c>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="19">
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52274,16 +52280,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="35" t="s">
+      <c r="A56" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B56" s="35">
+      <c r="B56" s="41">
         <v>100.0</v>
       </c>
-      <c r="C56" s="15">
+      <c r="C56" s="14">
         <v>1.0</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="14">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52299,8 +52305,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="36"/>
-      <c r="B57" s="36"/>
+      <c r="A57" s="42"/>
+      <c r="B57" s="42"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52314,10 +52320,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="35" t="s">
+      <c r="A58" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="B58" s="36"/>
+      <c r="B58" s="42"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52331,16 +52337,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="s">
-        <v>7</v>
+      <c r="A59" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B59" s="35">
+      <c r="B59" s="41">
         <v>50.0</v>
       </c>
-      <c r="C59" s="15">
+      <c r="C59" s="14">
         <v>20.0</v>
       </c>
-      <c r="D59" s="15">
+      <c r="D59" s="14">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52356,13 +52362,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="35" t="s">
+      <c r="A60" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="35">
+      <c r="B60" s="41">
         <v>15.0</v>
       </c>
-      <c r="C60" s="15">
+      <c r="C60" s="14">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52379,8 +52385,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="36"/>
-      <c r="B61" s="36"/>
+      <c r="A61" s="42"/>
+      <c r="B61" s="42"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52394,11 +52400,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="35" t="s">
+      <c r="A62" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B62" s="35" t="s">
-        <v>13</v>
+      <c r="B62" s="41" t="s">
+        <v>25</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -52415,16 +52421,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="35" t="s">
+      <c r="A63" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B63" s="35">
+      <c r="B63" s="41">
         <v>5.0</v>
       </c>
-      <c r="C63" s="15">
+      <c r="C63" s="14">
         <v>80.0</v>
       </c>
-      <c r="D63" s="15">
+      <c r="D63" s="14">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52440,16 +52446,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="35" t="s">
+      <c r="A64" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B64" s="35">
+      <c r="B64" s="41">
         <v>15.0</v>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="14">
         <v>10.0</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="14">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52465,16 +52471,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="35" t="s">
-        <v>20</v>
+      <c r="A65" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B65" s="35">
+      <c r="B65" s="41">
         <v>30.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="14">
         <v>10.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="14">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52490,8 +52496,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="36"/>
-      <c r="B66" s="36"/>
+      <c r="A66" s="42"/>
+      <c r="B66" s="42"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52505,10 +52511,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="35" t="s">
+      <c r="A67" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B67" s="35" t="s">
+      <c r="B67" s="41" t="s">
         <v>33</v>
       </c>
       <c r="C67" s="4"/>
@@ -52526,16 +52532,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="35" t="s">
+      <c r="A68" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B68" s="35">
+      <c r="B68" s="41">
         <v>5.0</v>
       </c>
-      <c r="C68" s="15">
+      <c r="C68" s="14">
         <v>80.0</v>
       </c>
-      <c r="D68" s="15">
+      <c r="D68" s="14">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52549,16 +52555,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="35" t="s">
+      <c r="A69" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B69" s="35">
+      <c r="B69" s="41">
         <v>15.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="14">
         <v>10.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="14">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52572,16 +52578,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="35" t="s">
-        <v>20</v>
+      <c r="A70" s="41" t="s">
+        <v>13</v>
       </c>
-      <c r="B70" s="35">
+      <c r="B70" s="41">
         <v>20.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="14">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="14">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52597,8 +52603,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="36"/>
-      <c r="B71" s="36"/>
+      <c r="A71" s="42"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52612,8 +52618,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="35"/>
-      <c r="B72" s="36"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="42"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52627,8 +52633,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="36"/>
-      <c r="B73" s="36"/>
+      <c r="A73" s="42"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-29T14:00:07.131Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -31,19 +31,31 @@
     <t>最後更新日期</t>
   </si>
   <si>
+    <t>0.3mm</t>
+  </si>
+  <si>
     <t>遮蓋膠紙</t>
   </si>
   <si>
-    <t>0.3mm</t>
+    <t>Line</t>
   </si>
   <si>
     <t>刀壓</t>
   </si>
   <si>
-    <t>Line</t>
+    <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut-1/2</t>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -52,34 +64,25 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
     <t>0.3 mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
+    <t>1mm</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
+    <t>Fill</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>1mm</t>
+    <t>2mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -88,13 +91,13 @@
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
     <t>3mm</t>
   </si>
   <si>
     <t>4mm</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
@@ -103,16 +106,13 @@
     <t>1.5mm</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>吉翁號刻線參數</t>
-  </si>
-  <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
+    <t>吉翁號刻線參數</t>
   </si>
   <si>
     <t>5mm</t>
@@ -181,14 +181,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14.0"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -336,9 +336,6 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -348,10 +345,7 @@
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -363,7 +357,22 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -372,28 +381,19 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -401,9 +401,6 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -415,26 +412,29 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -708,7 +708,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -723,18 +723,18 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -751,16 +751,16 @@
       <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>16</v>
+      <c r="A6" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>18</v>
+      <c r="B6" s="14" t="s">
+        <v>13</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -809,22 +809,22 @@
     </row>
     <row r="7">
       <c r="A7" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="14">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="14">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <v>1.0</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -837,20 +837,20 @@
       <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="14">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="14">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <v>1.0</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="25"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -895,22 +895,22 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -921,15 +921,15 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -947,13 +947,13 @@
       <c r="A13" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>24</v>
+      <c r="A15" s="13" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="15"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1003,18 +1003,18 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="14">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="14">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="14">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="15"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1029,16 +1029,16 @@
       <c r="A17" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="14">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="14">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="14">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="15"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="25"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1069,9 +1069,9 @@
       <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1085,15 +1085,15 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1111,9 +1111,9 @@
       <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1161,18 +1161,18 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="14">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="14">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="14">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1193,8 +1193,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="33"/>
-      <c r="E25" s="34"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>10</v>
+      <c r="A27" s="9" t="s">
+        <v>14</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>29</v>
+      <c r="B27" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="35">
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>8</v>
+      <c r="A28" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="35">
+      <c r="D28" s="16"/>
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>13</v>
+      <c r="A29" s="9" t="s">
+        <v>17</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="35">
+      <c r="D29" s="16"/>
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17128,7 +17128,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="4"/>
@@ -17144,18 +17144,18 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17173,13 +17173,13 @@
       <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
       <c r="E4" s="7"/>
@@ -17196,11 +17196,11 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -17215,21 +17215,21 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17242,19 +17242,19 @@
       <c r="A7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,12 +17281,12 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
-        <v>16</v>
+      <c r="A9" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
       <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -17301,15 +17301,15 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="14">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="14">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>1.0</v>
       </c>
       <c r="E10" s="21">
@@ -17330,13 +17330,13 @@
       <c r="A11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="14">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="14">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="14">
         <v>1.0</v>
       </c>
       <c r="E11" s="21">
@@ -17357,13 +17357,13 @@
       <c r="A12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="14">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="14">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="14">
         <v>1.0</v>
       </c>
       <c r="E12" s="21">
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17401,18 +17401,18 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="14">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="14">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="14">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="25"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17428,16 +17428,16 @@
       <c r="A15" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="14">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="14">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="14">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="25"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,7 +17450,7 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
+      <c r="A16" s="28"/>
       <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -17465,13 +17465,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
       <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -17486,15 +17486,15 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
       <c r="E18" s="7"/>
@@ -17513,13 +17513,13 @@
       <c r="A19" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
       <c r="E19" s="7"/>
@@ -17535,10 +17535,10 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
       <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>24</v>
+      <c r="A21" s="13" t="s">
+        <v>22</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17572,18 +17572,18 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="14">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="14">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="14">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17599,16 +17599,16 @@
       <c r="A23" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="14">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="14">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,10 +17621,10 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
       <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -17641,9 +17641,9 @@
       <c r="A25" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
       <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -17658,15 +17658,15 @@
     </row>
     <row r="26">
       <c r="A26" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
       <c r="E26" s="7"/>
@@ -17685,16 +17685,16 @@
       <c r="A27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,10 +17709,10 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17746,18 +17746,18 @@
     </row>
     <row r="30">
       <c r="A30" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="14">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="14">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="14">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="38" t="s">
+      <c r="A33" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="38">
+        <v>5.0</v>
+      </c>
+      <c r="C33" s="38">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="38">
+        <v>2.0</v>
+      </c>
+      <c r="E33" s="39">
+        <v>46043.55545597222</v>
+      </c>
+      <c r="F33" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="39">
-        <v>5.0</v>
-      </c>
-      <c r="C33" s="39">
-        <v>10.0</v>
-      </c>
-      <c r="D33" s="39">
-        <v>2.0</v>
-      </c>
-      <c r="E33" s="40">
-        <v>46043.55545597222</v>
-      </c>
-      <c r="F33" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>10</v>
+      <c r="A36" s="9" t="s">
+        <v>14</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>29</v>
+      <c r="B36" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>8</v>
+      <c r="A37" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="16"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>13</v>
+      <c r="A38" s="9" t="s">
+        <v>17</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="16"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -34608,18 +34608,18 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34634,18 +34634,20 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>10.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="10">
+        <v>46232.916719409724</v>
+      </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -34660,16 +34662,16 @@
       <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>20.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34684,18 +34686,18 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>20.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34710,9 +34712,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34725,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="s">
-        <v>16</v>
+      <c r="A8" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>18</v>
+      <c r="B8" s="14" t="s">
+        <v>13</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34746,22 +34748,22 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="14">
         <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="14">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <v>1.0</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34774,20 +34776,20 @@
       <c r="A10" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="14">
         <v>20.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="14">
         <v>10.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>1.0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34797,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="25"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="11"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34814,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34829,12 +34831,12 @@
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34849,16 +34851,16 @@
       <c r="A14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>20.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>10.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34873,12 +34875,12 @@
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34890,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="25"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="11"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34907,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="11"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34925,22 +34927,22 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34951,15 +34953,15 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>5.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>15.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34977,13 +34979,13 @@
       <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>32.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -34998,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="25"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35014,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="s">
-        <v>24</v>
+      <c r="A22" s="13" t="s">
+        <v>22</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="17"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35033,18 +35035,18 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="14">
         <v>5.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="14">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35059,16 +35061,16 @@
       <c r="A24" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="14">
         <v>50.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="14">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="14">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35080,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,9 +35101,9 @@
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35115,15 +35117,15 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>5.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35141,9 +35143,9 @@
       <c r="A28" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35156,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="25"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35172,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="17"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35191,18 +35193,18 @@
     </row>
     <row r="31">
       <c r="A31" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="14">
         <v>5.0</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="14">
         <v>5.0</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="14">
         <v>1.0</v>
       </c>
-      <c r="E31" s="17"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35223,8 +35225,8 @@
       <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="34"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35236,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="16"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35252,15 +35254,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>10</v>
+      <c r="A34" s="9" t="s">
+        <v>14</v>
       </c>
-      <c r="B34" s="10" t="s">
-        <v>29</v>
+      <c r="B34" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="35">
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35274,17 +35276,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>8</v>
+      <c r="A35" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="9">
         <v>2.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="35">
+      <c r="D35" s="16"/>
+      <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35298,17 +35300,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>13</v>
+      <c r="A36" s="9" t="s">
+        <v>17</v>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="9">
         <v>20.0</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="35">
+      <c r="D36" s="16"/>
+      <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35322,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35338,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51130,10 +51132,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51155,11 +51157,11 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="9"/>
       <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -51174,13 +51176,13 @@
       <c r="A3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="12">
         <v>60.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="12">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
       <c r="E3" s="7"/>
@@ -51195,9 +51197,9 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
       <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -51210,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51229,18 +51231,18 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>60.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51254,9 +51256,9 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
       <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -51269,11 +51271,11 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
       <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -51286,18 +51288,18 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="9">
         <v>10.0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="9">
         <v>45.0</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="9">
         <v>1.0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="11">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51311,18 +51313,18 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>11.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>20.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="11">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51336,10 +51338,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51350,15 +51352,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>15</v>
+      <c r="A12" s="24" t="s">
+        <v>18</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>19</v>
+      <c r="B12" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51372,16 +51374,16 @@
       <c r="A13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>5.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>60.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="11">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51395,18 +51397,18 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>30.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51418,22 +51420,22 @@
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>4.0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>23</v>
+      <c r="F15" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51445,18 +51447,18 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>12.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <v>20.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="11">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51470,10 +51472,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51485,11 +51487,11 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
       <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -51502,18 +51504,18 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="12">
         <v>6.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="12">
         <v>45.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="11">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51529,16 +51531,16 @@
       <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="12">
         <v>18.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="12">
         <v>20.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51552,9 +51554,9 @@
     </row>
     <row r="21">
       <c r="A21" s="8"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
       <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -51566,15 +51568,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="s">
-        <v>16</v>
+      <c r="A22" s="24" t="s">
+        <v>11</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>19</v>
+      <c r="B22" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="12">
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="11">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51590,16 +51592,16 @@
       <c r="A23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="12">
         <v>6.0</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="12">
         <v>50.0</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="9">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="11">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51613,18 +51615,18 @@
     </row>
     <row r="24">
       <c r="A24" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="12">
         <v>8.0</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="12">
         <v>30.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="11">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51638,22 +51640,22 @@
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="12">
         <v>10.0</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="12">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <v>4.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>23</v>
+      <c r="F25" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51665,18 +51667,18 @@
     </row>
     <row r="26">
       <c r="A26" s="8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="12">
         <v>17.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="12">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="11">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51690,9 +51692,9 @@
     </row>
     <row r="27">
       <c r="A27" s="8"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
       <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -51704,14 +51706,14 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -51726,16 +51728,16 @@
       <c r="A29" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="12">
         <v>6.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="12">
         <v>50.0</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="9">
         <v>1.0</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="11">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51749,15 +51751,15 @@
     </row>
     <row r="30">
       <c r="A30" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="12">
         <v>8.0</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="12">
         <v>30.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
       <c r="E30" s="7"/>
@@ -51774,16 +51776,16 @@
       <c r="A31" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="12">
         <v>15.0</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="12">
         <v>10.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="9">
         <v>2.0</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="11">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51797,9 +51799,9 @@
     </row>
     <row r="32">
       <c r="A32" s="8"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
       <c r="E32" s="7"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -51811,13 +51813,13 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="s">
-        <v>21</v>
+      <c r="A33" s="13" t="s">
+        <v>19</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="26"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51829,15 +51831,15 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B34" s="32" t="s">
-        <v>27</v>
+      <c r="B34" s="35" t="s">
+        <v>28</v>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="35">
         <v>40.0</v>
       </c>
-      <c r="D34" s="32">
+      <c r="D34" s="35">
         <v>1.0</v>
       </c>
       <c r="E34" s="21">
@@ -51856,16 +51858,16 @@
       <c r="A35" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="32">
+      <c r="B35" s="35">
         <v>30.0</v>
       </c>
-      <c r="C35" s="32">
+      <c r="C35" s="35">
         <v>15.0</v>
       </c>
-      <c r="D35" s="32">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51876,10 +51878,10 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="25"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
       <c r="E36" s="7"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -51892,11 +51894,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
       <c r="E37" s="7"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -51911,16 +51913,16 @@
       <c r="A38" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>40.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>15.0</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="9">
         <v>1.0</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="11">
         <v>46203.63427946759</v>
       </c>
       <c r="F38" s="4"/>
@@ -51934,9 +51936,9 @@
     </row>
     <row r="39">
       <c r="A39" s="5"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
       <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51949,11 +51951,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
       <c r="E40" s="7"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -51966,18 +51968,18 @@
     </row>
     <row r="41">
       <c r="A41" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="9">
         <v>9.0</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="9">
         <v>20.0</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="9">
         <v>1.0</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="11">
         <v>46006.95620635417</v>
       </c>
       <c r="F41" s="4"/>
@@ -51993,16 +51995,16 @@
       <c r="A42" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="9">
         <v>55.0</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="9">
         <v>20.0</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="9">
         <v>1.0</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="11">
         <v>46006.95627618056</v>
       </c>
       <c r="F42" s="4"/>
@@ -52016,22 +52018,22 @@
     </row>
     <row r="43">
       <c r="A43" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="9">
         <v>10.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="9">
         <v>250.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F43" s="14" t="s">
-        <v>30</v>
+      <c r="F43" s="17" t="s">
+        <v>32</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -52042,10 +52044,10 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="37"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
       <c r="E44" s="7"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
@@ -52057,12 +52059,12 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="37" t="s">
+      <c r="A45" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
       <c r="E45" s="7"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -52077,16 +52079,16 @@
       <c r="A46" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="9">
         <v>60.0</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="9">
         <v>10.0</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="9">
         <v>1.0</v>
       </c>
-      <c r="E46" s="12">
+      <c r="E46" s="11">
         <v>46203.63265940972</v>
       </c>
       <c r="F46" s="4"/>
@@ -52099,10 +52101,10 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="37"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
+      <c r="A47" s="42"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
       <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52114,12 +52116,12 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="37" t="s">
+      <c r="A48" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
       <c r="E48" s="7"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
@@ -52132,18 +52134,18 @@
     </row>
     <row r="49">
       <c r="A49" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="12">
         <v>70.0</v>
       </c>
-      <c r="C49" s="9">
+      <c r="C49" s="12">
         <v>300.0</v>
       </c>
-      <c r="D49" s="9">
+      <c r="D49" s="12">
         <v>1.0</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="11">
         <v>46223.80899857639</v>
       </c>
       <c r="F49" s="4"/>
@@ -52157,18 +52159,18 @@
     </row>
     <row r="50">
       <c r="A50" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="12">
         <v>10.0</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="12">
         <v>20.0</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="12">
         <v>1.0</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="11">
         <v>46223.80911148148</v>
       </c>
       <c r="F50" s="4"/>
@@ -52184,16 +52186,16 @@
       <c r="A51" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="12">
         <v>70.0</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="12">
         <v>10.0</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="12">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="11">
         <v>46207.72572512731</v>
       </c>
       <c r="F51" s="4"/>
@@ -52207,9 +52209,9 @@
     </row>
     <row r="52">
       <c r="A52" s="8"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
       <c r="E52" s="7"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52224,12 +52226,12 @@
       <c r="A53" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="12">
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="11">
         <v>45946.87875708334</v>
       </c>
       <c r="F53" s="4"/>
@@ -52245,12 +52247,12 @@
       <c r="A54" s="8">
         <v>50.0</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B54" s="9">
         <v>100.0</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="12">
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="11">
         <v>45946.87887299768</v>
       </c>
       <c r="F54" s="4"/>
@@ -52280,16 +52282,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="41" t="s">
+      <c r="A56" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B56" s="41">
+      <c r="B56" s="40">
         <v>100.0</v>
       </c>
-      <c r="C56" s="14">
+      <c r="C56" s="17">
         <v>1.0</v>
       </c>
-      <c r="D56" s="14">
+      <c r="D56" s="17">
         <v>2.0</v>
       </c>
       <c r="E56" s="46">
@@ -52305,8 +52307,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="42"/>
-      <c r="B57" s="42"/>
+      <c r="A57" s="41"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
@@ -52320,10 +52322,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52340,13 +52342,13 @@
       <c r="A59" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B59" s="41">
+      <c r="B59" s="40">
         <v>50.0</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="17">
         <v>20.0</v>
       </c>
-      <c r="D59" s="14">
+      <c r="D59" s="17">
         <v>1.0</v>
       </c>
       <c r="E59" s="46">
@@ -52362,13 +52364,13 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="41" t="s">
+      <c r="A60" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="41">
+      <c r="B60" s="40">
         <v>15.0</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="17">
         <v>16.0</v>
       </c>
       <c r="D60" s="4"/>
@@ -52385,8 +52387,8 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="42"/>
-      <c r="B61" s="42"/>
+      <c r="A61" s="41"/>
+      <c r="B61" s="41"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
@@ -52400,10 +52402,10 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B62" s="41" t="s">
+      <c r="B62" s="40" t="s">
         <v>25</v>
       </c>
       <c r="C62" s="4"/>
@@ -52421,16 +52423,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B63" s="41">
+      <c r="B63" s="40">
         <v>5.0</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="17">
         <v>80.0</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="17">
         <v>1.0</v>
       </c>
       <c r="E63" s="46">
@@ -52446,16 +52448,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B64" s="41">
+      <c r="B64" s="40">
         <v>15.0</v>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="17">
         <v>10.0</v>
       </c>
-      <c r="D64" s="14">
+      <c r="D64" s="17">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52471,16 +52473,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="41" t="s">
-        <v>13</v>
+      <c r="A65" s="40" t="s">
+        <v>17</v>
       </c>
-      <c r="B65" s="41">
+      <c r="B65" s="40">
         <v>30.0</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="17">
         <v>10.0</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="17">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52496,8 +52498,8 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="42"/>
-      <c r="B66" s="42"/>
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -52511,10 +52513,10 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B67" s="41" t="s">
+      <c r="B67" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C67" s="4"/>
@@ -52532,16 +52534,16 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="40">
         <v>5.0</v>
       </c>
-      <c r="C68" s="14">
+      <c r="C68" s="17">
         <v>80.0</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="17">
         <v>1.0</v>
       </c>
       <c r="E68" s="4"/>
@@ -52555,16 +52557,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="40">
         <v>15.0</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="17">
         <v>10.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="17">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52578,16 +52580,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="41" t="s">
-        <v>13</v>
+      <c r="A70" s="40" t="s">
+        <v>17</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="40">
         <v>20.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="17">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="17">
         <v>6.0</v>
       </c>
       <c r="E70" s="46">
@@ -52603,8 +52605,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="42"/>
-      <c r="B71" s="42"/>
+      <c r="A71" s="41"/>
+      <c r="B71" s="41"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -52618,8 +52620,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="42"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52633,8 +52635,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="42"/>
-      <c r="B73" s="42"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-30T06:41:09.189Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,7 +19,13 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -34,16 +40,16 @@
     <t>0.3mm</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>Line</t>
   </si>
   <si>
-    <t>刀壓</t>
+    <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut-1/2</t>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>FILL</t>
   </si>
   <si>
     <t>(PS)</t>
@@ -52,28 +58,19 @@
     <t>0.5mm</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
     <t>A4紙</t>
   </si>
   <si>
     <t>03mm</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>0.3 mm</t>
+    <t>(PS -3)</t>
   </si>
   <si>
-    <t>1mm</t>
+    <t>0.3 mm</t>
   </si>
   <si>
     <t>Fill</t>
@@ -82,7 +79,7 @@
     <t>PS</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>1mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -91,25 +88,28 @@
     <t>Keep Detail</t>
   </si>
   <si>
+    <t>2mm</t>
+  </si>
+  <si>
     <t>3mm</t>
   </si>
   <si>
     <t>4mm</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -330,13 +330,16 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -345,10 +348,13 @@
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -357,45 +363,39 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -403,19 +403,13 @@
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -432,6 +426,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -685,16 +685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -708,7 +708,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -722,19 +722,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +748,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15"/>
+      <c r="B6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
-        <v>7</v>
+      <c r="A7" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="22">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="10"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>7</v>
+      <c r="A11" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,16 +920,16 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>7</v>
+      <c r="A12" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -944,16 +944,16 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
+      <c r="A14" s="26"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>22</v>
+      <c r="A15" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="15"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
-        <v>7</v>
+      <c r="A16" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="15"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1069,9 +1069,9 @@
       <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1084,16 +1084,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>7</v>
+      <c r="A20" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1108,12 +1108,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
+      <c r="A22" s="26"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="15"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
-        <v>7</v>
+      <c r="A24" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1193,8 +1193,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>27</v>
+      <c r="B27" s="8" t="s">
+        <v>28</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="34">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
-        <v>7</v>
+      <c r="A28" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="34">
+      <c r="D28" s="13"/>
+      <c r="E28" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>17</v>
+      <c r="A29" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="34">
+      <c r="D29" s="13"/>
+      <c r="E29" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17104,16 +17104,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17128,9 +17128,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,19 +17143,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,19 +17170,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
+      <c r="A5" s="7" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>7</v>
+      <c r="A6" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>11</v>
+      <c r="A9" s="14" t="s">
+        <v>13</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
-        <v>7</v>
+      <c r="A10" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="20">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="20">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>20</v>
+      <c r="A12" s="19" t="s">
+        <v>19</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,12 +17381,12 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>10</v>
+      <c r="A13" s="19" t="s">
+        <v>12</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
       <c r="E13" s="25"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -17400,16 +17400,16 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
-        <v>7</v>
+      <c r="A14" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
       <c r="E14" s="25"/>
@@ -17425,16 +17425,16 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
       <c r="E15" s="25"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="7"/>
+      <c r="A16" s="27"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>10</v>
+      <c r="B17" s="28" t="s">
+        <v>12</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17485,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="7"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17510,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="7"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,12 +17552,12 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>22</v>
+      <c r="A21" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
       <c r="E21" s="25"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -17571,16 +17571,16 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
-        <v>7</v>
+      <c r="A22" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
       <c r="E22" s="25"/>
@@ -17596,16 +17596,16 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
       <c r="E23" s="25"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="7"/>
+      <c r="A24" s="26"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17641,10 +17641,10 @@
       <c r="A25" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="7"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,19 +17657,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>7</v>
+      <c r="A26" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="7"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,19 +17682,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,12 +17726,12 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
       <c r="E29" s="25"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -17745,16 +17745,16 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
-        <v>7</v>
+      <c r="A30" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
       <c r="E30" s="25"/>
@@ -17782,7 +17782,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="36"/>
+      <c r="E31" s="32"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
-        <v>30</v>
+      <c r="A33" s="35" t="s">
+        <v>27</v>
       </c>
-      <c r="B33" s="38">
+      <c r="B33" s="36">
         <v>5.0</v>
       </c>
-      <c r="C33" s="38">
+      <c r="C33" s="36">
         <v>10.0</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="36">
         <v>2.0</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="37">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="40" t="s">
-        <v>31</v>
+      <c r="F33" s="38" t="s">
+        <v>29</v>
       </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="39"/>
+      <c r="K33" s="39"/>
+      <c r="L33" s="39"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="39"/>
+      <c r="O33" s="39"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>27</v>
+      <c r="B36" s="8" t="s">
+        <v>28</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
-        <v>7</v>
+      <c r="A37" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="8">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="16"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
-        <v>17</v>
+      <c r="A38" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="16"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34570,16 +34570,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -34607,19 +34607,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34633,19 +34633,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>12</v>
+      <c r="A4" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>10.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>2.0</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="11">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34659,19 +34659,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>20.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="8">
         <v>1.0</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34685,19 +34685,19 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>16</v>
+      <c r="A6" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>20.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34712,9 +34712,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34727,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="14" t="s">
+      <c r="A8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="15"/>
+      <c r="B8" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
-        <v>7</v>
+      <c r="A9" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="16">
         <v>4.0</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="16">
         <v>20.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <v>10.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="22">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="10"/>
+      <c r="A11" s="26"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34830,13 +34830,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>7</v>
+      <c r="A13" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34848,19 +34848,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>20.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>10.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34874,13 +34874,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>16</v>
+      <c r="A15" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="20"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34926,23 +34926,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>7</v>
+      <c r="A18" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,16 +34952,16 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>7</v>
+      <c r="A19" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>5.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>15.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34976,16 +34976,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>32.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="20"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
+      <c r="A21" s="26"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35016,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>22</v>
+      <c r="A22" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="15"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35034,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
-        <v>7</v>
+      <c r="A23" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="16">
         <v>5.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="15"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35058,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="16">
         <v>50.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
+      <c r="A25" s="26"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35101,9 +35101,9 @@
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35116,16 +35116,16 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>7</v>
+      <c r="A27" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>5.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35140,12 +35140,12 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="20"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35174,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="15"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35192,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="s">
-        <v>7</v>
+      <c r="A31" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="16">
         <v>5.0</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="16">
         <v>5.0</v>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="16">
         <v>1.0</v>
       </c>
-      <c r="E31" s="15"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35225,8 +35225,8 @@
       <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="34"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,15 +35254,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>27</v>
+      <c r="B34" s="8" t="s">
+        <v>28</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="34">
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="40">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35276,17 +35276,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
-        <v>7</v>
+      <c r="A35" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>2.0</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="16"/>
-      <c r="E35" s="34">
+      <c r="D35" s="13"/>
+      <c r="E35" s="40">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35300,17 +35300,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>17</v>
+      <c r="A36" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>20.0</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="8">
         <v>100.0</v>
       </c>
-      <c r="D36" s="16"/>
-      <c r="E36" s="34">
+      <c r="D36" s="13"/>
+      <c r="E36" s="40">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="16"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="16"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51156,13 +51156,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>7</v>
+      <c r="A2" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="7"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51173,19 +51173,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="10">
         <v>60.0</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="9"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="7"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51217,9 +51217,9 @@
       <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51230,19 +51230,19 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>17</v>
+      <c r="A6" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>60.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51256,10 +51256,10 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="7"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51273,10 +51273,10 @@
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="9"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51287,19 +51287,19 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>7</v>
+      <c r="A9" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>10.0</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="8">
         <v>45.0</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>1.0</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51312,19 +51312,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>17</v>
+      <c r="A10" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>11.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>20.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51338,10 +51338,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="5"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="21"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51352,15 +51352,15 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>21</v>
+      <c r="B12" s="24" t="s">
+        <v>20</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51371,19 +51371,19 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" ht="20.25" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>20</v>
+      <c r="A13" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>5.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>60.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51396,19 +51396,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>7</v>
+      <c r="A14" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>30.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51419,23 +51419,23 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>23</v>
+      <c r="A15" s="7" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <v>4.0</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="17" t="s">
-        <v>24</v>
+      <c r="F15" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51446,19 +51446,19 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>17</v>
+      <c r="A16" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>12.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>20.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>1.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51472,10 +51472,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="21"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51487,12 +51487,12 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="7"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51503,19 +51503,19 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>7</v>
+      <c r="A19" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="10">
         <v>6.0</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="10">
         <v>45.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51528,19 +51528,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="10">
         <v>18.0</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="10">
         <v>20.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51553,11 +51553,11 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="7"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51568,15 +51568,15 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="s">
-        <v>11</v>
+      <c r="A22" s="23" t="s">
+        <v>13</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>21</v>
+      <c r="B22" s="24" t="s">
+        <v>20</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="11">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51589,19 +51589,19 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>20</v>
+      <c r="A23" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="10">
         <v>6.0</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="10">
         <v>50.0</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="8">
         <v>1.0</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51614,19 +51614,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>7</v>
+      <c r="A24" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="10">
         <v>8.0</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="10">
         <v>30.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51639,23 +51639,23 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>17</v>
+      <c r="A25" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="10">
         <v>10.0</v>
       </c>
-      <c r="C25" s="12">
+      <c r="C25" s="10">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="8">
         <v>4.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="17" t="s">
-        <v>24</v>
+      <c r="F25" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51666,19 +51666,19 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>17</v>
+      <c r="A26" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="10">
         <v>17.0</v>
       </c>
-      <c r="C26" s="12">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51691,11 +51691,11 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="7"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51706,15 +51706,15 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" s="26" t="s">
+      <c r="A28" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="7"/>
+      <c r="B28" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51725,19 +51725,19 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>20</v>
+      <c r="A29" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="10">
         <v>6.0</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="10">
         <v>50.0</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="8">
         <v>1.0</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51750,19 +51750,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>7</v>
+      <c r="A30" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="10">
         <v>8.0</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="10">
         <v>30.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="7"/>
+      <c r="E30" s="9"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51773,19 +51773,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="10">
         <v>15.0</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="10">
         <v>10.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="8">
         <v>2.0</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51798,11 +51798,11 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="7"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="9"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51813,12 +51813,12 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="s">
-        <v>19</v>
+      <c r="A33" s="14" t="s">
+        <v>21</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
       <c r="E33" s="25"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51830,19 +51830,19 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="s">
-        <v>7</v>
+      <c r="A34" s="19" t="s">
+        <v>8</v>
       </c>
-      <c r="B34" s="35" t="s">
-        <v>28</v>
+      <c r="B34" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="41">
         <v>40.0</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="41">
         <v>1.0</v>
       </c>
-      <c r="E34" s="21">
+      <c r="E34" s="20">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51855,16 +51855,16 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="35">
+      <c r="B35" s="41">
         <v>30.0</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="41">
         <v>15.0</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
       <c r="E35" s="25"/>
@@ -51878,11 +51878,11 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="20"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="7"/>
+      <c r="A36" s="26"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="9"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51893,13 +51893,11 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="7"/>
+      <c r="A37" s="26"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51910,21 +51908,13 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>9</v>
+      <c r="A38" s="5" t="s">
+        <v>31</v>
       </c>
-      <c r="B38" s="9">
-        <v>40.0</v>
-      </c>
-      <c r="C38" s="9">
-        <v>15.0</v>
-      </c>
-      <c r="D38" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E38" s="11">
-        <v>46203.63427946759</v>
-      </c>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="9"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51935,11 +51925,21 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="7"/>
+      <c r="A39" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="8">
+        <v>40.0</v>
+      </c>
+      <c r="C39" s="8">
+        <v>15.0</v>
+      </c>
+      <c r="D39" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E39" s="12">
+        <v>46203.63427946759</v>
+      </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51950,13 +51950,11 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" s="16"/>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="7"/>
+      <c r="A40" s="5"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="9"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51967,21 +51965,13 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="s">
-        <v>7</v>
+      <c r="A41" s="5" t="s">
+        <v>24</v>
       </c>
-      <c r="B41" s="9">
-        <v>9.0</v>
-      </c>
-      <c r="C41" s="9">
-        <v>20.0</v>
-      </c>
-      <c r="D41" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E41" s="11">
-        <v>46006.95620635417</v>
-      </c>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="9"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51992,20 +51982,20 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="s">
-        <v>9</v>
+      <c r="A42" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B42" s="9">
-        <v>55.0</v>
+      <c r="B42" s="8">
+        <v>9.0</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="8">
         <v>20.0</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="8">
         <v>1.0</v>
       </c>
-      <c r="E42" s="11">
-        <v>46006.95627618056</v>
+      <c r="E42" s="12">
+        <v>46006.95620635417</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -52017,24 +52007,22 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
-        <v>7</v>
+      <c r="A43" s="7" t="s">
+        <v>9</v>
       </c>
-      <c r="B43" s="9">
-        <v>10.0</v>
+      <c r="B43" s="8">
+        <v>55.0</v>
       </c>
-      <c r="C43" s="9">
-        <v>250.0</v>
+      <c r="C43" s="8">
+        <v>20.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
-        <v>46038.439073761576</v>
+      <c r="E43" s="12">
+        <v>46006.95627618056</v>
       </c>
-      <c r="F43" s="17" t="s">
-        <v>32</v>
-      </c>
+      <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
@@ -52044,12 +52032,24 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="42"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="4"/>
+      <c r="A44" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B44" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C44" s="8">
+        <v>250.0</v>
+      </c>
+      <c r="D44" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E44" s="12">
+        <v>46038.439073761576</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>32</v>
+      </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
@@ -52059,13 +52059,11 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="7"/>
+      <c r="A45" s="42"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="9"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52076,21 +52074,13 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="s">
-        <v>9</v>
+      <c r="A46" s="42" t="s">
+        <v>26</v>
       </c>
-      <c r="B46" s="9">
-        <v>60.0</v>
-      </c>
-      <c r="C46" s="9">
-        <v>10.0</v>
-      </c>
-      <c r="D46" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E46" s="11">
-        <v>46203.63265940972</v>
-      </c>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="9"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52101,11 +52091,21 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="42"/>
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="7"/>
+      <c r="A47" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="C47" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="D47" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E47" s="12">
+        <v>46203.63265940972</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52116,13 +52116,11 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="B48" s="16"/>
-      <c r="C48" s="16"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="7"/>
+      <c r="A48" s="42"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52133,21 +52131,13 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="s">
-        <v>16</v>
+      <c r="A49" s="42" t="s">
+        <v>33</v>
       </c>
-      <c r="B49" s="12">
-        <v>70.0</v>
-      </c>
-      <c r="C49" s="12">
-        <v>300.0</v>
-      </c>
-      <c r="D49" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="E49" s="11">
-        <v>46223.80899857639</v>
-      </c>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="9"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52158,20 +52148,20 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="s">
-        <v>7</v>
+      <c r="A50" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B50" s="12">
-        <v>10.0</v>
+      <c r="B50" s="10">
+        <v>70.0</v>
       </c>
-      <c r="C50" s="12">
-        <v>20.0</v>
+      <c r="C50" s="10">
+        <v>300.0</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="10">
         <v>1.0</v>
       </c>
-      <c r="E50" s="11">
-        <v>46223.80911148148</v>
+      <c r="E50" s="12">
+        <v>46223.80899857639</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52183,20 +52173,20 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="s">
-        <v>9</v>
+      <c r="A51" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B51" s="12">
-        <v>70.0</v>
-      </c>
-      <c r="C51" s="12">
+      <c r="B51" s="10">
         <v>10.0</v>
       </c>
-      <c r="D51" s="12">
+      <c r="C51" s="10">
+        <v>20.0</v>
+      </c>
+      <c r="D51" s="10">
         <v>1.0</v>
       </c>
-      <c r="E51" s="11">
-        <v>46207.72572512731</v>
+      <c r="E51" s="12">
+        <v>46223.80911148148</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -52208,11 +52198,21 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="8"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="7"/>
+      <c r="A52" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="10">
+        <v>70.0</v>
+      </c>
+      <c r="C52" s="10">
+        <v>10.0</v>
+      </c>
+      <c r="D52" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E52" s="12">
+        <v>46207.72572512731</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52223,17 +52223,11 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="11">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="A53" s="7"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="9"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52244,16 +52238,16 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="8">
-        <v>50.0</v>
+      <c r="A54" s="7" t="s">
+        <v>34</v>
       </c>
-      <c r="B54" s="9">
-        <v>100.0</v>
+      <c r="B54" s="8" t="s">
+        <v>35</v>
       </c>
-      <c r="C54" s="16"/>
-      <c r="D54" s="16"/>
-      <c r="E54" s="11">
-        <v>45946.87887299768</v>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="12">
+        <v>45946.87875708334</v>
       </c>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52265,13 +52259,17 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="43" t="s">
-        <v>36</v>
+      <c r="A55" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B55" s="44"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="12">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52282,21 +52280,13 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="40" t="s">
-        <v>37</v>
+      <c r="A56" s="43" t="s">
+        <v>36</v>
       </c>
-      <c r="B56" s="40">
-        <v>100.0</v>
-      </c>
-      <c r="C56" s="17">
-        <v>1.0</v>
-      </c>
-      <c r="D56" s="17">
-        <v>2.0</v>
-      </c>
-      <c r="E56" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B56" s="44"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="44"/>
+      <c r="E56" s="45"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -52307,11 +52297,21 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="41"/>
-      <c r="B57" s="41"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="A57" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B57" s="38">
+        <v>100.0</v>
+      </c>
+      <c r="C57" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D57" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E57" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52322,10 +52322,8 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="41"/>
+      <c r="A58" s="39"/>
+      <c r="B58" s="39"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52339,21 +52337,13 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="s">
-        <v>9</v>
+      <c r="A59" s="38" t="s">
+        <v>38</v>
       </c>
-      <c r="B59" s="40">
-        <v>50.0</v>
-      </c>
-      <c r="C59" s="17">
-        <v>20.0</v>
-      </c>
-      <c r="D59" s="17">
-        <v>1.0</v>
-      </c>
-      <c r="E59" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B59" s="39"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52364,18 +52354,20 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="s">
-        <v>39</v>
+      <c r="A60" s="7" t="s">
+        <v>9</v>
       </c>
-      <c r="B60" s="40">
-        <v>15.0</v>
+      <c r="B60" s="38">
+        <v>50.0</v>
       </c>
-      <c r="C60" s="17">
-        <v>16.0</v>
+      <c r="C60" s="15">
+        <v>20.0</v>
       </c>
-      <c r="D60" s="4"/>
+      <c r="D60" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E60" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
@@ -52387,11 +52379,19 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="41"/>
-      <c r="B61" s="41"/>
-      <c r="C61" s="4"/>
+      <c r="A61" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B61" s="38">
+        <v>15.0</v>
+      </c>
+      <c r="C61" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
+      <c r="E61" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52402,17 +52402,11 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B62" s="40" t="s">
-        <v>25</v>
-      </c>
+      <c r="A62" s="39"/>
+      <c r="B62" s="39"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52423,20 +52417,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="s">
-        <v>41</v>
+      <c r="A63" s="38" t="s">
+        <v>40</v>
       </c>
-      <c r="B63" s="40">
-        <v>5.0</v>
+      <c r="B63" s="38" t="s">
+        <v>25</v>
       </c>
-      <c r="C63" s="17">
-        <v>80.0</v>
-      </c>
-      <c r="D63" s="17">
-        <v>1.0</v>
-      </c>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
       <c r="E63" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
@@ -52448,20 +52438,20 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
-        <v>42</v>
+      <c r="A64" s="38" t="s">
+        <v>41</v>
       </c>
-      <c r="B64" s="40">
-        <v>15.0</v>
+      <c r="B64" s="38">
+        <v>5.0</v>
       </c>
-      <c r="C64" s="17">
-        <v>10.0</v>
+      <c r="C64" s="15">
+        <v>80.0</v>
       </c>
-      <c r="D64" s="17">
+      <c r="D64" s="15">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
@@ -52473,20 +52463,20 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="40" t="s">
-        <v>17</v>
+      <c r="A65" s="38" t="s">
+        <v>42</v>
       </c>
-      <c r="B65" s="40">
-        <v>30.0</v>
+      <c r="B65" s="38">
+        <v>15.0</v>
       </c>
-      <c r="C65" s="17">
+      <c r="C65" s="15">
         <v>10.0</v>
       </c>
-      <c r="D65" s="17">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -52498,11 +52488,21 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="41"/>
-      <c r="B66" s="41"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="A66" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="B66" s="38">
+        <v>30.0</v>
+      </c>
+      <c r="C66" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D66" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E66" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52513,17 +52513,11 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B67" s="40" t="s">
-        <v>33</v>
-      </c>
+      <c r="A67" s="39"/>
+      <c r="B67" s="39"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52534,19 +52528,17 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
-        <v>41</v>
+      <c r="A68" s="38" t="s">
+        <v>40</v>
       </c>
-      <c r="B68" s="40">
-        <v>5.0</v>
+      <c r="B68" s="38" t="s">
+        <v>33</v>
       </c>
-      <c r="C68" s="17">
-        <v>80.0</v>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D68" s="17">
-        <v>1.0</v>
-      </c>
-      <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -52557,16 +52549,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
-        <v>42</v>
+      <c r="A69" s="38" t="s">
+        <v>41</v>
       </c>
-      <c r="B69" s="40">
-        <v>15.0</v>
+      <c r="B69" s="38">
+        <v>5.0</v>
       </c>
-      <c r="C69" s="17">
-        <v>10.0</v>
+      <c r="C69" s="15">
+        <v>80.0</v>
       </c>
-      <c r="D69" s="17">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52580,21 +52572,19 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
-        <v>17</v>
+      <c r="A70" s="38" t="s">
+        <v>42</v>
       </c>
-      <c r="B70" s="40">
-        <v>20.0</v>
+      <c r="B70" s="38">
+        <v>15.0</v>
       </c>
-      <c r="C70" s="17">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="17">
-        <v>6.0</v>
+      <c r="D70" s="15">
+        <v>1.0</v>
       </c>
-      <c r="E70" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E70" s="4"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -52605,11 +52595,21 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="41"/>
-      <c r="B71" s="41"/>
-      <c r="C71" s="4"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="A71" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="B71" s="38">
+        <v>20.0</v>
+      </c>
+      <c r="C71" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D71" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E71" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -52620,8 +52620,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="41"/>
+      <c r="A72" s="39"/>
+      <c r="B72" s="39"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52635,8 +52635,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="41"/>
-      <c r="B73" s="41"/>
+      <c r="A73" s="38"/>
+      <c r="B73" s="39"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -52650,8 +52650,8 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="4"/>
-      <c r="B74" s="4"/>
+      <c r="A74" s="39"/>
+      <c r="B74" s="39"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
@@ -66719,6 +66719,21 @@
       <c r="L1011" s="4"/>
       <c r="M1011" s="4"/>
     </row>
+    <row r="1012">
+      <c r="A1012" s="4"/>
+      <c r="B1012" s="4"/>
+      <c r="C1012" s="4"/>
+      <c r="D1012" s="4"/>
+      <c r="E1012" s="4"/>
+      <c r="F1012" s="4"/>
+      <c r="G1012" s="4"/>
+      <c r="H1012" s="4"/>
+      <c r="I1012" s="4"/>
+      <c r="J1012" s="4"/>
+      <c r="K1012" s="4"/>
+      <c r="L1012" s="4"/>
+      <c r="M1012" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-30T06:41:17.317Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="43">
   <si>
     <t>項目</t>
   </si>
@@ -25,9 +25,6 @@
     <t>功率</t>
   </si>
   <si>
-    <t>刀壓</t>
-  </si>
-  <si>
     <t>速度</t>
   </si>
   <si>
@@ -35,6 +32,9 @@
   </si>
   <si>
     <t>最後更新日期</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>0.3mm</t>
@@ -49,28 +49,28 @@
     <t>Cut(detail)</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
     <t>A4紙</t>
   </si>
   <si>
     <t>03mm</t>
   </si>
   <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>(PS -3)</t>
+    <t>(PS)</t>
   </si>
   <si>
     <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>Fill</t>
@@ -82,13 +82,13 @@
     <t>1mm</t>
   </si>
   <si>
+    <t>2mm</t>
+  </si>
+  <si>
     <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
-  </si>
-  <si>
-    <t>2mm</t>
   </si>
   <si>
     <t>3mm</t>
@@ -97,16 +97,16 @@
     <t>4mm</t>
   </si>
   <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>６</t>
+  </si>
+  <si>
     <t>甲板紙</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -333,28 +333,25 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -363,16 +360,19 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -381,21 +381,21 @@
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -403,14 +403,20 @@
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -426,12 +432,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -688,13 +688,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -725,13 +725,13 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -751,13 +751,13 @@
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
       <c r="E4" s="11"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -791,12 +791,12 @@
       <c r="A6" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>17</v>
+      <c r="B6" s="15" t="s">
+        <v>18</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -811,20 +811,20 @@
       <c r="A7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
       <c r="E7" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -837,20 +837,20 @@
       <c r="A8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
       <c r="E8" s="22">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,10 +860,10 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="26"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
       <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -879,9 +879,9 @@
       <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="8"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="9"/>
       <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -897,20 +897,20 @@
       <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
       <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -923,13 +923,13 @@
       <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -947,13 +947,13 @@
       <c r="A13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="26"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -985,12 +985,12 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1005,16 +1005,16 @@
       <c r="A16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1029,16 +1029,16 @@
       <c r="A17" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="26"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1069,9 +1069,9 @@
       <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1087,13 +1087,13 @@
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1111,9 +1111,9 @@
       <c r="A21" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="26"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1145,10 +1145,10 @@
       <c r="A23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1163,16 +1163,16 @@
       <c r="A24" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1193,8 +1193,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="33"/>
-      <c r="E25" s="34"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>14</v>
+      <c r="A27" s="9" t="s">
+        <v>11</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>28</v>
+      <c r="B27" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="40">
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="40">
+      <c r="D28" s="12"/>
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>16</v>
+      <c r="A29" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="40">
+      <c r="D29" s="12"/>
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17107,13 +17107,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17146,16 +17146,16 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="13">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17173,16 +17173,16 @@
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17196,12 +17196,12 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17217,19 +17217,19 @@
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17242,19 +17242,19 @@
       <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="13"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17284,10 +17284,10 @@
       <c r="A9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17303,16 +17303,16 @@
       <c r="A10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17330,16 +17330,16 @@
       <c r="A11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17357,16 +17357,16 @@
       <c r="A12" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="25"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17403,16 +17403,16 @@
       <c r="A14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17428,16 +17428,16 @@
       <c r="A15" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
-      <c r="E16" s="9"/>
+      <c r="A16" s="28"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17467,12 +17467,12 @@
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="28" t="s">
-        <v>12</v>
+      <c r="B17" s="29" t="s">
+        <v>16</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17488,16 +17488,16 @@
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17513,16 +17513,16 @@
       <c r="A19" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="26"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="9"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17553,12 +17553,12 @@
     </row>
     <row r="21">
       <c r="A21" s="14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="25"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17574,16 +17574,16 @@
       <c r="A22" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="25"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17599,16 +17599,16 @@
       <c r="A23" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="25"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="26"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="9"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17641,10 +17641,10 @@
       <c r="A25" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17660,16 +17660,16 @@
       <c r="A26" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="9"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17685,16 +17685,16 @@
       <c r="A27" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="13">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="26"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17729,10 +17729,10 @@
       <c r="A29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="25"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17748,16 +17748,16 @@
       <c r="A30" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="25"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17782,7 +17782,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="35"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="35" t="s">
-        <v>27</v>
+      <c r="A33" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="36">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="37">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="38" t="s">
-        <v>29</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
-      <c r="K33" s="39"/>
-      <c r="L33" s="39"/>
-      <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
-      <c r="O33" s="39"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>14</v>
+      <c r="A36" s="9" t="s">
+        <v>11</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>28</v>
+      <c r="B36" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="12"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>16</v>
+      <c r="A38" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="12"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34573,13 +34573,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34610,13 +34610,13 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -34636,13 +34636,13 @@
       <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>10.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
       <c r="E4" s="11">
@@ -34662,13 +34662,13 @@
       <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>20.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
       <c r="E5" s="11">
@@ -34686,15 +34686,15 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>20.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
       <c r="E6" s="11">
@@ -34712,9 +34712,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34730,12 +34730,12 @@
       <c r="A8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>17</v>
+      <c r="B8" s="15" t="s">
+        <v>18</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34750,20 +34750,20 @@
       <c r="A9" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
       <c r="E9" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34776,20 +34776,20 @@
       <c r="A10" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>20.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>10.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
       <c r="E10" s="22">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,10 +34799,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="26"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
       <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34833,9 +34833,9 @@
       <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
       <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -34851,13 +34851,13 @@
       <c r="A14" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>20.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>10.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
       <c r="E14" s="11">
@@ -34875,11 +34875,11 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
       <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -34892,10 +34892,10 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="26"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34911,9 +34911,9 @@
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="8"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="9"/>
       <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -34929,20 +34929,20 @@
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
       <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34955,13 +34955,13 @@
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>5.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="9">
         <v>15.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34979,13 +34979,13 @@
       <c r="A20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>32.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="26"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35017,12 +35017,12 @@
     </row>
     <row r="22">
       <c r="A22" s="14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="17"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35037,16 +35037,16 @@
       <c r="A23" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>5.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35061,16 +35061,16 @@
       <c r="A24" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>50.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="26"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35101,9 +35101,9 @@
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35119,13 +35119,13 @@
       <c r="A27" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>5.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35143,9 +35143,9 @@
       <c r="A28" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="26"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35177,10 +35177,10 @@
       <c r="A30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="17"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35195,16 +35195,16 @@
       <c r="A31" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="15">
         <v>5.0</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="15">
         <v>5.0</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="15">
         <v>1.0</v>
       </c>
-      <c r="E31" s="17"/>
+      <c r="E31" s="16"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35225,8 +35225,8 @@
       <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="34"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,15 +35254,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>14</v>
+      <c r="A34" s="9" t="s">
+        <v>11</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>28</v>
+      <c r="B34" s="9" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="40">
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35276,17 +35276,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="9">
         <v>2.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="40">
+      <c r="D35" s="12"/>
+      <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35300,17 +35300,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>16</v>
+      <c r="A36" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="9">
         <v>20.0</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="40">
+      <c r="D36" s="12"/>
+      <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51135,16 +51135,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51159,10 +51159,10 @@
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51176,16 +51176,16 @@
       <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>60.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="9"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="13"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51231,18 +51231,18 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>60.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="13">
         <v>46156.860351111114</v>
       </c>
       <c r="F6" s="4"/>
@@ -51256,10 +51256,10 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="9"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -51271,12 +51271,12 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51290,16 +51290,16 @@
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <v>10.0</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <v>45.0</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <v>1.0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="13">
         <v>46106.73232292824</v>
       </c>
       <c r="F9" s="4"/>
@@ -51313,18 +51313,18 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <v>11.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="9">
         <v>20.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <v>46106.732369062505</v>
       </c>
       <c r="F10" s="4"/>
@@ -51341,7 +51341,7 @@
       <c r="B11" s="18"/>
       <c r="C11" s="18"/>
       <c r="D11" s="18"/>
-      <c r="E11" s="21"/>
+      <c r="E11" s="20"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -51353,14 +51353,14 @@
     </row>
     <row r="12">
       <c r="A12" s="23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="13"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51374,16 +51374,16 @@
       <c r="A13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>5.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>60.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="13">
         <v>46160.881155752315</v>
       </c>
       <c r="F13" s="4"/>
@@ -51399,16 +51399,16 @@
       <c r="A14" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>30.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12"/>
+      <c r="E14" s="13"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -51420,22 +51420,22 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="9">
         <v>4.0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="13">
         <v>46160.85381630787</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>23</v>
+      <c r="F15" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51447,18 +51447,18 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="9">
         <v>12.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="9">
         <v>20.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="9">
         <v>1.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="13">
         <v>46158.840069502316</v>
       </c>
       <c r="F16" s="4"/>
@@ -51475,7 +51475,7 @@
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
       <c r="D17" s="18"/>
-      <c r="E17" s="21"/>
+      <c r="E17" s="20"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -51489,10 +51489,10 @@
       <c r="A18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51506,16 +51506,16 @@
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="8">
         <v>6.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>45.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <v>46203.65718435185</v>
       </c>
       <c r="F19" s="4"/>
@@ -51531,16 +51531,16 @@
       <c r="A20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>18.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>20.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <v>46155.874796793985</v>
       </c>
       <c r="F20" s="4"/>
@@ -51554,10 +51554,10 @@
     </row>
     <row r="21">
       <c r="A21" s="7"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -51571,12 +51571,12 @@
       <c r="A22" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="12">
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="13">
         <v>46155.850816817125</v>
       </c>
       <c r="F22" s="4"/>
@@ -51592,16 +51592,16 @@
       <c r="A23" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="8">
         <v>6.0</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="8">
         <v>50.0</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="9">
         <v>1.0</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="13">
         <v>46155.86764509259</v>
       </c>
       <c r="F23" s="4"/>
@@ -51617,16 +51617,16 @@
       <c r="A24" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="8">
         <v>8.0</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <v>30.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="13">
         <v>46155.86212506944</v>
       </c>
       <c r="F24" s="4"/>
@@ -51640,22 +51640,22 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="8">
         <v>10.0</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="9">
         <v>4.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="13">
         <v>46156.84678416667</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>23</v>
+      <c r="F25" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -51667,18 +51667,18 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>17.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="13">
         <v>46155.877253784725</v>
       </c>
       <c r="F26" s="4"/>
@@ -51692,10 +51692,10 @@
     </row>
     <row r="27">
       <c r="A27" s="7"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="10"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -51709,12 +51709,12 @@
       <c r="A28" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51728,16 +51728,16 @@
       <c r="A29" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="8">
         <v>6.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="8">
         <v>50.0</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="9">
         <v>1.0</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <v>46155.89164559028</v>
       </c>
       <c r="F29" s="4"/>
@@ -51753,16 +51753,16 @@
       <c r="A30" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="8">
         <v>8.0</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="8">
         <v>30.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -51776,16 +51776,16 @@
       <c r="A31" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="10">
+      <c r="B31" s="8">
         <v>15.0</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31" s="8">
         <v>10.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="9">
         <v>2.0</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="13">
         <v>46176.957761134254</v>
       </c>
       <c r="F31" s="4"/>
@@ -51799,10 +51799,10 @@
     </row>
     <row r="32">
       <c r="A32" s="7"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="9"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="10"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -51816,10 +51816,10 @@
       <c r="A33" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="25"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51833,16 +51833,16 @@
       <c r="A34" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B34" s="41" t="s">
-        <v>30</v>
+      <c r="B34" s="36" t="s">
+        <v>28</v>
       </c>
-      <c r="C34" s="41">
+      <c r="C34" s="36">
         <v>40.0</v>
       </c>
-      <c r="D34" s="41">
+      <c r="D34" s="36">
         <v>1.0</v>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F34" s="4"/>
@@ -51858,16 +51858,16 @@
       <c r="A35" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="36">
         <v>30.0</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="36">
         <v>15.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="36">
         <v>1.0</v>
       </c>
-      <c r="E35" s="25"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -51878,11 +51878,13 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="26"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="9"/>
+      <c r="A36" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="10"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51893,11 +51895,11 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="26"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="9"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="10"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -51911,10 +51913,10 @@
       <c r="A38" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="9"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="10"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51928,16 +51930,16 @@
       <c r="A39" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="9">
         <v>40.0</v>
       </c>
-      <c r="C39" s="8">
+      <c r="C39" s="9">
         <v>15.0</v>
       </c>
-      <c r="D39" s="8">
+      <c r="D39" s="9">
         <v>1.0</v>
       </c>
-      <c r="E39" s="12">
+      <c r="E39" s="13">
         <v>46203.63427946759</v>
       </c>
       <c r="F39" s="4"/>
@@ -51951,10 +51953,10 @@
     </row>
     <row r="40">
       <c r="A40" s="5"/>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="9"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="10"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -51966,12 +51968,12 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="9"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="10"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51985,16 +51987,16 @@
       <c r="A42" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="9">
         <v>9.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="9">
         <v>20.0</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="9">
         <v>1.0</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="13">
         <v>46006.95620635417</v>
       </c>
       <c r="F42" s="4"/>
@@ -52010,16 +52012,16 @@
       <c r="A43" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>55.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="9">
         <v>20.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="13">
         <v>46006.95627618056</v>
       </c>
       <c r="F43" s="4"/>
@@ -52035,19 +52037,19 @@
       <c r="A44" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="9">
         <v>10.0</v>
       </c>
-      <c r="C44" s="8">
+      <c r="C44" s="9">
         <v>250.0</v>
       </c>
-      <c r="D44" s="8">
+      <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="13">
         <v>46038.439073761576</v>
       </c>
-      <c r="F44" s="15" t="s">
+      <c r="F44" s="17" t="s">
         <v>32</v>
       </c>
       <c r="G44" s="4"/>
@@ -52060,10 +52062,10 @@
     </row>
     <row r="45">
       <c r="A45" s="42"/>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="9"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="10"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52077,10 +52079,10 @@
       <c r="A46" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="9"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="10"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52094,16 +52096,16 @@
       <c r="A47" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B47" s="8">
+      <c r="B47" s="9">
         <v>60.0</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="9">
         <v>10.0</v>
       </c>
-      <c r="D47" s="8">
+      <c r="D47" s="9">
         <v>1.0</v>
       </c>
-      <c r="E47" s="12">
+      <c r="E47" s="13">
         <v>46203.63265940972</v>
       </c>
       <c r="F47" s="4"/>
@@ -52117,10 +52119,10 @@
     </row>
     <row r="48">
       <c r="A48" s="42"/>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="9"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="10"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -52134,10 +52136,10 @@
       <c r="A49" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="9"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="10"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52149,18 +52151,18 @@
     </row>
     <row r="50">
       <c r="A50" s="7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
-      <c r="B50" s="10">
+      <c r="B50" s="8">
         <v>70.0</v>
       </c>
-      <c r="C50" s="10">
+      <c r="C50" s="8">
         <v>300.0</v>
       </c>
-      <c r="D50" s="10">
+      <c r="D50" s="8">
         <v>1.0</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="13">
         <v>46223.80899857639</v>
       </c>
       <c r="F50" s="4"/>
@@ -52176,16 +52178,16 @@
       <c r="A51" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="8">
         <v>10.0</v>
       </c>
-      <c r="C51" s="10">
+      <c r="C51" s="8">
         <v>20.0</v>
       </c>
-      <c r="D51" s="10">
+      <c r="D51" s="8">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="13">
         <v>46223.80911148148</v>
       </c>
       <c r="F51" s="4"/>
@@ -52201,16 +52203,16 @@
       <c r="A52" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="8">
         <v>70.0</v>
       </c>
-      <c r="C52" s="10">
+      <c r="C52" s="8">
         <v>10.0</v>
       </c>
-      <c r="D52" s="10">
+      <c r="D52" s="8">
         <v>1.0</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="13">
         <v>46207.72572512731</v>
       </c>
       <c r="F52" s="4"/>
@@ -52224,10 +52226,10 @@
     </row>
     <row r="53">
       <c r="A53" s="7"/>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="9"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="10"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52241,12 +52243,12 @@
       <c r="A54" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="12">
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="13">
         <v>45946.87875708334</v>
       </c>
       <c r="F54" s="4"/>
@@ -52262,12 +52264,12 @@
       <c r="A55" s="7">
         <v>50.0</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="9">
         <v>100.0</v>
       </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="12">
+      <c r="C55" s="12"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="13">
         <v>45946.87887299768</v>
       </c>
       <c r="F55" s="4"/>
@@ -52297,16 +52299,16 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="38" t="s">
+      <c r="A57" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="38">
+      <c r="B57" s="40">
         <v>100.0</v>
       </c>
-      <c r="C57" s="15">
+      <c r="C57" s="17">
         <v>1.0</v>
       </c>
-      <c r="D57" s="15">
+      <c r="D57" s="17">
         <v>2.0</v>
       </c>
       <c r="E57" s="46">
@@ -52322,8 +52324,8 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="39"/>
-      <c r="B58" s="39"/>
+      <c r="A58" s="41"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
@@ -52337,10 +52339,10 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="38" t="s">
+      <c r="A59" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B59" s="39"/>
+      <c r="B59" s="41"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
@@ -52357,13 +52359,13 @@
       <c r="A60" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B60" s="38">
+      <c r="B60" s="40">
         <v>50.0</v>
       </c>
-      <c r="C60" s="15">
+      <c r="C60" s="17">
         <v>20.0</v>
       </c>
-      <c r="D60" s="15">
+      <c r="D60" s="17">
         <v>1.0</v>
       </c>
       <c r="E60" s="46">
@@ -52379,13 +52381,13 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="38" t="s">
+      <c r="A61" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B61" s="38">
+      <c r="B61" s="40">
         <v>15.0</v>
       </c>
-      <c r="C61" s="15">
+      <c r="C61" s="17">
         <v>16.0</v>
       </c>
       <c r="D61" s="4"/>
@@ -52402,8 +52404,8 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="39"/>
-      <c r="B62" s="39"/>
+      <c r="A62" s="41"/>
+      <c r="B62" s="41"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
@@ -52417,10 +52419,10 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="38" t="s">
+      <c r="A63" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B63" s="38" t="s">
+      <c r="B63" s="40" t="s">
         <v>25</v>
       </c>
       <c r="C63" s="4"/>
@@ -52438,16 +52440,16 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="38" t="s">
+      <c r="A64" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="38">
+      <c r="B64" s="40">
         <v>5.0</v>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="17">
         <v>80.0</v>
       </c>
-      <c r="D64" s="15">
+      <c r="D64" s="17">
         <v>1.0</v>
       </c>
       <c r="E64" s="46">
@@ -52463,16 +52465,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="38" t="s">
+      <c r="A65" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B65" s="38">
+      <c r="B65" s="40">
         <v>15.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="17">
         <v>10.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="17">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52488,16 +52490,16 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="38" t="s">
-        <v>16</v>
+      <c r="A66" s="40" t="s">
+        <v>15</v>
       </c>
-      <c r="B66" s="38">
+      <c r="B66" s="40">
         <v>30.0</v>
       </c>
-      <c r="C66" s="15">
+      <c r="C66" s="17">
         <v>10.0</v>
       </c>
-      <c r="D66" s="15">
+      <c r="D66" s="17">
         <v>1.0</v>
       </c>
       <c r="E66" s="46">
@@ -52513,8 +52515,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="39"/>
-      <c r="B67" s="39"/>
+      <c r="A67" s="41"/>
+      <c r="B67" s="41"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -52528,10 +52530,10 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="38" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="38" t="s">
+      <c r="B68" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C68" s="4"/>
@@ -52549,16 +52551,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="38" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="38">
+      <c r="B69" s="40">
         <v>5.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="17">
         <v>80.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="17">
         <v>1.0</v>
       </c>
       <c r="E69" s="4"/>
@@ -52572,16 +52574,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="38" t="s">
+      <c r="A70" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="38">
+      <c r="B70" s="40">
         <v>15.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="17">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="17">
         <v>1.0</v>
       </c>
       <c r="E70" s="4"/>
@@ -52595,16 +52597,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="38" t="s">
-        <v>16</v>
+      <c r="A71" s="40" t="s">
+        <v>15</v>
       </c>
-      <c r="B71" s="38">
+      <c r="B71" s="40">
         <v>20.0</v>
       </c>
-      <c r="C71" s="15">
+      <c r="C71" s="17">
         <v>10.0</v>
       </c>
-      <c r="D71" s="15">
+      <c r="D71" s="17">
         <v>6.0</v>
       </c>
       <c r="E71" s="46">
@@ -52620,8 +52622,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="39"/>
-      <c r="B72" s="39"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52635,8 +52637,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="38"/>
-      <c r="B73" s="39"/>
+      <c r="A73" s="40"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -52650,8 +52652,8 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="39"/>
-      <c r="B74" s="39"/>
+      <c r="A74" s="41"/>
+      <c r="B74" s="41"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-07-30T06:41:21.779Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -46,28 +46,28 @@
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
     <t>A4紙</t>
   </si>
   <si>
     <t>03mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
+    <t>(PS)</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>Cut(detail)</t>
   </si>
   <si>
     <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>FILL</t>
   </si>
   <si>
     <t>(PS -3)</t>
@@ -82,13 +82,13 @@
     <t>1mm</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
     <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
+  </si>
+  <si>
+    <t>2mm</t>
   </si>
   <si>
     <t>3mm</t>
@@ -100,16 +100,16 @@
     <t>(0.9 Power)</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>６</t>
   </si>
   <si>
-    <t>甲板紙</t>
+    <t>1.5mm</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>1.5mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -327,9 +327,6 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -342,13 +339,19 @@
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -360,42 +363,39 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -409,16 +409,16 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -710,7 +710,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -722,19 +722,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="13">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +748,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="13"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,10 +773,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="6"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>13</v>
+      <c r="A6" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -811,20 +811,20 @@
       <c r="A7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
       <c r="E7" s="22">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -837,20 +837,20 @@
       <c r="A8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
       <c r="E8" s="22">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="24"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="8"/>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
-      <c r="E9" s="11"/>
+      <c r="E9" s="13"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -881,8 +881,8 @@
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="11"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="13"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="13">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,19 +920,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -944,19 +944,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -968,11 +968,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="24"/>
+      <c r="A14" s="26"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
-      <c r="E14" s="6"/>
+      <c r="E14" s="10"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
-        <v>22</v>
+      <c r="A15" s="15" t="s">
+        <v>24</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1005,16 +1005,16 @@
       <c r="A16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1029,16 +1029,16 @@
       <c r="A17" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,11 +1050,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="24"/>
+      <c r="A18" s="26"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
-      <c r="E18" s="6"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1072,7 +1072,7 @@
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
-      <c r="E19" s="6"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1084,19 +1084,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1108,13 +1108,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
-      <c r="E21" s="6"/>
+      <c r="E21" s="10"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1126,11 +1126,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="24"/>
+      <c r="A22" s="26"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
-      <c r="E22" s="6"/>
+      <c r="E22" s="10"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1163,16 +1163,16 @@
       <c r="A24" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>11</v>
+      <c r="A27" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
-      <c r="E27" s="34">
+      <c r="E27" s="35">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="34">
+      <c r="E28" s="35">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>15</v>
+      <c r="A29" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
       <c r="D29" s="12"/>
-      <c r="E29" s="34">
+      <c r="E29" s="35">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,19 +17143,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,19 +17170,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>16</v>
+      <c r="A5" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="13"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>13</v>
+      <c r="A9" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17303,16 +17303,16 @@
       <c r="A10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="20">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17330,16 +17330,16 @@
       <c r="A11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="20">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17357,16 +17357,16 @@
       <c r="A12" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="23"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17403,16 +17403,16 @@
       <c r="A14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="23"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17428,16 +17428,16 @@
       <c r="A15" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="23"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="25"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17467,12 +17467,12 @@
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>16</v>
+      <c r="B17" s="28" t="s">
+        <v>12</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17485,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17510,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="24"/>
+      <c r="A20" s="26"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
-        <v>22</v>
+      <c r="A21" s="15" t="s">
+        <v>24</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="23"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17574,16 +17574,16 @@
       <c r="A22" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="23"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17599,16 +17599,16 @@
       <c r="A23" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C2